<commit_message>
fix(content): compose sky sign manifestations per unit
</commit_message>
<xml_diff>
--- a/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
+++ b/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2db42b0020f44a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="2" r:id="Rbffb474424db407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="3" r:id="R06881f7e0ea64581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="4" r:id="R82c351eb656b470b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="5" r:id="R5f112ff2d0294121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="6" r:id="R91995762d21a4ba2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="7" r:id="Rbdc1761f8d334e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcb49b968d3c246f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="2" r:id="Rcb9a994ffb3542e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="3" r:id="Rf2b3a4ee349d41e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="4" r:id="Rb4f3ffe799874882"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="5" r:id="R1adc9a1a678244b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="6" r:id="Rbec700f027334673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="7" r:id="Ra540c8d73f644231"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1020,9 +1020,9 @@
         <x:v>individual visibility depends on who moves first and claims the work</x:v>
       </x:c>
       <x:c r="E4" s="44" t="str">
-        <x:v>• individual credit being claimed before others agree
-• pressure to move first on visible contribution
-• delay around who represents the group being treated as lost control</x:v>
+        <x:v>• credit claimed before anyone agrees the work is finished
+• the person who starts the project becoming its public face
+• recognition following the first visible move rather than the longest contribution</x:v>
       </x:c>
       <x:c r="F4" s="44" t="str">
         <x:v>first moves and claimed visibility</x:v>
@@ -1054,9 +1054,9 @@
         <x:v>recognition is measured against tangible value and staying power</x:v>
       </x:c>
       <x:c r="E5" s="45" t="str">
-        <x:v>• individual credit measured against cost and durability
-• visible contribution slowed by what must be preserved
-• who represents the group judged by whether it can be maintained</x:v>
+        <x:v>• a contribution valued because it keeps producing something useful
+• recognition arriving only after the result proves it can last
+• public credit tied to who protected the budget or the material</x:v>
       </x:c>
       <x:c r="F5" s="45" t="str">
         <x:v>recognition tied to material worth and durability</x:v>
@@ -1088,9 +1088,9 @@
         <x:v>visibility shifts with who explains, compares, or names the contribution</x:v>
       </x:c>
       <x:c r="E6" s="45" t="str">
-        <x:v>• new information changing individual credit
-• several explanations competing around visible contribution
-• who represents the group being revised as the terms move</x:v>
+        <x:v>• the clearest explanation deciding who is seen as responsible
+• credit moving when a new version of the story circulates
+• several people making a plausible claim to the same idea</x:v>
       </x:c>
       <x:c r="F6" s="45" t="str">
         <x:v>credit shaped by language and comparison</x:v>
@@ -1122,9 +1122,9 @@
         <x:v>recognition is tied to care, belonging, and private loyalties</x:v>
       </x:c>
       <x:c r="E7" s="45" t="str">
-        <x:v>• care and belonging changing the handling of individual credit
-• private consequences shaping visible contribution
-• protection taking priority in decisions about who represents the group</x:v>
+        <x:v>• care work becoming the contribution everyone depends on
+• private loyalty shaping who receives public acknowledgment
+• someone representing the group because they remember its history</x:v>
       </x:c>
       <x:c r="F7" s="45" t="str">
         <x:v>recognition tied to care and private loyalty</x:v>
@@ -1190,9 +1190,9 @@
         <x:v>contribution is judged by usefulness, precision, and what gets corrected</x:v>
       </x:c>
       <x:c r="E9" s="45" t="str">
-        <x:v>• individual credit tested against the details
-• a correction changing visible contribution
-• usefulness becoming the measure of who represents the group</x:v>
+        <x:v>• the person who catches the error receiving the authority to fix it
+• useful work being noticed after a small failure exposes its value
+• recognition depending on precision rather than display</x:v>
       </x:c>
       <x:c r="F9" s="45" t="str">
         <x:v>useful contribution, precision, and correction</x:v>
@@ -1224,9 +1224,9 @@
         <x:v>individual credit matters inside agreements about fairness and shared terms</x:v>
       </x:c>
       <x:c r="E10" s="45" t="str">
-        <x:v>• fairness depending on who adjusts individual credit
-• visible contribution needing clearer shared terms
-• reciprocity becoming part of who represents the group</x:v>
+        <x:v>• credit divided according to the terms people agreed to
+• a public role changing hands to keep the arrangement fair
+• individual visibility negotiated alongside shared ownership</x:v>
       </x:c>
       <x:c r="F10" s="45" t="str">
         <x:v>individual credit inside fair agreements</x:v>
@@ -1258,9 +1258,9 @@
         <x:v>recognition carries questions of trust, privacy, and who holds leverage</x:v>
       </x:c>
       <x:c r="E11" s="45" t="str">
-        <x:v>• hidden leverage affecting individual credit
-• privacy determining access to visible contribution
-• who represents the group carrying consequences that are hard to reverse</x:v>
+        <x:v>• recognition withheld until trust and access are settled
+• the public representative carrying private obligations others cannot see
+• credit becoming leverage in a decision with lasting consequences</x:v>
       </x:c>
       <x:c r="F11" s="45" t="str">
         <x:v>recognition and public contribution tied to privacy, trust, and leverage</x:v>
@@ -1292,9 +1292,9 @@
         <x:v>visibility grows around conviction, reach, and the promise of a larger aim</x:v>
       </x:c>
       <x:c r="E12" s="45" t="str">
-        <x:v>• a larger promise stretching individual credit
-• conviction setting the direction for visible contribution
-• distance changing what seems possible for who represents the group</x:v>
+        <x:v>• a strong belief making one contribution stand for a larger cause
+• recognition extending beyond the original audience
+• the person who names the wider purpose becoming identified with it</x:v>
       </x:c>
       <x:c r="F12" s="45" t="str">
         <x:v>visible conviction and larger aims</x:v>
@@ -1326,9 +1326,9 @@
         <x:v>recognition is earned through responsibility, authority, and results that last</x:v>
       </x:c>
       <x:c r="E13" s="45" t="str">
-        <x:v>• authority setting the workable limit for individual credit
-• duty continuing after decisions about visible contribution
-• long-term consequence outweighing immediate relief in who represents the group</x:v>
+        <x:v>• authority granted after someone accepts responsibility for the outcome
+• a title reflecting work that has already survived scrutiny
+• recognition attached to the person expected to answer for the result</x:v>
       </x:c>
       <x:c r="F13" s="45" t="str">
         <x:v>recognition through authority and lasting results</x:v>
@@ -1360,9 +1360,9 @@
         <x:v>personal contribution is weighed against group standards and collective identity</x:v>
       </x:c>
       <x:c r="E14" s="45" t="str">
-        <x:v>• individual credit being measured against group policy
-• precedent shaping visible contribution
-• who represents the group being expected to apply equally</x:v>
+        <x:v>• individual credit weighed against what the group built together
+• a public face expected to represent rules that apply to everyone
+• recognition going to the contribution that changes the system</x:v>
       </x:c>
       <x:c r="F14" s="45" t="str">
         <x:v>individual contribution measured against group standards</x:v>
@@ -1394,9 +1394,9 @@
         <x:v>identity and visibility become more porous, idealized, or hard to define</x:v>
       </x:c>
       <x:c r="E15" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about individual credit
-• uncertainty making visible contribution difficult to define
-• porous boundaries complicating who represents the group</x:v>
+        <x:v>• authorship becoming unclear when many people shaped the same vision
+• recognition attaching to an idealized image rather than the actual work
+• personal contribution fading into a shared emotional response</x:v>
       </x:c>
       <x:c r="F15" s="45" t="str">
         <x:v>porous identity and idealized visibility</x:v>
@@ -1428,9 +1428,9 @@
         <x:v>needs become urgent enough to demand immediate action</x:v>
       </x:c>
       <x:c r="E16" s="45" t="str">
-        <x:v>• immediate needs being claimed before others agree
-• pressure to move first on care and protection
-• delay around a sense of belonging being treated as lost control</x:v>
+        <x:v>• an immediate need becoming impossible to postpone
+• care arriving as quick protection rather than discussion
+• belonging tested by who responds when something happens</x:v>
       </x:c>
       <x:c r="F16" s="45" t="str">
         <x:v>urgent needs and immediate emotional action</x:v>
@@ -1462,9 +1462,9 @@
         <x:v>security depends on what can be kept, afforded, and maintained</x:v>
       </x:c>
       <x:c r="E17" s="45" t="str">
-        <x:v>• immediate needs measured against cost and durability
-• care and protection slowed by what must be preserved
-• a sense of belonging judged by whether it can be maintained</x:v>
+        <x:v>• security measured by whether food, money, or shelter remains dependable
+• comfort preserved even when a faster change is available
+• a familiar routine carrying more emotional weight than the new option</x:v>
       </x:c>
       <x:c r="F17" s="45" t="str">
         <x:v>security through material continuity</x:v>
@@ -1496,9 +1496,9 @@
         <x:v>feelings change as information moves and several explanations remain open</x:v>
       </x:c>
       <x:c r="E18" s="45" t="str">
-        <x:v>• new information changing immediate needs
-• several explanations competing around care and protection
-• a sense of belonging being revised as the terms move</x:v>
+        <x:v>• a mood changing when one more fact enters the conversation
+• care taking the form of keeping people informed
+• belonging negotiated through several competing accounts of what happened</x:v>
       </x:c>
       <x:c r="F18" s="45" t="str">
         <x:v>changing information and changing feeling</x:v>
@@ -1532,9 +1532,9 @@
         <x:v>care and belonging set the emotional terms for everything else</x:v>
       </x:c>
       <x:c r="E19" s="45" t="str">
-        <x:v>• care and belonging changing the handling of immediate needs
-• private consequences shaping care and protection
-• protection taking priority in decisions about a sense of belonging</x:v>
+        <x:v>• private needs setting the terms before public plans can continue
+• care becoming more protective when belonging feels uncertain
+• family memory making a present response stronger than expected</x:v>
       </x:c>
       <x:c r="F19" s="45" t="str">
         <x:v>emotional needs, protection, and belonging made more immediate</x:v>
@@ -1566,9 +1566,9 @@
         <x:v>emotional security depends on being seen, valued, and personally acknowledged</x:v>
       </x:c>
       <x:c r="E20" s="45" t="str">
-        <x:v>• immediate needs needing visible acknowledgment
-• personal ownership becoming part of care and protection
-• a sense of belonging being distinguished from the group response</x:v>
+        <x:v>• emotional security rising when care is acknowledged openly
+• hurt becoming visible when appreciation is withheld
+• belonging tied to having a recognizable place in the group</x:v>
       </x:c>
       <x:c r="F20" s="45" t="str">
         <x:v>emotional security through recognition</x:v>
@@ -1600,9 +1600,9 @@
         <x:v>needs are sorted through practical care, useful routines, and correction</x:v>
       </x:c>
       <x:c r="E21" s="45" t="str">
-        <x:v>• immediate needs tested against the details
-• a correction changing care and protection
-• usefulness becoming the measure of a sense of belonging</x:v>
+        <x:v>• care appearing as the task that keeps a routine from failing
+• unease narrowing attention to the detail that can be corrected
+• emotional relief depending on whether practical help actually works</x:v>
       </x:c>
       <x:c r="F21" s="45" t="str">
         <x:v>practical care and corrected routines</x:v>
@@ -1636,9 +1636,9 @@
         <x:v>belonging depends on fairness, reciprocity, and whether everyone is considered</x:v>
       </x:c>
       <x:c r="E22" s="45" t="str">
-        <x:v>• fairness depending on who adjusts immediate needs
-• care and protection needing clearer shared terms
-• reciprocity becoming part of a sense of belonging</x:v>
+        <x:v>• someone feeling included only after their needs enter the agreement
+• care distributed so one person is not carrying all of it
+• belonging strained by a compromise that looks fair but feels uneven</x:v>
       </x:c>
       <x:c r="F22" s="45" t="str">
         <x:v>belonging through fairness and reciprocity</x:v>
@@ -1668,9 +1668,9 @@
         <x:v>emotional safety is tied to privacy, trust, and what cannot be taken back</x:v>
       </x:c>
       <x:c r="E23" s="45" t="str">
-        <x:v>• hidden leverage affecting immediate needs
-• privacy determining access to care and protection
-• a sense of belonging carrying consequences that are hard to reverse</x:v>
+        <x:v>• emotional safety depending on who is trusted with private information
+• care becoming guarded after something cannot be taken back
+• belonging deepening where people share the risk of being known</x:v>
       </x:c>
       <x:c r="F23" s="45" t="str">
         <x:v>emotional safety, privacy, and trust</x:v>
@@ -1704,9 +1704,9 @@
         <x:v>mood lifts or strains around freedom, conviction, and room to go farther</x:v>
       </x:c>
       <x:c r="E24" s="45" t="str">
-        <x:v>• a larger promise stretching immediate needs
-• conviction setting the direction for care and protection
-• distance changing what seems possible for a sense of belonging</x:v>
+        <x:v>• a change of place restoring emotional room
+• belonging widening around a shared belief rather than a shared history
+• care expressed by making space for a larger possibility</x:v>
       </x:c>
       <x:c r="F24" s="45" t="str">
         <x:v>emotional freedom and larger meaning</x:v>
@@ -1740,9 +1740,9 @@
         <x:v>needs are managed through duty, restraint, and what must still be done</x:v>
       </x:c>
       <x:c r="E25" s="45" t="str">
-        <x:v>• authority setting the workable limit for immediate needs
-• duty continuing after decisions about care and protection
-• long-term consequence outweighing immediate relief in a sense of belonging</x:v>
+        <x:v>• needs being postponed until the required work is done
+• care shown by taking responsibility when feelings stay private
+• belonging secured through reliability rather than reassurance</x:v>
       </x:c>
       <x:c r="F25" s="45" t="str">
         <x:v>emotional needs managed through duty and restraint</x:v>
@@ -1774,9 +1774,9 @@
         <x:v>belonging is filtered through group values, distance, and room for independence</x:v>
       </x:c>
       <x:c r="E26" s="45" t="str">
-        <x:v>• immediate needs being measured against group policy
-• precedent shaping care and protection
-• a sense of belonging being expected to apply equally</x:v>
+        <x:v>• emotional distance protecting room to remain part of the group
+• belonging depending on whether difference is allowed without explanation
+• care organized through a shared system instead of personal closeness</x:v>
       </x:c>
       <x:c r="F26" s="45" t="str">
         <x:v>belonging with distance and independence</x:v>
@@ -1808,9 +1808,9 @@
         <x:v>feeling, empathy, and uncertainty spill into each other easily</x:v>
       </x:c>
       <x:c r="E27" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about immediate needs
-• uncertainty making care and protection difficult to define
-• porous boundaries complicating a sense of belonging</x:v>
+        <x:v>• one person's mood spreading before anyone names it
+• care extending past the point where responsibility is clear
+• belonging felt through empathy even when facts remain uncertain</x:v>
       </x:c>
       <x:c r="F27" s="45" t="str">
         <x:v>feeling, empathy, and porous boundaries</x:v>
@@ -1844,9 +1844,9 @@
         <x:v>information becomes a reason to decide or speak before delay takes over</x:v>
       </x:c>
       <x:c r="E28" s="45" t="str">
-        <x:v>• the stated facts being claimed before others agree
-• pressure to move first on the decision language
-• delay around the terms being exchanged being treated as lost control</x:v>
+        <x:v>• a decision announced before every objection has been heard
+• the first explanation setting the terms of the debate
+• new facts treated as reasons to act now rather than wait</x:v>
       </x:c>
       <x:c r="F28" s="45" t="str">
         <x:v>direct speech and immediate decisions</x:v>
@@ -1880,9 +1880,9 @@
         <x:v>decisions slow down until terms feel concrete, useful, and durable</x:v>
       </x:c>
       <x:c r="E29" s="45" t="str">
-        <x:v>• the stated facts measured against cost and durability
-• the decision language slowed by what must be preserved
-• the terms being exchanged judged by whether it can be maintained</x:v>
+        <x:v>• an agreement slowing until the price and practical terms are clear
+• a repeated fact carrying more weight than a clever argument
+• decisions holding once they are written in concrete language</x:v>
       </x:c>
       <x:c r="F29" s="45" t="str">
         <x:v>concrete terms and durable decisions</x:v>
@@ -1914,9 +1914,9 @@
         <x:v>language multiplies the available facts, comparisons, and ways forward</x:v>
       </x:c>
       <x:c r="E30" s="45" t="str">
-        <x:v>• new information changing the stated facts
-• several explanations competing around the decision language
-• the terms being exchanged being revised as the terms move</x:v>
+        <x:v>• several versions of the same information remaining active at once
+• the wording changing as quickly as the facts
+• a decision staying open because another comparison is still possible</x:v>
       </x:c>
       <x:c r="F30" s="45" t="str">
         <x:v>information and language multiplying their own possible answers</x:v>
@@ -1950,9 +1950,9 @@
         <x:v>communication carries memory, care, and the private consequences of what is said</x:v>
       </x:c>
       <x:c r="E31" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the stated facts
-• private consequences shaping the decision language
-• protection taking priority in decisions about the terms being exchanged</x:v>
+        <x:v>• a practical question carrying the memory of an earlier conversation
+• private consequences changing what can be said in public
+• information being trusted because it arrives through care</x:v>
       </x:c>
       <x:c r="F31" s="45" t="str">
         <x:v>language carrying memory and private consequence</x:v>
@@ -1984,9 +1984,9 @@
         <x:v>words become a claim to visibility, authority, or personal credit</x:v>
       </x:c>
       <x:c r="E32" s="45" t="str">
-        <x:v>• the stated facts needing visible acknowledgment
-• personal ownership becoming part of the decision language
-• the terms being exchanged being distinguished from the group response</x:v>
+        <x:v>• an opinion becoming inseparable from who said it
+• the clearest speaker taking visible ownership of the decision
+• language used to defend personal credit as well as the point itself</x:v>
       </x:c>
       <x:c r="F32" s="45" t="str">
         <x:v>speech as visible personal claim</x:v>
@@ -2020,9 +2020,9 @@
         <x:v>thought narrows toward precision, usefulness, and correcting what does not add up</x:v>
       </x:c>
       <x:c r="E33" s="45" t="str">
-        <x:v>• the stated facts tested against the details
-• a correction changing the decision language
-• usefulness becoming the measure of the terms being exchanged</x:v>
+        <x:v>• one inconsistency changing the whole decision
+• the useful correction mattering more than the impressive explanation
+• terms narrowed until every part can be checked</x:v>
       </x:c>
       <x:c r="F33" s="45" t="str">
         <x:v>precise thought and useful correction</x:v>
@@ -2054,9 +2054,9 @@
         <x:v>decisions are negotiated through fairness, response, and shared terms</x:v>
       </x:c>
       <x:c r="E34" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the stated facts
-• the decision language needing clearer shared terms
-• reciprocity becoming part of the terms being exchanged</x:v>
+        <x:v>• a decision moving only after both replies enter the record
+• wording revised to distribute responsibility more fairly
+• the agreement depending on whether each side can answer the same terms</x:v>
       </x:c>
       <x:c r="F34" s="45" t="str">
         <x:v>negotiated decisions and shared terms</x:v>
@@ -2088,9 +2088,9 @@
         <x:v>information is measured by trust, privacy, and who knows what</x:v>
       </x:c>
       <x:c r="E35" s="45" t="str">
-        <x:v>• hidden leverage affecting the stated facts
-• privacy determining access to the decision language
-• the terms being exchanged carrying consequences that are hard to reverse</x:v>
+        <x:v>• access to private information deciding who can act
+• a withheld fact gaining power as the stakes rise
+• language becoming exact because the consequence cannot be reversed</x:v>
       </x:c>
       <x:c r="F35" s="45" t="str">
         <x:v>private information and trusted access</x:v>
@@ -2122,9 +2122,9 @@
         <x:v>language reaches for the larger claim, the principle, or the distant possibility</x:v>
       </x:c>
       <x:c r="E36" s="45" t="str">
-        <x:v>• a larger promise stretching the stated facts
-• conviction setting the direction for the decision language
-• distance changing what seems possible for the terms being exchanged</x:v>
+        <x:v>• one principle organizing facts that point in several directions
+• a distant possibility changing the immediate decision
+• the larger claim traveling farther than its supporting detail</x:v>
       </x:c>
       <x:c r="F36" s="45" t="str">
         <x:v>language reaching toward principle and distance</x:v>
@@ -2156,9 +2156,9 @@
         <x:v>communication becomes formal, consequential, and accountable to structure</x:v>
       </x:c>
       <x:c r="E37" s="45" t="str">
-        <x:v>• authority setting the workable limit for the stated facts
-• duty continuing after decisions about the decision language
-• long-term consequence outweighing immediate relief in the terms being exchanged</x:v>
+        <x:v>• formal wording assigning responsibility that continues after the meeting
+• a decision becoming real when an authority records it
+• communication judged by whether it can support a lasting structure</x:v>
       </x:c>
       <x:c r="F37" s="45" t="str">
         <x:v>formal language and accountable decisions</x:v>
@@ -2190,9 +2190,9 @@
         <x:v>ideas are judged by the system they could change and the group they would affect</x:v>
       </x:c>
       <x:c r="E38" s="45" t="str">
-        <x:v>• the stated facts being measured against group policy
-• precedent shaping the decision language
-• the terms being exchanged being expected to apply equally</x:v>
+        <x:v>• an idea evaluated by the system it would alter
+• information shared widely enough to change who holds access
+• the group adopting language that makes a new rule possible</x:v>
       </x:c>
       <x:c r="F38" s="45" t="str">
         <x:v>system-changing ideas and group consequence</x:v>
@@ -2224,9 +2224,9 @@
         <x:v>information moves through impression, implication, and facts that are hard to pin down</x:v>
       </x:c>
       <x:c r="E39" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the stated facts
-• uncertainty making the decision language difficult to define
-• porous boundaries complicating the terms being exchanged</x:v>
+        <x:v>• meaning carried by tone when the stated facts remain incomplete
+• an implication spreading faster than anyone can verify it
+• a decision blurred by sympathy for several incompatible accounts</x:v>
       </x:c>
       <x:c r="F39" s="45" t="str">
         <x:v>implied meaning and uncertain facts</x:v>
@@ -2260,9 +2260,9 @@
         <x:v>attraction and agreement move toward direct preference and a quick yes or no</x:v>
       </x:c>
       <x:c r="E40" s="45" t="str">
-        <x:v>• shared value being claimed before others agree
-• pressure to move first on fair agreement
-• delay around what remains worth preserving being treated as lost control</x:v>
+        <x:v>• a preference stated clearly enough to force a quick answer
+• attraction growing through direct pursuit instead of careful agreement
+• value assigned to the choice that shows immediate commitment</x:v>
       </x:c>
       <x:c r="F40" s="45" t="str">
         <x:v>direct preference and quick agreement</x:v>
@@ -2294,9 +2294,9 @@
         <x:v>value settles around what feels good, costs what it is worth, and can last</x:v>
       </x:c>
       <x:c r="E41" s="45" t="str">
-        <x:v>• shared value measured against cost and durability
-• fair agreement slowed by what must be preserved
-• what remains worth preserving judged by whether it can be maintained</x:v>
+        <x:v>• an agreement holding because the exchange feels materially worthwhile
+• comfort becoming part of how value is measured
+• affection shown by preserving what people already share</x:v>
       </x:c>
       <x:c r="F41" s="45" t="str">
         <x:v>lasting value, comfort, and material worth</x:v>
@@ -2330,9 +2330,9 @@
         <x:v>connection depends on conversation, variety, and terms that can keep moving</x:v>
       </x:c>
       <x:c r="E42" s="45" t="str">
-        <x:v>• new information changing shared value
-• several explanations competing around fair agreement
-• what remains worth preserving being revised as the terms move</x:v>
+        <x:v>• connection growing through the conversation that keeps changing shape
+• interest sustained by more than one possible arrangement
+• shared value revised when people compare what each option offers</x:v>
       </x:c>
       <x:c r="F42" s="45" t="str">
         <x:v>connection through varied conversation</x:v>
@@ -2366,9 +2366,9 @@
         <x:v>value is measured through care, loyalty, and whether people feel included</x:v>
       </x:c>
       <x:c r="E43" s="45" t="str">
-        <x:v>• care and belonging changing the handling of shared value
-• private consequences shaping fair agreement
-• protection taking priority in decisions about what remains worth preserving</x:v>
+        <x:v>• affection expressed through inclusion in private life
+• an agreement valued because it protects belonging
+• care determining what people are willing to preserve together</x:v>
       </x:c>
       <x:c r="F43" s="45" t="str">
         <x:v>care, loyalty, and inclusive value</x:v>
@@ -2400,9 +2400,9 @@
         <x:v>affection and agreement carry a need for warmth, visibility, and personal appreciation</x:v>
       </x:c>
       <x:c r="E44" s="45" t="str">
-        <x:v>• shared value needing visible acknowledgment
-• personal ownership becoming part of fair agreement
-• what remains worth preserving being distinguished from the group response</x:v>
+        <x:v>• appreciation becoming real when it is shown where others can see it
+• affection tied to being chosen distinctly rather than generally included
+• a shared value represented through visible generosity</x:v>
       </x:c>
       <x:c r="F44" s="45" t="str">
         <x:v>visible affection and personal appreciation</x:v>
@@ -2436,9 +2436,9 @@
         <x:v>care is shown through usefulness, attention, and fixing what creates strain</x:v>
       </x:c>
       <x:c r="E45" s="45" t="str">
-        <x:v>• shared value tested against the details
-• a correction changing fair agreement
-• usefulness becoming the measure of what remains worth preserving</x:v>
+        <x:v>• care demonstrated by noticing the strain and reducing it
+• an agreement improved through one practical adjustment
+• value measured by whether attention makes daily life work better</x:v>
       </x:c>
       <x:c r="F45" s="45" t="str">
         <x:v>care through practical attention</x:v>
@@ -2472,9 +2472,9 @@
         <x:v>fairness and mutual response become the terms of connection itself</x:v>
       </x:c>
       <x:c r="E46" s="45" t="str">
-        <x:v>• fairness depending on who adjusts shared value
-• fair agreement needing clearer shared terms
-• reciprocity becoming part of what remains worth preserving</x:v>
+        <x:v>• mutual response becoming the evidence that an agreement is fair
+• affection sustained by terms neither person has to disappear inside
+• shared value defined through balance rather than identical contribution</x:v>
       </x:c>
       <x:c r="F46" s="45" t="str">
         <x:v>fairness and mutuality becoming the terms of connection</x:v>
@@ -2508,9 +2508,9 @@
         <x:v>attraction deepens around trust, privacy, and the risk of giving up leverage</x:v>
       </x:c>
       <x:c r="E47" s="45" t="str">
-        <x:v>• hidden leverage affecting shared value
-• privacy determining access to fair agreement
-• what remains worth preserving carrying consequences that are hard to reverse</x:v>
+        <x:v>• desire deepening after trust survives a private disclosure
+• an agreement carrying the risk of giving someone real leverage
+• value concentrating around what cannot be casually replaced</x:v>
       </x:c>
       <x:c r="F47" s="45" t="str">
         <x:v>desire tied to privacy and trust</x:v>
@@ -2542,9 +2542,9 @@
         <x:v>value follows openness, conviction, and the room to want more</x:v>
       </x:c>
       <x:c r="E48" s="45" t="str">
-        <x:v>• a larger promise stretching shared value
-• conviction setting the direction for fair agreement
-• distance changing what seems possible for what remains worth preserving</x:v>
+        <x:v>• connection widening through a shared horizon rather than a fixed plan
+• value following the choice that leaves more room to grow
+• affection expressed by supporting a belief with visible reach</x:v>
       </x:c>
       <x:c r="F48" s="45" t="str">
         <x:v>open value and expansive desire</x:v>
@@ -2578,9 +2578,9 @@
         <x:v>agreement is tested by responsibility, status, and whether it can hold over time</x:v>
       </x:c>
       <x:c r="E49" s="45" t="str">
-        <x:v>• authority setting the workable limit for shared value
-• duty continuing after decisions about fair agreement
-• long-term consequence outweighing immediate relief in what remains worth preserving</x:v>
+        <x:v>• an agreement earning value because it can carry responsibility over time
+• affection shown through commitments that survive inconvenience
+• shared worth measured against consequence, status, and durability</x:v>
       </x:c>
       <x:c r="F49" s="45" t="str">
         <x:v>durable agreement and social responsibility</x:v>
@@ -2614,9 +2614,9 @@
         <x:v>connection needs enough independence to coexist with group commitments</x:v>
       </x:c>
       <x:c r="E50" s="45" t="str">
-        <x:v>• shared value being measured against group policy
-• precedent shaping fair agreement
-• what remains worth preserving being expected to apply equally</x:v>
+        <x:v>• connection remaining possible because independence is built into the terms
+• shared value forming around a group commitment rather than private closeness
+• affection making room for a difference the old agreement could not hold</x:v>
       </x:c>
       <x:c r="F50" s="45" t="str">
         <x:v>independent connection within group commitments</x:v>
@@ -2648,9 +2648,9 @@
         <x:v>affection can become generous, idealized, or difficult to separate from longing</x:v>
       </x:c>
       <x:c r="E51" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about shared value
-• uncertainty making fair agreement difficult to define
-• porous boundaries complicating what remains worth preserving</x:v>
+        <x:v>• longing adding value to an arrangement before its limits are visible
+• affection extending beyond what either person has clearly promised
+• shared ideals making unequal terms difficult to notice</x:v>
       </x:c>
       <x:c r="F51" s="45" t="str">
         <x:v>idealized affection and porous longing</x:v>
@@ -2682,9 +2682,9 @@
         <x:v>action becomes immediate, direct, and difficult to contain once begun</x:v>
       </x:c>
       <x:c r="E52" s="45" t="str">
-        <x:v>• the first action being claimed before others agree
-• pressure to move first on open pressure
-• delay around the result being pursued being treated as lost control</x:v>
+        <x:v>• the first move establishing who controls the pace
+• pressure turning directly into action before a process is agreed
+• a visible result pursued without waiting for broader support</x:v>
       </x:c>
       <x:c r="F52" s="45" t="str">
         <x:v>direct action reinforcing its own urgency</x:v>
@@ -2718,9 +2718,9 @@
         <x:v>pressure builds slowly around resources, limits, and what will not be moved</x:v>
       </x:c>
       <x:c r="E53" s="45" t="str">
-        <x:v>• the first action measured against cost and durability
-• open pressure slowed by what must be preserved
-• the result being pursued judged by whether it can be maintained</x:v>
+        <x:v>• effort continuing at the same point until a material limit gives way
+• conflict gathering around a resource no one wants to surrender
+• action delayed until the result can be kept</x:v>
       </x:c>
       <x:c r="F53" s="45" t="str">
         <x:v>slow pressure around resources and fixed limits</x:v>
@@ -2754,9 +2754,9 @@
         <x:v>action scatters through words, errands, comparisons, and changing targets</x:v>
       </x:c>
       <x:c r="E54" s="45" t="str">
-        <x:v>• new information changing the first action
-• several explanations competing around open pressure
-• the result being pursued being revised as the terms move</x:v>
+        <x:v>• effort divided among several messages, errands, or targets
+• conflict moving with the wording instead of staying on one issue
+• a new comparison redirecting action already underway</x:v>
       </x:c>
       <x:c r="F54" s="45" t="str">
         <x:v>scattered action and changing targets</x:v>
@@ -2790,9 +2790,9 @@
         <x:v>conflict protects home, belonging, and private vulnerability before it explains itself</x:v>
       </x:c>
       <x:c r="E55" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the first action
-• private consequences shaping open pressure
-• protection taking priority in decisions about the result being pursued</x:v>
+        <x:v>• defense beginning when home or belonging feels exposed
+• action taken to protect someone before the reason is explained
+• conflict carrying a private vulnerability into a public decision</x:v>
       </x:c>
       <x:c r="F55" s="45" t="str">
         <x:v>action and conflict organized around care and private belonging</x:v>
@@ -2826,9 +2826,9 @@
         <x:v>action seeks a visible result and personal ownership of the move</x:v>
       </x:c>
       <x:c r="E56" s="45" t="str">
-        <x:v>• the first action needing visible acknowledgment
-• personal ownership becoming part of open pressure
-• the result being pursued being distinguished from the group response</x:v>
+        <x:v>• a bold action tying the outcome to one visible person
+• effort intensifying when pride and recognition are on the line
+• the result pursued in a way that makes ownership unmistakable</x:v>
       </x:c>
       <x:c r="F56" s="45" t="str">
         <x:v>visible action and ownership of the result</x:v>
@@ -2862,9 +2862,9 @@
         <x:v>effort goes into fixing, sorting, and making the method work</x:v>
       </x:c>
       <x:c r="E57" s="45" t="str">
-        <x:v>• the first action tested against the details
-• a correction changing open pressure
-• usefulness becoming the measure of the result being pursued</x:v>
+        <x:v>• energy concentrating on the fault that can actually be repaired
+• conflict narrowing into a dispute about method
+• action continuing through small corrections rather than one large move</x:v>
       </x:c>
       <x:c r="F57" s="45" t="str">
         <x:v>effort focused on repair and method</x:v>
@@ -2898,9 +2898,9 @@
         <x:v>the urge to act is checked by fairness, response, and the cost of open conflict</x:v>
       </x:c>
       <x:c r="E58" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the first action
-• open pressure needing clearer shared terms
-• reciprocity becoming part of the result being pursued</x:v>
+        <x:v>• the urge to act slowing long enough to measure the other response
+• conflict entering negotiation before either side gets its preferred result
+• effort redirected toward terms that do not leave one party carrying the cost</x:v>
       </x:c>
       <x:c r="F58" s="45" t="str">
         <x:v>action negotiated through fairness and response</x:v>
@@ -2934,9 +2934,9 @@
         <x:v>pursuit becomes strategic where trust, control, and irreversible consequences are involved</x:v>
       </x:c>
       <x:c r="E59" s="45" t="str">
-        <x:v>• hidden leverage affecting the first action
-• privacy determining access to open pressure
-• the result being pursued carrying consequences that are hard to reverse</x:v>
+        <x:v>• action withheld until the source of control becomes clear
+• pressure applied where trust and private access are already at stake
+• a result pursued carefully because it cannot be undone</x:v>
       </x:c>
       <x:c r="F59" s="45" t="str">
         <x:v>strategic pursuit, trust, and control</x:v>
@@ -2968,9 +2968,9 @@
         <x:v>action pushes toward distance, conviction, and the next larger possibility</x:v>
       </x:c>
       <x:c r="E60" s="45" t="str">
-        <x:v>• a larger promise stretching the first action
-• conviction setting the direction for open pressure
-• distance changing what seems possible for the result being pursued</x:v>
+        <x:v>• effort extending toward the larger target before the near one is settled
+• action gaining force from conviction rather than immediate proof
+• conflict widening when freedom of movement is restricted</x:v>
       </x:c>
       <x:c r="F60" s="45" t="str">
         <x:v>action driven by conviction and distance</x:v>
@@ -3002,9 +3002,9 @@
         <x:v>effort is disciplined by duty, authority, and a result that can endure</x:v>
       </x:c>
       <x:c r="E61" s="45" t="str">
-        <x:v>• authority setting the workable limit for the first action
-• duty continuing after decisions about open pressure
-• long-term consequence outweighing immediate relief in the result being pursued</x:v>
+        <x:v>• effort organized around the result an authority will accept
+• pressure sustained through duty after urgency has passed
+• action measured by whether it creates a durable outcome</x:v>
       </x:c>
       <x:c r="F61" s="45" t="str">
         <x:v>disciplined effort and durable results</x:v>
@@ -3038,9 +3038,9 @@
         <x:v>pressure builds around independence, shared rules, and changing the system</x:v>
       </x:c>
       <x:c r="E62" s="45" t="str">
-        <x:v>• the first action being measured against group policy
-• precedent shaping open pressure
-• the result being pursued being expected to apply equally</x:v>
+        <x:v>• conflict gathering around a rule that limits independence
+• action aimed at changing the system rather than winning one exception
+• group pressure building behind a different arrangement</x:v>
       </x:c>
       <x:c r="F62" s="45" t="str">
         <x:v>pressure for independence and system change</x:v>
@@ -3072,9 +3072,9 @@
         <x:v>action follows feeling and instinct even when the boundary or target is unclear</x:v>
       </x:c>
       <x:c r="E63" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the first action
-• uncertainty making open pressure difficult to define
-• porous boundaries complicating the result being pursued</x:v>
+        <x:v>• effort following an emotional current before the target is defined
+• conflict spreading because the boundary of responsibility stays unclear
+• action losing force when several needs merge into one another</x:v>
       </x:c>
       <x:c r="F63" s="45" t="str">
         <x:v>instinctive action with an unclear target</x:v>
@@ -3108,9 +3108,9 @@
         <x:v>growth is measured by the freedom to begin, take a risk, and move first</x:v>
       </x:c>
       <x:c r="E64" s="45" t="str">
-        <x:v>• the promised growth being claimed before others agree
-• pressure to move first on a wider opportunity
-• delay around confidence in what is possible being treated as lost control</x:v>
+        <x:v>• a new opening becoming larger because someone risks moving first
+• confidence building through action before certainty arrives
+• growth attached to the option that expands independence</x:v>
       </x:c>
       <x:c r="F64" s="45" t="str">
         <x:v>growth through risk and first moves</x:v>
@@ -3144,9 +3144,9 @@
         <x:v>opportunity expands through resources, value, and what can be sustained</x:v>
       </x:c>
       <x:c r="E65" s="45" t="str">
-        <x:v>• the promised growth measured against cost and durability
-• a wider opportunity slowed by what must be preserved
-• confidence in what is possible judged by whether it can be maintained</x:v>
+        <x:v>• opportunity increasing the resources people can actually maintain
+• a larger promise tested against cost before it is trusted
+• growth appearing in what becomes more secure or materially useful</x:v>
       </x:c>
       <x:c r="F65" s="45" t="str">
         <x:v>sustainable opportunity and material value</x:v>
@@ -3178,9 +3178,9 @@
         <x:v>possibility multiplies through information, comparison, and several open routes</x:v>
       </x:c>
       <x:c r="E66" s="45" t="str">
-        <x:v>• new information changing the promised growth
-• several explanations competing around a wider opportunity
-• confidence in what is possible being revised as the terms move</x:v>
+        <x:v>• several small openings becoming available through new information
+• confidence rising as people compare more than one route
+• possibility expanding faster than the decision can narrow</x:v>
       </x:c>
       <x:c r="F66" s="45" t="str">
         <x:v>multiple possibilities through information</x:v>
@@ -3214,9 +3214,9 @@
         <x:v>growth takes the form of protection, care, and a wider sense of belonging</x:v>
       </x:c>
       <x:c r="E67" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the promised growth
-• private consequences shaping a wider opportunity
-• protection taking priority in decisions about confidence in what is possible</x:v>
+        <x:v>• growth taking the form of wider protection or belonging
+• an opportunity becoming meaningful because it includes people previously left out
+• confidence increasing where care has made risk feel survivable</x:v>
       </x:c>
       <x:c r="F67" s="45" t="str">
         <x:v>growth through care and belonging</x:v>
@@ -3248,9 +3248,9 @@
         <x:v>confidence grows through visible contribution, generosity, and recognition</x:v>
       </x:c>
       <x:c r="E68" s="45" t="str">
-        <x:v>• the promised growth needing visible acknowledgment
-• personal ownership becoming part of a wider opportunity
-• confidence in what is possible being distinguished from the group response</x:v>
+        <x:v>• generosity making an individual contribution more visible
+• a larger role becoming possible after someone is publicly trusted
+• confidence spreading through recognition that feels personally earned</x:v>
       </x:c>
       <x:c r="F68" s="45" t="str">
         <x:v>confidence through visible generosity</x:v>
@@ -3282,9 +3282,9 @@
         <x:v>expansion is tested by usefulness, detail, and what can actually be improved</x:v>
       </x:c>
       <x:c r="E69" s="45" t="str">
-        <x:v>• the promised growth tested against the details
-• a correction changing a wider opportunity
-• usefulness becoming the measure of confidence in what is possible</x:v>
+        <x:v>• an opportunity proving itself through a useful improvement
+• growth limited to what the details can support
+• confidence increasing after the method produces a measurable result</x:v>
       </x:c>
       <x:c r="F69" s="45" t="str">
         <x:v>useful expansion tested by detail</x:v>
@@ -3316,9 +3316,9 @@
         <x:v>opportunity depends on fair terms, cooperation, and benefits shared across the agreement</x:v>
       </x:c>
       <x:c r="E70" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the promised growth
-• a wider opportunity needing clearer shared terms
-• reciprocity becoming part of confidence in what is possible</x:v>
+        <x:v>• benefit widening when the terms distribute it more fairly
+• an agreement creating an opportunity neither side could reach alone
+• confidence resting on cooperation that remains reciprocal</x:v>
       </x:c>
       <x:c r="F70" s="45" t="str">
         <x:v>shared opportunity through fair terms</x:v>
@@ -3352,9 +3352,9 @@
         <x:v>growth carries questions of trust, leverage, and how much change can be reversed</x:v>
       </x:c>
       <x:c r="E71" s="45" t="str">
-        <x:v>• hidden leverage affecting the promised growth
-• privacy determining access to a wider opportunity
-• confidence in what is possible carrying consequences that are hard to reverse</x:v>
+        <x:v>• growth requiring enough trust to share real leverage
+• a larger opportunity carrying consequences that cannot be easily reversed
+• confidence changing when hidden stakes become visible</x:v>
       </x:c>
       <x:c r="F71" s="45" t="str">
         <x:v>growth through trust and reversible stakes</x:v>
@@ -3386,9 +3386,9 @@
         <x:v>belief, reach, and possibility expand until limits become easy to overlook</x:v>
       </x:c>
       <x:c r="E72" s="45" t="str">
-        <x:v>• a larger promise stretching the promised growth
-• conviction setting the direction for a wider opportunity
-• distance changing what seems possible for confidence in what is possible</x:v>
+        <x:v>• belief enlarging the horizon beyond the current limit
+• an opportunity reaching farther because its meaning is widely shared
+• confidence rising faster than practical constraints can answer</x:v>
       </x:c>
       <x:c r="F72" s="45" t="str">
         <x:v>growth and belief expanding past visible limits</x:v>
@@ -3420,9 +3420,9 @@
         <x:v>ambition grows inside duty, hierarchy, and consequences that take time</x:v>
       </x:c>
       <x:c r="E73" s="45" t="str">
-        <x:v>• authority setting the workable limit for the promised growth
-• duty continuing after decisions about a wider opportunity
-• long-term consequence outweighing immediate relief in confidence in what is possible</x:v>
+        <x:v>• ambition expanding through duties that increase authority
+• an opportunity becoming credible when it fits a long structure
+• growth measured by what can still stand after accountability arrives</x:v>
       </x:c>
       <x:c r="F73" s="45" t="str">
         <x:v>ambition inside duty and hierarchy</x:v>
@@ -3456,9 +3456,9 @@
         <x:v>possibility attaches to reform, group aims, and systems meant to reach more people</x:v>
       </x:c>
       <x:c r="E74" s="45" t="str">
-        <x:v>• the promised growth being measured against group policy
-• precedent shaping a wider opportunity
-• confidence in what is possible being expected to apply equally</x:v>
+        <x:v>• possibility widening through a reform meant to reach the whole group
+• confidence gathering around a system people believe can change
+• an opportunity emerging from shared access rather than private advantage</x:v>
       </x:c>
       <x:c r="F74" s="45" t="str">
         <x:v>collective reform and wider opportunity</x:v>
@@ -3490,9 +3490,9 @@
         <x:v>hope and meaning expand through empathy, imagination, and boundaries that loosen</x:v>
       </x:c>
       <x:c r="E75" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the promised growth
-• uncertainty making a wider opportunity difficult to define
-• porous boundaries complicating confidence in what is possible</x:v>
+        <x:v>• hope expanding where empathy loosens an old boundary
+• possibility becoming larger than anyone can yet define
+• confidence attaching to a shared ideal before its limits are clear</x:v>
       </x:c>
       <x:c r="F75" s="45" t="str">
         <x:v>expansive hope and porous boundaries</x:v>
@@ -3524,9 +3524,9 @@
         <x:v>limits confront the demand to act now and prove independence</x:v>
       </x:c>
       <x:c r="E76" s="45" t="str">
-        <x:v>• the active limit being claimed before others agree
-• pressure to move first on assigned responsibility
-• delay around the standard being enforced being treated as lost control</x:v>
+        <x:v>• a limit stopping the first move until responsibility is assigned
+• independence tested by a consequence that cannot be rushed
+• authority requiring proof before action receives backing</x:v>
       </x:c>
       <x:c r="F76" s="45" t="str">
         <x:v>limits against immediate independence</x:v>
@@ -3558,9 +3558,9 @@
         <x:v>responsibility settles around resources, endurance, and what must be maintained</x:v>
       </x:c>
       <x:c r="E77" s="45" t="str">
-        <x:v>• the active limit measured against cost and durability
-• assigned responsibility slowed by what must be preserved
-• the standard being enforced judged by whether it can be maintained</x:v>
+        <x:v>• responsibility settling on the resource that must not run out
+• a material limit forcing people to maintain what they already have
+• progress measured by endurance rather than speed</x:v>
       </x:c>
       <x:c r="F77" s="45" t="str">
         <x:v>responsibility for material continuity</x:v>
@@ -3594,9 +3594,9 @@
         <x:v>standards tighten around facts, wording, and decisions that keep changing</x:v>
       </x:c>
       <x:c r="E78" s="45" t="str">
-        <x:v>• new information changing the active limit
-• several explanations competing around assigned responsibility
-• the standard being enforced being revised as the terms move</x:v>
+        <x:v>• changing language held to a standard that must remain consistent
+• a decision delayed while conflicting facts are documented
+• responsibility attached to the version that enters the record</x:v>
       </x:c>
       <x:c r="F78" s="45" t="str">
         <x:v>standards for changing facts and language</x:v>
@@ -3630,9 +3630,9 @@
         <x:v>duty weighs on care, belonging, and the private costs people carry</x:v>
       </x:c>
       <x:c r="E79" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the active limit
-• private consequences shaping assigned responsibility
-• protection taking priority in decisions about the standard being enforced</x:v>
+        <x:v>• duty falling on the person who protects private continuity
+• care narrowed by a limit on time, money, or capacity
+• belonging tested by obligations that are not distributed equally</x:v>
       </x:c>
       <x:c r="F79" s="45" t="str">
         <x:v>duty carrying private emotional cost</x:v>
@@ -3664,9 +3664,9 @@
         <x:v>authority tests how recognition is earned and how much individual pride can bend</x:v>
       </x:c>
       <x:c r="E80" s="45" t="str">
-        <x:v>• the active limit needing visible acknowledgment
-• personal ownership becoming part of assigned responsibility
-• the standard being enforced being distinguished from the group response</x:v>
+        <x:v>• recognition withheld until the visible contribution meets the standard
+• authority limiting how much pride can direct the decision
+• a public role carrying consequences that personal confidence cannot erase</x:v>
       </x:c>
       <x:c r="F80" s="45" t="str">
         <x:v>authority testing pride and recognition</x:v>
@@ -3698,9 +3698,9 @@
         <x:v>responsibility concentrates in routines, corrections, and work that must be exact</x:v>
       </x:c>
       <x:c r="E81" s="45" t="str">
-        <x:v>• the active limit tested against the details
-• a correction changing assigned responsibility
-• usefulness becoming the measure of the standard being enforced</x:v>
+        <x:v>• responsibility concentrating in the detail no one else can ignore
+• a routine becoming stricter after an avoidable error
+• progress depending on correction that can be repeated reliably</x:v>
       </x:c>
       <x:c r="F81" s="45" t="str">
         <x:v>exact routines and corrective responsibility</x:v>
@@ -3732,9 +3732,9 @@
         <x:v>obligations are negotiated through fairness, shared terms, and equal accountability</x:v>
       </x:c>
       <x:c r="E82" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the active limit
-• assigned responsibility needing clearer shared terms
-• reciprocity becoming part of the standard being enforced</x:v>
+        <x:v>• obligation divided according to terms both sides must answer to
+• fairness tested by who carries the consequence of compromise
+• an agreement becoming binding when accountability is shared</x:v>
       </x:c>
       <x:c r="F82" s="45" t="str">
         <x:v>fair obligation and shared accountability</x:v>
@@ -3766,9 +3766,9 @@
         <x:v>limits become questions of trust, control, and consequences that cannot be undone</x:v>
       </x:c>
       <x:c r="E83" s="45" t="str">
-        <x:v>• hidden leverage affecting the active limit
-• privacy determining access to assigned responsibility
-• the standard being enforced carrying consequences that are hard to reverse</x:v>
+        <x:v>• a limit protecting access to information that cannot be taken back
+• responsibility increasing where control and trust are intertwined
+• authority settling a consequence people had hoped to postpone</x:v>
       </x:c>
       <x:c r="F83" s="45" t="str">
         <x:v>limits tied to trust and irreversible consequence</x:v>
@@ -3800,9 +3800,9 @@
         <x:v>belief and large promises meet the boundary of what can be proved or delivered</x:v>
       </x:c>
       <x:c r="E84" s="45" t="str">
-        <x:v>• a larger promise stretching the active limit
-• conviction setting the direction for assigned responsibility
-• distance changing what seems possible for the standard being enforced</x:v>
+        <x:v>• a large promise reduced to what can be proved and delivered
+• belief tested by the boundary of an institution or law
+• responsibility following the claim farther than confidence expected</x:v>
       </x:c>
       <x:c r="F84" s="45" t="str">
         <x:v>belief tested by proof and delivery</x:v>
@@ -3836,9 +3836,9 @@
         <x:v>duty, authority, and long-term consequence become the measure of progress</x:v>
       </x:c>
       <x:c r="E85" s="45" t="str">
-        <x:v>• authority setting the workable limit for the active limit
-• duty continuing after decisions about assigned responsibility
-• long-term consequence outweighing immediate relief in the standard being enforced</x:v>
+        <x:v>• authority consolidating around the person who can carry the duty
+• long consequences deciding which ambition remains workable
+• progress becoming inseparable from structure and accountability</x:v>
       </x:c>
       <x:c r="F85" s="45" t="str">
         <x:v>duty and consequence reinforcing structure and authority</x:v>
@@ -3904,9 +3904,9 @@
         <x:v>structure is asked to contain uncertainty, compassion, and boundaries that do not stay firm</x:v>
       </x:c>
       <x:c r="E87" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the active limit
-• uncertainty making assigned responsibility difficult to define
-• porous boundaries complicating the standard being enforced</x:v>
+        <x:v>• a formal boundary trying to contain a need that has no clean edge
+• responsibility becoming hard to assign when compassion is widely shared
+• structure holding only where uncertainty is named rather than denied</x:v>
       </x:c>
       <x:c r="F87" s="45" t="str">
         <x:v>structure containing compassion and uncertainty</x:v>
@@ -3938,9 +3938,9 @@
         <x:v>disruption arrives through a sudden claim of independence or an unexpected first move</x:v>
       </x:c>
       <x:c r="E88" s="45" t="str">
-        <x:v>• the proposed change being claimed before others agree
-• pressure to move first on room for independence
-• delay around the arrangement being revised being treated as lost control</x:v>
+        <x:v>• an unexpected first move changing who has room to act
+• independence claimed before the existing process can respond
+• a sudden break creating an opening that did not exist a moment earlier</x:v>
       </x:c>
       <x:c r="F88" s="45" t="str">
         <x:v>unexpected initiative and sudden independence</x:v>
@@ -3974,9 +3974,9 @@
         <x:v>change reaches the resources, values, and routines assumed to be secure</x:v>
       </x:c>
       <x:c r="E89" s="45" t="str">
-        <x:v>• the proposed change measured against cost and durability
-• room for independence slowed by what must be preserved
-• the arrangement being revised judged by whether it can be maintained</x:v>
+        <x:v>• a secure resource becoming the site of an unexpected revision
+• material routines changing after stability proves less fixed than assumed
+• independence requiring a new way to preserve what still matters</x:v>
       </x:c>
       <x:c r="F89" s="45" t="str">
         <x:v>disruption of material security</x:v>
@@ -4008,9 +4008,9 @@
         <x:v>new information rapidly alters the terms, routes, and available explanations</x:v>
       </x:c>
       <x:c r="E90" s="45" t="str">
-        <x:v>• new information changing the proposed change
-• several explanations competing around room for independence
-• the arrangement being revised being revised as the terms move</x:v>
+        <x:v>• new information altering the available routes almost immediately
+• a revised term changing who can participate
+• independence spreading through access to a different explanation</x:v>
       </x:c>
       <x:c r="F90" s="45" t="str">
         <x:v>rapidly revised information and terms</x:v>
@@ -4044,9 +4044,9 @@
         <x:v>independence unsettles familiar patterns of care, home, and belonging</x:v>
       </x:c>
       <x:c r="E91" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the proposed change
-• private consequences shaping room for independence
-• protection taking priority in decisions about the arrangement being revised</x:v>
+        <x:v>• a household pattern changing because someone needs more room
+• belonging reorganized around a form of care no longer kept private
+• independence unsettling the role that once guaranteed emotional safety</x:v>
       </x:c>
       <x:c r="F91" s="45" t="str">
         <x:v>independence disrupting care and belonging</x:v>
@@ -4078,9 +4078,9 @@
         <x:v>change breaks into questions of visibility, recognition, and who gets to stand apart</x:v>
       </x:c>
       <x:c r="E92" s="45" t="str">
-        <x:v>• the proposed change needing visible acknowledgment
-• personal ownership becoming part of room for independence
-• the arrangement being revised being distinguished from the group response</x:v>
+        <x:v>• visible difference interrupting the expected public role
+• recognition shifting toward the contribution that breaks precedent
+• independence becoming impossible to separate from personal visibility</x:v>
       </x:c>
       <x:c r="F92" s="45" t="str">
         <x:v>visible difference and personal freedom</x:v>
@@ -4112,9 +4112,9 @@
         <x:v>revision targets routines, methods, and details that no longer work</x:v>
       </x:c>
       <x:c r="E93" s="45" t="str">
-        <x:v>• the proposed change tested against the details
-• a correction changing room for independence
-• usefulness becoming the measure of the arrangement being revised</x:v>
+        <x:v>• a routine revised when the old method stops solving the problem
+• one technical change altering how the work is distributed
+• independence gained through a more useful process</x:v>
       </x:c>
       <x:c r="F93" s="45" t="str">
         <x:v>revision of routines and methods</x:v>
@@ -4146,9 +4146,9 @@
         <x:v>freedom pressures agreements to change their terms of fairness and reciprocity</x:v>
       </x:c>
       <x:c r="E94" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the proposed change
-• room for independence needing clearer shared terms
-• reciprocity becoming part of the arrangement being revised</x:v>
+        <x:v>• an agreement reopening because equal treatment no longer produces a fair result
+• independence changing the terms of mutual obligation
+• a different arrangement becoming possible once reciprocity is redefined</x:v>
       </x:c>
       <x:c r="F94" s="45" t="str">
         <x:v>freedom changing fair agreements</x:v>
@@ -4180,9 +4180,9 @@
         <x:v>disruption exposes hidden leverage, private stakes, and arrangements that cannot be restored</x:v>
       </x:c>
       <x:c r="E95" s="45" t="str">
-        <x:v>• hidden leverage affecting the proposed change
-• privacy determining access to room for independence
-• the arrangement being revised carrying consequences that are hard to reverse</x:v>
+        <x:v>• hidden leverage exposed by a change no one can reverse
+• private access disrupted before trust can be renegotiated
+• independence altering who controls the most consequential information</x:v>
       </x:c>
       <x:c r="F95" s="45" t="str">
         <x:v>disruption exposing private leverage</x:v>
@@ -4214,9 +4214,9 @@
         <x:v>independence widens the horizon faster than existing beliefs or plans can contain</x:v>
       </x:c>
       <x:c r="E96" s="45" t="str">
-        <x:v>• a larger promise stretching the proposed change
-• conviction setting the direction for room for independence
-• distance changing what seems possible for the arrangement being revised</x:v>
+        <x:v>• a sudden opening widening the distance people can imagine crossing
+• independence challenging a belief that once set the horizon
+• change moving farther than the original plan was built to contain</x:v>
       </x:c>
       <x:c r="F96" s="45" t="str">
         <x:v>independence widening belief and distance</x:v>
@@ -4250,9 +4250,9 @@
         <x:v>change challenges authority, duty, and structures built to last</x:v>
       </x:c>
       <x:c r="E97" s="45" t="str">
-        <x:v>• authority setting the workable limit for the proposed change
-• duty continuing after decisions about room for independence
-• long-term consequence outweighing immediate relief in the arrangement being revised</x:v>
+        <x:v>• a long-standing authority losing control of the structure it maintained
+• independence forced into a system designed to resist quick revision
+• change becoming durable only after responsibility is reassigned</x:v>
       </x:c>
       <x:c r="F97" s="45" t="str">
         <x:v>change confronting authority and structure</x:v>
@@ -4284,9 +4284,9 @@
         <x:v>independence and system change reinforce each other until the old arrangement cannot hold</x:v>
       </x:c>
       <x:c r="E98" s="45" t="str">
-        <x:v>• the proposed change being measured against group policy
-• precedent shaping room for independence
-• the arrangement being revised being expected to apply equally</x:v>
+        <x:v>• a group redesigning the rule that once limited its own independence
+• system change spreading because the exception reveals a wider problem
+• difference becoming part of the shared arrangement rather than outside it</x:v>
       </x:c>
       <x:c r="F98" s="45" t="str">
         <x:v>independence and system change reinforcing each other</x:v>
@@ -4318,9 +4318,9 @@
         <x:v>disruption moves through intuition, uncertainty, and boundaries already hard to define</x:v>
       </x:c>
       <x:c r="E99" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the proposed change
-• uncertainty making room for independence difficult to define
-• porous boundaries complicating the arrangement being revised</x:v>
+        <x:v>• a sudden intuition disrupting a boundary that was already unclear
+• independence appearing where people had mistaken sympathy for agreement
+• change moving through a shared feeling before anyone can define the plan</x:v>
       </x:c>
       <x:c r="F99" s="45" t="str">
         <x:v>intuitive disruption and uncertain boundaries</x:v>
@@ -4352,9 +4352,9 @@
         <x:v>imagination rushes toward a beginning before the direction is fully clear</x:v>
       </x:c>
       <x:c r="E100" s="45" t="str">
-        <x:v>• the hoped-for outcome being claimed before others agree
-• pressure to move first on uncertain information
-• delay around the boundary in question being treated as lost control</x:v>
+        <x:v>• a collective hope rushing into action before its direction is understood
+• an ideal making the first move feel clearer than the evidence does
+• uncertainty hidden by the urgency of beginning</x:v>
       </x:c>
       <x:c r="F100" s="45" t="str">
         <x:v>collective ideals rushing toward an uncertain beginning</x:v>
@@ -4388,9 +4388,9 @@
         <x:v>ideals attach to comfort, value, and material security in ways that can blur the true cost</x:v>
       </x:c>
       <x:c r="E101" s="45" t="str">
-        <x:v>• the hoped-for outcome measured against cost and durability
-• uncertain information slowed by what must be preserved
-• the boundary in question judged by whether it can be maintained</x:v>
+        <x:v>• comfort carrying an idealized value that obscures the real cost
+• material security trusted because it feels familiar rather than verified
+• a shared hope attaching to something people want to preserve</x:v>
       </x:c>
       <x:c r="F101" s="45" t="str">
         <x:v>idealized security and uncertain value</x:v>
@@ -4424,9 +4424,9 @@
         <x:v>uncertainty spreads through information, comparison, and explanations that keep changing</x:v>
       </x:c>
       <x:c r="E102" s="45" t="str">
-        <x:v>• new information changing the hoped-for outcome
-• several explanations competing around uncertain information
-• the boundary in question being revised as the terms move</x:v>
+        <x:v>• several plausible explanations blurring which fact deserves trust
+• an implied meaning circulating without a stable source
+• information becoming more persuasive as its boundaries become less exact</x:v>
       </x:c>
       <x:c r="F102" s="45" t="str">
         <x:v>uncertainty spreading through information</x:v>
@@ -4460,9 +4460,9 @@
         <x:v>feeling and memory soften the line between care, loyalty, and projection</x:v>
       </x:c>
       <x:c r="E103" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the hoped-for outcome
-• private consequences shaping uncertain information
-• protection taking priority in decisions about the boundary in question</x:v>
+        <x:v>• memory softening the difference between care and projection
+• a private longing shaping what the group believes it needs
+• belonging idealized until unequal emotional labor becomes hard to see</x:v>
       </x:c>
       <x:c r="F103" s="45" t="str">
         <x:v>memory, care, and projection</x:v>
@@ -4494,9 +4494,9 @@
         <x:v>visibility can carry hope, glamour, or an idealized picture of individual contribution</x:v>
       </x:c>
       <x:c r="E104" s="45" t="str">
-        <x:v>• the hoped-for outcome needing visible acknowledgment
-• personal ownership becoming part of uncertain information
-• the boundary in question being distinguished from the group response</x:v>
+        <x:v>• a public image carrying more hope than the contribution can support
+• recognition attaching to the story people want to believe
+• individual visibility becoming a screen for a collective ideal</x:v>
       </x:c>
       <x:c r="F104" s="45" t="str">
         <x:v>idealized visibility and contribution</x:v>
@@ -4530,9 +4530,9 @@
         <x:v>ideals meet the demand for useful details, workable methods, and proof</x:v>
       </x:c>
       <x:c r="E105" s="45" t="str">
-        <x:v>• the hoped-for outcome tested against the details
-• a correction changing uncertain information
-• usefulness becoming the measure of the boundary in question</x:v>
+        <x:v>• an ideal meeting the practical detail it cannot explain away
+• uncertainty exposed when the method has to produce a usable result
+• compassion losing clarity around what actually needs correction</x:v>
       </x:c>
       <x:c r="F105" s="45" t="str">
         <x:v>ideals tested by practical proof</x:v>
@@ -4564,9 +4564,9 @@
         <x:v>agreement becomes shaped by an ideal of fairness that may hide unequal terms</x:v>
       </x:c>
       <x:c r="E106" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the hoped-for outcome
-• uncertain information needing clearer shared terms
-• reciprocity becoming part of the boundary in question</x:v>
+        <x:v>• an image of fairness hiding which side keeps absorbing the cost
+• agreement sustained by avoiding the unequal term underneath it
+• shared ideals blurring the point where reciprocity stopped</x:v>
       </x:c>
       <x:c r="F106" s="45" t="str">
         <x:v>ideal fairness and unequal terms</x:v>
@@ -4598,9 +4598,9 @@
         <x:v>uncertainty deepens around trust, privacy, and power that is difficult to name</x:v>
       </x:c>
       <x:c r="E107" s="45" t="str">
-        <x:v>• hidden leverage affecting the hoped-for outcome
-• privacy determining access to uncertain information
-• the boundary in question carrying consequences that are hard to reverse</x:v>
+        <x:v>• trust deepening around a motive no one can fully name
+• private power becoming harder to locate as boundaries soften
+• an irreversible choice shaped by information that remains uncertain</x:v>
       </x:c>
       <x:c r="F107" s="45" t="str">
         <x:v>uncertain trust and hidden power</x:v>
@@ -4634,9 +4634,9 @@
         <x:v>belief and possibility expand beyond what the supporting facts can hold</x:v>
       </x:c>
       <x:c r="E108" s="45" t="str">
-        <x:v>• a larger promise stretching the hoped-for outcome
-• conviction setting the direction for uncertain information
-• distance changing what seems possible for the boundary in question</x:v>
+        <x:v>• a belief growing beyond what its supporting facts can carry
+• hope widening the horizon while obscuring the practical distance
+• a collective ideal becoming difficult to separate from certainty</x:v>
       </x:c>
       <x:c r="F108" s="45" t="str">
         <x:v>belief outrunning supporting facts</x:v>
@@ -4668,9 +4668,9 @@
         <x:v>ideals are pressed against authority, duty, and consequences that require clear limits</x:v>
       </x:c>
       <x:c r="E109" s="45" t="str">
-        <x:v>• authority setting the workable limit for the hoped-for outcome
-• duty continuing after decisions about uncertain information
-• long-term consequence outweighing immediate relief in the boundary in question</x:v>
+        <x:v>• an institution asked to formalize a need it cannot clearly define
+• authority lending certainty to an ideal that still lacks limits
+• responsibility blurred by a structure built around appearances</x:v>
       </x:c>
       <x:c r="F109" s="45" t="str">
         <x:v>ideals pressed against duty and consequence</x:v>
@@ -4702,9 +4702,9 @@
         <x:v>collective hopes gather around systems, reform, and futures not yet defined</x:v>
       </x:c>
       <x:c r="E110" s="45" t="str">
-        <x:v>• the hoped-for outcome being measured against group policy
-• precedent shaping uncertain information
-• the boundary in question being expected to apply equally</x:v>
+        <x:v>• collective hope gathering around a system that does not yet exist
+• an imagined reform obscuring who would carry its actual cost
+• group ideals making uncertain access feel universally available</x:v>
       </x:c>
       <x:c r="F110" s="45" t="str">
         <x:v>collective hope and imagined reform</x:v>
@@ -4736,9 +4736,9 @@
         <x:v>imagination, empathy, and uncertainty become difficult to separate from one another</x:v>
       </x:c>
       <x:c r="E111" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the hoped-for outcome
-• uncertainty making uncertain information difficult to define
-• porous boundaries complicating the boundary in question</x:v>
+        <x:v>• empathy dissolving the line between shared feeling and shared duty
+• imagination expanding where facts cannot set a firm boundary
+• a collective longing becoming the atmosphere around the decision</x:v>
       </x:c>
       <x:c r="F111" s="45" t="str">
         <x:v>imagination and uncertainty dissolving the boundary between them</x:v>
@@ -4770,9 +4770,9 @@
         <x:v>power concentrates in who moves first, takes control, or refuses to wait</x:v>
       </x:c>
       <x:c r="E112" s="45" t="str">
-        <x:v>• the source of leverage being claimed before others agree
-• pressure to move first on control of the decision
-• delay around the change that cannot be reversed being treated as lost control</x:v>
+        <x:v>• leverage taken before anyone agrees it is in play
+• the first decisive move concentrating control around one actor
+• power revealed by who can act without waiting for consent</x:v>
       </x:c>
       <x:c r="F112" s="45" t="str">
         <x:v>power in the first move</x:v>
@@ -4804,9 +4804,9 @@
         <x:v>control settles around money, resources, and what people cannot afford to lose</x:v>
       </x:c>
       <x:c r="E113" s="45" t="str">
-        <x:v>• the source of leverage measured against cost and durability
-• control of the decision slowed by what must be preserved
-• the change that cannot be reversed judged by whether it can be maintained</x:v>
+        <x:v>• control settling around the resource people cannot afford to lose
+• a material dependency giving one side durable leverage
+• power becoming visible when security can no longer be assumed</x:v>
       </x:c>
       <x:c r="F113" s="45" t="str">
         <x:v>control of resources and material security</x:v>
@@ -4840,9 +4840,9 @@
         <x:v>leverage moves through information, access, and who controls the explanation</x:v>
       </x:c>
       <x:c r="E114" s="45" t="str">
-        <x:v>• new information changing the source of leverage
-• several explanations competing around control of the decision
-• the change that cannot be reversed being revised as the terms move</x:v>
+        <x:v>• access to the explanation deciding who can shape the outcome
+• one version of the facts becoming leverage over the others
+• control shifting when information reaches a wider audience</x:v>
       </x:c>
       <x:c r="F114" s="45" t="str">
         <x:v>information as leverage</x:v>
@@ -4874,9 +4874,9 @@
         <x:v>power reaches into care, family loyalty, and the private bonds that shape belonging</x:v>
       </x:c>
       <x:c r="E115" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the source of leverage
-• private consequences shaping control of the decision
-• protection taking priority in decisions about the change that cannot be reversed</x:v>
+        <x:v>• family loyalty giving private influence public consequence
+• care turning into leverage where belonging feels conditional
+• control hidden inside the role that protects the household</x:v>
       </x:c>
       <x:c r="F115" s="45" t="str">
         <x:v>power inside care and family loyalty</x:v>
@@ -4908,9 +4908,9 @@
         <x:v>control becomes visible through recognition, authority, and ownership of the public role</x:v>
       </x:c>
       <x:c r="E116" s="45" t="str">
-        <x:v>• the source of leverage needing visible acknowledgment
-• personal ownership becoming part of control of the decision
-• the change that cannot be reversed being distinguished from the group response</x:v>
+        <x:v>• ownership of the public role becoming a source of control
+• recognition deciding whose authority appears legitimate
+• power concentrating around the person identified with the outcome</x:v>
       </x:c>
       <x:c r="F116" s="45" t="str">
         <x:v>visible authority and ownership</x:v>
@@ -4942,9 +4942,9 @@
         <x:v>pressure exposes who sets the method, defines usefulness, and decides what must be corrected</x:v>
       </x:c>
       <x:c r="E117" s="45" t="str">
-        <x:v>• the source of leverage tested against the details
-• a correction changing control of the decision
-• usefulness becoming the measure of the change that cannot be reversed</x:v>
+        <x:v>• control exercised through the method everyone must use
+• one required correction exposing who defines acceptable work
+• leverage appearing in the power to call something defective</x:v>
       </x:c>
       <x:c r="F117" s="45" t="str">
         <x:v>control of methods and correction</x:v>
@@ -4978,9 +4978,9 @@
         <x:v>power enters agreements through fairness claims, compromise, and who keeps yielding</x:v>
       </x:c>
       <x:c r="E118" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the source of leverage
-• control of the decision needing clearer shared terms
-• reciprocity becoming part of the change that cannot be reversed</x:v>
+        <x:v>• compromise revealing which side has been yielding to preserve the agreement
+• fairness language used to conceal unequal control
+• power shifting when reciprocal terms become enforceable</x:v>
       </x:c>
       <x:c r="F118" s="45" t="str">
         <x:v>power hidden inside compromise</x:v>
@@ -5012,9 +5012,9 @@
         <x:v>privacy, leverage, and irreversible change intensify each other</x:v>
       </x:c>
       <x:c r="E119" s="45" t="str">
-        <x:v>• hidden leverage affecting the source of leverage
-• privacy determining access to control of the decision
-• the change that cannot be reversed carrying consequences that are hard to reverse</x:v>
+        <x:v>• private leverage intensifying because the consequence cannot be reversed
+• control depending on access to what others cannot safely disclose
+• power becoming undeniable when trust and survival meet</x:v>
       </x:c>
       <x:c r="F119" s="45" t="str">
         <x:v>privacy and leverage carrying irreversible stakes</x:v>
@@ -5048,9 +5048,9 @@
         <x:v>conviction and larger aims reveal who can define the truth or extend the reach</x:v>
       </x:c>
       <x:c r="E120" s="45" t="str">
-        <x:v>• a larger promise stretching the source of leverage
-• conviction setting the direction for control of the decision
-• distance changing what seems possible for the change that cannot be reversed</x:v>
+        <x:v>• authority growing around who can define the larger truth
+• a belief extending power beyond its original boundary
+• control moving through the institution that grants wider reach</x:v>
       </x:c>
       <x:c r="F120" s="45" t="str">
         <x:v>conviction defining truth and reach</x:v>
@@ -5082,9 +5082,9 @@
         <x:v>control works through institutions, duty, and structures with lasting consequence</x:v>
       </x:c>
       <x:c r="E121" s="45" t="str">
-        <x:v>• authority setting the workable limit for the source of leverage
-• duty continuing after decisions about control of the decision
-• long-term consequence outweighing immediate relief in the change that cannot be reversed</x:v>
+        <x:v>• institutional power becoming visible in who assigns lasting duty
+• control secured through a structure that outlives the immediate dispute
+• authority concentrating where consequences are formally enforced</x:v>
       </x:c>
       <x:c r="F121" s="45" t="str">
         <x:v>institutional control and lasting consequence</x:v>
@@ -5116,9 +5116,9 @@
         <x:v>power shifts through groups, systems, and the rules governing independence</x:v>
       </x:c>
       <x:c r="E122" s="45" t="str">
-        <x:v>• the source of leverage being measured against group policy
-• precedent shaping control of the decision
-• the change that cannot be reversed being expected to apply equally</x:v>
+        <x:v>• group rules redistributing power across an entire system
+• collective pressure exposing who benefits from the current arrangement
+• control changing hands when independence becomes structurally possible</x:v>
       </x:c>
       <x:c r="F122" s="45" t="str">
         <x:v>power shifting through groups and systems</x:v>
@@ -5150,9 +5150,9 @@
         <x:v>control becomes harder to locate where boundaries, ideals, and collective feeling blur</x:v>
       </x:c>
       <x:c r="E123" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the source of leverage
-• uncertainty making control of the decision difficult to define
-• porous boundaries complicating the change that cannot be reversed</x:v>
+        <x:v>• power becoming difficult to locate inside a shared emotional field
+• control operating through an ideal no single person appears to own
+• leverage increasing where boundaries and responsibility remain diffuse</x:v>
       </x:c>
       <x:c r="F123" s="45" t="str">
         <x:v>diffuse control inside collective feeling</x:v>
@@ -5184,9 +5184,9 @@
         <x:v>sensitivity gathers around the right to act, begin, and assert independence</x:v>
       </x:c>
       <x:c r="E124" s="45" t="str">
-        <x:v>• the sensitive point being claimed before others agree
-• pressure to move first on an old defense
-• delay around the pain still shaping the response being treated as lost control</x:v>
+        <x:v>• hesitation around acting first after initiative was once punished
+• a strong reaction when independence is treated as selfishness
+• pain resurfacing at the moment someone has to claim the right to begin</x:v>
       </x:c>
       <x:c r="F124" s="45" t="str">
         <x:v>sensitivity around action and independence</x:v>
@@ -5218,9 +5218,9 @@
         <x:v>pain becomes attached to worth, material security, and what feels safe to keep</x:v>
       </x:c>
       <x:c r="E125" s="45" t="str">
-        <x:v>• the sensitive point measured against cost and durability
-• an old defense slowed by what must be preserved
-• the pain still shaping the response judged by whether it can be maintained</x:v>
+        <x:v>• worth becoming sensitive where material safety has been unreliable
+• difficulty trusting comfort that could still be taken away
+• an old defense returning when resources determine who gets to stay secure</x:v>
       </x:c>
       <x:c r="F125" s="45" t="str">
         <x:v>pain tied to worth and material security</x:v>
@@ -5252,9 +5252,9 @@
         <x:v>sensitivity is carried through language, understanding, and the fear of being misread</x:v>
       </x:c>
       <x:c r="E126" s="45" t="str">
-        <x:v>• new information changing the sensitive point
-• several explanations competing around an old defense
-• the pain still shaping the response being revised as the terms move</x:v>
+        <x:v>• careful wording shaped by the fear of being misunderstood again
+• a question carrying the memory of not being believed
+• sensitivity appearing when several explanations exclude the lived one</x:v>
       </x:c>
       <x:c r="F126" s="45" t="str">
         <x:v>sensitivity around language and being understood</x:v>
@@ -5286,9 +5286,9 @@
         <x:v>old pain and the need to belong reinforce each other through care and family memory</x:v>
       </x:c>
       <x:c r="E127" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the sensitive point
-• private consequences shaping an old defense
-• protection taking priority in decisions about the pain still shaping the response</x:v>
+        <x:v>• care becoming protective where belonging once felt conditional
+• family memory sharpening a present need for safety
+• old pain returning when private loyalty is asked to prove itself</x:v>
       </x:c>
       <x:c r="F127" s="45" t="str">
         <x:v>belonging pain carried through family memory</x:v>
@@ -5320,9 +5320,9 @@
         <x:v>hurt becomes visible around recognition, pride, and whether contribution is valued</x:v>
       </x:c>
       <x:c r="E128" s="45" t="str">
-        <x:v>• the sensitive point needing visible acknowledgment
-• personal ownership becoming part of an old defense
-• the pain still shaping the response being distinguished from the group response</x:v>
+        <x:v>• recognition touching the earlier fear that contribution would be dismissed
+• visible pride covering uncertainty about whether appreciation will last
+• hurt surfacing when the person doing the work is not named</x:v>
       </x:c>
       <x:c r="F128" s="45" t="str">
         <x:v>visible hurt around recognition</x:v>
@@ -5354,9 +5354,9 @@
         <x:v>sensitivity gathers around usefulness, correction, and the fear of getting it wrong</x:v>
       </x:c>
       <x:c r="E129" s="45" t="str">
-        <x:v>• the sensitive point tested against the details
-• a correction changing an old defense
-• usefulness becoming the measure of the pain still shaping the response</x:v>
+        <x:v>• a small correction reopening the fear of never being useful enough
+• competence becoming a defense against being judged as a burden
+• sensitivity gathering around the detail that others call insignificant</x:v>
       </x:c>
       <x:c r="F129" s="45" t="str">
         <x:v>sensitivity around usefulness and correction</x:v>
@@ -5388,9 +5388,9 @@
         <x:v>pain surfaces in fairness, agreement, and the effort to keep relationships balanced</x:v>
       </x:c>
       <x:c r="E130" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the sensitive point
-• an old defense needing clearer shared terms
-• reciprocity becoming part of the pain still shaping the response</x:v>
+        <x:v>• an unfair term touching an older habit of preserving peace at personal cost
+• pain appearing where agreement requires repeated self-adjustment
+• balance becoming fragile when one side's need is treated as disruption</x:v>
       </x:c>
       <x:c r="F130" s="45" t="str">
         <x:v>pain inside fairness and agreement</x:v>
@@ -5422,9 +5422,9 @@
         <x:v>old pain sits close to trust, privacy, and experiences that cannot be undone</x:v>
       </x:c>
       <x:c r="E131" s="45" t="str">
-        <x:v>• hidden leverage affecting the sensitive point
-• privacy determining access to an old defense
-• the pain still shaping the response carrying consequences that are hard to reverse</x:v>
+        <x:v>• trust activating the memory of a disclosure that carried consequences
+• privacy guarded because some experiences cannot be made harmless afterward
+• old pain shaping how much leverage anyone is allowed to hold</x:v>
       </x:c>
       <x:c r="F131" s="45" t="str">
         <x:v>old pain, privacy, and irreversible experience</x:v>
@@ -5456,9 +5456,9 @@
         <x:v>sensitivity touches belief, meaning, and the freedom to imagine a larger life</x:v>
       </x:c>
       <x:c r="E132" s="45" t="str">
-        <x:v>• a larger promise stretching the sensitive point
-• conviction setting the direction for an old defense
-• distance changing what seems possible for the pain still shaping the response</x:v>
+        <x:v>• a larger promise touching the fear that hope will be punished again
+• belief becoming sensitive when one story is declared universally true
+• pain entering the question of who is free to imagine a different future</x:v>
       </x:c>
       <x:c r="F132" s="45" t="str">
         <x:v>sensitivity around belief and meaning</x:v>
@@ -5490,9 +5490,9 @@
         <x:v>pain is managed through competence, duty, and the pressure to need less</x:v>
       </x:c>
       <x:c r="E133" s="45" t="str">
-        <x:v>• authority setting the workable limit for the sensitive point
-• duty continuing after decisions about an old defense
-• long-term consequence outweighing immediate relief in the pain still shaping the response</x:v>
+        <x:v>• competence used to hide the cost of carrying too much responsibility
+• an old hurt returning when need is treated as failure
+• duty becoming the place where vulnerability is least allowed</x:v>
       </x:c>
       <x:c r="F133" s="45" t="str">
         <x:v>pain managed through duty and competence</x:v>
@@ -5524,9 +5524,9 @@
         <x:v>sensitivity gathers around exclusion, difference, and belonging inside a group</x:v>
       </x:c>
       <x:c r="E134" s="45" t="str">
-        <x:v>• the sensitive point being measured against group policy
-• precedent shaping an old defense
-• the pain still shaping the response being expected to apply equally</x:v>
+        <x:v>• group belonging tested by whether difference is tolerated in practice
+• exclusion remembered when a shared rule erases a particular need
+• sensitivity gathering around being useful to the group but not known by it</x:v>
       </x:c>
       <x:c r="F134" s="45" t="str">
         <x:v>sensitivity around exclusion and group belonging</x:v>
@@ -5558,9 +5558,9 @@
         <x:v>old pain can blur into empathy, longing, and the wish to make suffering meaningful</x:v>
       </x:c>
       <x:c r="E135" s="45" t="str">
-        <x:v>• feeling affecting what can be promised about the sensitive point
-• uncertainty making an old defense difficult to define
-• porous boundaries complicating the pain still shaping the response</x:v>
+        <x:v>• empathy reopening pain that has not been clearly separated from others
+• longing making an old loss feel collectively meaningful
+• sensitivity spreading where care has no agreed boundary</x:v>
       </x:c>
       <x:c r="F135" s="45" t="str">
         <x:v>pain diffused through empathy and longing</x:v>
@@ -5592,9 +5592,9 @@
         <x:v>refusal becomes a direct claim to act without waiting for approval</x:v>
       </x:c>
       <x:c r="E136" s="45" t="str">
-        <x:v>• the refusal being claimed before others agree
-• pressure to move first on the excluded position
-• delay around the demand deemed unacceptable being treated as lost control</x:v>
+        <x:v>• a refusal stated before anyone grants the right to object
+• autonomy claimed through the act others call premature
+• the excluded position forcing its way into the decision</x:v>
       </x:c>
       <x:c r="F136" s="45" t="str">
         <x:v>direct refusal and autonomous action</x:v>
@@ -5624,9 +5624,9 @@
         <x:v>autonomy gathers around the body, resources, and what will not be surrendered</x:v>
       </x:c>
       <x:c r="E137" s="45" t="str">
-        <x:v>• the refusal measured against cost and durability
-• the excluded position slowed by what must be preserved
-• the demand deemed unacceptable judged by whether it can be maintained</x:v>
+        <x:v>• a boundary forming around the body or resource others expect to use
+• refusal becoming firm when security requires surrender
+• autonomy measured by what can be kept without apology</x:v>
       </x:c>
       <x:c r="F137" s="45" t="str">
         <x:v>bodily autonomy and protected resources</x:v>
@@ -5656,9 +5656,9 @@
         <x:v>refusal moves through naming the contradiction and rejecting a single approved version</x:v>
       </x:c>
       <x:c r="E138" s="45" t="str">
-        <x:v>• new information changing the refusal
-• several explanations competing around the excluded position
-• the demand deemed unacceptable being revised as the terms move</x:v>
+        <x:v>• a contradiction spoken after the approved explanation stops holding
+• refusal moving between versions that authority wanted reduced to one
+• autonomy preserved through naming what the official language leaves out</x:v>
       </x:c>
       <x:c r="F138" s="45" t="str">
         <x:v>refusal through contradiction and alternate versions</x:v>
@@ -5688,9 +5688,9 @@
         <x:v>autonomy protects private feeling, belonging, and the right not to perform care</x:v>
       </x:c>
       <x:c r="E139" s="45" t="str">
-        <x:v>• care and belonging changing the handling of the refusal
-• private consequences shaping the excluded position
-• protection taking priority in decisions about the demand deemed unacceptable</x:v>
+        <x:v>• care withheld from a role that expects feeling to be performed
+• private belonging protected from demands for emotional access
+• refusal appearing when loyalty is used to override autonomy</x:v>
       </x:c>
       <x:c r="F139" s="45" t="str">
         <x:v>private autonomy and nonperformed care</x:v>
@@ -5720,9 +5720,9 @@
         <x:v>refusal becomes visible where recognition depends on making oneself acceptable</x:v>
       </x:c>
       <x:c r="E140" s="45" t="str">
-        <x:v>• the refusal needing visible acknowledgment
-• personal ownership becoming part of the excluded position
-• the demand deemed unacceptable being distinguished from the group response</x:v>
+        <x:v>• visibility claimed without making the contribution more acceptable first
+• recognition rejected when it depends on shrinking the difficult part
+• autonomy becoming public where approval had set the terms</x:v>
       </x:c>
       <x:c r="F140" s="45" t="str">
         <x:v>visible refusal of conditional recognition</x:v>
@@ -5752,9 +5752,9 @@
         <x:v>autonomy rejects standards that turn usefulness or purity into a condition of worth</x:v>
       </x:c>
       <x:c r="E141" s="45" t="str">
-        <x:v>• the refusal tested against the details
-• a correction changing the excluded position
-• usefulness becoming the measure of the demand deemed unacceptable</x:v>
+        <x:v>• a standard refused because usefulness has become a condition of worth
+• autonomy defended against correction aimed at making difference manageable
+• the excluded need exposing what the approved method cannot serve</x:v>
       </x:c>
       <x:c r="F141" s="45" t="str">
         <x:v>refusal of purity and usefulness standards</x:v>
@@ -5784,9 +5784,9 @@
         <x:v>refusal exposes agreements that call repeated self-erasure fairness</x:v>
       </x:c>
       <x:c r="E142" s="45" t="str">
-        <x:v>• fairness depending on who adjusts the refusal
-• the excluded position needing clearer shared terms
-• reciprocity becoming part of the demand deemed unacceptable</x:v>
+        <x:v>• an agreement challenged after fairness becomes repeated self-erasure
+• refusal entering the negotiation where politeness had hidden the cost
+• autonomy requiring terms that do not depend on one side yielding</x:v>
       </x:c>
       <x:c r="F142" s="45" t="str">
         <x:v>autonomy exposing unfair agreement</x:v>
@@ -5816,9 +5816,9 @@
         <x:v>autonomy protects desire, privacy, and the right to keep power from being taken</x:v>
       </x:c>
       <x:c r="E143" s="45" t="str">
-        <x:v>• hidden leverage affecting the refusal
-• privacy determining access to the excluded position
-• the demand deemed unacceptable carrying consequences that are hard to reverse</x:v>
+        <x:v>• desire protected from someone else's claim to private access
+• refusal becoming final where trust has been used as leverage
+• autonomy holding back what cannot be safely recovered once given</x:v>
       </x:c>
       <x:c r="F143" s="45" t="str">
         <x:v>protected desire, privacy, and power</x:v>
@@ -5848,9 +5848,9 @@
         <x:v>refusal breaks with beliefs or rules that make freedom conditional</x:v>
       </x:c>
       <x:c r="E144" s="45" t="str">
-        <x:v>• a larger promise stretching the refusal
-• conviction setting the direction for the excluded position
-• distance changing what seems possible for the demand deemed unacceptable</x:v>
+        <x:v>• a rule rejected when belief is used to make freedom conditional
+• autonomy widening beyond the story that defined acceptable desire
+• refusal exposing who was allowed to name the larger truth</x:v>
       </x:c>
       <x:c r="F144" s="45" t="str">
         <x:v>freedom refusing conditional belief</x:v>
@@ -5880,9 +5880,9 @@
         <x:v>autonomy confronts authority, duty, and respectability used as control</x:v>
       </x:c>
       <x:c r="E145" s="45" t="str">
-        <x:v>• authority setting the workable limit for the refusal
-• duty continuing after decisions about the excluded position
-• long-term consequence outweighing immediate relief in the demand deemed unacceptable</x:v>
+        <x:v>• authority confronted where respectability has been used as control
+• a duty refused because compliance would erase the person carrying it
+• autonomy becoming visible in the consequence someone chooses to accept</x:v>
       </x:c>
       <x:c r="F145" s="45" t="str">
         <x:v>autonomy against authority and respectability</x:v>
@@ -5912,9 +5912,9 @@
         <x:v>refusal tests group norms that praise difference only when it stays manageable</x:v>
       </x:c>
       <x:c r="E146" s="45" t="str">
-        <x:v>• the refusal being measured against group policy
-• precedent shaping the excluded position
-• the demand deemed unacceptable being expected to apply equally</x:v>
+        <x:v>• a group norm challenged for welcoming difference only in approved forms
+• refusal revealing who remains excluded by a supposedly universal rule
+• autonomy protected from collective pressure to become easier to manage</x:v>
       </x:c>
       <x:c r="F146" s="45" t="str">
         <x:v>refusal inside conditional group belonging</x:v>
@@ -5944,9 +5944,9 @@
         <x:v>autonomy resists being absorbed into other people's feelings, ideals, or need for rescue</x:v>
       </x:c>
       <x:c r="E147" s="46" t="str">
-        <x:v>• feeling affecting what can be promised about the refusal
-• uncertainty making the excluded position difficult to define
-• porous boundaries complicating the demand deemed unacceptable</x:v>
+        <x:v>• an emotional demand refused before empathy becomes absorption
+• autonomy held where other people's ideals blur personal boundaries
+• the excluded feeling named without turning it into a request for rescue</x:v>
       </x:c>
       <x:c r="F147" s="46" t="str">
         <x:v>autonomy against emotional absorption</x:v>
@@ -5977,7 +5977,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f4d033756054ad0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9939ef307de4265"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6209,7 +6209,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R397045f1fdf9464e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15de5eab2f0f499a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6555,7 +6555,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73e76d5187ad41ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ba895a27a7d4106"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7051,7 +7051,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b9db36d1ca84240"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cc2e559d5f04ef9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7249,23 +7249,43 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+      <x:c r="A11" s="26" t="str">
         <x:v>Verbatim component emission</x:v>
       </x:c>
-      <x:c r="B11" s="27" t="str">
+      <x:c r="B11" s="26" t="str">
         <x:v>All components</x:v>
       </x:c>
-      <x:c r="C11" s="27" t="n">
+      <x:c r="C11" s="26" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D11" s="27" t="str">
+      <x:c r="D11" s="26" t="str">
         <x:v>Composer paraphrases and integrates</x:v>
       </x:c>
-      <x:c r="E11" s="27" t="str">
+      <x:c r="E11" s="26" t="str">
         <x:v>A stored component appears as a full sentence</x:v>
       </x:c>
-      <x:c r="F11" s="27" t="str">
+      <x:c r="F11" s="26" t="str">
         <x:v>Components govern meaning, not prose</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
+        <x:v>Manifestation shape reuse</x:v>
+      </x:c>
+      <x:c r="B12" s="27" t="str">
+        <x:v>Sign-unit manifestations</x:v>
+      </x:c>
+      <x:c r="C12" s="27" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D12" s="27" t="str">
+        <x:v>Planet-sign events use distinct grammar</x:v>
+      </x:c>
+      <x:c r="E12" s="27" t="str">
+        <x:v>A sign frame survives after planet nouns are stripped</x:v>
+      </x:c>
+      <x:c r="F12" s="27" t="str">
+        <x:v>String uniqueness alone does not catch slot templates</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7286,6 +7306,9 @@
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="3" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="64" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -7304,22 +7327,40 @@
       <x:c r="E1" s="3" t="str">
         <x:v>Wording-layer QA</x:v>
       </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, or opener monoculture have returned.</x:v>
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, or opener monoculture have returned.</x:v>
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, or opener monoculture have returned.</x:v>
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, or opener monoculture have returned.</x:v>
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, or opener monoculture have returned.</x:v>
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -7338,6 +7379,12 @@
       <x:c r="E4" s="9" t="str">
         <x:v>Distinct bullets</x:v>
       </x:c>
+      <x:c r="G4" s="9" t="str">
+        <x:v>Skeleton occurrence count</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="str">
+        <x:v>Distinct skeletons</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="14" t="str">
@@ -7355,6 +7402,12 @@
       <x:c r="E5" s="10" t="n">
         <x:v>432</x:v>
       </x:c>
+      <x:c r="G5" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H5" s="10" t="n">
+        <x:v>432</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="15" t="str">
@@ -7402,23 +7455,34 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="15" t="str">
-        <x:v>Maximum details-language use</x:v>
+        <x:v>Maximum manifestation skeleton use</x:v>
       </x:c>
       <x:c r="B10" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C10" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="15" t="str">
+        <x:v>Maximum details-language use</x:v>
+      </x:c>
+      <x:c r="B11" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="15" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
+    <x:row r="12">
+      <x:c r="A12" s="16" t="str">
         <x:v>Maximum connective n-gram use</x:v>
       </x:c>
-      <x:c r="B11" s="16" t="n">
+      <x:c r="B12" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C11" s="16" t="n">
+      <x:c r="C12" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -7435,6 +7499,12 @@
       <x:c r="E13" s="9" t="str">
         <x:v>Uses</x:v>
       </x:c>
+      <x:c r="G13" s="9" t="str">
+        <x:v>Manifestation skeleton</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="str">
+        <x:v>Uses</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="19" t="str">
@@ -7449,6 +7519,12 @@
       <x:c r="E14" s="19" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="G14" s="19" t="str">
+        <x:v>{planet} aimed at changing the system rather than winning one exception</x:v>
+      </x:c>
+      <x:c r="H14" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="20" t="str">
@@ -7463,6 +7539,12 @@
       <x:c r="E15" s="20" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="G15" s="20" t="str">
+        <x:v>{planet} altering who controls the most consequential information</x:v>
+      </x:c>
+      <x:c r="H15" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="20" t="str">
@@ -7477,6 +7559,12 @@
       <x:c r="E16" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="G16" s="20" t="str">
+        <x:v>{planet} appearing as the task that keeps a routine from failing</x:v>
+      </x:c>
+      <x:c r="H16" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="20" t="str">
@@ -7491,6 +7579,12 @@
       <x:c r="E17" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="G17" s="20" t="str">
+        <x:v>{planet} appearing in the {planet} to call something defective</x:v>
+      </x:c>
+      <x:c r="H17" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="20" t="str">
@@ -7505,6 +7599,12 @@
       <x:c r="E18" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="G18" s="20" t="str">
+        <x:v>{planet} appearing in what becomes more secure or materially useful</x:v>
+      </x:c>
+      <x:c r="H18" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="20" t="str">
@@ -7519,6 +7619,12 @@
       <x:c r="E19" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="G19" s="20" t="str">
+        <x:v>{planet} appearing when loyalty is used to override {planet}</x:v>
+      </x:c>
+      <x:c r="H19" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="20" t="str">
@@ -7533,6 +7639,12 @@
       <x:c r="E20" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G20" s="20" t="str">
+        <x:v>{planet} appearing when several explanations exclude the lived one</x:v>
+      </x:c>
+      <x:c r="H20" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="20" t="str">
@@ -7547,6 +7659,12 @@
       <x:c r="E21" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G21" s="20" t="str">
+        <x:v>{planet} appearing where agreement requires repeated self adjustment</x:v>
+      </x:c>
+      <x:c r="H21" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="20" t="str">
@@ -7561,6 +7679,12 @@
       <x:c r="E22" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G22" s="20" t="str">
+        <x:v>{planet} appearing where people had mistaken sympathy for agreement</x:v>
+      </x:c>
+      <x:c r="H22" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="20" t="str">
@@ -7575,6 +7699,12 @@
       <x:c r="E23" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G23" s="20" t="str">
+        <x:v>{planet} applied where trust and private access are already at stake</x:v>
+      </x:c>
+      <x:c r="H23" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="20" t="str">
@@ -7589,6 +7719,12 @@
       <x:c r="E24" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G24" s="20" t="str">
+        <x:v>{planet} arriving as quick {planet} rather than discussion</x:v>
+      </x:c>
+      <x:c r="H24" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="20" t="str">
@@ -7603,6 +7739,12 @@
       <x:c r="E25" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G25" s="20" t="str">
+        <x:v>{planet} arriving only after the result proves it can last</x:v>
+      </x:c>
+      <x:c r="H25" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="20" t="str">
@@ -7617,6 +7759,12 @@
       <x:c r="E26" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G26" s="20" t="str">
+        <x:v>{planet} assigned to the choice that shows immediate commitment</x:v>
+      </x:c>
+      <x:c r="H26" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="20" t="str">
@@ -7631,6 +7779,12 @@
       <x:c r="E27" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G27" s="20" t="str">
+        <x:v>{planet} attached to the option that expands independence</x:v>
+      </x:c>
+      <x:c r="H27" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="20" t="str">
@@ -7645,6 +7799,12 @@
       <x:c r="E28" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G28" s="20" t="str">
+        <x:v>{planet} attached to the person expected to answer for the result</x:v>
+      </x:c>
+      <x:c r="H28" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="20" t="str">
@@ -7659,6 +7819,12 @@
       <x:c r="E29" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G29" s="20" t="str">
+        <x:v>{planet} attached to the version that enters the record</x:v>
+      </x:c>
+      <x:c r="H29" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="20" t="str">
@@ -7673,6 +7839,12 @@
       <x:c r="E30" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G30" s="20" t="str">
+        <x:v>{planet} attaching to a shared ideal before its limits are clear</x:v>
+      </x:c>
+      <x:c r="H30" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="20" t="str">
@@ -7687,6 +7859,12 @@
       <x:c r="E31" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G31" s="20" t="str">
+        <x:v>{planet} attaching to an idealized image rather than the actual work</x:v>
+      </x:c>
+      <x:c r="H31" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="20" t="str">
@@ -7701,6 +7879,12 @@
       <x:c r="E32" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G32" s="20" t="str">
+        <x:v>{planet} becoming difficult to locate inside a shared emotional field</x:v>
+      </x:c>
+      <x:c r="H32" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="21" t="str">
@@ -7715,11 +7899,17 @@
       <x:c r="E33" s="21" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="G33" s="21" t="str">
+        <x:v>{planet} becoming durable only after responsibility is reassigned</x:v>
+      </x:c>
+      <x:c r="H33" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:E1"/>
-    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(content): rebuild sky aspect composer v2
</commit_message>
<xml_diff>
--- a/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
+++ b/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2b3e64317f774323"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R14958f6717af420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="Rcdce18c9bf8841ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="4" r:id="R53810ebad924402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="5" r:id="R532b1acd96a440dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="6" r:id="R6349c11e7588440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="7" r:id="R2ff3d032e67541b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="8" r:id="Re11082fc5a0a4d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R99b6b2bef8a54d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R915f1c8416d641c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="Rbf75f1bc4cf04c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="4" r:id="R3bf92c83c2f14c0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="5" r:id="Rb2e1d239ecf0452d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="6" r:id="Re8a4acaf45054423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="7" r:id="R21a9e752c588470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="8" r:id="R5f7c5e084afb40ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -682,10 +682,10 @@
         <x:v>Reader order</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
-        <x:v>4 beats</x:v>
+        <x:v>Forecast 4 / Details 3</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
-        <x:v>What may happen; why it matters; why it sticks or moves; what can move.</x:v>
+        <x:v>Forecast concludes with four hidden meanings. Details explains what may happen, why it matters, and why it sticks or moves.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -8061,7 +8061,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a37e772598a41c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4637b5410a484765"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8293,7 +8293,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe272f37e46b47e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8f56d744aed41a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8639,7 +8639,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re333998586e748b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64755ed10f0f42e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9135,7 +9135,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62b090e4993544e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8109d60c763045f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9174,22 +9174,22 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Beats are required. Connective wording is not. The future composer must vary openers and connective constructions across the corpus.</x:v>
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>Beats are required. Connective wording is not. The future composer must vary openers and connective constructions across the corpus.</x:v>
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Beats are required. Connective wording is not. The future composer must vary openers and connective constructions across the corpus.</x:v>
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>Beats are required. Connective wording is not. The future composer must vary openers and connective constructions across the corpus.</x:v>
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Beats are required. Connective wording is not. The future composer must vary openers and connective constructions across the corpus.</x:v>
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>Beats are required. Connective wording is not. The future composer must vary openers and connective constructions across the corpus.</x:v>
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -9320,16 +9320,16 @@
         <x:v>Each Details block</x:v>
       </x:c>
       <x:c r="C10" s="26" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
-        <x:v>Reader order preserved</x:v>
+        <x:v>Explanation ends after behavior</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
-        <x:v>Planet-by-planet concatenation</x:v>
+        <x:v>Forecast conclusion repeated in Details</x:v>
       </x:c>
       <x:c r="F10" s="26" t="str">
-        <x:v>Astrology explains the reader beats</x:v>
+        <x:v>Forecast concludes; Details explains</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
fix(content): rework sky meaning components
</commit_message>
<xml_diff>
--- a/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
+++ b/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R99b6b2bef8a54d33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R915f1c8416d641c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="Rbf75f1bc4cf04c32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="4" r:id="R3bf92c83c2f14c0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="5" r:id="Rb2e1d239ecf0452d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="6" r:id="Re8a4acaf45054423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="7" r:id="R21a9e752c588470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="8" r:id="R5f7c5e084afb40ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re01cad737e9247b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="Ra122e62e6cf84d77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="R9f74f7a85e5e4bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="4" r:id="R76bfbb742f264571"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="5" r:id="R713bc8c58c7547ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="6" r:id="Re5e3e2eaa2134931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="7" r:id="R182553d3e494424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="8" r:id="R20c75948f1d44dd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -672,10 +672,10 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="13" t="str">
+      <x:c r="A9" s="12" t="str">
         <x:v>Total</x:v>
       </x:c>
-      <x:c r="B9" s="13" t="n">
+      <x:c r="B9" s="12" t="n">
         <x:v>174</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
@@ -688,161 +688,113 @@
         <x:v>Forecast concludes with four hidden meanings. Details explains what may happen, why it matters, and why it sticks or moves.</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="12" t="str">
+        <x:v>Units rechecked</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="n">
+        <x:v>174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="12" t="str">
+        <x:v>Units changed</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="n">
+        <x:v>138</x:v>
+      </x:c>
+    </x:row>
     <x:row r="12">
-      <x:c r="A12" s="17" t="str">
+      <x:c r="A12" s="12" t="str">
+        <x:v>One-sided before pass</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="n">
+        <x:v>39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>One-sided after pass</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="17" t="str">
         <x:v>Field definitions</x:v>
       </x:c>
-      <x:c r="B12" s="17" t="str">
+      <x:c r="B16" s="17" t="str">
         <x:v>Field definitions</x:v>
       </x:c>
-      <x:c r="C12" s="17" t="str">
+      <x:c r="C16" s="17" t="str">
         <x:v>Field definitions</x:v>
       </x:c>
-      <x:c r="D12" s="17" t="str">
+      <x:c r="D16" s="17" t="str">
         <x:v>Field definitions</x:v>
       </x:c>
-      <x:c r="E12" s="17" t="str">
+      <x:c r="E16" s="17" t="str">
         <x:v>Field definitions</x:v>
       </x:c>
-      <x:c r="F12" s="17" t="str">
+      <x:c r="F16" s="17" t="str">
         <x:v>Field definitions</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="18" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="18" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="B13" s="18" t="str">
+      <x:c r="B17" s="18" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C13" s="18" t="str">
+      <x:c r="C17" s="18" t="str">
         <x:v>Purpose</x:v>
       </x:c>
-      <x:c r="D13" s="18" t="str">
+      <x:c r="D17" s="18" t="str">
         <x:v>May render verbatim?</x:v>
       </x:c>
-      <x:c r="E13" s="18" t="str">
+      <x:c r="E17" s="18" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F13" s="18" t="str">
+      <x:c r="F17" s="18" t="str">
         <x:v>Owner action</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="25" t="str">
+    <x:row r="18">
+      <x:c r="A18" s="25" t="str">
         <x:v>planet_function</x:v>
       </x:c>
-      <x:c r="B14" s="25" t="str">
+      <x:c r="B18" s="25" t="str">
         <x:v>Sign</x:v>
       </x:c>
-      <x:c r="C14" s="25" t="str">
+      <x:c r="C18" s="25" t="str">
         <x:v>What the planet governs in this placement</x:v>
       </x:c>
-      <x:c r="D14" s="25" t="str">
+      <x:c r="D18" s="25" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="E14" s="25" t="str">
+      <x:c r="E18" s="25" t="str">
         <x:v>Approved rows and matrices</x:v>
       </x:c>
-      <x:c r="F14" s="25" t="str">
-        <x:v>Approve, revise, or reject</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="26" t="str">
-        <x:v>sign_expression</x:v>
-      </x:c>
-      <x:c r="B15" s="26" t="str">
-        <x:v>Sign</x:v>
-      </x:c>
-      <x:c r="C15" s="26" t="str">
-        <x:v>How the sign changes that function</x:v>
-      </x:c>
-      <x:c r="D15" s="26" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E15" s="26" t="str">
-        <x:v>Approved rows and matrices</x:v>
-      </x:c>
-      <x:c r="F15" s="26" t="str">
-        <x:v>Approve, revise, or reject</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="26" t="str">
-        <x:v>combined_position</x:v>
-      </x:c>
-      <x:c r="B16" s="26" t="str">
-        <x:v>Sign</x:v>
-      </x:c>
-      <x:c r="C16" s="26" t="str">
-        <x:v>Bounded synthesis of planet and sign</x:v>
-      </x:c>
-      <x:c r="D16" s="26" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E16" s="26" t="str">
-        <x:v>Approved rows and matrices</x:v>
-      </x:c>
-      <x:c r="F16" s="26" t="str">
-        <x:v>Approve, revise, or reject</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="26" t="str">
-        <x:v>reader_manifestations</x:v>
-      </x:c>
-      <x:c r="B17" s="26" t="str">
-        <x:v>Sign</x:v>
-      </x:c>
-      <x:c r="C17" s="26" t="str">
-        <x:v>Possible lived forms available to the composer</x:v>
-      </x:c>
-      <x:c r="D17" s="26" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E17" s="26" t="str">
-        <x:v>Approved rows and matrices</x:v>
-      </x:c>
-      <x:c r="F17" s="26" t="str">
-        <x:v>Approve, revise, or reject</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="26" t="str">
-        <x:v>details_language</x:v>
-      </x:c>
-      <x:c r="B18" s="26" t="str">
-        <x:v>Sign</x:v>
-      </x:c>
-      <x:c r="C18" s="26" t="str">
-        <x:v>Compact astrology language for Details</x:v>
-      </x:c>
-      <x:c r="D18" s="26" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E18" s="26" t="str">
-        <x:v>Approved rows and matrices</x:v>
-      </x:c>
-      <x:c r="F18" s="26" t="str">
+      <x:c r="F18" s="25" t="str">
         <x:v>Approve, revise, or reject</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="26" t="str">
-        <x:v>reader_effect</x:v>
+        <x:v>sign_expression</x:v>
       </x:c>
       <x:c r="B19" s="26" t="str">
-        <x:v>Aspect</x:v>
+        <x:v>Sign</x:v>
       </x:c>
       <x:c r="C19" s="26" t="str">
-        <x:v>What becomes noticeable</x:v>
+        <x:v>How the sign changes that function</x:v>
       </x:c>
       <x:c r="D19" s="26" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="E19" s="26" t="str">
-        <x:v>Approved aspect primitive</x:v>
+        <x:v>Approved rows and matrices</x:v>
       </x:c>
       <x:c r="F19" s="26" t="str">
         <x:v>Approve, revise, or reject</x:v>
@@ -850,41 +802,121 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="26" t="str">
-        <x:v>conflict_behavior</x:v>
+        <x:v>combined_position</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Aspect/How</x:v>
+        <x:v>Sign</x:v>
       </x:c>
       <x:c r="C20" s="26" t="str">
-        <x:v>Why the pressure behaves this way</x:v>
+        <x:v>Bounded synthesis of planet and sign</x:v>
       </x:c>
       <x:c r="D20" s="26" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="E20" s="26" t="str">
-        <x:v>Approved aspect, mode, or element evidence</x:v>
+        <x:v>Approved rows and matrices</x:v>
       </x:c>
       <x:c r="F20" s="26" t="str">
         <x:v>Approve, revise, or reject</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="27" t="str">
+      <x:c r="A21" s="26" t="str">
+        <x:v>reader_manifestations</x:v>
+      </x:c>
+      <x:c r="B21" s="26" t="str">
+        <x:v>Sign</x:v>
+      </x:c>
+      <x:c r="C21" s="26" t="str">
+        <x:v>Possible lived forms available to the composer</x:v>
+      </x:c>
+      <x:c r="D21" s="26" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E21" s="26" t="str">
+        <x:v>Approved rows and matrices</x:v>
+      </x:c>
+      <x:c r="F21" s="26" t="str">
+        <x:v>Approve, revise, or reject</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="26" t="str">
+        <x:v>details_language</x:v>
+      </x:c>
+      <x:c r="B22" s="26" t="str">
+        <x:v>Sign</x:v>
+      </x:c>
+      <x:c r="C22" s="26" t="str">
+        <x:v>Compact astrology language for Details</x:v>
+      </x:c>
+      <x:c r="D22" s="26" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E22" s="26" t="str">
+        <x:v>Approved rows and matrices</x:v>
+      </x:c>
+      <x:c r="F22" s="26" t="str">
+        <x:v>Approve, revise, or reject</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="26" t="str">
+        <x:v>reader_effect</x:v>
+      </x:c>
+      <x:c r="B23" s="26" t="str">
+        <x:v>Aspect</x:v>
+      </x:c>
+      <x:c r="C23" s="26" t="str">
+        <x:v>What becomes noticeable</x:v>
+      </x:c>
+      <x:c r="D23" s="26" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E23" s="26" t="str">
+        <x:v>Approved aspect primitive</x:v>
+      </x:c>
+      <x:c r="F23" s="26" t="str">
+        <x:v>Approve, revise, or reject</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="26" t="str">
+        <x:v>conflict_behavior</x:v>
+      </x:c>
+      <x:c r="B24" s="26" t="str">
+        <x:v>Aspect/How</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>Why the pressure behaves this way</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="str">
+        <x:v>Approved aspect, mode, or element evidence</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="str">
+        <x:v>Approve, revise, or reject</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="27" t="str">
         <x:v>movement_bias</x:v>
       </x:c>
-      <x:c r="B21" s="27" t="str">
+      <x:c r="B25" s="27" t="str">
         <x:v>Aspect/How</x:v>
       </x:c>
-      <x:c r="C21" s="27" t="str">
+      <x:c r="C25" s="27" t="str">
         <x:v>What kind of change is supported</x:v>
       </x:c>
-      <x:c r="D21" s="27" t="str">
+      <x:c r="D25" s="27" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="E21" s="27" t="str">
+      <x:c r="E25" s="27" t="str">
         <x:v>Approved aspect, mode, or element evidence</x:v>
       </x:c>
-      <x:c r="F21" s="27" t="str">
+      <x:c r="F25" s="27" t="str">
         <x:v>Approve, revise, or reject</x:v>
       </x:c>
     </x:row>
@@ -892,7 +924,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A12:F12"/>
+    <x:mergeCell ref="A16:F16"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1402,9 +1434,9 @@
         <x:v>whoever moves first often becomes the face of the work</x:v>
       </x:c>
       <x:c r="E4" s="44" t="str">
-        <x:v>• credit claimed before anyone agrees the work is finished
+        <x:v>• someone claiming credit before anyone agrees the work is finished
 • the person who starts the project becoming its public face
-• recognition following the first visible move rather than the longest contribution</x:v>
+• people recognizing the first visible move instead of the person who carried the work longest</x:v>
       </x:c>
       <x:c r="F4" s="44" t="str">
         <x:v>first moves and claimed visibility</x:v>
@@ -1446,7 +1478,7 @@
       </x:c>
       <x:c r="E5" s="45" t="str">
         <x:v>• a contribution valued because it keeps producing something useful
-• recognition arriving only after the result proves it can last
+• people waiting to give credit until the result proves it can last
 • public credit tied to who protected the budget or the material</x:v>
       </x:c>
       <x:c r="F5" s="45" t="str">
@@ -1489,7 +1521,7 @@
       </x:c>
       <x:c r="E6" s="45" t="str">
         <x:v>• the clearest explanation deciding who is seen as responsible
-• credit moving when a new version of the story circulates
+• people changing who gets credit when a new version of the story circulates
 • several people making a plausible claim to the same idea</x:v>
       </x:c>
       <x:c r="F6" s="45" t="str">
@@ -1531,8 +1563,8 @@
         <x:v>the care people provide in private starts deciding who represents the group</x:v>
       </x:c>
       <x:c r="E7" s="45" t="str">
-        <x:v>• care work becoming the contribution everyone depends on
-• private loyalty shaping who receives public acknowledgment
+        <x:v>• someone doing the care work that everyone else depends on
+• family members using private loyalty to influence who gets acknowledged publicly
 • someone representing the group because they remember its history</x:v>
       </x:c>
       <x:c r="F7" s="45" t="str">
@@ -1619,7 +1651,7 @@
       <x:c r="E9" s="45" t="str">
         <x:v>• the person who catches the error receiving the authority to fix it
 • useful work being noticed after a small failure exposes its value
-• recognition depending on precision rather than display</x:v>
+• people giving credit to the person who got the detail right instead of the best performer</x:v>
       </x:c>
       <x:c r="F9" s="45" t="str">
         <x:v>useful contribution, precision, and correction</x:v>
@@ -1660,7 +1692,7 @@
         <x:v>people have to divide credit without erasing the shared work</x:v>
       </x:c>
       <x:c r="E10" s="45" t="str">
-        <x:v>• credit divided according to the terms people agreed to
+        <x:v>• people dividing credit according to the terms they agreed to
 • a public role changing hands to keep the arrangement fair
 • individual visibility negotiated alongside shared ownership</x:v>
       </x:c>
@@ -1703,9 +1735,9 @@
         <x:v>who gets named publicly depends on trust, privacy, and leverage behind the scenes</x:v>
       </x:c>
       <x:c r="E11" s="45" t="str">
-        <x:v>• recognition withheld until trust and access are settled
+        <x:v>• someone withholding recognition until trust and access are settled
 • the public representative carrying private obligations others cannot see
-• credit becoming leverage in a decision with lasting consequences</x:v>
+• someone using public credit as leverage in a decision with lasting consequences</x:v>
       </x:c>
       <x:c r="F11" s="45" t="str">
         <x:v>recognition and public contribution tied to privacy, trust, and leverage</x:v>
@@ -1747,7 +1779,7 @@
       </x:c>
       <x:c r="E12" s="45" t="str">
         <x:v>• a strong belief making one contribution stand for a larger cause
-• recognition extending beyond the original audience
+• people carrying someone's work to an audience it was not made for
 • the person who names the wider purpose becoming identified with it</x:v>
       </x:c>
       <x:c r="F12" s="45" t="str">
@@ -1789,9 +1821,9 @@
         <x:v>a title goes to the person expected to carry the result</x:v>
       </x:c>
       <x:c r="E13" s="45" t="str">
-        <x:v>• authority granted after someone accepts responsibility for the outcome
+        <x:v>• someone gaining authority after accepting responsibility for the outcome
 • a title reflecting work that has already survived scrutiny
-• recognition attached to the person expected to answer for the result</x:v>
+• people giving credit to the person expected to answer for the result</x:v>
       </x:c>
       <x:c r="F13" s="45" t="str">
         <x:v>recognition through authority and lasting results</x:v>
@@ -1834,7 +1866,7 @@
       <x:c r="E14" s="45" t="str">
         <x:v>• individual credit weighed against what the group built together
 • a public face expected to represent rules that apply to everyone
-• recognition going to the contribution that changes the system</x:v>
+• people crediting the contribution that changes the system</x:v>
       </x:c>
       <x:c r="F14" s="45" t="str">
         <x:v>individual contribution measured against group standards</x:v>
@@ -1876,7 +1908,7 @@
       </x:c>
       <x:c r="E15" s="45" t="str">
         <x:v>• authorship becoming unclear when many people shaped the same vision
-• recognition attaching to an idealized image rather than the actual work
+• people crediting the image they want to believe instead of the work that was done
 • personal contribution fading into a shared emotional response</x:v>
       </x:c>
       <x:c r="F15" s="45" t="str">
@@ -1919,8 +1951,8 @@
       </x:c>
       <x:c r="E16" s="45" t="str">
         <x:v>• an immediate need becoming impossible to postpone
-• care arriving as quick protection rather than discussion
-• belonging tested by who responds when something happens</x:v>
+• someone protecting the person involved before asking what happened
+• someone treating every strong feeling like an emergency that everyone must answer</x:v>
       </x:c>
       <x:c r="F16" s="45" t="str">
         <x:v>urgent needs and immediate emotional action</x:v>
@@ -1965,8 +1997,8 @@
         <x:v>people reach for what they can keep, afford, and count on whenever the mood changes</x:v>
       </x:c>
       <x:c r="E17" s="45" t="str">
-        <x:v>• security measured by whether food, money, or shelter remains dependable
-• comfort preserved even when a faster change is available
+        <x:v>• people judging their security by whether food, money, or shelter remains dependable
+• someone keeping the familiar arrangement even when a faster change is available
 • a familiar routine carrying more emotional weight than the new option</x:v>
       </x:c>
       <x:c r="F17" s="45" t="str">
@@ -2013,8 +2045,8 @@
       </x:c>
       <x:c r="E18" s="45" t="str">
         <x:v>• a mood changing when one more fact enters the conversation
-• care taking the form of keeping people informed
-• belonging negotiated through several competing accounts of what happened</x:v>
+• someone showing care by keeping people informed
+• someone explaining the feeling repeatedly instead of admitting that they are hurt</x:v>
       </x:c>
       <x:c r="F18" s="45" t="str">
         <x:v>changing information and changing feeling</x:v>
@@ -2061,8 +2093,8 @@
         <x:v>the people who remember and provide care set the emotional terms</x:v>
       </x:c>
       <x:c r="E19" s="45" t="str">
-        <x:v>• private needs setting the terms before public plans can continue
-• care becoming more protective when belonging feels uncertain
+        <x:v>• someone bringing a private need into the room before the public plan can continue
+• someone holding the family closer when they are unsure who still belongs
 • family memory making a present response stronger than expected</x:v>
       </x:c>
       <x:c r="F19" s="45" t="str">
@@ -2108,9 +2140,9 @@
         <x:v>someone needs their feeling acknowledged so the group can move on</x:v>
       </x:c>
       <x:c r="E20" s="45" t="str">
-        <x:v>• emotional security rising when care is acknowledged openly
-• hurt becoming visible when appreciation is withheld
-• belonging tied to having a recognizable place in the group</x:v>
+        <x:v>• someone feeling safer after the care they provided is acknowledged openly
+• someone showing their hurt when the expected appreciation never arrives
+• someone feeling they belong after the group gives them a recognizable place</x:v>
       </x:c>
       <x:c r="F20" s="45" t="str">
         <x:v>emotional security through recognition</x:v>
@@ -2155,9 +2187,9 @@
         <x:v>people calm the mood by fixing a practical problem they can name</x:v>
       </x:c>
       <x:c r="E21" s="45" t="str">
-        <x:v>• care appearing as the task that keeps a routine from failing
+        <x:v>• someone doing the overlooked task that keeps the routine from failing
 • unease narrowing attention to the detail that can be corrected
-• emotional relief depending on whether practical help actually works</x:v>
+• someone relaxing only after the practical help actually works</x:v>
       </x:c>
       <x:c r="F21" s="45" t="str">
         <x:v>practical care and corrected routines</x:v>
@@ -2205,8 +2237,8 @@
       </x:c>
       <x:c r="E22" s="45" t="str">
         <x:v>• someone feeling included only after their needs enter the agreement
-• care distributed so one person is not carrying all of it
-• belonging strained by a compromise that looks fair but feels uneven</x:v>
+• people dividing the care so one person is not carrying all of it
+• someone agreeing to keep the peace and swallowing the need that would complicate it</x:v>
       </x:c>
       <x:c r="F22" s="45" t="str">
         <x:v>belonging through fairness and reciprocity</x:v>
@@ -2249,9 +2281,9 @@
         <x:v>people hold back and wait to see who can be trusted with the full feeling</x:v>
       </x:c>
       <x:c r="E23" s="45" t="str">
-        <x:v>• emotional safety depending on who is trusted with private information
-• care becoming guarded after something cannot be taken back
-• belonging deepening where people share the risk of being known</x:v>
+        <x:v>• someone deciding how safe they feel by who can be trusted with private information
+• someone offering less care after a private disclosure changes the trust
+• people feeling closer after each person risks being known honestly</x:v>
       </x:c>
       <x:c r="F23" s="45" t="str">
         <x:v>emotional safety, privacy, and trust</x:v>
@@ -2299,8 +2331,8 @@
       </x:c>
       <x:c r="E24" s="45" t="str">
         <x:v>• a change of place restoring emotional room
-• belonging widening around a shared belief rather than a shared history
-• care expressed by making space for a larger possibility</x:v>
+• people making room for newcomers who share the belief but not the history
+• someone leaving or turning pain into a lesson before they have felt it</x:v>
       </x:c>
       <x:c r="F24" s="45" t="str">
         <x:v>emotional freedom and larger meaning</x:v>
@@ -2347,9 +2379,9 @@
         <x:v>people put the duty first and deal with the feeling after the work is done</x:v>
       </x:c>
       <x:c r="E25" s="45" t="str">
-        <x:v>• needs being postponed until the required work is done
-• care shown by taking responsibility when feelings stay private
-• belonging secured through reliability rather than reassurance</x:v>
+        <x:v>• someone postponing their needs until the required work is done
+• someone showing care by taking responsibility while keeping their feelings private
+• someone relying on repeated follow-through instead of reassurance to know they belong</x:v>
       </x:c>
       <x:c r="F25" s="45" t="str">
         <x:v>emotional needs managed through duty and restraint</x:v>
@@ -2394,9 +2426,9 @@
         <x:v>the group makes room for feeling by stepping back and looking at the pattern</x:v>
       </x:c>
       <x:c r="E26" s="45" t="str">
-        <x:v>• emotional distance protecting room to remain part of the group
-• belonging depending on whether difference is allowed without explanation
-• care organized through a shared system instead of personal closeness</x:v>
+        <x:v>• someone stepping back emotionally so they can remain part of the group
+• people deciding who belongs by whether difference can remain unexplained
+• someone analyzing the group's needs while acting as if they have none</x:v>
       </x:c>
       <x:c r="F26" s="45" t="str">
         <x:v>belonging with distance and independence</x:v>
@@ -2442,8 +2474,8 @@
       </x:c>
       <x:c r="E27" s="45" t="str">
         <x:v>• one person's mood spreading before anyone names it
-• care extending past the point where responsibility is clear
-• belonging felt through empathy even when facts remain uncertain</x:v>
+• someone continuing to help after no one can say who is responsible
+• people feeling connected through empathy even while the facts remain uncertain</x:v>
       </x:c>
       <x:c r="F27" s="45" t="str">
         <x:v>feeling, empathy, and porous boundaries</x:v>
@@ -2492,7 +2524,7 @@
       <x:c r="E28" s="45" t="str">
         <x:v>• a decision announced before every objection has been heard
 • the first explanation setting the terms of the debate
-• new facts treated as reasons to act now rather than wait</x:v>
+• someone deciding before listening and turning the reply into a verbal fight</x:v>
       </x:c>
       <x:c r="F28" s="45" t="str">
         <x:v>direct speech and immediate decisions</x:v>
@@ -2541,7 +2573,7 @@
       <x:c r="E29" s="45" t="str">
         <x:v>• an agreement slowing until the price and practical terms are clear
 • a repeated fact carrying more weight than a clever argument
-• decisions holding once they are written in concrete language</x:v>
+• someone rejecting a new fact because the older explanation feels safer</x:v>
       </x:c>
       <x:c r="F29" s="45" t="str">
         <x:v>concrete terms and durable decisions</x:v>
@@ -2634,8 +2666,8 @@
       </x:c>
       <x:c r="E31" s="45" t="str">
         <x:v>• a practical question carrying the memory of an earlier conversation
-• private consequences changing what can be said in public
-• information being trusted because it arrives through care</x:v>
+• someone changing what they say publicly because the private consequences are real
+• people trusting the information because someone they rely on delivers it carefully</x:v>
       </x:c>
       <x:c r="F31" s="45" t="str">
         <x:v>language carrying memory and private consequence</x:v>
@@ -2680,7 +2712,7 @@
       <x:c r="E32" s="45" t="str">
         <x:v>• an opinion becoming inseparable from who said it
 • the clearest speaker taking visible ownership of the decision
-• language used to defend personal credit as well as the point itself</x:v>
+• someone exaggerating the point because being admired matters more than being understood</x:v>
       </x:c>
       <x:c r="F32" s="45" t="str">
         <x:v>speech as visible personal claim</x:v>
@@ -2774,7 +2806,7 @@
       <x:c r="E34" s="45" t="str">
         <x:v>• a decision moving only after both replies enter the record
 • wording revised to distribute responsibility more fairly
-• the agreement depending on whether each side can answer the same terms</x:v>
+• someone softening the truth until the decision no longer says what it means</x:v>
       </x:c>
       <x:c r="F34" s="45" t="str">
         <x:v>negotiated decisions and shared terms</x:v>
@@ -2819,7 +2851,7 @@
       <x:c r="E35" s="45" t="str">
         <x:v>• access to private information deciding who can act
 • a withheld fact gaining power as the stakes rise
-• language becoming exact because the consequence cannot be reversed</x:v>
+• someone choosing exact words because the consequence cannot be reversed</x:v>
       </x:c>
       <x:c r="F35" s="45" t="str">
         <x:v>private information and trusted access</x:v>
@@ -2909,7 +2941,7 @@
       <x:c r="E37" s="45" t="str">
         <x:v>• formal wording assigning responsibility that continues after the meeting
 • a decision becoming real when an authority records it
-• communication judged by whether it can support a lasting structure</x:v>
+• someone withholding the words until the message sounds colder than intended</x:v>
       </x:c>
       <x:c r="F37" s="45" t="str">
         <x:v>formal language and accountable decisions</x:v>
@@ -2953,8 +2985,8 @@
       </x:c>
       <x:c r="E38" s="45" t="str">
         <x:v>• an idea evaluated by the system it would alter
-• information shared widely enough to change who holds access
-• the group adopting language that makes a new rule possible</x:v>
+• someone sharing information widely enough to change who holds access
+• someone defending the clever idea while ignoring how it lands on the person hearing it</x:v>
       </x:c>
       <x:c r="F38" s="45" t="str">
         <x:v>system-changing ideas and group consequence</x:v>
@@ -2997,7 +3029,7 @@
         <x:v>people understand the tone or image sooner than they agree on the facts</x:v>
       </x:c>
       <x:c r="E39" s="45" t="str">
-        <x:v>• meaning carried by tone when the stated facts remain incomplete
+        <x:v>• people reading the tone when the stated facts remain incomplete
 • an implication spreading faster than anyone can verify it
 • a decision blurred by sympathy for several incompatible accounts</x:v>
       </x:c>
@@ -3047,8 +3079,8 @@
       </x:c>
       <x:c r="E40" s="45" t="str">
         <x:v>• a preference stated clearly enough to force a quick answer
-• attraction growing through direct pursuit instead of careful agreement
-• value assigned to the choice that shows immediate commitment</x:v>
+• someone pursuing the person they want before the terms are clear
+• someone losing interest when the chase becomes an actual relationship</x:v>
       </x:c>
       <x:c r="F40" s="45" t="str">
         <x:v>direct preference and quick agreement</x:v>
@@ -3092,8 +3124,8 @@
       </x:c>
       <x:c r="E41" s="45" t="str">
         <x:v>• an agreement holding because the exchange feels materially worthwhile
-• comfort becoming part of how value is measured
-• affection shown by preserving what people already share</x:v>
+• people counting comfort as part of what makes the agreement worthwhile
+• someone keeping a comfortable arrangement after it has stopped helping either person grow</x:v>
       </x:c>
       <x:c r="F41" s="45" t="str">
         <x:v>lasting value, comfort, and material worth</x:v>
@@ -3140,9 +3172,9 @@
         <x:v>people stay connected through conversation even as the terms remain open</x:v>
       </x:c>
       <x:c r="E42" s="45" t="str">
-        <x:v>• connection growing through the conversation that keeps changing shape
-• interest sustained by more than one possible arrangement
-• shared value revised when people compare what each option offers</x:v>
+        <x:v>• people staying interested because the conversation keeps changing shape
+• people staying interested because more than one arrangement remains possible
+• someone sending mixed signals because every new option feels easier than choosing</x:v>
       </x:c>
       <x:c r="F42" s="45" t="str">
         <x:v>connection through varied conversation</x:v>
@@ -3189,9 +3221,9 @@
         <x:v>people judge the agreement by whether care and loyalty are returned</x:v>
       </x:c>
       <x:c r="E43" s="45" t="str">
-        <x:v>• affection expressed through inclusion in private life
+        <x:v>• someone showing affection by including another person in private life
 • an agreement valued because it protects belonging
-• care determining what people are willing to preserve together</x:v>
+• someone offering care in a way that makes the other person feel obligated to stay</x:v>
       </x:c>
       <x:c r="F43" s="45" t="str">
         <x:v>care, loyalty, and inclusive value</x:v>
@@ -3235,8 +3267,8 @@
       </x:c>
       <x:c r="E44" s="45" t="str">
         <x:v>• appreciation becoming real when it is shown where others can see it
-• affection tied to being chosen distinctly rather than generally included
-• a shared value represented through visible generosity</x:v>
+• someone needing to be chosen distinctly instead of generally included
+• someone creating drama because ordinary affection does not feel like enough proof</x:v>
       </x:c>
       <x:c r="F44" s="45" t="str">
         <x:v>visible affection and personal appreciation</x:v>
@@ -3283,9 +3315,9 @@
         <x:v>someone shows care by fixing the detail that makes life harder</x:v>
       </x:c>
       <x:c r="E45" s="45" t="str">
-        <x:v>• care demonstrated by noticing the strain and reducing it
+        <x:v>• someone showing care by noticing the strain and reducing it
 • an agreement improved through one practical adjustment
-• value measured by whether attention makes daily life work better</x:v>
+• people judging the relationship by whether that attention makes daily life work better</x:v>
       </x:c>
       <x:c r="F45" s="45" t="str">
         <x:v>care through practical attention</x:v>
@@ -3332,9 +3364,9 @@
         <x:v>each side keeps checking whether the exchange is fair and mutual</x:v>
       </x:c>
       <x:c r="E46" s="45" t="str">
-        <x:v>• mutual response becoming the evidence that an agreement is fair
-• affection sustained by terms neither person has to disappear inside
-• shared value defined through balance rather than identical contribution</x:v>
+        <x:v>• both sides responding in ways that show whether the agreement is fair
+• people keeping affection alive through terms that do not erase either person
+• people valuing different contributions when the overall exchange remains balanced</x:v>
       </x:c>
       <x:c r="F46" s="45" t="str">
         <x:v>fairness and mutuality becoming the terms of connection</x:v>
@@ -3381,9 +3413,9 @@
         <x:v>people want closeness but guard the trust and leverage that come with it</x:v>
       </x:c>
       <x:c r="E47" s="45" t="str">
-        <x:v>• desire deepening after trust survives a private disclosure
+        <x:v>• someone wanting more closeness after trust survives a private disclosure
 • an agreement carrying the risk of giving someone real leverage
-• value concentrating around what cannot be casually replaced</x:v>
+• people valuing the bond more once they understand what cannot be replaced</x:v>
       </x:c>
       <x:c r="F47" s="45" t="str">
         <x:v>desire tied to privacy and trust</x:v>
@@ -3426,9 +3458,9 @@
         <x:v>people choose the agreement that leaves more room to grow and explore</x:v>
       </x:c>
       <x:c r="E48" s="45" t="str">
-        <x:v>• connection widening through a shared horizon rather than a fixed plan
-• value following the choice that leaves more room to grow
-• affection expressed by supporting a belief with visible reach</x:v>
+        <x:v>• people choosing each other because they can imagine a wider life together
+• people choosing the option that leaves more room to grow
+• someone leaving when accountability starts to feel like a limit on freedom</x:v>
       </x:c>
       <x:c r="F48" s="45" t="str">
         <x:v>open value and expansive desire</x:v>
@@ -3476,8 +3508,8 @@
       </x:c>
       <x:c r="E49" s="45" t="str">
         <x:v>• an agreement earning value because it can carry responsibility over time
-• affection shown through commitments that survive inconvenience
-• shared worth measured against consequence, status, and durability</x:v>
+• someone showing affection through commitments that survive inconvenience
+• someone treating affection like a transaction because control feels safer than uncertainty</x:v>
       </x:c>
       <x:c r="F49" s="45" t="str">
         <x:v>durable agreement and social responsibility</x:v>
@@ -3524,9 +3556,9 @@
         <x:v>people stay connected by giving each other room inside the group</x:v>
       </x:c>
       <x:c r="E50" s="45" t="str">
-        <x:v>• connection remaining possible because independence is built into the terms
-• shared value forming around a group commitment rather than private closeness
-• affection making room for a difference the old agreement could not hold</x:v>
+        <x:v>• people staying connected because the agreement leaves room for independence
+• people finding common value in a group commitment instead of private closeness
+• someone acting detached while still expecting the connection to remain available</x:v>
       </x:c>
       <x:c r="F50" s="45" t="str">
         <x:v>independent connection within group commitments</x:v>
@@ -3569,9 +3601,9 @@
         <x:v>people can fall for the hope of connection before its actual terms are clear</x:v>
       </x:c>
       <x:c r="E51" s="45" t="str">
-        <x:v>• longing adding value to an arrangement before its limits are visible
-• affection extending beyond what either person has clearly promised
-• shared ideals making unequal terms difficult to notice</x:v>
+        <x:v>• someone valuing an arrangement more because they long for what it could become
+• someone giving more affection than either person has actually promised
+• people overlooking unequal terms because they share the same ideal</x:v>
       </x:c>
       <x:c r="F51" s="45" t="str">
         <x:v>idealized affection and porous longing</x:v>
@@ -3615,7 +3647,7 @@
       </x:c>
       <x:c r="E52" s="45" t="str">
         <x:v>• the first move establishing who controls the pace
-• pressure turning directly into action before a process is agreed
+• someone acting on the pressure before the group agrees on a process
 • a visible result pursued without waiting for broader support</x:v>
       </x:c>
       <x:c r="F52" s="45" t="str">
@@ -3663,9 +3695,9 @@
         <x:v>people keep pushing the same point until a material limit finally moves</x:v>
       </x:c>
       <x:c r="E53" s="45" t="str">
-        <x:v>• effort continuing at the same point until a material limit gives way
-• conflict gathering around a resource no one wants to surrender
-• action delayed until the result can be kept</x:v>
+        <x:v>• someone working the same point until a material limit gives way
+• people arguing over the resource no one wants to surrender
+• someone delaying action until they can keep the result</x:v>
       </x:c>
       <x:c r="F53" s="45" t="str">
         <x:v>slow pressure around resources and fixed limits</x:v>
@@ -3712,8 +3744,8 @@
         <x:v>people spread their effort across messages, errands, debates, and several moving targets</x:v>
       </x:c>
       <x:c r="E54" s="45" t="str">
-        <x:v>• effort divided among several messages, errands, or targets
-• conflict moving with the wording instead of staying on one issue
+        <x:v>• someone dividing their effort among several messages, errands, or targets
+• people changing the argument each time the wording changes
 • a new comparison redirecting action already underway</x:v>
       </x:c>
       <x:c r="F54" s="45" t="str">
@@ -3762,8 +3794,8 @@
       </x:c>
       <x:c r="E55" s="45" t="str">
         <x:v>• defense beginning when home or belonging feels exposed
-• action taken to protect someone before the reason is explained
-• conflict carrying a private vulnerability into a public decision</x:v>
+• someone acting to protect another person before explaining why
+• someone defending a private vulnerability inside a public decision</x:v>
       </x:c>
       <x:c r="F55" s="45" t="str">
         <x:v>action and conflict organized around care and private belonging</x:v>
@@ -3811,8 +3843,8 @@
       </x:c>
       <x:c r="E56" s="45" t="str">
         <x:v>• a bold action tying the outcome to one visible person
-• effort intensifying when pride and recognition are on the line
-• the result pursued in a way that makes ownership unmistakable</x:v>
+• someone pushing harder when pride and recognition are on the line
+• someone turning a disagreement into a contest over who gets respect and attention</x:v>
       </x:c>
       <x:c r="F56" s="45" t="str">
         <x:v>visible action and ownership of the result</x:v>
@@ -3859,9 +3891,9 @@
         <x:v>someone reaches for the tool, finds the flaw, and keeps working until the method functions</x:v>
       </x:c>
       <x:c r="E57" s="45" t="str">
-        <x:v>• energy concentrating on the fault that can actually be repaired
-• conflict narrowing into a dispute about method
-• action continuing through small corrections rather than one large move</x:v>
+        <x:v>• someone putting their energy into the fault that can actually be repaired
+• people narrowing the conflict to a dispute about method
+• someone continuing through small corrections instead of making one large move</x:v>
       </x:c>
       <x:c r="F57" s="45" t="str">
         <x:v>effort focused on repair and method</x:v>
@@ -3909,8 +3941,8 @@
       </x:c>
       <x:c r="E58" s="45" t="str">
         <x:v>• the urge to act slowing long enough to measure the other response
-• conflict entering negotiation before either side gets its preferred result
-• effort redirected toward terms that do not leave one party carrying the cost</x:v>
+• people negotiating the disagreement before either side gets its preferred result
+• people redirecting their effort toward terms that do not leave one party carrying the cost</x:v>
       </x:c>
       <x:c r="F58" s="45" t="str">
         <x:v>action negotiated through fairness and response</x:v>
@@ -3957,8 +3989,8 @@
         <x:v>someone acts carefully because trust, control, and lasting consequences are involved</x:v>
       </x:c>
       <x:c r="E59" s="45" t="str">
-        <x:v>• action withheld until the source of control becomes clear
-• pressure applied where trust and private access are already at stake
+        <x:v>• someone withholding action until the source of control becomes clear
+• someone applying pressure where trust and private access are already at stake
 • a result pursued carefully because it cannot be undone</x:v>
       </x:c>
       <x:c r="F59" s="45" t="str">
@@ -4004,9 +4036,9 @@
         <x:v>people spend energy on the plan that reaches farther and supports a larger claim</x:v>
       </x:c>
       <x:c r="E60" s="45" t="str">
-        <x:v>• effort extending toward the larger target before the near one is settled
-• action gaining force from conviction rather than immediate proof
-• conflict widening when freedom of movement is restricted</x:v>
+        <x:v>• someone reaching for the larger target before finishing the nearer one
+• someone acting more forcefully because conviction matters more than immediate proof
+• people widening the fight when a rule limits where they can go</x:v>
       </x:c>
       <x:c r="F60" s="45" t="str">
         <x:v>action driven by conviction and distance</x:v>
@@ -4051,9 +4083,9 @@
         <x:v>a long deadline rewards the person who can pace the work and carry the result</x:v>
       </x:c>
       <x:c r="E61" s="45" t="str">
-        <x:v>• effort organized around the result an authority will accept
-• pressure sustained through duty after urgency has passed
-• action measured by whether it creates a durable outcome</x:v>
+        <x:v>• someone organizing the work around the result an authority will accept
+• someone sustaining the pressure through duty after the urgency has passed
+• people judging the action by whether it creates a durable outcome</x:v>
       </x:c>
       <x:c r="F61" s="45" t="str">
         <x:v>disciplined effort and durable results</x:v>
@@ -4100,9 +4132,9 @@
         <x:v>people challenge the rule when the old system blocks a different way of acting</x:v>
       </x:c>
       <x:c r="E62" s="45" t="str">
-        <x:v>• conflict gathering around a rule that limits independence
-• action aimed at changing the system rather than winning one exception
-• group pressure building behind a different arrangement</x:v>
+        <x:v>• people challenging the rule that limits how they can act
+• people acting to change the system instead of winning one exception
+• a group pressing for a different arrangement</x:v>
       </x:c>
       <x:c r="F62" s="45" t="str">
         <x:v>pressure for independence and system change</x:v>
@@ -4147,9 +4179,9 @@
         <x:v>someone senses the need to act although the target or boundary is still unclear</x:v>
       </x:c>
       <x:c r="E63" s="45" t="str">
-        <x:v>• effort following an emotional current before the target is defined
-• conflict spreading because the boundary of responsibility stays unclear
-• action losing force when several needs merge into one another</x:v>
+        <x:v>• someone acting on the feeling before they can name the target
+• people drawing more people into the conflict because no one knows who is responsible
+• someone losing momentum when several needs merge into one another</x:v>
       </x:c>
       <x:c r="F63" s="45" t="str">
         <x:v>instinctive action with an unclear target</x:v>
@@ -4197,8 +4229,8 @@
       </x:c>
       <x:c r="E64" s="45" t="str">
         <x:v>• a new opening becoming larger because someone risks moving first
-• confidence building through action before certainty arrives
-• growth attached to the option that expands independence</x:v>
+• someone becoming more confident by acting before certainty arrives
+• people choosing the option that gives them more room to act independently</x:v>
       </x:c>
       <x:c r="F64" s="45" t="str">
         <x:v>growth through risk and first moves</x:v>
@@ -4245,9 +4277,9 @@
         <x:v>people use extra room to build, buy, or preserve what can actually last</x:v>
       </x:c>
       <x:c r="E65" s="45" t="str">
-        <x:v>• opportunity increasing the resources people can actually maintain
+        <x:v>• people using a new opportunity to increase the resources they can maintain
 • a larger promise tested against cost before it is trusted
-• growth appearing in what becomes more secure or materially useful</x:v>
+• people measuring the improvement by what becomes safer or more useful</x:v>
       </x:c>
       <x:c r="F65" s="45" t="str">
         <x:v>sustainable opportunity and material value</x:v>
@@ -4293,8 +4325,8 @@
       </x:c>
       <x:c r="E66" s="45" t="str">
         <x:v>• several small openings becoming available through new information
-• confidence rising as people compare more than one route
-• possibility expanding faster than the decision can narrow</x:v>
+• people getting more confident as they compare more than one route
+• people opening more routes than they have time or attention to follow</x:v>
       </x:c>
       <x:c r="F66" s="45" t="str">
         <x:v>multiple possibilities through information</x:v>
@@ -4341,9 +4373,9 @@
         <x:v>people make more room for care, protection, and a wider sense of belonging</x:v>
       </x:c>
       <x:c r="E67" s="45" t="str">
-        <x:v>• growth taking the form of wider protection or belonging
+        <x:v>• people using new resources to protect or include more of the group
 • an opportunity becoming meaningful because it includes people previously left out
-• confidence increasing where care has made risk feel survivable</x:v>
+• people taking a larger risk after someone makes the consequences feel survivable</x:v>
       </x:c>
       <x:c r="F67" s="45" t="str">
         <x:v>growth through care and belonging</x:v>
@@ -4388,9 +4420,9 @@
         <x:v>people give more freely, and one visible contribution can seem larger</x:v>
       </x:c>
       <x:c r="E68" s="45" t="str">
-        <x:v>• generosity making an individual contribution more visible
+        <x:v>• someone giving enough support to make another person's contribution more visible
 • a larger role becoming possible after someone is publicly trusted
-• confidence spreading through recognition that feels personally earned</x:v>
+• someone promising more than the work can support because the applause feels convincing</x:v>
       </x:c>
       <x:c r="F68" s="45" t="str">
         <x:v>confidence through visible generosity</x:v>
@@ -4436,8 +4468,8 @@
       </x:c>
       <x:c r="E69" s="45" t="str">
         <x:v>• an opportunity proving itself through a useful improvement
-• growth limited to what the details can support
-• confidence increasing after the method produces a measurable result</x:v>
+• people limiting the larger plan to what the details can support
+• people adding corrections until the larger opportunity becomes too small to matter</x:v>
       </x:c>
       <x:c r="F69" s="45" t="str">
         <x:v>useful expansion tested by detail</x:v>
@@ -4482,9 +4514,9 @@
         <x:v>people find more room to move when the terms spread the benefit fairly</x:v>
       </x:c>
       <x:c r="E70" s="45" t="str">
-        <x:v>• benefit widening when the terms distribute it more fairly
+        <x:v>• more people benefiting after the terms distribute the opportunity more fairly
 • an agreement creating an opportunity neither side could reach alone
-• confidence resting on cooperation that remains reciprocal</x:v>
+• people accommodating every side until no one can tell what was actually agreed</x:v>
       </x:c>
       <x:c r="F70" s="45" t="str">
         <x:v>shared opportunity through fair terms</x:v>
@@ -4531,9 +4563,9 @@
         <x:v>people take a larger risk only after trust and leverage are clear</x:v>
       </x:c>
       <x:c r="E71" s="45" t="str">
-        <x:v>• growth requiring enough trust to share real leverage
+        <x:v>• people taking a larger step only after there is enough trust to share real leverage
 • a larger opportunity carrying consequences that cannot be easily reversed
-• confidence changing when hidden stakes become visible</x:v>
+• people changing the size of the risk when the hidden stakes become visible</x:v>
       </x:c>
       <x:c r="F71" s="45" t="str">
         <x:v>growth through trust and reversible stakes</x:v>
@@ -4578,9 +4610,9 @@
         <x:v>people trust the promise enough to keep enlarging it until the limit is easy to miss</x:v>
       </x:c>
       <x:c r="E72" s="45" t="str">
-        <x:v>• belief enlarging the horizon beyond the current limit
+        <x:v>• people looking beyond the current limit because they believe a larger option exists
 • an opportunity reaching farther because its meaning is widely shared
-• confidence rising faster than practical constraints can answer</x:v>
+• people enlarging the promise faster than the practical limits can answer</x:v>
       </x:c>
       <x:c r="F72" s="45" t="str">
         <x:v>growth and belief expanding past visible limits</x:v>
@@ -4625,9 +4657,9 @@
         <x:v>a larger project succeeds only if the budget, timing, and duty can support it</x:v>
       </x:c>
       <x:c r="E73" s="45" t="str">
-        <x:v>• ambition expanding through duties that increase authority
+        <x:v>• someone accepting more responsibility because it also increases their authority
 • an opportunity becoming credible when it fits a long structure
-• growth measured by what can still stand after accountability arrives</x:v>
+• someone lowering the aim early because the first limit looks permanent</x:v>
       </x:c>
       <x:c r="F73" s="45" t="str">
         <x:v>ambition inside duty and hierarchy</x:v>
@@ -4671,12 +4703,12 @@
         <x:v>the group asks whether the same rule applies to everyone</x:v>
       </x:c>
       <x:c r="D74" s="45" t="str">
-        <x:v>people back the reform that promises to reach more of the group</x:v>
+        <x:v>a bigger opportunity gets support when more people can actually use it</x:v>
       </x:c>
       <x:c r="E74" s="45" t="str">
-        <x:v>• possibility widening through a reform meant to reach the whole group
-• confidence gathering around a system people believe can change
-• an opportunity emerging from shared access rather than private advantage</x:v>
+        <x:v>• a program, policy, or opportunity expanding because access is opened to more people
+• a group getting confident enough to challenge a rule that only worked for a few
+• people promising broader access before the system is ready to deliver it</x:v>
       </x:c>
       <x:c r="F74" s="45" t="str">
         <x:v>collective reform and wider opportunity</x:v>
@@ -4721,9 +4753,9 @@
         <x:v>people make more room for compassion while the practical boundary becomes harder to see</x:v>
       </x:c>
       <x:c r="E75" s="45" t="str">
-        <x:v>• hope expanding where empathy loosens an old boundary
-• possibility becoming larger than anyone can yet define
-• confidence attaching to a shared ideal before its limits are clear</x:v>
+        <x:v>• people hoping for more after empathy loosens an old boundary
+• people supporting a possibility no one can define clearly yet
+• people trusting a shared ideal before anyone names its limits</x:v>
       </x:c>
       <x:c r="F75" s="45" t="str">
         <x:v>expansive hope and porous boundaries</x:v>
@@ -4769,8 +4801,8 @@
       </x:c>
       <x:c r="E76" s="45" t="str">
         <x:v>• a limit stopping the first move until responsibility is assigned
-• independence tested by a consequence that cannot be rushed
-• authority requiring proof before action receives backing</x:v>
+• someone proving they can act independently while carrying a consequence that cannot be rushed
+• an authority requiring proof before backing the action</x:v>
       </x:c>
       <x:c r="F76" s="45" t="str">
         <x:v>a deadline against a rushed first move</x:v>
@@ -4815,9 +4847,9 @@
         <x:v>a smaller budget makes people decide what is worth maintaining</x:v>
       </x:c>
       <x:c r="E77" s="45" t="str">
-        <x:v>• responsibility settling on the resource that must not run out
+        <x:v>• someone taking responsibility for the resource that must not run out
 • a material limit forcing people to maintain what they already have
-• progress measured by endurance rather than speed</x:v>
+• people judging progress by endurance instead of speed</x:v>
       </x:c>
       <x:c r="F77" s="45" t="str">
         <x:v>a smaller budget and what must be maintained</x:v>
@@ -4866,7 +4898,7 @@
       <x:c r="E78" s="45" t="str">
         <x:v>• changing language held to a standard that must remain consistent
 • a decision delayed while conflicting facts are documented
-• responsibility attached to the version that enters the record</x:v>
+• someone using skepticism to close the discussion before a new idea can be tested</x:v>
       </x:c>
       <x:c r="F78" s="45" t="str">
         <x:v>rewritten words and decisions with consequences</x:v>
@@ -4913,9 +4945,9 @@
         <x:v>a named responsibility leaves less room for private needs and care</x:v>
       </x:c>
       <x:c r="E79" s="45" t="str">
-        <x:v>• duty falling on the person who protects private continuity
-• care narrowed by a limit on time, money, or capacity
-• belonging tested by obligations that are not distributed equally</x:v>
+        <x:v>• the person protecting private continuity also carrying the duty
+• someone providing less care because time, money, or capacity has reached a limit
+• people questioning whether they belong when the obligations are not distributed equally</x:v>
       </x:c>
       <x:c r="F79" s="45" t="str">
         <x:v>named duty and the private needs it leaves behind</x:v>
@@ -4960,9 +4992,9 @@
         <x:v>anyone seeking recognition has to show they can carry the result</x:v>
       </x:c>
       <x:c r="E80" s="45" t="str">
-        <x:v>• recognition withheld until the visible contribution meets the standard
-• authority limiting how much pride can direct the decision
-• a public role carrying consequences that personal confidence cannot erase</x:v>
+        <x:v>• an authority withholding recognition until the visible contribution meets the standard
+• an authority limiting how much personal pride can direct the decision
+• someone withholding their contribution because uncertain recognition feels too risky</x:v>
       </x:c>
       <x:c r="F80" s="45" t="str">
         <x:v>recognition tested by the ability to carry the result</x:v>
@@ -5007,9 +5039,9 @@
         <x:v>the work improves through repetition, correction, and attention to the small failure</x:v>
       </x:c>
       <x:c r="E81" s="45" t="str">
-        <x:v>• responsibility concentrating in the detail no one else can ignore
+        <x:v>• someone becoming responsible for the detail no one else can ignore
 • a routine becoming stricter after an avoidable error
-• progress depending on correction that can be repeated reliably</x:v>
+• someone correcting every small flaw until the work becomes punishing to finish</x:v>
       </x:c>
       <x:c r="F81" s="45" t="str">
         <x:v>repetition, correction, and work that has to be exact</x:v>
@@ -5055,7 +5087,7 @@
       </x:c>
       <x:c r="E82" s="45" t="str">
         <x:v>• obligation divided according to terms both sides must answer to
-• fairness tested by who carries the consequence of compromise
+• people judging fairness by who carries the consequence of the compromise
 • an agreement becoming binding when accountability is shared</x:v>
       </x:c>
       <x:c r="F82" s="45" t="str">
@@ -5102,8 +5134,8 @@
       </x:c>
       <x:c r="E83" s="45" t="str">
         <x:v>• a limit protecting access to information that cannot be taken back
-• responsibility increasing where control and trust are intertwined
-• authority settling a consequence people had hoped to postpone</x:v>
+• someone carrying more responsibility because they also control the access
+• an authority making the consequence official after people tried to postpone it</x:v>
       </x:c>
       <x:c r="F83" s="45" t="str">
         <x:v>hard limits, controlled access, and lasting consequences</x:v>
@@ -5149,8 +5181,8 @@
       </x:c>
       <x:c r="E84" s="45" t="str">
         <x:v>• a large promise reduced to what can be proved and delivered
-• belief tested by the boundary of an institution or law
-• responsibility following the claim farther than confidence expected</x:v>
+• someone testing a belief against the boundary of an institution or law
+• someone preaching freedom while refusing responsibility for where the claim leads</x:v>
       </x:c>
       <x:c r="F84" s="45" t="str">
         <x:v>large promises tested by proof and delivery</x:v>
@@ -5197,9 +5229,9 @@
         <x:v>the deadline, the duty, and the long result decide whether the structure can hold</x:v>
       </x:c>
       <x:c r="E85" s="45" t="str">
-        <x:v>• authority consolidating around the person who can carry the duty
+        <x:v>• people giving more authority to the person who can carry the duty
 • long consequences deciding which ambition remains workable
-• progress becoming inseparable from structure and accountability</x:v>
+• people making progress only after the work has structure and accountability</x:v>
       </x:c>
       <x:c r="F85" s="45" t="str">
         <x:v>deadlines, duty, and results that take time</x:v>
@@ -5292,8 +5324,8 @@
       </x:c>
       <x:c r="E87" s="45" t="str">
         <x:v>• a formal boundary trying to contain a need that has no clean edge
-• responsibility becoming hard to assign when compassion is widely shared
-• structure holding only where uncertainty is named rather than denied</x:v>
+• people struggling to assign responsibility because everyone feels for the person involved
+• people keeping the plan intact by naming what remains uncertain</x:v>
       </x:c>
       <x:c r="F87" s="45" t="str">
         <x:v>firm boundaries around a changing need</x:v>
@@ -5339,7 +5371,7 @@
       </x:c>
       <x:c r="E88" s="45" t="str">
         <x:v>• an unexpected first move changing who has room to act
-• independence claimed before the existing process can respond
+• someone claiming independence before the existing process can respond
 • a sudden break creating an opening that did not exist a moment earlier</x:v>
       </x:c>
       <x:c r="F88" s="45" t="str">
@@ -5389,7 +5421,7 @@
       <x:c r="E89" s="45" t="str">
         <x:v>• a secure resource becoming the site of an unexpected revision
 • material routines changing after stability proves less fixed than assumed
-• independence requiring a new way to preserve what still matters</x:v>
+• someone finding a new way to preserve what matters without giving up independence</x:v>
       </x:c>
       <x:c r="F89" s="45" t="str">
         <x:v>disruption of material security</x:v>
@@ -5436,7 +5468,7 @@
       <x:c r="E90" s="45" t="str">
         <x:v>• new information altering the available routes almost immediately
 • a revised term changing who can participate
-• independence spreading through access to a different explanation</x:v>
+• people acting more independently after a different explanation becomes available</x:v>
       </x:c>
       <x:c r="F90" s="45" t="str">
         <x:v>rapidly revised information and terms</x:v>
@@ -5484,8 +5516,8 @@
       </x:c>
       <x:c r="E91" s="45" t="str">
         <x:v>• a household pattern changing because someone needs more room
-• belonging reorganized around a form of care no longer kept private
-• independence unsettling the role that once guaranteed emotional safety</x:v>
+• people reorganizing who belongs after private care becomes a public concern
+• someone leaving the role that once guaranteed emotional safety</x:v>
       </x:c>
       <x:c r="F91" s="45" t="str">
         <x:v>independence disrupting care and belonging</x:v>
@@ -5531,8 +5563,8 @@
       </x:c>
       <x:c r="E92" s="45" t="str">
         <x:v>• visible difference interrupting the expected public role
-• recognition shifting toward the contribution that breaks precedent
-• independence becoming impossible to separate from personal visibility</x:v>
+• people giving credit to the contribution that breaks precedent
+• someone making their independence visible because the old role no longer fits</x:v>
       </x:c>
       <x:c r="F92" s="45" t="str">
         <x:v>visible difference and personal freedom</x:v>
@@ -5579,7 +5611,7 @@
       <x:c r="E93" s="45" t="str">
         <x:v>• a routine revised when the old method stops solving the problem
 • one technical change altering how the work is distributed
-• independence gained through a more useful process</x:v>
+• people gaining independence by using a more useful process</x:v>
       </x:c>
       <x:c r="F93" s="45" t="str">
         <x:v>revision of routines and methods</x:v>
@@ -5625,7 +5657,7 @@
       </x:c>
       <x:c r="E94" s="45" t="str">
         <x:v>• an agreement reopening because equal treatment no longer produces a fair result
-• independence changing the terms of mutual obligation
+• someone asking to change what each side owes so there is more room to act alone
 • a different arrangement becoming possible once reciprocity is redefined</x:v>
       </x:c>
       <x:c r="F94" s="45" t="str">
@@ -5672,8 +5704,8 @@
       </x:c>
       <x:c r="E95" s="45" t="str">
         <x:v>• hidden leverage exposed by a change no one can reverse
-• private access disrupted before trust can be renegotiated
-• independence altering who controls the most consequential information</x:v>
+• someone disrupting private access before trust can be renegotiated
+• someone acting independently and changing who controls the most consequential information</x:v>
       </x:c>
       <x:c r="F95" s="45" t="str">
         <x:v>disruption exposing private leverage</x:v>
@@ -5719,8 +5751,8 @@
       </x:c>
       <x:c r="E96" s="45" t="str">
         <x:v>• a sudden opening widening the distance people can imagine crossing
-• independence challenging a belief that once set the horizon
-• change moving farther than the original plan was built to contain</x:v>
+• someone acting independently of the belief that once set the horizon
+• people carrying a change farther than the original plan was built to contain</x:v>
       </x:c>
       <x:c r="F96" s="45" t="str">
         <x:v>independence widening belief and distance</x:v>
@@ -5768,8 +5800,8 @@
       </x:c>
       <x:c r="E97" s="45" t="str">
         <x:v>• a long-standing authority losing control of the structure it maintained
-• independence forced into a system designed to resist quick revision
-• change becoming durable only after responsibility is reassigned</x:v>
+• someone trying to act independently inside a system designed to resist quick revision
+• people making the change last by reassigning responsibility</x:v>
       </x:c>
       <x:c r="F97" s="45" t="str">
         <x:v>change confronting authority and structure</x:v>
@@ -5816,7 +5848,7 @@
       <x:c r="E98" s="45" t="str">
         <x:v>• a group redesigning the rule that once limited its own independence
 • system change spreading because the exception reveals a wider problem
-• difference becoming part of the shared arrangement rather than outside it</x:v>
+• a group changing the system so quickly that people lose the support the old one provided</x:v>
       </x:c>
       <x:c r="F98" s="45" t="str">
         <x:v>independence and system change reinforcing each other</x:v>
@@ -5862,8 +5894,8 @@
       </x:c>
       <x:c r="E99" s="45" t="str">
         <x:v>• a sudden intuition disrupting a boundary that was already unclear
-• independence appearing where people had mistaken sympathy for agreement
-• change moving through a shared feeling before anyone can define the plan</x:v>
+• someone stepping away after others mistook sympathy for agreement
+• people changing course together before anyone can define the plan</x:v>
       </x:c>
       <x:c r="F99" s="45" t="str">
         <x:v>intuitive disruption and uncertain boundaries</x:v>
@@ -5910,7 +5942,7 @@
       <x:c r="E100" s="45" t="str">
         <x:v>• a collective hope rushing into action before its direction is understood
 • an ideal making the first move feel clearer than the evidence does
-• uncertainty hidden by the urgency of beginning</x:v>
+• people starting quickly so they do not have to admit the direction is uncertain</x:v>
       </x:c>
       <x:c r="F100" s="45" t="str">
         <x:v>collective ideals rushing toward an uncertain beginning</x:v>
@@ -5957,7 +5989,7 @@
         <x:v>a beautiful or reassuring plan can hide what it will actually cost</x:v>
       </x:c>
       <x:c r="E101" s="45" t="str">
-        <x:v>• comfort carrying an idealized value that obscures the real cost
+        <x:v>• people choosing the reassuring option while overlooking its real cost
 • material security trusted because it feels familiar rather than verified
 • a shared hope attaching to something people want to preserve</x:v>
       </x:c>
@@ -6008,7 +6040,7 @@
       <x:c r="E102" s="45" t="str">
         <x:v>• several plausible explanations blurring which fact deserves trust
 • an implied meaning circulating without a stable source
-• information becoming more persuasive as its boundaries become less exact</x:v>
+• people trusting an appealing explanation more as its boundaries become less exact</x:v>
       </x:c>
       <x:c r="F102" s="45" t="str">
         <x:v>uncertainty spreading through information</x:v>
@@ -6057,7 +6089,7 @@
       <x:c r="E103" s="45" t="str">
         <x:v>• memory softening the difference between care and projection
 • a private longing shaping what the group believes it needs
-• belonging idealized until unequal emotional labor becomes hard to see</x:v>
+• people idealizing the family bond until they stop seeing who carries the emotional labor</x:v>
       </x:c>
       <x:c r="F103" s="45" t="str">
         <x:v>memory, care, and projection</x:v>
@@ -6103,8 +6135,8 @@
       </x:c>
       <x:c r="E104" s="45" t="str">
         <x:v>• a public image carrying more hope than the contribution can support
-• recognition attaching to the story people want to believe
-• individual visibility becoming a screen for a collective ideal</x:v>
+• people crediting the story they want to believe instead of checking the work
+• people trusting the impressive image after it has stopped matching the work behind it</x:v>
       </x:c>
       <x:c r="F104" s="45" t="str">
         <x:v>idealized visibility and contribution</x:v>
@@ -6152,8 +6184,8 @@
       </x:c>
       <x:c r="E105" s="45" t="str">
         <x:v>• an ideal meeting the practical detail it cannot explain away
-• uncertainty exposed when the method has to produce a usable result
-• compassion losing clarity around what actually needs correction</x:v>
+• people seeing the uncertainty once the method has to produce a usable result
+• people correcting the plan repeatedly because no real version can match the ideal</x:v>
       </x:c>
       <x:c r="F105" s="45" t="str">
         <x:v>ideals tested by practical proof</x:v>
@@ -6199,8 +6231,8 @@
       </x:c>
       <x:c r="E106" s="45" t="str">
         <x:v>• an image of fairness hiding which side keeps absorbing the cost
-• agreement sustained by avoiding the unequal term underneath it
-• shared ideals blurring the point where reciprocity stopped</x:v>
+• people keeping an agreement by avoiding the unequal term underneath it
+• people overlooking where reciprocity stopped because they still share the ideal</x:v>
       </x:c>
       <x:c r="F106" s="45" t="str">
         <x:v>ideal fairness and unequal terms</x:v>
@@ -6246,7 +6278,7 @@
       </x:c>
       <x:c r="E107" s="45" t="str">
         <x:v>• trust deepening around a motive no one can fully name
-• private power becoming harder to locate as boundaries soften
+• people losing track of who holds private power as the boundaries soften
 • an irreversible choice shaped by information that remains uncertain</x:v>
       </x:c>
       <x:c r="F107" s="45" t="str">
@@ -6295,7 +6327,7 @@
       </x:c>
       <x:c r="E108" s="45" t="str">
         <x:v>• a belief growing beyond what its supporting facts can carry
-• hope widening the horizon while obscuring the practical distance
+• people looking farther ahead while overlooking the practical distance
 • a collective ideal becoming difficult to separate from certainty</x:v>
       </x:c>
       <x:c r="F108" s="45" t="str">
@@ -6342,8 +6374,8 @@
       </x:c>
       <x:c r="E109" s="45" t="str">
         <x:v>• an institution asked to formalize a need it cannot clearly define
-• authority lending certainty to an ideal that still lacks limits
-• responsibility blurred by a structure built around appearances</x:v>
+• an authority making an ideal sound settled before anyone has named its limits
+• people losing track of responsibility inside a structure built around appearances</x:v>
       </x:c>
       <x:c r="F109" s="45" t="str">
         <x:v>ideals pressed against duty and consequence</x:v>
@@ -6388,9 +6420,9 @@
         <x:v>a group gathers around the future it wants while the system still lacks a workable shape</x:v>
       </x:c>
       <x:c r="E110" s="45" t="str">
-        <x:v>• collective hope gathering around a system that does not yet exist
+        <x:v>• a group supporting a system that does not yet exist because it answers a shared hope
 • an imagined reform obscuring who would carry its actual cost
-• group ideals making uncertain access feel universally available</x:v>
+• a group assuming everyone has access because the ideal says they should</x:v>
       </x:c>
       <x:c r="F110" s="45" t="str">
         <x:v>collective hope and imagined reform</x:v>
@@ -6435,8 +6467,8 @@
         <x:v>people share a feeling or hope before anyone can tell where it began or what it asks</x:v>
       </x:c>
       <x:c r="E111" s="45" t="str">
-        <x:v>• empathy dissolving the line between shared feeling and shared duty
-• imagination expanding where facts cannot set a firm boundary
+        <x:v>• people treating a shared feeling as if it creates the same duty for everyone
+• people imagining more because the facts do not set a firm boundary
 • a collective longing becoming the atmosphere around the decision</x:v>
       </x:c>
       <x:c r="F111" s="45" t="str">
@@ -6482,9 +6514,9 @@
         <x:v>whoever moves first can seize leverage before anyone agrees it is in play</x:v>
       </x:c>
       <x:c r="E112" s="45" t="str">
-        <x:v>• leverage taken before anyone agrees it is in play
+        <x:v>• someone taking leverage before anyone agrees it is in play
 • the first decisive move concentrating control around one actor
-• power revealed by who can act without waiting for consent</x:v>
+• people seeing who has power by who can act without waiting for consent</x:v>
       </x:c>
       <x:c r="F112" s="45" t="str">
         <x:v>power in the first move</x:v>
@@ -6529,9 +6561,9 @@
         <x:v>who controls the money or material people cannot lose can control the decision</x:v>
       </x:c>
       <x:c r="E113" s="45" t="str">
-        <x:v>• control settling around the resource people cannot afford to lose
+        <x:v>• someone gaining control by holding the resource others cannot afford to lose
 • a material dependency giving one side durable leverage
-• power becoming visible when security can no longer be assumed</x:v>
+• people seeing who has power after the expected security disappears</x:v>
       </x:c>
       <x:c r="F113" s="45" t="str">
         <x:v>control of resources and material security</x:v>
@@ -6580,7 +6612,7 @@
       <x:c r="E114" s="45" t="str">
         <x:v>• access to the explanation deciding who can shape the outcome
 • one version of the facts becoming leverage over the others
-• control shifting when information reaches a wider audience</x:v>
+• someone losing control after the information reaches a wider audience</x:v>
       </x:c>
       <x:c r="F114" s="45" t="str">
         <x:v>information as leverage</x:v>
@@ -6622,12 +6654,12 @@
         <x:v>people respond through care, memory, and private loyalties</x:v>
       </x:c>
       <x:c r="D115" s="45" t="str">
-        <x:v>people give private loyalty enough weight to shape a decision that reaches the whole group</x:v>
+        <x:v>family loyalty or private influence starts deciding what happens to everyone else</x:v>
       </x:c>
       <x:c r="E115" s="45" t="str">
-        <x:v>• family loyalty giving private influence public consequence
-• care turning into leverage where belonging feels conditional
-• control hidden inside the role that protects the household</x:v>
+        <x:v>• family loyalty influencing a decision that affects people outside the family
+• someone using care, access, or obligation to make it harder for another person to say no
+• the person who protects the household also deciding who belongs and what loyalty requires</x:v>
       </x:c>
       <x:c r="F115" s="45" t="str">
         <x:v>power inside care and family loyalty</x:v>
@@ -6673,8 +6705,8 @@
       </x:c>
       <x:c r="E116" s="45" t="str">
         <x:v>• ownership of the public role becoming a source of control
-• recognition deciding whose authority appears legitimate
-• power concentrating around the person identified with the outcome</x:v>
+• people treating one person's authority as legitimate because that person receives recognition
+• people giving more power to the person identified with the outcome</x:v>
       </x:c>
       <x:c r="F116" s="45" t="str">
         <x:v>visible authority and ownership</x:v>
@@ -6719,9 +6751,9 @@
         <x:v>whoever defines the flaw can also control the method used to fix it</x:v>
       </x:c>
       <x:c r="E117" s="45" t="str">
-        <x:v>• control exercised through the method everyone must use
+        <x:v>• someone controlling the outcome through the method everyone must use
 • one required correction exposing who defines acceptable work
-• leverage appearing in the power to call something defective</x:v>
+• someone gaining leverage by deciding what counts as defective</x:v>
       </x:c>
       <x:c r="F117" s="45" t="str">
         <x:v>control of methods and correction</x:v>
@@ -6769,8 +6801,8 @@
       </x:c>
       <x:c r="E118" s="45" t="str">
         <x:v>• compromise revealing which side has been yielding to preserve the agreement
-• fairness language used to conceal unequal control
-• power shifting when reciprocal terms become enforceable</x:v>
+• someone using the language of fairness to conceal unequal control
+• people changing who holds power by making reciprocal terms enforceable</x:v>
       </x:c>
       <x:c r="F118" s="45" t="str">
         <x:v>power hidden inside compromise</x:v>
@@ -6815,9 +6847,9 @@
         <x:v>people protect private information because giving it up would change the balance of power</x:v>
       </x:c>
       <x:c r="E119" s="45" t="str">
-        <x:v>• private leverage intensifying because the consequence cannot be reversed
-• control depending on access to what others cannot safely disclose
-• power becoming undeniable when trust and survival meet</x:v>
+        <x:v>• someone gaining more private leverage because the consequence cannot be reversed
+• someone keeping control because others cannot safely disclose what they know
+• people seeing who has power when trust and survival depend on the same decision</x:v>
       </x:c>
       <x:c r="F119" s="45" t="str">
         <x:v>privacy and leverage carrying irreversible stakes</x:v>
@@ -6864,9 +6896,9 @@
         <x:v>whoever defines the larger truth can extend their reach over the decision</x:v>
       </x:c>
       <x:c r="E120" s="45" t="str">
-        <x:v>• authority growing around who can define the larger truth
+        <x:v>• someone gaining authority by defining the larger truth
 • a belief extending power beyond its original boundary
-• control moving through the institution that grants wider reach</x:v>
+• an institution controlling who gets the wider reach</x:v>
       </x:c>
       <x:c r="F120" s="45" t="str">
         <x:v>conviction defining truth and reach</x:v>
@@ -6911,9 +6943,9 @@
         <x:v>an institution assigns duty in ways that reveal who can make the lasting rule</x:v>
       </x:c>
       <x:c r="E121" s="45" t="str">
-        <x:v>• institutional power becoming visible in who assigns lasting duty
-• control secured through a structure that outlives the immediate dispute
-• authority concentrating where consequences are formally enforced</x:v>
+        <x:v>• people seeing institutional power in who gets to assign lasting duty
+• someone securing control through a structure that outlives the immediate dispute
+• the person who enforces the consequence gaining more authority</x:v>
       </x:c>
       <x:c r="F121" s="45" t="str">
         <x:v>institutional control and lasting consequence</x:v>
@@ -6958,9 +6990,9 @@
         <x:v>a group changes the rules when the current system keeps power in the same hands</x:v>
       </x:c>
       <x:c r="E122" s="45" t="str">
-        <x:v>• group rules redistributing power across an entire system
-• collective pressure exposing who benefits from the current arrangement
-• control changing hands when independence becomes structurally possible</x:v>
+        <x:v>• a group rewriting its rules and redistributing power across the system
+• a group pressing the issue until everyone can see who benefits from the current arrangement
+• people changing who controls the system once independence becomes possible</x:v>
       </x:c>
       <x:c r="F122" s="45" t="str">
         <x:v>power shifting through groups and systems</x:v>
@@ -7005,9 +7037,9 @@
         <x:v>people can feel the pressure without being able to name who controls it</x:v>
       </x:c>
       <x:c r="E123" s="45" t="str">
-        <x:v>• power becoming difficult to locate inside a shared emotional field
-• control operating through an ideal no single person appears to own
-• leverage increasing where boundaries and responsibility remain diffuse</x:v>
+        <x:v>• people feeling controlled without being able to name who is doing it
+• people enforcing an ideal while each person denies owning it
+• someone gaining leverage because no one has named the boundary or responsibility</x:v>
       </x:c>
       <x:c r="F123" s="45" t="str">
         <x:v>diffuse control inside collective feeling</x:v>
@@ -7049,12 +7081,12 @@
         <x:v>someone moves first and asks everyone else to catch up</x:v>
       </x:c>
       <x:c r="D124" s="45" t="str">
-        <x:v>someone hesitates to begin because taking the lead once carried a painful cost</x:v>
+        <x:v>someone hangs back on the first move because going first has gone badly before</x:v>
       </x:c>
       <x:c r="E124" s="45" t="str">
-        <x:v>• hesitation around acting first after initiative was once punished
-• a strong reaction when independence is treated as selfishness
-• pain resurfacing at the moment someone has to claim the right to begin</x:v>
+        <x:v>• hesitating to volunteer, apply, speak first, or take the lead after being punished for it before
+• reacting strongly when independence is treated as selfishness
+• wanting to act but checking for permission first because taking initiative used to come with consequences</x:v>
       </x:c>
       <x:c r="F124" s="45" t="str">
         <x:v>sensitivity around action and independence</x:v>
@@ -7140,7 +7172,7 @@
       <x:c r="E126" s="45" t="str">
         <x:v>• careful wording shaped by the fear of being misunderstood again
 • a question carrying the memory of not being believed
-• sensitivity appearing when several explanations exclude the lived one</x:v>
+• someone reacting after every official explanation leaves out what they lived through</x:v>
       </x:c>
       <x:c r="F126" s="45" t="str">
         <x:v>sensitivity around language and being understood</x:v>
@@ -7181,7 +7213,7 @@
         <x:v>people ask for care differently when an old family hurt enters the room</x:v>
       </x:c>
       <x:c r="E127" s="45" t="str">
-        <x:v>• care becoming protective where belonging once felt conditional
+        <x:v>• someone protecting the person whose belonging was once treated as conditional
 • family memory sharpening a present need for safety
 • old pain returning when private loyalty is asked to prove itself</x:v>
       </x:c>
@@ -7224,9 +7256,9 @@
         <x:v>someone wants the work recognized without having the old hurt exposed with it</x:v>
       </x:c>
       <x:c r="E128" s="45" t="str">
-        <x:v>• recognition touching the earlier fear that contribution would be dismissed
+        <x:v>• someone receiving recognition and still expecting their contribution to be dismissed
 • visible pride covering uncertainty about whether appreciation will last
-• hurt surfacing when the person doing the work is not named</x:v>
+• someone reacting strongly when the person doing the work is not named</x:v>
       </x:c>
       <x:c r="F128" s="45" t="str">
         <x:v>visible hurt around recognition</x:v>
@@ -7269,7 +7301,7 @@
       <x:c r="E129" s="45" t="str">
         <x:v>• a small correction reopening the fear of never being useful enough
 • competence becoming a defense against being judged as a burden
-• sensitivity gathering around the detail that others call insignificant</x:v>
+• someone focusing on the detail others dismiss because it once carried a real cost</x:v>
       </x:c>
       <x:c r="F129" s="45" t="str">
         <x:v>sensitivity around usefulness and correction</x:v>
@@ -7311,7 +7343,7 @@
       </x:c>
       <x:c r="E130" s="45" t="str">
         <x:v>• an unfair term touching an older habit of preserving peace at personal cost
-• pain appearing where agreement requires repeated self-adjustment
+• someone feeling an older hurt each time the agreement asks them to adjust again
 • balance becoming fragile when one side's need is treated as disruption</x:v>
       </x:c>
       <x:c r="F130" s="45" t="str">
@@ -7354,7 +7386,7 @@
       </x:c>
       <x:c r="E131" s="45" t="str">
         <x:v>• trust activating the memory of a disclosure that carried consequences
-• privacy guarded because some experiences cannot be made harmless afterward
+• someone guarding their privacy because disclosure cannot be made harmless afterward
 • old pain shaping how much leverage anyone is allowed to hold</x:v>
       </x:c>
       <x:c r="F131" s="45" t="str">
@@ -7397,8 +7429,8 @@
       </x:c>
       <x:c r="E132" s="45" t="str">
         <x:v>• a larger promise touching the fear that hope will be punished again
-• belief becoming sensitive when one story is declared universally true
-• pain entering the question of who is free to imagine a different future</x:v>
+• someone reacting when one story is treated as the only truth
+• someone holding back a different future because hope once brought consequences</x:v>
       </x:c>
       <x:c r="F132" s="45" t="str">
         <x:v>sensitivity around belief and meaning</x:v>
@@ -7441,7 +7473,7 @@
       <x:c r="E133" s="45" t="str">
         <x:v>• competence used to hide the cost of carrying too much responsibility
 • an old hurt returning when need is treated as failure
-• duty becoming the place where vulnerability is least allowed</x:v>
+• someone hiding vulnerability whenever duty has to be performed</x:v>
       </x:c>
       <x:c r="F133" s="45" t="str">
         <x:v>pain managed through duty and competence</x:v>
@@ -7482,9 +7514,9 @@
         <x:v>a shared rule can reopen the memory of being useful to the group but never fully included</x:v>
       </x:c>
       <x:c r="E134" s="45" t="str">
-        <x:v>• group belonging tested by whether difference is tolerated in practice
-• exclusion remembered when a shared rule erases a particular need
-• sensitivity gathering around being useful to the group but not known by it</x:v>
+        <x:v>• someone testing whether the group actually tolerates their difference
+• someone remembering an earlier exclusion when a shared rule erases their need
+• someone leaving the group first because exclusion feels easier to control when it is chosen</x:v>
       </x:c>
       <x:c r="F134" s="45" t="str">
         <x:v>sensitivity around exclusion and group belonging</x:v>
@@ -7525,9 +7557,9 @@
         <x:v>people can absorb an old pain from the room without knowing what belongs to whom</x:v>
       </x:c>
       <x:c r="E135" s="45" t="str">
-        <x:v>• empathy reopening pain that has not been clearly separated from others
-• longing making an old loss feel collectively meaningful
-• sensitivity spreading where care has no agreed boundary</x:v>
+        <x:v>• someone feeling another person's pain and reopening their own
+• people giving an old loss shared meaning because they still long for what was lost
+• someone absorbing more pain because no one has agreed where care ends</x:v>
       </x:c>
       <x:c r="F135" s="45" t="str">
         <x:v>pain diffused through empathy and longing</x:v>
@@ -7569,8 +7601,8 @@
       </x:c>
       <x:c r="E136" s="45" t="str">
         <x:v>• a refusal stated before anyone grants the right to object
-• autonomy claimed through the act others call premature
-• the excluded position forcing its way into the decision</x:v>
+• someone claiming the right to act even when others call the move premature
+• someone starting a confrontation just to prove that no one can tell them what to do</x:v>
       </x:c>
       <x:c r="F136" s="45" t="str">
         <x:v>direct refusal and autonomous action</x:v>
@@ -7610,8 +7642,8 @@
       </x:c>
       <x:c r="E137" s="45" t="str">
         <x:v>• a boundary forming around the body or resource others expect to use
-• refusal becoming firm when security requires surrender
-• autonomy measured by what can be kept without apology</x:v>
+• someone refusing the security offered because it requires surrender
+• someone judging their freedom by what they can keep without apology</x:v>
       </x:c>
       <x:c r="F137" s="45" t="str">
         <x:v>bodily autonomy and protected resources</x:v>
@@ -7651,8 +7683,8 @@
       </x:c>
       <x:c r="E138" s="45" t="str">
         <x:v>• a contradiction spoken after the approved explanation stops holding
-• refusal moving between versions that authority wanted reduced to one
-• autonomy preserved through naming what the official language leaves out</x:v>
+• someone offering several versions after an authority demands one approved account
+• someone changing the story whenever the last version begins to carry consequences</x:v>
       </x:c>
       <x:c r="F138" s="45" t="str">
         <x:v>refusal through contradiction and alternate versions</x:v>
@@ -7691,9 +7723,9 @@
         <x:v>people refuse a role that demands care or feeling on command</x:v>
       </x:c>
       <x:c r="E139" s="45" t="str">
-        <x:v>• care withheld from a role that expects feeling to be performed
-• private belonging protected from demands for emotional access
-• refusal appearing when loyalty is used to override autonomy</x:v>
+        <x:v>• someone withholding care from a role that expects feeling on command
+• someone protecting private belonging from demands for emotional access
+• someone letting an old family hurt color every present request for care</x:v>
       </x:c>
       <x:c r="F139" s="45" t="str">
         <x:v>private autonomy and nonperformed care</x:v>
@@ -7732,9 +7764,9 @@
         <x:v>someone claims visibility without making the difficult part more acceptable first</x:v>
       </x:c>
       <x:c r="E140" s="45" t="str">
-        <x:v>• visibility claimed without making the contribution more acceptable first
-• recognition rejected when it depends on shrinking the difficult part
-• autonomy becoming public where approval had set the terms</x:v>
+        <x:v>• someone claiming visibility without making the contribution more acceptable first
+• someone rejecting recognition that depends on shrinking the difficult part
+• someone making the whole conflict about them because shame is harder to name directly</x:v>
       </x:c>
       <x:c r="F140" s="45" t="str">
         <x:v>visible refusal of conditional recognition</x:v>
@@ -7774,7 +7806,7 @@
       </x:c>
       <x:c r="E141" s="45" t="str">
         <x:v>• a standard refused because usefulness has become a condition of worth
-• autonomy defended against correction aimed at making difference manageable
+• someone defending their difference against correction meant to make it manageable
 • the excluded need exposing what the approved method cannot serve</x:v>
       </x:c>
       <x:c r="F141" s="45" t="str">
@@ -7815,8 +7847,8 @@
       </x:c>
       <x:c r="E142" s="45" t="str">
         <x:v>• an agreement challenged after fairness becomes repeated self-erasure
-• refusal entering the negotiation where politeness had hidden the cost
-• autonomy requiring terms that do not depend on one side yielding</x:v>
+• someone naming the cost that polite negotiation kept hidden
+• someone demanding terms that do not depend on one side yielding</x:v>
       </x:c>
       <x:c r="F142" s="45" t="str">
         <x:v>autonomy exposing unfair agreement</x:v>
@@ -7855,9 +7887,9 @@
         <x:v>people protect desire and private access from someone trying to take control</x:v>
       </x:c>
       <x:c r="E143" s="45" t="str">
-        <x:v>• desire protected from someone else's claim to private access
-• refusal becoming final where trust has been used as leverage
-• autonomy holding back what cannot be safely recovered once given</x:v>
+        <x:v>• someone protecting desire from another person's claim to private access
+• someone ending the agreement after trust is used as leverage
+• someone keeping private what they could not safely recover once given</x:v>
       </x:c>
       <x:c r="F143" s="45" t="str">
         <x:v>protected desire, privacy, and power</x:v>
@@ -7897,8 +7929,8 @@
       </x:c>
       <x:c r="E144" s="45" t="str">
         <x:v>• a rule rejected when belief is used to make freedom conditional
-• autonomy widening beyond the story that defined acceptable desire
-• refusal exposing who was allowed to name the larger truth</x:v>
+• someone wanting more than the approved story allowed them to name
+• someone refusing the approved story and exposing who was allowed to define the truth</x:v>
       </x:c>
       <x:c r="F144" s="45" t="str">
         <x:v>freedom refusing conditional belief</x:v>
@@ -7937,9 +7969,9 @@
         <x:v>people confront an authority that uses duty or respectability to demand compliance</x:v>
       </x:c>
       <x:c r="E145" s="45" t="str">
-        <x:v>• authority confronted where respectability has been used as control
+        <x:v>• someone confronting an authority that has used respectability as control
 • a duty refused because compliance would erase the person carrying it
-• autonomy becoming visible in the consequence someone chooses to accept</x:v>
+• someone accepting the consequence rather than obeying the demand</x:v>
       </x:c>
       <x:c r="F145" s="45" t="str">
         <x:v>autonomy against authority and respectability</x:v>
@@ -7979,8 +8011,8 @@
       </x:c>
       <x:c r="E146" s="45" t="str">
         <x:v>• a group norm challenged for welcoming difference only in approved forms
-• refusal revealing who remains excluded by a supposedly universal rule
-• autonomy protected from collective pressure to become easier to manage</x:v>
+• someone challenging a universal rule and showing who it still excludes
+• someone rebelling against the group rule even when the rebellion leaves them more isolated</x:v>
       </x:c>
       <x:c r="F146" s="45" t="str">
         <x:v>refusal inside conditional group belonging</x:v>
@@ -8020,7 +8052,7 @@
       </x:c>
       <x:c r="E147" s="46" t="str">
         <x:v>• an emotional demand refused before empathy becomes absorption
-• autonomy held where other people's ideals blur personal boundaries
+• someone holding a personal boundary while other people treat their ideals as shared
 • the excluded feeling named without turning it into a request for rescue</x:v>
       </x:c>
       <x:c r="F147" s="46" t="str">
@@ -8061,7 +8093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4637b5410a484765"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R477c1a59473c459a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8293,7 +8325,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8f56d744aed41a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9398035ddb8b41bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8639,7 +8671,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64755ed10f0f42e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38cd79d77d2641e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9135,7 +9167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8109d60c763045f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3e8512c442648a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9393,22 +9425,62 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="27" t="str">
+      <x:c r="A14" s="26" t="str">
+        <x:v>Manifestation actor or act</x:v>
+      </x:c>
+      <x:c r="B14" s="26" t="str">
+        <x:v>All sign manifestations</x:v>
+      </x:c>
+      <x:c r="C14" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="26" t="str">
+        <x:v>A person acts or a concrete act is visible</x:v>
+      </x:c>
+      <x:c r="E14" s="26" t="str">
+        <x:v>Care turns into leverage</x:v>
+      </x:c>
+      <x:c r="F14" s="26" t="str">
+        <x:v>An abstraction may not perform the behavior</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="26" t="str">
+        <x:v>Source shadow coverage</x:v>
+      </x:c>
+      <x:c r="B15" s="26" t="str">
+        <x:v>All sign units</x:v>
+      </x:c>
+      <x:c r="C15" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="26" t="str">
+        <x:v>A supported cost or overreach remains available</x:v>
+      </x:c>
+      <x:c r="E15" s="26" t="str">
+        <x:v>Jupiter becomes uniformly beneficial</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="str">
+        <x:v>The component may not erase source challenge, shadow, or cost</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="27" t="str">
         <x:v>Owner-source conversion</x:v>
       </x:c>
-      <x:c r="B14" s="27" t="str">
+      <x:c r="B16" s="27" t="str">
         <x:v>All owner-voice evidence</x:v>
       </x:c>
-      <x:c r="C14" s="27" t="n">
+      <x:c r="C16" s="27" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D14" s="27" t="str">
+      <x:c r="D16" s="27" t="str">
         <x:v>Personal source meaning is converted for collective Sky</x:v>
       </x:c>
-      <x:c r="E14" s="27" t="str">
+      <x:c r="E16" s="27" t="str">
         <x:v>Eight or more source words are copied verbatim</x:v>
       </x:c>
-      <x:c r="F14" s="27" t="str">
+      <x:c r="F16" s="27" t="str">
         <x:v>Owner voice governs without leaking second-person source prose</x:v>
       </x:c>
     </x:row>
@@ -9622,171 +9694,126 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="16" t="str">
+      <x:c r="A14" s="15" t="str">
+        <x:v>Manifestation plainness violations</x:v>
+      </x:c>
+      <x:c r="B14" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="15" t="str">
         <x:v>Owner-source verbatim matches (8+ words)</x:v>
       </x:c>
-      <x:c r="B14" s="16" t="n">
+      <x:c r="B15" s="15" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C14" s="16" t="n">
+      <x:c r="C15" s="15" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="9" t="str">
+      <x:c r="A16" s="15" t="str">
+        <x:v>Units rechecked</x:v>
+      </x:c>
+      <x:c r="B16" s="15" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="C16" s="15" t="n">
+        <x:v>174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="15" t="str">
+        <x:v>Units changed</x:v>
+      </x:c>
+      <x:c r="B17" s="15" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C17" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="15" t="str">
+        <x:v>One-sided before source-shadow pass</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C18" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="16" t="str">
+        <x:v>One-sided after source-shadow pass</x:v>
+      </x:c>
+      <x:c r="B19" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="9" t="str">
         <x:v>Opening construction</x:v>
       </x:c>
-      <x:c r="B16" s="9" t="str">
+      <x:c r="B21" s="9" t="str">
         <x:v>Uses</x:v>
       </x:c>
-      <x:c r="D16" s="9" t="str">
+      <x:c r="D21" s="9" t="str">
         <x:v>Repeated connective n-gram</x:v>
       </x:c>
-      <x:c r="E16" s="9" t="str">
+      <x:c r="E21" s="9" t="str">
         <x:v>Uses</x:v>
       </x:c>
-      <x:c r="G16" s="9" t="str">
+      <x:c r="G21" s="9" t="str">
         <x:v>Manifestation skeleton</x:v>
       </x:c>
-      <x:c r="H16" s="9" t="str">
+      <x:c r="H21" s="9" t="str">
         <x:v>Uses</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="19" t="str">
+    <x:row r="22">
+      <x:c r="A22" s="19" t="str">
         <x:v>people can</x:v>
       </x:c>
-      <x:c r="B17" s="19" t="n">
+      <x:c r="B22" s="19" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D17" s="19" t="str">
+      <x:c r="D22" s="19" t="str">
         <x:v>as the</x:v>
       </x:c>
-      <x:c r="E17" s="19" t="n">
+      <x:c r="E22" s="19" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G17" s="19" t="str">
-        <x:v>{planet} aimed at changing the system rather than winning one exception</x:v>
-      </x:c>
-      <x:c r="H17" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="20" t="str">
-        <x:v>a group</x:v>
-      </x:c>
-      <x:c r="B18" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D18" s="20" t="str">
-        <x:v>before anyone</x:v>
-      </x:c>
-      <x:c r="E18" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G18" s="20" t="str">
-        <x:v>{planet} altering who controls the most consequential information</x:v>
-      </x:c>
-      <x:c r="H18" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="20" t="str">
-        <x:v>a larger</x:v>
-      </x:c>
-      <x:c r="B19" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D19" s="20" t="str">
-        <x:v>until the</x:v>
-      </x:c>
-      <x:c r="E19" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G19" s="20" t="str">
-        <x:v>{planet} appearing as the task that keeps a routine from failing</x:v>
-      </x:c>
-      <x:c r="H19" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="20" t="str">
-        <x:v>a new</x:v>
-      </x:c>
-      <x:c r="B20" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D20" s="20" t="str">
-        <x:v>when the</x:v>
-      </x:c>
-      <x:c r="E20" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G20" s="20" t="str">
-        <x:v>{planet} appearing in the {planet} to call something defective</x:v>
-      </x:c>
-      <x:c r="H20" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="20" t="str">
-        <x:v>people give</x:v>
-      </x:c>
-      <x:c r="B21" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D21" s="20" t="str">
-        <x:v>while the</x:v>
-      </x:c>
-      <x:c r="E21" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G21" s="20" t="str">
-        <x:v>{planet} appearing in what becomes more secure or materially useful</x:v>
-      </x:c>
-      <x:c r="H21" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="20" t="str">
-        <x:v>people protect</x:v>
-      </x:c>
-      <x:c r="B22" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D22" s="20" t="str">
-        <x:v>with it</x:v>
-      </x:c>
-      <x:c r="E22" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G22" s="20" t="str">
-        <x:v>{planet} appearing when loyalty is used to override {planet}</x:v>
-      </x:c>
-      <x:c r="H22" s="20" t="n">
+      <x:c r="G22" s="19" t="str">
+        <x:v>{planet} becoming real when it is shown where others can see it</x:v>
+      </x:c>
+      <x:c r="H22" s="19" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="20" t="str">
-        <x:v>a sudden</x:v>
+        <x:v>a group</x:v>
       </x:c>
       <x:c r="B23" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D23" s="20" t="str">
-        <x:v>with the</x:v>
+        <x:v>before anyone</x:v>
       </x:c>
       <x:c r="E23" s="20" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G23" s="20" t="str">
-        <x:v>{planet} appearing when several explanations exclude the lived one</x:v>
+        <x:v>{planet} becoming unclear when many people shaped the same vision</x:v>
       </x:c>
       <x:c r="H23" s="20" t="n">
         <x:v>1</x:v>
@@ -9794,19 +9821,19 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="20" t="str">
-        <x:v>each side</x:v>
+        <x:v>a larger</x:v>
       </x:c>
       <x:c r="B24" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D24" s="20" t="str">
-        <x:v>after the</x:v>
+        <x:v>until the</x:v>
       </x:c>
       <x:c r="E24" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G24" s="20" t="str">
-        <x:v>{planet} appearing where agreement requires repeated self adjustment</x:v>
+        <x:v>{planet} divided according to terms both sides must answer to</x:v>
       </x:c>
       <x:c r="H24" s="20" t="n">
         <x:v>1</x:v>
@@ -9814,19 +9841,19 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="20" t="str">
-        <x:v>people have</x:v>
+        <x:v>a new</x:v>
       </x:c>
       <x:c r="B25" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D25" s="20" t="str">
-        <x:v>around a</x:v>
+        <x:v>when the</x:v>
       </x:c>
       <x:c r="E25" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G25" s="20" t="str">
-        <x:v>{planet} appearing where people had mistaken sympathy for agreement</x:v>
+        <x:v>{planet} narrowed until every part can be checked</x:v>
       </x:c>
       <x:c r="H25" s="20" t="n">
         <x:v>1</x:v>
@@ -9834,19 +9861,19 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="20" t="str">
-        <x:v>people keep</x:v>
+        <x:v>people protect</x:v>
       </x:c>
       <x:c r="B26" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D26" s="20" t="str">
-        <x:v>around the</x:v>
+        <x:v>while the</x:v>
       </x:c>
       <x:c r="E26" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G26" s="20" t="str">
-        <x:v>{planet} applied where trust and private access are already at stake</x:v>
+        <x:v>{planet} revised to distribute responsibility more fairly</x:v>
       </x:c>
       <x:c r="H26" s="20" t="n">
         <x:v>1</x:v>
@@ -9854,19 +9881,19 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="20" t="str">
-        <x:v>people make</x:v>
+        <x:v>a sudden</x:v>
       </x:c>
       <x:c r="B27" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D27" s="20" t="str">
-        <x:v>before anyone can</x:v>
+        <x:v>with it</x:v>
       </x:c>
       <x:c r="E27" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G27" s="20" t="str">
-        <x:v>{planet} arriving as quick {planet} rather than discussion</x:v>
+        <x:v>{planet} spreading because the exception reveals a wider problem</x:v>
       </x:c>
       <x:c r="H27" s="20" t="n">
         <x:v>1</x:v>
@@ -9874,19 +9901,19 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="20" t="str">
-        <x:v>people refuse</x:v>
+        <x:v>each side</x:v>
       </x:c>
       <x:c r="B28" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D28" s="20" t="str">
-        <x:v>boundary around</x:v>
+        <x:v>with the</x:v>
       </x:c>
       <x:c r="E28" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G28" s="20" t="str">
-        <x:v>{planet} arriving only after the result proves it can last</x:v>
+        <x:v>a {planet} announced before every objection has been heard</x:v>
       </x:c>
       <x:c r="H28" s="20" t="n">
         <x:v>1</x:v>
@@ -9894,19 +9921,19 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="20" t="str">
-        <x:v>people stay</x:v>
+        <x:v>people give</x:v>
       </x:c>
       <x:c r="B29" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D29" s="20" t="str">
-        <x:v>by fixing</x:v>
+        <x:v>after the</x:v>
       </x:c>
       <x:c r="E29" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G29" s="20" t="str">
-        <x:v>{planet} assigned to the choice that shows immediate commitment</x:v>
+        <x:v>a {planet} becoming real when an authority records it</x:v>
       </x:c>
       <x:c r="H29" s="20" t="n">
         <x:v>1</x:v>
@@ -9914,19 +9941,19 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="20" t="str">
-        <x:v>someone acts</x:v>
+        <x:v>people have</x:v>
       </x:c>
       <x:c r="B30" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D30" s="21" t="str">
-        <x:v>when it</x:v>
-      </x:c>
-      <x:c r="E30" s="21" t="n">
+      <x:c r="D30" s="20" t="str">
+        <x:v>around a</x:v>
+      </x:c>
+      <x:c r="E30" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="20" t="str">
-        <x:v>{planet} attached to the option that expands independence</x:v>
+        <x:v>a {planet} blurred by sympathy for several incompatible {planet}</x:v>
       </x:c>
       <x:c r="H30" s="20" t="n">
         <x:v>1</x:v>
@@ -9934,13 +9961,19 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="20" t="str">
-        <x:v>the group</x:v>
+        <x:v>people keep</x:v>
       </x:c>
       <x:c r="B31" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="D31" s="20" t="str">
+        <x:v>around the</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="G31" s="20" t="str">
-        <x:v>{planet} attached to the person expected to answer for the result</x:v>
+        <x:v>a {planet} changing when one more fact enters the conversation</x:v>
       </x:c>
       <x:c r="H31" s="20" t="n">
         <x:v>1</x:v>
@@ -9948,13 +9981,19 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="20" t="str">
-        <x:v>whoever defines</x:v>
+        <x:v>people make</x:v>
       </x:c>
       <x:c r="B32" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="D32" s="20" t="str">
+        <x:v>before anyone can</x:v>
+      </x:c>
+      <x:c r="E32" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="G32" s="20" t="str">
-        <x:v>{planet} attached to the version that enters the record</x:v>
+        <x:v>a {planet} forming around the body or resource others expect to use</x:v>
       </x:c>
       <x:c r="H32" s="20" t="n">
         <x:v>1</x:v>
@@ -9962,13 +10001,19 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="20" t="str">
-        <x:v>whoever moves</x:v>
+        <x:v>people refuse</x:v>
       </x:c>
       <x:c r="B33" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="D33" s="20" t="str">
+        <x:v>boundary around</x:v>
+      </x:c>
+      <x:c r="E33" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="G33" s="20" t="str">
-        <x:v>{planet} attaching to a shared ideal before its limits are clear</x:v>
+        <x:v>a {planet} meant to apply equally</x:v>
       </x:c>
       <x:c r="H33" s="20" t="n">
         <x:v>1</x:v>
@@ -9976,13 +10021,19 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="20" t="str">
-        <x:v>a beautiful</x:v>
+        <x:v>people stay</x:v>
       </x:c>
       <x:c r="B34" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D34" s="20" t="str">
+        <x:v>by fixing</x:v>
+      </x:c>
+      <x:c r="E34" s="20" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G34" s="20" t="str">
-        <x:v>{planet} attaching to an idealized image rather than the actual work</x:v>
+        <x:v>a {planet} moving only after both replies enter the record</x:v>
       </x:c>
       <x:c r="H34" s="20" t="n">
         <x:v>1</x:v>
@@ -9990,29 +10041,105 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="20" t="str">
-        <x:v>a choice</x:v>
+        <x:v>someone acts</x:v>
       </x:c>
       <x:c r="B35" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D35" s="21" t="str">
+        <x:v>when it</x:v>
+      </x:c>
+      <x:c r="E35" s="21" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G35" s="20" t="str">
-        <x:v>{planet} becoming difficult to locate inside a shared emotional field</x:v>
+        <x:v>a {planet} protecting access to information that cannot be taken back</x:v>
       </x:c>
       <x:c r="H35" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="21" t="str">
-        <x:v>a deadline</x:v>
-      </x:c>
-      <x:c r="B36" s="21" t="n">
+      <x:c r="A36" s="20" t="str">
+        <x:v>the group</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G36" s="20" t="str">
+        <x:v>a {planet} pursued carefully because it cannot be undone</x:v>
+      </x:c>
+      <x:c r="H36" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G36" s="21" t="str">
-        <x:v>{planet} becoming durable only after responsibility is reassigned</x:v>
-      </x:c>
-      <x:c r="H36" s="21" t="n">
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="20" t="str">
+        <x:v>whoever defines</x:v>
+      </x:c>
+      <x:c r="B37" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G37" s="20" t="str">
+        <x:v>a {planet} stated before anyone grants the right to object</x:v>
+      </x:c>
+      <x:c r="H37" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="20" t="str">
+        <x:v>whoever moves</x:v>
+      </x:c>
+      <x:c r="B38" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G38" s="20" t="str">
+        <x:v>a {planet} stated clearly enough to force a quick answer</x:v>
+      </x:c>
+      <x:c r="H38" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="20" t="str">
+        <x:v>a beautiful</x:v>
+      </x:c>
+      <x:c r="B39" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G39" s="20" t="str">
+        <x:v>a {planet} staying open because another comparison is still possible</x:v>
+      </x:c>
+      <x:c r="H39" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="20" t="str">
+        <x:v>a bigger</x:v>
+      </x:c>
+      <x:c r="B40" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G40" s="20" t="str">
+        <x:v>a {planet} stopping the first move until {planet} is assigned</x:v>
+      </x:c>
+      <x:c r="H40" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="21" t="str">
+        <x:v>a choice</x:v>
+      </x:c>
+      <x:c r="B41" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G41" s="21" t="str">
+        <x:v>a {planet} valued because it keeps producing something useful</x:v>
+      </x:c>
+      <x:c r="H41" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
fix(content): classify sky realization pools
</commit_message>
<xml_diff>
--- a/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
+++ b/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re5d3a92e997d4a9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="Rd88c63735a234057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="Rfc51b2568dc04def"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="4" r:id="R03536c44c96c49c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="5" r:id="Rdacd6eaa5e164ba4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="6" r:id="R000fd17d821b4395"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="7" r:id="R53dbae0e5bc94813"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="8" r:id="Rb3d1f597956743a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb684352f9c9f4ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R220ea213da0a49c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="R870abf1da4f94b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Audit" sheetId="4" r:id="R45d92f15683c4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="5" r:id="Rc281c90b3cc34604"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="6" r:id="R9c32c81bca8a43f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="7" r:id="R8715e384e81f417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="8" r:id="R6d6d32ac2d8d462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="9" r:id="Rd60192ed22d94cac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -225,7 +226,18 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="5">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF6B4F00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF7E8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -298,26 +310,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AspectMechanismsTable" displayName="AspectMechanismsTable" ref="A3:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClassificationAuditTable" displayName="ClassificationAuditTable" ref="A3:K72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
-    <x:tableColumn id="2" name="Reader effect"/>
-    <x:tableColumn id="3" name="Conflict behavior"/>
-    <x:tableColumn id="4" name="Movement bias"/>
-    <x:tableColumn id="5" name="Supportive realizations"/>
-    <x:tableColumn id="6" name="Neutral realizations"/>
-    <x:tableColumn id="7" name="Shadow realizations"/>
-    <x:tableColumn id="8" name="Source IDs"/>
-    <x:tableColumn id="9" name="Source hashes"/>
-    <x:tableColumn id="10" name="Owner review status"/>
-    <x:tableColumn id="11" name="Owner notes"/>
+    <x:tableColumn id="2" name="Reviewed population"/>
+    <x:tableColumn id="3" name="Before shape"/>
+    <x:tableColumn id="4" name="After shape"/>
+    <x:tableColumn id="5" name="Realization"/>
+    <x:tableColumn id="6" name="Before type"/>
+    <x:tableColumn id="7" name="After type"/>
+    <x:tableColumn id="8" name="Changed?"/>
+    <x:tableColumn id="9" name="Evidence finding"/>
+    <x:tableColumn id="10" name="Supportive-pool finding"/>
+    <x:tableColumn id="11" name="Evidence pointers"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ModalityUnitsTable" displayName="ModalityUnitsTable" ref="A3:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AspectMechanismsTable" displayName="AspectMechanismsTable" ref="A3:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Reader effect"/>
@@ -336,7 +348,26 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ElementUnitsTable" displayName="ElementUnitsTable" ref="A3:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ModalityUnitsTable" displayName="ModalityUnitsTable" ref="A3:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Key"/>
+    <x:tableColumn id="2" name="Reader effect"/>
+    <x:tableColumn id="3" name="Conflict behavior"/>
+    <x:tableColumn id="4" name="Movement bias"/>
+    <x:tableColumn id="5" name="Supportive realizations"/>
+    <x:tableColumn id="6" name="Neutral realizations"/>
+    <x:tableColumn id="7" name="Shadow realizations"/>
+    <x:tableColumn id="8" name="Source IDs"/>
+    <x:tableColumn id="9" name="Source hashes"/>
+    <x:tableColumn id="10" name="Owner review status"/>
+    <x:tableColumn id="11" name="Owner notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ElementUnitsTable" displayName="ElementUnitsTable" ref="A3:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Reader effect"/>
@@ -724,11 +755,27 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="13" t="str">
+      <x:c r="A13" s="12" t="str">
         <x:v>One-sided after pass</x:v>
       </x:c>
-      <x:c r="B13" s="13" t="n">
+      <x:c r="B13" s="12" t="n">
         <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="12" t="str">
+        <x:v>Realizations reclassified</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="n">
+        <x:v>44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>Empty supportive pools</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="n">
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1641,13 +1688,15 @@
       <x:c r="D7" s="45" t="str">
         <x:v>the care people provide in private starts deciding who represents the group</x:v>
       </x:c>
-      <x:c r="E7" s="45" t="str"/>
+      <x:c r="E7" s="45" t="str">
+        <x:v>• someone doing the care work that everyone else depends on</x:v>
+      </x:c>
       <x:c r="F7" s="45" t="str">
-        <x:v>• someone doing the care work that everyone else depends on
-• family members using private loyalty to influence who gets acknowledged publicly
-• someone representing the group because they remember its history</x:v>
-      </x:c>
-      <x:c r="G7" s="45" t="str"/>
+        <x:v>• someone representing the group because they remember its history</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>• family members using private loyalty to influence who gets acknowledged publicly</x:v>
+      </x:c>
       <x:c r="H7" s="45" t="str">
         <x:v>recognition tied to care and private loyalty</x:v>
       </x:c>
@@ -1826,10 +1875,11 @@
         <x:v>who gets named publicly depends on trust, privacy, and leverage behind the scenes</x:v>
       </x:c>
       <x:c r="E11" s="45" t="str"/>
-      <x:c r="F11" s="45" t="str"/>
+      <x:c r="F11" s="45" t="str">
+        <x:v>• the public representative carrying private obligations others cannot see</x:v>
+      </x:c>
       <x:c r="G11" s="45" t="str">
         <x:v>• someone withholding recognition until trust and access are settled
-• the public representative carrying private obligations others cannot see
 • someone using public credit as leverage in a decision with lasting consequences</x:v>
       </x:c>
       <x:c r="H11" s="45" t="str">
@@ -1870,13 +1920,15 @@
       <x:c r="D12" s="45" t="str">
         <x:v>whoever names the larger purpose can become the face of it</x:v>
       </x:c>
-      <x:c r="E12" s="45" t="str"/>
+      <x:c r="E12" s="45" t="str">
+        <x:v>• a strong belief making one contribution stand for a larger cause</x:v>
+      </x:c>
       <x:c r="F12" s="45" t="str">
-        <x:v>• a strong belief making one contribution stand for a larger cause
-• people carrying someone's work to an audience it was not made for
-• the person who names the wider purpose becoming identified with it</x:v>
-      </x:c>
-      <x:c r="G12" s="45" t="str"/>
+        <x:v>• the person who names the wider purpose becoming identified with it</x:v>
+      </x:c>
+      <x:c r="G12" s="45" t="str">
+        <x:v>• people carrying someone's work to an audience it was not made for</x:v>
+      </x:c>
       <x:c r="H12" s="45" t="str">
         <x:v>visible conviction and larger aims</x:v>
       </x:c>
@@ -2513,13 +2565,15 @@
       <x:c r="D25" s="45" t="str">
         <x:v>people put the duty first and deal with the feeling after the work is done</x:v>
       </x:c>
-      <x:c r="E25" s="45" t="str"/>
+      <x:c r="E25" s="45" t="str">
+        <x:v>• someone relying on repeated follow-through instead of reassurance to know they belong</x:v>
+      </x:c>
       <x:c r="F25" s="45" t="str">
-        <x:v>• someone postponing their needs until the required work is done
-• someone showing care by taking responsibility while keeping their feelings private
-• someone relying on repeated follow-through instead of reassurance to know they belong</x:v>
-      </x:c>
-      <x:c r="G25" s="45" t="str"/>
+        <x:v>• someone showing care by taking responsibility while keeping their feelings private</x:v>
+      </x:c>
+      <x:c r="G25" s="45" t="str">
+        <x:v>• someone postponing their needs until the required work is done</x:v>
+      </x:c>
       <x:c r="H25" s="45" t="str">
         <x:v>emotional needs managed through duty and restraint</x:v>
       </x:c>
@@ -3207,13 +3261,14 @@
       <x:c r="D39" s="45" t="str">
         <x:v>people understand the tone or image sooner than they agree on the facts</x:v>
       </x:c>
-      <x:c r="E39" s="45" t="str"/>
-      <x:c r="F39" s="45" t="str">
-        <x:v>• people reading the tone when the stated facts remain incomplete
-• an implication spreading faster than anyone can verify it
+      <x:c r="E39" s="45" t="str">
+        <x:v>• people reading the tone when the stated facts remain incomplete</x:v>
+      </x:c>
+      <x:c r="F39" s="45" t="str"/>
+      <x:c r="G39" s="45" t="str">
+        <x:v>• an implication spreading faster than anyone can verify it
 • a decision blurred by sympathy for several incompatible accounts</x:v>
       </x:c>
-      <x:c r="G39" s="45" t="str"/>
       <x:c r="H39" s="45" t="str">
         <x:v>implied meaning and uncertain facts</x:v>
       </x:c>
@@ -3866,12 +3921,14 @@
       <x:c r="D52" s="45" t="str">
         <x:v>someone acts as soon as the problem appears and everyone else has to respond</x:v>
       </x:c>
-      <x:c r="E52" s="45" t="str"/>
-      <x:c r="F52" s="45" t="str"/>
+      <x:c r="E52" s="45" t="str">
+        <x:v>• a visible result pursued without waiting for broader support</x:v>
+      </x:c>
+      <x:c r="F52" s="45" t="str">
+        <x:v>• the first move establishing who controls the pace</x:v>
+      </x:c>
       <x:c r="G52" s="45" t="str">
-        <x:v>• the first move establishing who controls the pace
-• someone acting on the pressure before the group agrees on a process
-• a visible result pursued without waiting for broader support</x:v>
+        <x:v>• someone acting on the pressure before the group agrees on a process</x:v>
       </x:c>
       <x:c r="H52" s="45" t="str">
         <x:v>direct action reinforcing its own urgency</x:v>
@@ -3917,12 +3974,14 @@
       <x:c r="D53" s="45" t="str">
         <x:v>people keep pushing the same point until a material limit finally moves</x:v>
       </x:c>
-      <x:c r="E53" s="45" t="str"/>
-      <x:c r="F53" s="45" t="str"/>
+      <x:c r="E53" s="45" t="str">
+        <x:v>• someone working the same point until a material limit gives way</x:v>
+      </x:c>
+      <x:c r="F53" s="45" t="str">
+        <x:v>• someone delaying action until they can keep the result</x:v>
+      </x:c>
       <x:c r="G53" s="45" t="str">
-        <x:v>• someone working the same point until a material limit gives way
-• people arguing over the resource no one wants to surrender
-• someone delaying action until they can keep the result</x:v>
+        <x:v>• people arguing over the resource no one wants to surrender</x:v>
       </x:c>
       <x:c r="H53" s="45" t="str">
         <x:v>slow pressure around resources and fixed limits</x:v>
@@ -3968,13 +4027,14 @@
       <x:c r="D54" s="45" t="str">
         <x:v>people spread their effort across messages, errands, debates, and several moving targets</x:v>
       </x:c>
-      <x:c r="E54" s="45" t="str"/>
-      <x:c r="F54" s="45" t="str">
+      <x:c r="E54" s="45" t="str">
+        <x:v>• a new comparison redirecting action already underway</x:v>
+      </x:c>
+      <x:c r="F54" s="45" t="str"/>
+      <x:c r="G54" s="45" t="str">
         <x:v>• someone dividing their effort among several messages, errands, or targets
-• people changing the argument each time the wording changes
-• a new comparison redirecting action already underway</x:v>
-      </x:c>
-      <x:c r="G54" s="45" t="str"/>
+• people changing the argument each time the wording changes</x:v>
+      </x:c>
       <x:c r="H54" s="45" t="str">
         <x:v>scattered action and changing targets</x:v>
       </x:c>
@@ -4228,12 +4288,14 @@
       <x:c r="D59" s="45" t="str">
         <x:v>someone acts carefully because trust, control, and lasting consequences are involved</x:v>
       </x:c>
-      <x:c r="E59" s="45" t="str"/>
-      <x:c r="F59" s="45" t="str"/>
+      <x:c r="E59" s="45" t="str">
+        <x:v>• a result pursued carefully because it cannot be undone</x:v>
+      </x:c>
+      <x:c r="F59" s="45" t="str">
+        <x:v>• someone withholding action until the source of control becomes clear</x:v>
+      </x:c>
       <x:c r="G59" s="45" t="str">
-        <x:v>• someone withholding action until the source of control becomes clear
-• someone applying pressure where trust and private access are already at stake
-• a result pursued carefully because it cannot be undone</x:v>
+        <x:v>• someone applying pressure where trust and private access are already at stake</x:v>
       </x:c>
       <x:c r="H59" s="45" t="str">
         <x:v>strategic pursuit, trust, and control</x:v>
@@ -5300,10 +5362,11 @@
         <x:v>anyone seeking recognition has to show they can carry the result</x:v>
       </x:c>
       <x:c r="E80" s="45" t="str"/>
-      <x:c r="F80" s="45" t="str"/>
+      <x:c r="F80" s="45" t="str">
+        <x:v>• an authority limiting how much personal pride can direct the decision</x:v>
+      </x:c>
       <x:c r="G80" s="45" t="str">
         <x:v>• an authority withholding recognition until the visible contribution meets the standard
-• an authority limiting how much personal pride can direct the decision
 • someone withholding their contribution because uncertain recognition feels too risky</x:v>
       </x:c>
       <x:c r="H80" s="45" t="str">
@@ -5448,12 +5511,14 @@
       <x:c r="D83" s="45" t="str">
         <x:v>a hard limit reveals who controls access and who carries the lasting consequence</x:v>
       </x:c>
-      <x:c r="E83" s="45" t="str"/>
-      <x:c r="F83" s="45" t="str"/>
+      <x:c r="E83" s="45" t="str">
+        <x:v>• a limit protecting access to information that cannot be taken back</x:v>
+      </x:c>
+      <x:c r="F83" s="45" t="str">
+        <x:v>• someone carrying more responsibility because they also control the access</x:v>
+      </x:c>
       <x:c r="G83" s="45" t="str">
-        <x:v>• a limit protecting access to information that cannot be taken back
-• someone carrying more responsibility because they also control the access
-• an authority making the consequence official after people tried to postpone it</x:v>
+        <x:v>• an authority making the consequence official after people tried to postpone it</x:v>
       </x:c>
       <x:c r="H83" s="45" t="str">
         <x:v>hard limits, controlled access, and lasting consequences</x:v>
@@ -5599,11 +5664,12 @@
       <x:c r="D86" s="45" t="str">
         <x:v>the same rule is expected to apply across the group, even when one case resists it</x:v>
       </x:c>
-      <x:c r="E86" s="45" t="str"/>
+      <x:c r="E86" s="45" t="str">
+        <x:v>• a standard meant to apply equally</x:v>
+      </x:c>
       <x:c r="F86" s="45" t="str">
         <x:v>• policy applied across the group
-• precedent
-• a standard meant to apply equally</x:v>
+• precedent</x:v>
       </x:c>
       <x:c r="G86" s="45" t="str"/>
       <x:c r="H86" s="45" t="str">
@@ -5648,13 +5714,15 @@
       <x:c r="D87" s="45" t="str">
         <x:v>people try to set a firm boundary around a need that keeps changing shape</x:v>
       </x:c>
-      <x:c r="E87" s="45" t="str"/>
+      <x:c r="E87" s="45" t="str">
+        <x:v>• people keeping the plan intact by naming what remains uncertain</x:v>
+      </x:c>
       <x:c r="F87" s="45" t="str">
-        <x:v>• a formal boundary trying to contain a need that has no clean edge
-• people struggling to assign responsibility because everyone feels for the person involved
-• people keeping the plan intact by naming what remains uncertain</x:v>
-      </x:c>
-      <x:c r="G87" s="45" t="str"/>
+        <x:v>• a formal boundary trying to contain a need that has no clean edge</x:v>
+      </x:c>
+      <x:c r="G87" s="45" t="str">
+        <x:v>• people struggling to assign responsibility because everyone feels for the person involved</x:v>
+      </x:c>
       <x:c r="H87" s="45" t="str">
         <x:v>firm boundaries around a changing need</x:v>
       </x:c>
@@ -5851,13 +5919,15 @@
       <x:c r="D91" s="45" t="str">
         <x:v>an unexpected need for distance changes how care and belonging are arranged</x:v>
       </x:c>
-      <x:c r="E91" s="45" t="str"/>
+      <x:c r="E91" s="45" t="str">
+        <x:v>• a household pattern changing because someone needs more room</x:v>
+      </x:c>
       <x:c r="F91" s="45" t="str">
-        <x:v>• a household pattern changing because someone needs more room
-• people reorganizing who belongs after private care becomes a public concern
-• someone leaving the role that once guaranteed emotional safety</x:v>
-      </x:c>
-      <x:c r="G91" s="45" t="str"/>
+        <x:v>• people reorganizing who belongs after private care becomes a public concern</x:v>
+      </x:c>
+      <x:c r="G91" s="45" t="str">
+        <x:v>• someone leaving the role that once guaranteed emotional safety</x:v>
+      </x:c>
       <x:c r="H91" s="45" t="str">
         <x:v>independence disrupting care and belonging</x:v>
       </x:c>
@@ -6252,13 +6322,15 @@
       <x:c r="D99" s="45" t="str">
         <x:v>the change arrives through a hunch or mood before anyone can draw a clean boundary around it</x:v>
       </x:c>
-      <x:c r="E99" s="45" t="str"/>
+      <x:c r="E99" s="45" t="str">
+        <x:v>• someone stepping away after others mistook sympathy for agreement</x:v>
+      </x:c>
       <x:c r="F99" s="45" t="str">
-        <x:v>• a sudden intuition disrupting a boundary that was already unclear
-• someone stepping away after others mistook sympathy for agreement
-• people changing course together before anyone can define the plan</x:v>
-      </x:c>
-      <x:c r="G99" s="45" t="str"/>
+        <x:v>• a sudden intuition disrupting a boundary that was already unclear</x:v>
+      </x:c>
+      <x:c r="G99" s="45" t="str">
+        <x:v>• people changing course together before anyone can define the plan</x:v>
+      </x:c>
       <x:c r="H99" s="45" t="str">
         <x:v>intuitive disruption and uncertain boundaries</x:v>
       </x:c>
@@ -6459,11 +6531,12 @@
       </x:c>
       <x:c r="E103" s="45" t="str"/>
       <x:c r="F103" s="45" t="str">
+        <x:v>• a private longing shaping what the group believes it needs</x:v>
+      </x:c>
+      <x:c r="G103" s="45" t="str">
         <x:v>• memory softening the difference between care and projection
-• a private longing shaping what the group believes it needs
 • people idealizing the family bond until they stop seeing who carries the emotional labor</x:v>
       </x:c>
-      <x:c r="G103" s="45" t="str"/>
       <x:c r="H103" s="45" t="str">
         <x:v>memory, care, and projection</x:v>
       </x:c>
@@ -6659,11 +6732,12 @@
       </x:c>
       <x:c r="E107" s="45" t="str"/>
       <x:c r="F107" s="45" t="str">
-        <x:v>• trust deepening around a motive no one can fully name
-• people losing track of who holds private power as the boundaries soften
+        <x:v>• trust deepening around a motive no one can fully name</x:v>
+      </x:c>
+      <x:c r="G107" s="45" t="str">
+        <x:v>• people losing track of who holds private power as the boundaries soften
 • an irreversible choice shaped by information that remains uncertain</x:v>
       </x:c>
-      <x:c r="G107" s="45" t="str"/>
       <x:c r="H107" s="45" t="str">
         <x:v>uncertain trust and hidden power</x:v>
       </x:c>
@@ -6859,13 +6933,15 @@
       <x:c r="D111" s="45" t="str">
         <x:v>people share a feeling or hope before anyone can tell where it began or what it asks</x:v>
       </x:c>
-      <x:c r="E111" s="45" t="str"/>
+      <x:c r="E111" s="45" t="str">
+        <x:v>• people imagining more because the facts do not set a firm boundary</x:v>
+      </x:c>
       <x:c r="F111" s="45" t="str">
-        <x:v>• people treating a shared feeling as if it creates the same duty for everyone
-• people imagining more because the facts do not set a firm boundary
-• a collective longing becoming the atmosphere around the decision</x:v>
-      </x:c>
-      <x:c r="G111" s="45" t="str"/>
+        <x:v>• a collective longing becoming the atmosphere around the decision</x:v>
+      </x:c>
+      <x:c r="G111" s="45" t="str">
+        <x:v>• people treating a shared feeling as if it creates the same duty for everyone</x:v>
+      </x:c>
       <x:c r="H111" s="45" t="str">
         <x:v>imagination and uncertainty dissolving the boundary between them</x:v>
       </x:c>
@@ -7611,10 +7687,11 @@
       <x:c r="E126" s="45" t="str"/>
       <x:c r="F126" s="45" t="str">
         <x:v>• careful wording shaped by the fear of being misunderstood again
-• a question carrying the memory of not being believed
-• someone reacting after every official explanation leaves out what they lived through</x:v>
-      </x:c>
-      <x:c r="G126" s="45" t="str"/>
+• a question carrying the memory of not being believed</x:v>
+      </x:c>
+      <x:c r="G126" s="45" t="str">
+        <x:v>• someone reacting after every official explanation leaves out what they lived through</x:v>
+      </x:c>
       <x:c r="H126" s="45" t="str">
         <x:v>sensitivity around language and being understood</x:v>
       </x:c>
@@ -8243,12 +8320,13 @@
       <x:c r="D140" s="45" t="str">
         <x:v>someone claims visibility without making the difficult part more acceptable first</x:v>
       </x:c>
-      <x:c r="E140" s="45" t="str"/>
+      <x:c r="E140" s="45" t="str">
+        <x:v>• someone claiming visibility without making the contribution more acceptable first
+• someone rejecting recognition that depends on shrinking the difficult part</x:v>
+      </x:c>
       <x:c r="F140" s="45" t="str"/>
       <x:c r="G140" s="45" t="str">
-        <x:v>• someone claiming visibility without making the contribution more acceptable first
-• someone rejecting recognition that depends on shrinking the difficult part
-• someone making the whole conflict about them because shame is harder to name directly</x:v>
+        <x:v>• someone making the whole conflict about them because shame is harder to name directly</x:v>
       </x:c>
       <x:c r="H140" s="45" t="str">
         <x:v>visible refusal of conditional recognition</x:v>
@@ -8286,13 +8364,14 @@
       <x:c r="D141" s="45" t="str">
         <x:v>people reject a standard that treats usefulness or purity as the price of worth</x:v>
       </x:c>
-      <x:c r="E141" s="45" t="str"/>
-      <x:c r="F141" s="45" t="str"/>
-      <x:c r="G141" s="45" t="str">
+      <x:c r="E141" s="45" t="str">
         <x:v>• a standard refused because usefulness has become a condition of worth
-• someone defending their difference against correction meant to make it manageable
-• the excluded need exposing what the approved method cannot serve</x:v>
-      </x:c>
+• someone defending their difference against correction meant to make it manageable</x:v>
+      </x:c>
+      <x:c r="F141" s="45" t="str">
+        <x:v>• the excluded need exposing what the approved method cannot serve</x:v>
+      </x:c>
+      <x:c r="G141" s="45" t="str"/>
       <x:c r="H141" s="45" t="str">
         <x:v>refusal of purity and usefulness standards</x:v>
       </x:c>
@@ -8462,13 +8541,14 @@
       <x:c r="D145" s="45" t="str">
         <x:v>people confront an authority that uses duty or respectability to demand compliance</x:v>
       </x:c>
-      <x:c r="E145" s="45" t="str"/>
-      <x:c r="F145" s="45" t="str"/>
-      <x:c r="G145" s="45" t="str">
+      <x:c r="E145" s="45" t="str">
         <x:v>• someone confronting an authority that has used respectability as control
-• a duty refused because compliance would erase the person carrying it
-• someone accepting the consequence rather than obeying the demand</x:v>
-      </x:c>
+• a duty refused because compliance would erase the person carrying it</x:v>
+      </x:c>
+      <x:c r="F145" s="45" t="str">
+        <x:v>• someone accepting the consequence rather than obeying the demand</x:v>
+      </x:c>
+      <x:c r="G145" s="45" t="str"/>
       <x:c r="H145" s="45" t="str">
         <x:v>autonomy against authority and respectability</x:v>
       </x:c>
@@ -8595,12 +8675,2639 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf415532dbe2f44b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaa587e4387c4ddd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="62" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="68" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="72" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="I1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="J1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+      <x:c r="K1" s="3" t="str">
+        <x:v>Realization classification audit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="I2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="J2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+      <x:c r="K2" s="7" t="str">
+        <x:v>Classification only: wording and evidence are unchanged. The 10-unit prompt count refers to all-shadow units; 81 units originally had no supportive realization.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B3" s="35" t="str">
+        <x:v>Reviewed population</x:v>
+      </x:c>
+      <x:c r="C3" s="35" t="str">
+        <x:v>Before shape</x:v>
+      </x:c>
+      <x:c r="D3" s="35" t="str">
+        <x:v>After shape</x:v>
+      </x:c>
+      <x:c r="E3" s="35" t="str">
+        <x:v>Realization</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>Before type</x:v>
+      </x:c>
+      <x:c r="G3" s="35" t="str">
+        <x:v>After type</x:v>
+      </x:c>
+      <x:c r="H3" s="35" t="str">
+        <x:v>Changed?</x:v>
+      </x:c>
+      <x:c r="I3" s="35" t="str">
+        <x:v>Evidence finding</x:v>
+      </x:c>
+      <x:c r="J3" s="35" t="str">
+        <x:v>Supportive-pool finding</x:v>
+      </x:c>
+      <x:c r="K3" s="36" t="str">
+        <x:v>Evidence pointers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="44" t="str">
+        <x:v>sky-sign/sun/cancer</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C4" s="44" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D4" s="44" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E4" s="44" t="str">
+        <x:v>someone doing the care work that everyone else depends on</x:v>
+      </x:c>
+      <x:c r="F4" s="44" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G4" s="44" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H4" s="44" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I4" s="44" t="str">
+        <x:v>Care work that others depend on is supportive; private loyalty deciding public recognition carries a source-supported cost.</x:v>
+      </x:c>
+      <x:c r="J4" s="44" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K4" s="44" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!803</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>sky-sign/sun/cancer</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>family members using private loyalty to influence who gets acknowledged publicly</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="str">
+        <x:v>Care work that others depend on is supportive; private loyalty deciding public recognition carries a source-supported cost.</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K5" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!803</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="45" t="str">
+        <x:v>sky-sign/sun/cancer</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E6" s="45" t="str">
+        <x:v>someone representing the group because they remember its history</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="str">
+        <x:v>Care work that others depend on is supportive; private loyalty deciding public recognition carries a source-supported cost.</x:v>
+      </x:c>
+      <x:c r="J6" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K6" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!803</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="45" t="str">
+        <x:v>sky-sign/sun/sagittarius</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="str">
+        <x:v>a strong belief making one contribution stand for a larger cause</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="str">
+        <x:v>A larger purpose can support reach, while carrying work to an audience it was not made for carries the source warning about certainty outrunning facts.</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K7" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/sagittarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!845</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="45" t="str">
+        <x:v>sky-sign/sun/sagittarius</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E8" s="45" t="str">
+        <x:v>people carrying someone's work to an audience it was not made for</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="str">
+        <x:v>A larger purpose can support reach, while carrying work to an audience it was not made for carries the source warning about certainty outrunning facts.</x:v>
+      </x:c>
+      <x:c r="J8" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K8" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/sagittarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!845</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="45" t="str">
+        <x:v>sky-sign/sun/sagittarius</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="str">
+        <x:v>the person who names the wider purpose becoming identified with it</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="str">
+        <x:v>A larger purpose can support reach, while carrying work to an audience it was not made for carries the source warning about certainty outrunning facts.</x:v>
+      </x:c>
+      <x:c r="J9" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K9" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/sagittarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!845</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="45" t="str">
+        <x:v>sky-sign/moon/capricorn</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E10" s="45" t="str">
+        <x:v>someone postponing their needs until the required work is done</x:v>
+      </x:c>
+      <x:c r="F10" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="str">
+        <x:v>Postponing needs carries the source cost; dependable follow-through is the supportive form already present in the wording.</x:v>
+      </x:c>
+      <x:c r="J10" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K10" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/moon/capricorn
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="45" t="str">
+        <x:v>sky-sign/moon/capricorn</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="str">
+        <x:v>someone showing care by taking responsibility while keeping their feelings private</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I11" s="45" t="str">
+        <x:v>Postponing needs carries the source cost; dependable follow-through is the supportive form already present in the wording.</x:v>
+      </x:c>
+      <x:c r="J11" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K11" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/moon/capricorn
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="45" t="str">
+        <x:v>sky-sign/moon/capricorn</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C12" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D12" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E12" s="45" t="str">
+        <x:v>someone relying on repeated follow-through instead of reassurance to know they belong</x:v>
+      </x:c>
+      <x:c r="F12" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G12" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H12" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I12" s="45" t="str">
+        <x:v>Postponing needs carries the source cost; dependable follow-through is the supportive form already present in the wording.</x:v>
+      </x:c>
+      <x:c r="J12" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K12" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/moon/capricorn
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="45" t="str">
+        <x:v>sky-sign/mercury/pisces</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="str">
+        <x:v>1/0/2</x:v>
+      </x:c>
+      <x:c r="E13" s="45" t="str">
+        <x:v>people reading the tone when the stated facts remain incomplete</x:v>
+      </x:c>
+      <x:c r="F13" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G13" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I13" s="45" t="str">
+        <x:v>Reading tone can carry the source-supported intuitive strength; unverified implication and blurred decisions carry its translation and verification costs.</x:v>
+      </x:c>
+      <x:c r="J13" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K13" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mercury/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!466
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="45" t="str">
+        <x:v>sky-sign/mercury/pisces</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C14" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="str">
+        <x:v>1/0/2</x:v>
+      </x:c>
+      <x:c r="E14" s="45" t="str">
+        <x:v>an implication spreading faster than anyone can verify it</x:v>
+      </x:c>
+      <x:c r="F14" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I14" s="45" t="str">
+        <x:v>Reading tone can carry the source-supported intuitive strength; unverified implication and blurred decisions carry its translation and verification costs.</x:v>
+      </x:c>
+      <x:c r="J14" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K14" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mercury/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!466
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="45" t="str">
+        <x:v>sky-sign/mercury/pisces</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D15" s="45" t="str">
+        <x:v>1/0/2</x:v>
+      </x:c>
+      <x:c r="E15" s="45" t="str">
+        <x:v>a decision blurred by sympathy for several incompatible accounts</x:v>
+      </x:c>
+      <x:c r="F15" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H15" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I15" s="45" t="str">
+        <x:v>Reading tone can carry the source-supported intuitive strength; unverified implication and blurred decisions carry its translation and verification costs.</x:v>
+      </x:c>
+      <x:c r="J15" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K15" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mercury/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!466
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="45" t="str">
+        <x:v>sky-sign/mars/gemini</x:v>
+      </x:c>
+      <x:c r="B16" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C16" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D16" s="45" t="str">
+        <x:v>1/0/2</x:v>
+      </x:c>
+      <x:c r="E16" s="45" t="str">
+        <x:v>someone dividing their effort among several messages, errands, or targets</x:v>
+      </x:c>
+      <x:c r="F16" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G16" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H16" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I16" s="45" t="str">
+        <x:v>Scattered effort and a moving argument carry the concentration cost; a new comparison redirecting action carries the source-supported adaptive opening.</x:v>
+      </x:c>
+      <x:c r="J16" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K16" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!147
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="45" t="str">
+        <x:v>sky-sign/mars/gemini</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C17" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D17" s="45" t="str">
+        <x:v>1/0/2</x:v>
+      </x:c>
+      <x:c r="E17" s="45" t="str">
+        <x:v>people changing the argument each time the wording changes</x:v>
+      </x:c>
+      <x:c r="F17" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G17" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H17" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I17" s="45" t="str">
+        <x:v>Scattered effort and a moving argument carry the concentration cost; a new comparison redirecting action carries the source-supported adaptive opening.</x:v>
+      </x:c>
+      <x:c r="J17" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K17" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!147
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="45" t="str">
+        <x:v>sky-sign/mars/gemini</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C18" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D18" s="45" t="str">
+        <x:v>1/0/2</x:v>
+      </x:c>
+      <x:c r="E18" s="45" t="str">
+        <x:v>a new comparison redirecting action already underway</x:v>
+      </x:c>
+      <x:c r="F18" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G18" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H18" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I18" s="45" t="str">
+        <x:v>Scattered effort and a moving argument carry the concentration cost; a new comparison redirecting action carries the source-supported adaptive opening.</x:v>
+      </x:c>
+      <x:c r="J18" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K18" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!147
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="45" t="str">
+        <x:v>sky-sign/saturn/aquarius</x:v>
+      </x:c>
+      <x:c r="B19" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C19" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D19" s="45" t="str">
+        <x:v>1/2/0</x:v>
+      </x:c>
+      <x:c r="E19" s="45" t="str">
+        <x:v>policy applied across the group</x:v>
+      </x:c>
+      <x:c r="F19" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G19" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H19" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I19" s="45" t="str">
+        <x:v>An equal standard is the supportive form. Policy and precedent remain neutral because their effect depends on the card's argument shape.</x:v>
+      </x:c>
+      <x:c r="J19" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K19" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/aquarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!719</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="45" t="str">
+        <x:v>sky-sign/saturn/aquarius</x:v>
+      </x:c>
+      <x:c r="B20" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C20" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D20" s="45" t="str">
+        <x:v>1/2/0</x:v>
+      </x:c>
+      <x:c r="E20" s="45" t="str">
+        <x:v>precedent</x:v>
+      </x:c>
+      <x:c r="F20" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G20" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H20" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I20" s="45" t="str">
+        <x:v>An equal standard is the supportive form. Policy and precedent remain neutral because their effect depends on the card's argument shape.</x:v>
+      </x:c>
+      <x:c r="J20" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K20" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/aquarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!719</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="45" t="str">
+        <x:v>sky-sign/saturn/aquarius</x:v>
+      </x:c>
+      <x:c r="B21" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C21" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D21" s="45" t="str">
+        <x:v>1/2/0</x:v>
+      </x:c>
+      <x:c r="E21" s="45" t="str">
+        <x:v>a standard meant to apply equally</x:v>
+      </x:c>
+      <x:c r="F21" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G21" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H21" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I21" s="45" t="str">
+        <x:v>An equal standard is the supportive form. Policy and precedent remain neutral because their effect depends on the card's argument shape.</x:v>
+      </x:c>
+      <x:c r="J21" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K21" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/aquarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!719</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="45" t="str">
+        <x:v>sky-sign/saturn/pisces</x:v>
+      </x:c>
+      <x:c r="B22" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C22" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D22" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E22" s="45" t="str">
+        <x:v>a formal boundary trying to contain a need that has no clean edge</x:v>
+      </x:c>
+      <x:c r="F22" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G22" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H22" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I22" s="45" t="str">
+        <x:v>Difficulty assigning responsibility carries the cost; naming uncertainty so the plan can hold is the supported constructive form.</x:v>
+      </x:c>
+      <x:c r="J22" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K22" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!733</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="45" t="str">
+        <x:v>sky-sign/saturn/pisces</x:v>
+      </x:c>
+      <x:c r="B23" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C23" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D23" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E23" s="45" t="str">
+        <x:v>people struggling to assign responsibility because everyone feels for the person involved</x:v>
+      </x:c>
+      <x:c r="F23" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G23" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H23" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I23" s="45" t="str">
+        <x:v>Difficulty assigning responsibility carries the cost; naming uncertainty so the plan can hold is the supported constructive form.</x:v>
+      </x:c>
+      <x:c r="J23" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K23" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!733</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="45" t="str">
+        <x:v>sky-sign/saturn/pisces</x:v>
+      </x:c>
+      <x:c r="B24" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C24" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D24" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E24" s="45" t="str">
+        <x:v>people keeping the plan intact by naming what remains uncertain</x:v>
+      </x:c>
+      <x:c r="F24" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G24" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H24" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I24" s="45" t="str">
+        <x:v>Difficulty assigning responsibility carries the cost; naming uncertainty so the plan can hold is the supported constructive form.</x:v>
+      </x:c>
+      <x:c r="J24" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K24" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!733</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="45" t="str">
+        <x:v>sky-sign/uranus/cancer</x:v>
+      </x:c>
+      <x:c r="B25" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C25" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D25" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E25" s="45" t="str">
+        <x:v>a household pattern changing because someone needs more room</x:v>
+      </x:c>
+      <x:c r="F25" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G25" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H25" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I25" s="45" t="str">
+        <x:v>Making room through a changed household pattern is supportive; leaving a role that once guaranteed safety carries the source cost of disruption.</x:v>
+      </x:c>
+      <x:c r="J25" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K25" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!939</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="45" t="str">
+        <x:v>sky-sign/uranus/cancer</x:v>
+      </x:c>
+      <x:c r="B26" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C26" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D26" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E26" s="45" t="str">
+        <x:v>people reorganizing who belongs after private care becomes a public concern</x:v>
+      </x:c>
+      <x:c r="F26" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G26" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H26" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I26" s="45" t="str">
+        <x:v>Making room through a changed household pattern is supportive; leaving a role that once guaranteed safety carries the source cost of disruption.</x:v>
+      </x:c>
+      <x:c r="J26" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K26" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!939</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="45" t="str">
+        <x:v>sky-sign/uranus/cancer</x:v>
+      </x:c>
+      <x:c r="B27" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C27" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D27" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E27" s="45" t="str">
+        <x:v>someone leaving the role that once guaranteed emotional safety</x:v>
+      </x:c>
+      <x:c r="F27" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G27" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H27" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I27" s="45" t="str">
+        <x:v>Making room through a changed household pattern is supportive; leaving a role that once guaranteed safety carries the source cost of disruption.</x:v>
+      </x:c>
+      <x:c r="J27" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K27" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!939</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="45" t="str">
+        <x:v>sky-sign/uranus/pisces</x:v>
+      </x:c>
+      <x:c r="B28" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C28" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D28" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E28" s="45" t="str">
+        <x:v>a sudden intuition disrupting a boundary that was already unclear</x:v>
+      </x:c>
+      <x:c r="F28" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G28" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H28" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I28" s="45" t="str">
+        <x:v>Stepping away after sympathy was mistaken for agreement is a supported boundary correction; changing course before a plan exists carries the disruption cost.</x:v>
+      </x:c>
+      <x:c r="J28" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K28" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!955</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="45" t="str">
+        <x:v>sky-sign/uranus/pisces</x:v>
+      </x:c>
+      <x:c r="B29" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C29" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D29" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E29" s="45" t="str">
+        <x:v>someone stepping away after others mistook sympathy for agreement</x:v>
+      </x:c>
+      <x:c r="F29" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G29" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H29" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I29" s="45" t="str">
+        <x:v>Stepping away after sympathy was mistaken for agreement is a supported boundary correction; changing course before a plan exists carries the disruption cost.</x:v>
+      </x:c>
+      <x:c r="J29" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K29" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!955</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="45" t="str">
+        <x:v>sky-sign/uranus/pisces</x:v>
+      </x:c>
+      <x:c r="B30" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C30" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D30" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E30" s="45" t="str">
+        <x:v>people changing course together before anyone can define the plan</x:v>
+      </x:c>
+      <x:c r="F30" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G30" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H30" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I30" s="45" t="str">
+        <x:v>Stepping away after sympathy was mistaken for agreement is a supported boundary correction; changing course before a plan exists carries the disruption cost.</x:v>
+      </x:c>
+      <x:c r="J30" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K30" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!955</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="45" t="str">
+        <x:v>sky-sign/neptune/cancer</x:v>
+      </x:c>
+      <x:c r="B31" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C31" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D31" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E31" s="45" t="str">
+        <x:v>memory softening the difference between care and projection</x:v>
+      </x:c>
+      <x:c r="F31" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G31" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H31" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I31" s="45" t="str">
+        <x:v>Blurred care and projection and unseen emotional labor both carry the source's idealization cost; private longing shaping a group need remains neutral.</x:v>
+      </x:c>
+      <x:c r="J31" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K31" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!537</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="45" t="str">
+        <x:v>sky-sign/neptune/cancer</x:v>
+      </x:c>
+      <x:c r="B32" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C32" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D32" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E32" s="45" t="str">
+        <x:v>a private longing shaping what the group believes it needs</x:v>
+      </x:c>
+      <x:c r="F32" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G32" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H32" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I32" s="45" t="str">
+        <x:v>Blurred care and projection and unseen emotional labor both carry the source's idealization cost; private longing shaping a group need remains neutral.</x:v>
+      </x:c>
+      <x:c r="J32" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K32" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!537</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="45" t="str">
+        <x:v>sky-sign/neptune/cancer</x:v>
+      </x:c>
+      <x:c r="B33" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C33" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D33" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E33" s="45" t="str">
+        <x:v>people idealizing the family bond until they stop seeing who carries the emotional labor</x:v>
+      </x:c>
+      <x:c r="F33" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G33" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H33" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I33" s="45" t="str">
+        <x:v>Blurred care and projection and unseen emotional labor both carry the source's idealization cost; private longing shaping a group need remains neutral.</x:v>
+      </x:c>
+      <x:c r="J33" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K33" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!537</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="45" t="str">
+        <x:v>sky-sign/neptune/scorpio</x:v>
+      </x:c>
+      <x:c r="B34" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C34" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D34" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E34" s="45" t="str">
+        <x:v>trust deepening around a motive no one can fully name</x:v>
+      </x:c>
+      <x:c r="F34" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G34" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H34" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I34" s="45" t="str">
+        <x:v>Unclear motive remains neutral; lost track of private power and an irreversible choice made with uncertain information carry the governed boundary and discernment costs.</x:v>
+      </x:c>
+      <x:c r="J34" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K34" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!545
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!247</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="45" t="str">
+        <x:v>sky-sign/neptune/scorpio</x:v>
+      </x:c>
+      <x:c r="B35" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C35" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D35" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E35" s="45" t="str">
+        <x:v>people losing track of who holds private power as the boundaries soften</x:v>
+      </x:c>
+      <x:c r="F35" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G35" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H35" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I35" s="45" t="str">
+        <x:v>Unclear motive remains neutral; lost track of private power and an irreversible choice made with uncertain information carry the governed boundary and discernment costs.</x:v>
+      </x:c>
+      <x:c r="J35" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K35" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!545
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!247</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="45" t="str">
+        <x:v>sky-sign/neptune/scorpio</x:v>
+      </x:c>
+      <x:c r="B36" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C36" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D36" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E36" s="45" t="str">
+        <x:v>an irreversible choice shaped by information that remains uncertain</x:v>
+      </x:c>
+      <x:c r="F36" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G36" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H36" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I36" s="45" t="str">
+        <x:v>Unclear motive remains neutral; lost track of private power and an irreversible choice made with uncertain information carry the governed boundary and discernment costs.</x:v>
+      </x:c>
+      <x:c r="J36" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K36" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!545
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!247</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="45" t="str">
+        <x:v>sky-sign/neptune/pisces</x:v>
+      </x:c>
+      <x:c r="B37" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C37" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D37" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E37" s="45" t="str">
+        <x:v>people treating a shared feeling as if it creates the same duty for everyone</x:v>
+      </x:c>
+      <x:c r="F37" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G37" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H37" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I37" s="45" t="str">
+        <x:v>Treating one feeling as the same duty for everyone carries a cost; imagining beyond a firm factual boundary carries the creative opening supported by the source.</x:v>
+      </x:c>
+      <x:c r="J37" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K37" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!555</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="45" t="str">
+        <x:v>sky-sign/neptune/pisces</x:v>
+      </x:c>
+      <x:c r="B38" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C38" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D38" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E38" s="45" t="str">
+        <x:v>people imagining more because the facts do not set a firm boundary</x:v>
+      </x:c>
+      <x:c r="F38" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G38" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H38" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I38" s="45" t="str">
+        <x:v>Treating one feeling as the same duty for everyone carries a cost; imagining beyond a firm factual boundary carries the creative opening supported by the source.</x:v>
+      </x:c>
+      <x:c r="J38" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K38" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!555</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="45" t="str">
+        <x:v>sky-sign/neptune/pisces</x:v>
+      </x:c>
+      <x:c r="B39" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C39" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D39" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E39" s="45" t="str">
+        <x:v>a collective longing becoming the atmosphere around the decision</x:v>
+      </x:c>
+      <x:c r="F39" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G39" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H39" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I39" s="45" t="str">
+        <x:v>Treating one feeling as the same duty for everyone carries a cost; imagining beyond a firm factual boundary carries the creative opening supported by the source.</x:v>
+      </x:c>
+      <x:c r="J39" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K39" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!555</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="45" t="str">
+        <x:v>sky-sign/chiron/gemini</x:v>
+      </x:c>
+      <x:c r="B40" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C40" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D40" s="45" t="str">
+        <x:v>0/2/1</x:v>
+      </x:c>
+      <x:c r="E40" s="45" t="str">
+        <x:v>careful wording shaped by the fear of being misunderstood again</x:v>
+      </x:c>
+      <x:c r="F40" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G40" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H40" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I40" s="45" t="str">
+        <x:v>Careful wording and a question shaped by prior disbelief remain neutral; reacting after repeated omission carries the source-supported cost.</x:v>
+      </x:c>
+      <x:c r="J40" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K40" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/chiron/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="45" t="str">
+        <x:v>sky-sign/chiron/gemini</x:v>
+      </x:c>
+      <x:c r="B41" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C41" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D41" s="45" t="str">
+        <x:v>0/2/1</x:v>
+      </x:c>
+      <x:c r="E41" s="45" t="str">
+        <x:v>a question carrying the memory of not being believed</x:v>
+      </x:c>
+      <x:c r="F41" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G41" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H41" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I41" s="45" t="str">
+        <x:v>Careful wording and a question shaped by prior disbelief remain neutral; reacting after repeated omission carries the source-supported cost.</x:v>
+      </x:c>
+      <x:c r="J41" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K41" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/chiron/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="45" t="str">
+        <x:v>sky-sign/chiron/gemini</x:v>
+      </x:c>
+      <x:c r="B42" s="45" t="str">
+        <x:v>all_neutral</x:v>
+      </x:c>
+      <x:c r="C42" s="45" t="str">
+        <x:v>0/3/0</x:v>
+      </x:c>
+      <x:c r="D42" s="45" t="str">
+        <x:v>0/2/1</x:v>
+      </x:c>
+      <x:c r="E42" s="45" t="str">
+        <x:v>someone reacting after every official explanation leaves out what they lived through</x:v>
+      </x:c>
+      <x:c r="F42" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="G42" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H42" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I42" s="45" t="str">
+        <x:v>Careful wording and a question shaped by prior disbelief remain neutral; reacting after repeated omission carries the source-supported cost.</x:v>
+      </x:c>
+      <x:c r="J42" s="45" t="str">
+        <x:v>not part of all-shadow review</x:v>
+      </x:c>
+      <x:c r="K42" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/chiron/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="45" t="str">
+        <x:v>sky-sign/sun/scorpio</x:v>
+      </x:c>
+      <x:c r="B43" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C43" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D43" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E43" s="45" t="str">
+        <x:v>someone withholding recognition until trust and access are settled</x:v>
+      </x:c>
+      <x:c r="F43" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G43" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H43" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I43" s="45" t="str">
+        <x:v>Private obligations that others cannot see are a neutral condition, not automatically a cost.</x:v>
+      </x:c>
+      <x:c r="J43" s="45" t="str">
+        <x:v>The source carries a constructive truth-naming form, but no current realization expresses it; nothing was invented during this check.</x:v>
+      </x:c>
+      <x:c r="K43" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!838</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="45" t="str">
+        <x:v>sky-sign/sun/scorpio</x:v>
+      </x:c>
+      <x:c r="B44" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C44" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D44" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E44" s="45" t="str">
+        <x:v>the public representative carrying private obligations others cannot see</x:v>
+      </x:c>
+      <x:c r="F44" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G44" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H44" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I44" s="45" t="str">
+        <x:v>Private obligations that others cannot see are a neutral condition, not automatically a cost.</x:v>
+      </x:c>
+      <x:c r="J44" s="45" t="str">
+        <x:v>The source carries a constructive truth-naming form, but no current realization expresses it; nothing was invented during this check.</x:v>
+      </x:c>
+      <x:c r="K44" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!838</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="45" t="str">
+        <x:v>sky-sign/sun/scorpio</x:v>
+      </x:c>
+      <x:c r="B45" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C45" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D45" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E45" s="45" t="str">
+        <x:v>someone using public credit as leverage in a decision with lasting consequences</x:v>
+      </x:c>
+      <x:c r="F45" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G45" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H45" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I45" s="45" t="str">
+        <x:v>Private obligations that others cannot see are a neutral condition, not automatically a cost.</x:v>
+      </x:c>
+      <x:c r="J45" s="45" t="str">
+        <x:v>The source carries a constructive truth-naming form, but no current realization expresses it; nothing was invented during this check.</x:v>
+      </x:c>
+      <x:c r="K45" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!838</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="45" t="str">
+        <x:v>sky-sign/mars/aries</x:v>
+      </x:c>
+      <x:c r="B46" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C46" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D46" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E46" s="45" t="str">
+        <x:v>the first move establishing who controls the pace</x:v>
+      </x:c>
+      <x:c r="F46" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G46" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H46" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I46" s="45" t="str">
+        <x:v>The first move setting pace is neutral; acting before a process exists remains shadow.</x:v>
+      </x:c>
+      <x:c r="J46" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: direct pursuit of a visible result carries the source's initiative and renewed-momentum strength.</x:v>
+      </x:c>
+      <x:c r="K46" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/aries
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!128
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="45" t="str">
+        <x:v>sky-sign/mars/aries</x:v>
+      </x:c>
+      <x:c r="B47" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C47" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D47" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E47" s="45" t="str">
+        <x:v>someone acting on the pressure before the group agrees on a process</x:v>
+      </x:c>
+      <x:c r="F47" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G47" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H47" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I47" s="45" t="str">
+        <x:v>The first move setting pace is neutral; acting before a process exists remains shadow.</x:v>
+      </x:c>
+      <x:c r="J47" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: direct pursuit of a visible result carries the source's initiative and renewed-momentum strength.</x:v>
+      </x:c>
+      <x:c r="K47" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/aries
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!128
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="45" t="str">
+        <x:v>sky-sign/mars/aries</x:v>
+      </x:c>
+      <x:c r="B48" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C48" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D48" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E48" s="45" t="str">
+        <x:v>a visible result pursued without waiting for broader support</x:v>
+      </x:c>
+      <x:c r="F48" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G48" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H48" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I48" s="45" t="str">
+        <x:v>The first move setting pace is neutral; acting before a process exists remains shadow.</x:v>
+      </x:c>
+      <x:c r="J48" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: direct pursuit of a visible result carries the source's initiative and renewed-momentum strength.</x:v>
+      </x:c>
+      <x:c r="K48" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/aries
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!128
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="45" t="str">
+        <x:v>sky-sign/mars/taurus</x:v>
+      </x:c>
+      <x:c r="B49" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C49" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D49" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E49" s="45" t="str">
+        <x:v>someone working the same point until a material limit gives way</x:v>
+      </x:c>
+      <x:c r="F49" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G49" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H49" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I49" s="45" t="str">
+        <x:v>Resource conflict remains shadow; delaying until a result can be kept is neutral.</x:v>
+      </x:c>
+      <x:c r="J49" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: sustained work on one point carries the source's persistence and craftsmanship strength.</x:v>
+      </x:c>
+      <x:c r="K49" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!140
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="45" t="str">
+        <x:v>sky-sign/mars/taurus</x:v>
+      </x:c>
+      <x:c r="B50" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C50" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D50" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E50" s="45" t="str">
+        <x:v>people arguing over the resource no one wants to surrender</x:v>
+      </x:c>
+      <x:c r="F50" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G50" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H50" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I50" s="45" t="str">
+        <x:v>Resource conflict remains shadow; delaying until a result can be kept is neutral.</x:v>
+      </x:c>
+      <x:c r="J50" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: sustained work on one point carries the source's persistence and craftsmanship strength.</x:v>
+      </x:c>
+      <x:c r="K50" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!140
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="45" t="str">
+        <x:v>sky-sign/mars/taurus</x:v>
+      </x:c>
+      <x:c r="B51" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C51" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D51" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E51" s="45" t="str">
+        <x:v>someone delaying action until they can keep the result</x:v>
+      </x:c>
+      <x:c r="F51" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G51" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H51" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I51" s="45" t="str">
+        <x:v>Resource conflict remains shadow; delaying until a result can be kept is neutral.</x:v>
+      </x:c>
+      <x:c r="J51" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: sustained work on one point carries the source's persistence and craftsmanship strength.</x:v>
+      </x:c>
+      <x:c r="K51" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!140
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="45" t="str">
+        <x:v>sky-sign/mars/scorpio</x:v>
+      </x:c>
+      <x:c r="B52" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C52" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D52" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E52" s="45" t="str">
+        <x:v>someone withholding action until the source of control becomes clear</x:v>
+      </x:c>
+      <x:c r="F52" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G52" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H52" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I52" s="45" t="str">
+        <x:v>Waiting for control to become clear is neutral; pressure around trust and access remains shadow.</x:v>
+      </x:c>
+      <x:c r="J52" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: careful pursuit of an irreversible result carries the source's strategic use of information gained during delay.</x:v>
+      </x:c>
+      <x:c r="K52" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!194</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="45" t="str">
+        <x:v>sky-sign/mars/scorpio</x:v>
+      </x:c>
+      <x:c r="B53" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C53" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D53" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E53" s="45" t="str">
+        <x:v>someone applying pressure where trust and private access are already at stake</x:v>
+      </x:c>
+      <x:c r="F53" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G53" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H53" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I53" s="45" t="str">
+        <x:v>Waiting for control to become clear is neutral; pressure around trust and access remains shadow.</x:v>
+      </x:c>
+      <x:c r="J53" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: careful pursuit of an irreversible result carries the source's strategic use of information gained during delay.</x:v>
+      </x:c>
+      <x:c r="K53" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!194</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="45" t="str">
+        <x:v>sky-sign/mars/scorpio</x:v>
+      </x:c>
+      <x:c r="B54" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C54" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D54" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E54" s="45" t="str">
+        <x:v>a result pursued carefully because it cannot be undone</x:v>
+      </x:c>
+      <x:c r="F54" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G54" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H54" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I54" s="45" t="str">
+        <x:v>Waiting for control to become clear is neutral; pressure around trust and access remains shadow.</x:v>
+      </x:c>
+      <x:c r="J54" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: careful pursuit of an irreversible result carries the source's strategic use of information gained during delay.</x:v>
+      </x:c>
+      <x:c r="K54" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!194</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="45" t="str">
+        <x:v>sky-sign/saturn/leo</x:v>
+      </x:c>
+      <x:c r="B55" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C55" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D55" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E55" s="45" t="str">
+        <x:v>an authority withholding recognition until the visible contribution meets the standard</x:v>
+      </x:c>
+      <x:c r="F55" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G55" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H55" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I55" s="45" t="str">
+        <x:v>Limiting how much pride directs a decision is neutral; withheld recognition and withheld contribution remain costs.</x:v>
+      </x:c>
+      <x:c r="J55" s="45" t="str">
+        <x:v>The source carries earned confidence and recognition for completed work, but no current realization expresses it; nothing was invented during this check.</x:v>
+      </x:c>
+      <x:c r="K55" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/leo
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!671</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="45" t="str">
+        <x:v>sky-sign/saturn/leo</x:v>
+      </x:c>
+      <x:c r="B56" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C56" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D56" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E56" s="45" t="str">
+        <x:v>an authority limiting how much personal pride can direct the decision</x:v>
+      </x:c>
+      <x:c r="F56" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G56" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H56" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I56" s="45" t="str">
+        <x:v>Limiting how much pride directs a decision is neutral; withheld recognition and withheld contribution remain costs.</x:v>
+      </x:c>
+      <x:c r="J56" s="45" t="str">
+        <x:v>The source carries earned confidence and recognition for completed work, but no current realization expresses it; nothing was invented during this check.</x:v>
+      </x:c>
+      <x:c r="K56" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/leo
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!671</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="45" t="str">
+        <x:v>sky-sign/saturn/leo</x:v>
+      </x:c>
+      <x:c r="B57" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C57" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D57" s="45" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="E57" s="45" t="str">
+        <x:v>someone withholding their contribution because uncertain recognition feels too risky</x:v>
+      </x:c>
+      <x:c r="F57" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G57" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H57" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I57" s="45" t="str">
+        <x:v>Limiting how much pride directs a decision is neutral; withheld recognition and withheld contribution remain costs.</x:v>
+      </x:c>
+      <x:c r="J57" s="45" t="str">
+        <x:v>The source carries earned confidence and recognition for completed work, but no current realization expresses it; nothing was invented during this check.</x:v>
+      </x:c>
+      <x:c r="K57" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/leo
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!671</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="45" t="str">
+        <x:v>sky-sign/saturn/scorpio</x:v>
+      </x:c>
+      <x:c r="B58" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C58" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D58" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E58" s="45" t="str">
+        <x:v>a limit protecting access to information that cannot be taken back</x:v>
+      </x:c>
+      <x:c r="F58" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G58" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H58" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I58" s="45" t="str">
+        <x:v>Responsibility attached to access remains neutral; making a postponed consequence official remains shadow.</x:v>
+      </x:c>
+      <x:c r="J58" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: a limit that protects irreversible information carries the source's constructive boundary function.</x:v>
+      </x:c>
+      <x:c r="K58" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!684</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="45" t="str">
+        <x:v>sky-sign/saturn/scorpio</x:v>
+      </x:c>
+      <x:c r="B59" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C59" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D59" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E59" s="45" t="str">
+        <x:v>someone carrying more responsibility because they also control the access</x:v>
+      </x:c>
+      <x:c r="F59" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G59" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H59" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I59" s="45" t="str">
+        <x:v>Responsibility attached to access remains neutral; making a postponed consequence official remains shadow.</x:v>
+      </x:c>
+      <x:c r="J59" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: a limit that protects irreversible information carries the source's constructive boundary function.</x:v>
+      </x:c>
+      <x:c r="K59" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!684</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="45" t="str">
+        <x:v>sky-sign/saturn/scorpio</x:v>
+      </x:c>
+      <x:c r="B60" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C60" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D60" s="45" t="str">
+        <x:v>1/1/1</x:v>
+      </x:c>
+      <x:c r="E60" s="45" t="str">
+        <x:v>an authority making the consequence official after people tried to postpone it</x:v>
+      </x:c>
+      <x:c r="F60" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G60" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H60" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I60" s="45" t="str">
+        <x:v>Responsibility attached to access remains neutral; making a postponed consequence official remains shadow.</x:v>
+      </x:c>
+      <x:c r="J60" s="45" t="str">
+        <x:v>A supportive realization existed but was misclassified: a limit that protects irreversible information carries the source's constructive boundary function.</x:v>
+      </x:c>
+      <x:c r="K60" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!684</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="45" t="str">
+        <x:v>sky-sign/neptune/libra</x:v>
+      </x:c>
+      <x:c r="B61" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C61" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D61" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="E61" s="45" t="str">
+        <x:v>an image of fairness hiding which side keeps absorbing the cost</x:v>
+      </x:c>
+      <x:c r="F61" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G61" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H61" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I61" s="45" t="str">
+        <x:v>All three current realizations explicitly carry idealization, unequal cost, or lost reciprocity.</x:v>
+      </x:c>
+      <x:c r="J61" s="45" t="str">
+        <x:v>The source carries an honest fairness check beyond the fantasy, but no current realization expresses it; the all-shadow classification is correct for the three realizations actually present.</x:v>
+      </x:c>
+      <x:c r="K61" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/libra
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!543</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="45" t="str">
+        <x:v>sky-sign/neptune/libra</x:v>
+      </x:c>
+      <x:c r="B62" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C62" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D62" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="E62" s="45" t="str">
+        <x:v>people keeping an agreement by avoiding the unequal term underneath it</x:v>
+      </x:c>
+      <x:c r="F62" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G62" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H62" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I62" s="45" t="str">
+        <x:v>All three current realizations explicitly carry idealization, unequal cost, or lost reciprocity.</x:v>
+      </x:c>
+      <x:c r="J62" s="45" t="str">
+        <x:v>The source carries an honest fairness check beyond the fantasy, but no current realization expresses it; the all-shadow classification is correct for the three realizations actually present.</x:v>
+      </x:c>
+      <x:c r="K62" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/libra
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!543</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="45" t="str">
+        <x:v>sky-sign/neptune/libra</x:v>
+      </x:c>
+      <x:c r="B63" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C63" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D63" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="E63" s="45" t="str">
+        <x:v>people overlooking where reciprocity stopped because they still share the ideal</x:v>
+      </x:c>
+      <x:c r="F63" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G63" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H63" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I63" s="45" t="str">
+        <x:v>All three current realizations explicitly carry idealization, unequal cost, or lost reciprocity.</x:v>
+      </x:c>
+      <x:c r="J63" s="45" t="str">
+        <x:v>The source carries an honest fairness check beyond the fantasy, but no current realization expresses it; the all-shadow classification is correct for the three realizations actually present.</x:v>
+      </x:c>
+      <x:c r="K63" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/libra
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!543</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="45" t="str">
+        <x:v>sky-sign/lilith/leo</x:v>
+      </x:c>
+      <x:c r="B64" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C64" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D64" s="45" t="str">
+        <x:v>2/0/1</x:v>
+      </x:c>
+      <x:c r="E64" s="45" t="str">
+        <x:v>someone claiming visibility without making the contribution more acceptable first</x:v>
+      </x:c>
+      <x:c r="F64" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G64" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H64" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I64" s="45" t="str">
+        <x:v>Turning the whole conflict into a substitute for naming shame remains shadow.</x:v>
+      </x:c>
+      <x:c r="J64" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: claiming visibility and rejecting recognition that requires self-erasure follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K64" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/leo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="45" t="str">
+        <x:v>sky-sign/lilith/leo</x:v>
+      </x:c>
+      <x:c r="B65" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C65" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D65" s="45" t="str">
+        <x:v>2/0/1</x:v>
+      </x:c>
+      <x:c r="E65" s="45" t="str">
+        <x:v>someone rejecting recognition that depends on shrinking the difficult part</x:v>
+      </x:c>
+      <x:c r="F65" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G65" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H65" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I65" s="45" t="str">
+        <x:v>Turning the whole conflict into a substitute for naming shame remains shadow.</x:v>
+      </x:c>
+      <x:c r="J65" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: claiming visibility and rejecting recognition that requires self-erasure follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K65" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/leo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="45" t="str">
+        <x:v>sky-sign/lilith/leo</x:v>
+      </x:c>
+      <x:c r="B66" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C66" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D66" s="45" t="str">
+        <x:v>2/0/1</x:v>
+      </x:c>
+      <x:c r="E66" s="45" t="str">
+        <x:v>someone making the whole conflict about them because shame is harder to name directly</x:v>
+      </x:c>
+      <x:c r="F66" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G66" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="H66" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="I66" s="45" t="str">
+        <x:v>Turning the whole conflict into a substitute for naming shame remains shadow.</x:v>
+      </x:c>
+      <x:c r="J66" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: claiming visibility and rejecting recognition that requires self-erasure follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K66" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/leo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="45" t="str">
+        <x:v>sky-sign/lilith/virgo</x:v>
+      </x:c>
+      <x:c r="B67" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C67" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D67" s="45" t="str">
+        <x:v>2/1/0</x:v>
+      </x:c>
+      <x:c r="E67" s="45" t="str">
+        <x:v>a standard refused because usefulness has become a condition of worth</x:v>
+      </x:c>
+      <x:c r="F67" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G67" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H67" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I67" s="45" t="str">
+        <x:v>The excluded need exposing a method's limit is a neutral diagnostic condition.</x:v>
+      </x:c>
+      <x:c r="J67" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: refusing conditional worth and defending difference follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K67" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/virgo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="45" t="str">
+        <x:v>sky-sign/lilith/virgo</x:v>
+      </x:c>
+      <x:c r="B68" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C68" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D68" s="45" t="str">
+        <x:v>2/1/0</x:v>
+      </x:c>
+      <x:c r="E68" s="45" t="str">
+        <x:v>someone defending their difference against correction meant to make it manageable</x:v>
+      </x:c>
+      <x:c r="F68" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G68" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H68" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I68" s="45" t="str">
+        <x:v>The excluded need exposing a method's limit is a neutral diagnostic condition.</x:v>
+      </x:c>
+      <x:c r="J68" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: refusing conditional worth and defending difference follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K68" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/virgo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="45" t="str">
+        <x:v>sky-sign/lilith/virgo</x:v>
+      </x:c>
+      <x:c r="B69" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C69" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D69" s="45" t="str">
+        <x:v>2/1/0</x:v>
+      </x:c>
+      <x:c r="E69" s="45" t="str">
+        <x:v>the excluded need exposing what the approved method cannot serve</x:v>
+      </x:c>
+      <x:c r="F69" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G69" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H69" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I69" s="45" t="str">
+        <x:v>The excluded need exposing a method's limit is a neutral diagnostic condition.</x:v>
+      </x:c>
+      <x:c r="J69" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: refusing conditional worth and defending difference follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K69" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/virgo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="45" t="str">
+        <x:v>sky-sign/lilith/capricorn</x:v>
+      </x:c>
+      <x:c r="B70" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C70" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D70" s="45" t="str">
+        <x:v>2/1/0</x:v>
+      </x:c>
+      <x:c r="E70" s="45" t="str">
+        <x:v>someone confronting an authority that has used respectability as control</x:v>
+      </x:c>
+      <x:c r="F70" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G70" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H70" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I70" s="45" t="str">
+        <x:v>Accepting a consequence rather than obeying remains neutral because the source does not promise benefit.</x:v>
+      </x:c>
+      <x:c r="J70" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: confronting respectability used as control and refusing an erasing duty follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K70" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/capricorn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="45" t="str">
+        <x:v>sky-sign/lilith/capricorn</x:v>
+      </x:c>
+      <x:c r="B71" s="45" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C71" s="45" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D71" s="45" t="str">
+        <x:v>2/1/0</x:v>
+      </x:c>
+      <x:c r="E71" s="45" t="str">
+        <x:v>a duty refused because compliance would erase the person carrying it</x:v>
+      </x:c>
+      <x:c r="F71" s="45" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G71" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="H71" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I71" s="45" t="str">
+        <x:v>Accepting a consequence rather than obeying remains neutral because the source does not promise benefit.</x:v>
+      </x:c>
+      <x:c r="J71" s="45" t="str">
+        <x:v>Two supportive realizations were misclassified: confronting respectability used as control and refusing an erasing duty follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K71" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/capricorn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="46" t="str">
+        <x:v>sky-sign/lilith/capricorn</x:v>
+      </x:c>
+      <x:c r="B72" s="46" t="str">
+        <x:v>all_shadow</x:v>
+      </x:c>
+      <x:c r="C72" s="46" t="str">
+        <x:v>0/0/3</x:v>
+      </x:c>
+      <x:c r="D72" s="46" t="str">
+        <x:v>2/1/0</x:v>
+      </x:c>
+      <x:c r="E72" s="46" t="str">
+        <x:v>someone accepting the consequence rather than obeying the demand</x:v>
+      </x:c>
+      <x:c r="F72" s="46" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="G72" s="46" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H72" s="46" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="I72" s="46" t="str">
+        <x:v>Accepting a consequence rather than obeying remains neutral because the source does not promise benefit.</x:v>
+      </x:c>
+      <x:c r="J72" s="46" t="str">
+        <x:v>Two supportive realizations were misclassified: confronting respectability used as control and refusing an erasing duty follow the owner-approved source directly.</x:v>
+      </x:c>
+      <x:c r="K72" s="46" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/capricorn</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="A4:K72">
+    <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="PENDING OWNER"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c89b2aeea0047d0"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -8893,7 +11600,7 @@
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:K8">
-    <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="PENDING OWNER"/>
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="PENDING OWNER"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="J4:J8">
@@ -8902,464 +11609,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bec9eafa3bd4670"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="J1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="D2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="E2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="F2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="G2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="H2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="I2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="J2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="K2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="34" t="str">
-        <x:v>Key</x:v>
-      </x:c>
-      <x:c r="B3" s="35" t="str">
-        <x:v>Reader effect</x:v>
-      </x:c>
-      <x:c r="C3" s="35" t="str">
-        <x:v>Conflict behavior</x:v>
-      </x:c>
-      <x:c r="D3" s="35" t="str">
-        <x:v>Movement bias</x:v>
-      </x:c>
-      <x:c r="E3" s="35" t="str">
-        <x:v>Supportive realizations</x:v>
-      </x:c>
-      <x:c r="F3" s="35" t="str">
-        <x:v>Neutral realizations</x:v>
-      </x:c>
-      <x:c r="G3" s="35" t="str">
-        <x:v>Shadow realizations</x:v>
-      </x:c>
-      <x:c r="H3" s="35" t="str">
-        <x:v>Source IDs</x:v>
-      </x:c>
-      <x:c r="I3" s="35" t="str">
-        <x:v>Source hashes</x:v>
-      </x:c>
-      <x:c r="J3" s="35" t="str">
-        <x:v>Owner review status</x:v>
-      </x:c>
-      <x:c r="K3" s="36" t="str">
-        <x:v>Owner notes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="44" t="str">
-        <x:v>sky-how/modality/cardinal/cardinal</x:v>
-      </x:c>
-      <x:c r="B4" s="44" t="str">
-        <x:v>two attempts to set direction become visible at once</x:v>
-      </x:c>
-      <x:c r="C4" s="44" t="str">
-        <x:v>both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
-      </x:c>
-      <x:c r="D4" s="44" t="str">
-        <x:v>both sides need a shared first step or a clear decision about who leads</x:v>
-      </x:c>
-      <x:c r="E4" s="44" t="str">
-        <x:v>• both sides need a shared first step or a clear decision about who leads</x:v>
-      </x:c>
-      <x:c r="F4" s="44" t="str">
-        <x:v>• two attempts to set direction become visible at once</x:v>
-      </x:c>
-      <x:c r="G4" s="44" t="str">
-        <x:v>• both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
-      </x:c>
-      <x:c r="H4" s="44" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I4" s="44" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J4" s="44" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K4" s="44" t="str"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="45" t="str">
-        <x:v>sky-how/modality/cardinal/fixed</x:v>
-      </x:c>
-      <x:c r="B5" s="45" t="str">
-        <x:v>an immediate push runs into a limit meant to hold</x:v>
-      </x:c>
-      <x:c r="C5" s="45" t="str">
-        <x:v>one position keeps initiating while the other protects what cannot be surrendered</x:v>
-      </x:c>
-      <x:c r="D5" s="45" t="str">
-        <x:v>people need an action that preserves the fixed position's central limit</x:v>
-      </x:c>
-      <x:c r="E5" s="45" t="str">
-        <x:v>• people need an action that preserves the fixed position's central limit</x:v>
-      </x:c>
-      <x:c r="F5" s="45" t="str">
-        <x:v>• an immediate push runs into a limit meant to hold</x:v>
-      </x:c>
-      <x:c r="G5" s="45" t="str">
-        <x:v>• one position keeps initiating while the other protects what cannot be surrendered</x:v>
-      </x:c>
-      <x:c r="H5" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I5" s="45" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J5" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K5" s="45" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="45" t="str">
-        <x:v>sky-how/modality/cardinal/mutable</x:v>
-      </x:c>
-      <x:c r="B6" s="45" t="str">
-        <x:v>a first move keeps meeting revised terms</x:v>
-      </x:c>
-      <x:c r="C6" s="45" t="str">
-        <x:v>one position wants a decision while the other adapts as new conditions appear</x:v>
-      </x:c>
-      <x:c r="D6" s="45" t="str">
-        <x:v>the first step has to leave room for a defined adjustment</x:v>
-      </x:c>
-      <x:c r="E6" s="45" t="str">
-        <x:v>• the first step has to leave room for a defined adjustment</x:v>
-      </x:c>
-      <x:c r="F6" s="45" t="str">
-        <x:v>• a first move keeps meeting revised terms</x:v>
-      </x:c>
-      <x:c r="G6" s="45" t="str">
-        <x:v>• one position wants a decision while the other adapts as new conditions appear</x:v>
-      </x:c>
-      <x:c r="H6" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I6" s="45" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J6" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K6" s="45" t="str"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="45" t="str">
-        <x:v>sky-how/modality/fixed/cardinal</x:v>
-      </x:c>
-      <x:c r="B7" s="45" t="str">
-        <x:v>a protected position is pressed for immediate action</x:v>
-      </x:c>
-      <x:c r="C7" s="45" t="str">
-        <x:v>one side holds its ground while the other treats movement as urgent</x:v>
-      </x:c>
-      <x:c r="D7" s="45" t="str">
-        <x:v>the proposed action must work inside the limit that is not moving</x:v>
-      </x:c>
-      <x:c r="E7" s="45" t="str">
-        <x:v>• the proposed action must work inside the limit that is not moving</x:v>
-      </x:c>
-      <x:c r="F7" s="45" t="str">
-        <x:v>• a protected position is pressed for immediate action</x:v>
-      </x:c>
-      <x:c r="G7" s="45" t="str">
-        <x:v>• one side holds its ground while the other treats movement as urgent</x:v>
-      </x:c>
-      <x:c r="H7" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I7" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J7" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K7" s="45" t="str"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="45" t="str">
-        <x:v>sky-how/modality/fixed/fixed</x:v>
-      </x:c>
-      <x:c r="B8" s="45" t="str">
-        <x:v>the disagreement settles around two positions neither side considers expendable</x:v>
-      </x:c>
-      <x:c r="C8" s="45" t="str">
-        <x:v>neither side gives ground easily under pressure</x:v>
-      </x:c>
-      <x:c r="D8" s="45" t="str">
-        <x:v>people are more likely to change the terms or structure than to make either side back down</x:v>
-      </x:c>
-      <x:c r="E8" s="45" t="str">
-        <x:v>• people are more likely to change the terms or structure than to make either side back down</x:v>
-      </x:c>
-      <x:c r="F8" s="45" t="str">
-        <x:v>• the disagreement settles around two positions neither side considers expendable</x:v>
-      </x:c>
-      <x:c r="G8" s="45" t="str">
-        <x:v>• neither side gives ground easily under pressure</x:v>
-      </x:c>
-      <x:c r="H8" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I8" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J8" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K8" s="45" t="str"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="45" t="str">
-        <x:v>sky-how/modality/fixed/mutable</x:v>
-      </x:c>
-      <x:c r="B9" s="45" t="str">
-        <x:v>a firm limit keeps meeting a changing response</x:v>
-      </x:c>
-      <x:c r="C9" s="45" t="str">
-        <x:v>one position holds the line while the other revises around it</x:v>
-      </x:c>
-      <x:c r="D9" s="45" t="str">
-        <x:v>people have to name the nonnegotiable point instead of revising around it</x:v>
-      </x:c>
-      <x:c r="E9" s="45" t="str">
-        <x:v>• people have to name the nonnegotiable point instead of revising around it</x:v>
-      </x:c>
-      <x:c r="F9" s="45" t="str">
-        <x:v>• a firm limit keeps meeting a changing response</x:v>
-      </x:c>
-      <x:c r="G9" s="45" t="str">
-        <x:v>• one position holds the line while the other revises around it</x:v>
-      </x:c>
-      <x:c r="H9" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I9" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J9" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K9" s="45" t="str"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="45" t="str">
-        <x:v>sky-how/modality/mutable/cardinal</x:v>
-      </x:c>
-      <x:c r="B10" s="45" t="str">
-        <x:v>changing conditions are pushed toward a decision</x:v>
-      </x:c>
-      <x:c r="C10" s="45" t="str">
-        <x:v>one position keeps revising while the other insists that action cannot wait</x:v>
-      </x:c>
-      <x:c r="D10" s="45" t="str">
-        <x:v>a decision can move if it includes a defined point for review</x:v>
-      </x:c>
-      <x:c r="E10" s="45" t="str">
-        <x:v>• a decision can move if it includes a defined point for review</x:v>
-      </x:c>
-      <x:c r="F10" s="45" t="str">
-        <x:v>• changing conditions are pushed toward a decision</x:v>
-      </x:c>
-      <x:c r="G10" s="45" t="str">
-        <x:v>• one position keeps revising while the other insists that action cannot wait</x:v>
-      </x:c>
-      <x:c r="H10" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I10" s="45" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J10" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K10" s="45" t="str"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="45" t="str">
-        <x:v>sky-how/modality/mutable/fixed</x:v>
-      </x:c>
-      <x:c r="B11" s="45" t="str">
-        <x:v>continued adjustment reaches a demand that will not move</x:v>
-      </x:c>
-      <x:c r="C11" s="45" t="str">
-        <x:v>one position adapts repeatedly while the other protects a fixed requirement</x:v>
-      </x:c>
-      <x:c r="D11" s="45" t="str">
-        <x:v>people can move once the flexible side stops revising around an unnamed demand</x:v>
-      </x:c>
-      <x:c r="E11" s="45" t="str">
-        <x:v>• people can move once the flexible side stops revising around an unnamed demand</x:v>
-      </x:c>
-      <x:c r="F11" s="45" t="str">
-        <x:v>• continued adjustment reaches a demand that will not move</x:v>
-      </x:c>
-      <x:c r="G11" s="45" t="str">
-        <x:v>• one position adapts repeatedly while the other protects a fixed requirement</x:v>
-      </x:c>
-      <x:c r="H11" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I11" s="45" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J11" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K11" s="45" t="str"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="46" t="str">
-        <x:v>sky-how/modality/mutable/mutable</x:v>
-      </x:c>
-      <x:c r="B12" s="46" t="str">
-        <x:v>the terms remain open because both positions keep changing with the conditions</x:v>
-      </x:c>
-      <x:c r="C12" s="46" t="str">
-        <x:v>each answer creates another possible version before the last one can be tested</x:v>
-      </x:c>
-      <x:c r="D12" s="46" t="str">
-        <x:v>one workable version has to remain in place long enough to show what it does</x:v>
-      </x:c>
-      <x:c r="E12" s="46" t="str">
-        <x:v>• one workable version has to remain in place long enough to show what it does</x:v>
-      </x:c>
-      <x:c r="F12" s="46" t="str">
-        <x:v>• the terms remain open because both positions keep changing with the conditions</x:v>
-      </x:c>
-      <x:c r="G12" s="46" t="str">
-        <x:v>• each answer creates another possible version before the last one can be tested</x:v>
-      </x:c>
-      <x:c r="H12" s="46" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I12" s="46" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J12" s="46" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K12" s="46" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="A4:K12">
-    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="PENDING OWNER"/>
-  </x:conditionalFormatting>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="J4:J12">
-      <x:formula1>"PENDING OWNER,APPROVED,REVISE,REJECTED"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf198ba0838e64664"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bb15ea325aa46db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9383,6 +11633,463 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="I1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="J1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="K1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="I2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="J2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="K2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B3" s="35" t="str">
+        <x:v>Reader effect</x:v>
+      </x:c>
+      <x:c r="C3" s="35" t="str">
+        <x:v>Conflict behavior</x:v>
+      </x:c>
+      <x:c r="D3" s="35" t="str">
+        <x:v>Movement bias</x:v>
+      </x:c>
+      <x:c r="E3" s="35" t="str">
+        <x:v>Supportive realizations</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>Neutral realizations</x:v>
+      </x:c>
+      <x:c r="G3" s="35" t="str">
+        <x:v>Shadow realizations</x:v>
+      </x:c>
+      <x:c r="H3" s="35" t="str">
+        <x:v>Source IDs</x:v>
+      </x:c>
+      <x:c r="I3" s="35" t="str">
+        <x:v>Source hashes</x:v>
+      </x:c>
+      <x:c r="J3" s="35" t="str">
+        <x:v>Owner review status</x:v>
+      </x:c>
+      <x:c r="K3" s="36" t="str">
+        <x:v>Owner notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="44" t="str">
+        <x:v>sky-how/modality/cardinal/cardinal</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
+        <x:v>two attempts to set direction become visible at once</x:v>
+      </x:c>
+      <x:c r="C4" s="44" t="str">
+        <x:v>both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
+      </x:c>
+      <x:c r="D4" s="44" t="str">
+        <x:v>both sides need a shared first step or a clear decision about who leads</x:v>
+      </x:c>
+      <x:c r="E4" s="44" t="str">
+        <x:v>• both sides need a shared first step or a clear decision about who leads</x:v>
+      </x:c>
+      <x:c r="F4" s="44" t="str">
+        <x:v>• two attempts to set direction become visible at once</x:v>
+      </x:c>
+      <x:c r="G4" s="44" t="str">
+        <x:v>• both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
+      </x:c>
+      <x:c r="H4" s="44" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I4" s="44" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J4" s="44" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K4" s="44" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>sky-how/modality/cardinal/fixed</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>an immediate push runs into a limit meant to hold</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>one position keeps initiating while the other protects what cannot be surrendered</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>people need an action that preserves the fixed position's central limit</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>• people need an action that preserves the fixed position's central limit</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>• an immediate push runs into a limit meant to hold</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>• one position keeps initiating while the other protects what cannot be surrendered</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K5" s="45" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="45" t="str">
+        <x:v>sky-how/modality/cardinal/mutable</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>a first move keeps meeting revised terms</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>one position wants a decision while the other adapts as new conditions appear</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="str">
+        <x:v>the first step has to leave room for a defined adjustment</x:v>
+      </x:c>
+      <x:c r="E6" s="45" t="str">
+        <x:v>• the first step has to leave room for a defined adjustment</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="str">
+        <x:v>• a first move keeps meeting revised terms</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="str">
+        <x:v>• one position wants a decision while the other adapts as new conditions appear</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J6" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K6" s="45" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="45" t="str">
+        <x:v>sky-how/modality/fixed/cardinal</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>a protected position is pressed for immediate action</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>one side holds its ground while the other treats movement as urgent</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="str">
+        <x:v>the proposed action must work inside the limit that is not moving</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="str">
+        <x:v>• the proposed action must work inside the limit that is not moving</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str">
+        <x:v>• a protected position is pressed for immediate action</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>• one side holds its ground while the other treats movement as urgent</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K7" s="45" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="45" t="str">
+        <x:v>sky-how/modality/fixed/fixed</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>the disagreement settles around two positions neither side considers expendable</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="str">
+        <x:v>neither side gives ground easily under pressure</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="str">
+        <x:v>people are more likely to change the terms or structure than to make either side back down</x:v>
+      </x:c>
+      <x:c r="E8" s="45" t="str">
+        <x:v>• people are more likely to change the terms or structure than to make either side back down</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="str">
+        <x:v>• the disagreement settles around two positions neither side considers expendable</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="str">
+        <x:v>• neither side gives ground easily under pressure</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J8" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K8" s="45" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="45" t="str">
+        <x:v>sky-how/modality/fixed/mutable</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>a firm limit keeps meeting a changing response</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>one position holds the line while the other revises around it</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="str">
+        <x:v>people have to name the nonnegotiable point instead of revising around it</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="str">
+        <x:v>• people have to name the nonnegotiable point instead of revising around it</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="str">
+        <x:v>• a firm limit keeps meeting a changing response</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="str">
+        <x:v>• one position holds the line while the other revises around it</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J9" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K9" s="45" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="45" t="str">
+        <x:v>sky-how/modality/mutable/cardinal</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="str">
+        <x:v>changing conditions are pushed toward a decision</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="str">
+        <x:v>one position keeps revising while the other insists that action cannot wait</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="str">
+        <x:v>a decision can move if it includes a defined point for review</x:v>
+      </x:c>
+      <x:c r="E10" s="45" t="str">
+        <x:v>• a decision can move if it includes a defined point for review</x:v>
+      </x:c>
+      <x:c r="F10" s="45" t="str">
+        <x:v>• changing conditions are pushed toward a decision</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="str">
+        <x:v>• one position keeps revising while the other insists that action cannot wait</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J10" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K10" s="45" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="45" t="str">
+        <x:v>sky-how/modality/mutable/fixed</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>continued adjustment reaches a demand that will not move</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>one position adapts repeatedly while the other protects a fixed requirement</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="str">
+        <x:v>people can move once the flexible side stops revising around an unnamed demand</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="str">
+        <x:v>• people can move once the flexible side stops revising around an unnamed demand</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="str">
+        <x:v>• continued adjustment reaches a demand that will not move</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="str">
+        <x:v>• one position adapts repeatedly while the other protects a fixed requirement</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I11" s="45" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J11" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K11" s="45" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="46" t="str">
+        <x:v>sky-how/modality/mutable/mutable</x:v>
+      </x:c>
+      <x:c r="B12" s="46" t="str">
+        <x:v>the terms remain open because both positions keep changing with the conditions</x:v>
+      </x:c>
+      <x:c r="C12" s="46" t="str">
+        <x:v>each answer creates another possible version before the last one can be tested</x:v>
+      </x:c>
+      <x:c r="D12" s="46" t="str">
+        <x:v>one workable version has to remain in place long enough to show what it does</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="str">
+        <x:v>• one workable version has to remain in place long enough to show what it does</x:v>
+      </x:c>
+      <x:c r="F12" s="46" t="str">
+        <x:v>• the terms remain open because both positions keep changing with the conditions</x:v>
+      </x:c>
+      <x:c r="G12" s="46" t="str">
+        <x:v>• each answer creates another possible version before the last one can be tested</x:v>
+      </x:c>
+      <x:c r="H12" s="46" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I12" s="46" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J12" s="46" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K12" s="46" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="A4:K12">
+    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="PENDING OWNER"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="J4:J12">
+      <x:formula1>"PENDING OWNER,APPROVED,REVISE,REJECTED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b8e15b03b2b4b57"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
         <x:v>Element units (16)</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
@@ -10020,7 +12727,7 @@
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:K19">
-    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="PENDING OWNER"/>
+    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="PENDING OWNER"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="J4:J19">
@@ -10029,12 +12736,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23e14c3ae71e47e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61c4d23d2e42401e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10375,7 +13082,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10657,7 +13364,7 @@
         <x:v>Typed-array count shapes</x:v>
       </x:c>
       <x:c r="B21" s="15" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C21" s="15" t="str">
         <x:v>&gt;= 2</x:v>

</xml_diff>

<commit_message>
fix(content): verify sky realization classifications
</commit_message>
<xml_diff>
--- a/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
+++ b/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0f951c7c90314cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R3b9783b4e5fc4d25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="R71f9d37f91254455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Audit" sheetId="4" r:id="Rd87397e3688e4d0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="5" r:id="R58eb7e31d26c46bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="6" r:id="R1701aebd25c54e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="7" r:id="Re5d090a3758f48d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="8" r:id="Ra6d3ed9980924991"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="9" r:id="R8424677bd0224adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re59bc0001e1b4ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R7699e6c81c824914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="R1b8a6c53e2454533"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Audit" sheetId="4" r:id="Rd25e47f202c5411b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeted Verification" sheetId="5" r:id="R6c4dcb0abb9d4a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="6" r:id="Rdc456446029c4507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="7" r:id="Rbc676e3729324001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="8" r:id="R9fc7a54080334053"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="9" r:id="R7dd328c624554cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="10" r:id="R97efc298562e40bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +227,29 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="5">
+  <x:dxfs count="7">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF6B4F00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF7E8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF6B4F00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF7E8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -330,7 +353,34 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AspectMechanismsTable" displayName="AspectMechanismsTable" ref="A3:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TargetedVerificationTable" displayName="TargetedVerificationTable" ref="A3:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="Key"/>
+    <x:tableColumn id="2" name="Realization"/>
+    <x:tableColumn id="3" name="Prior type"/>
+    <x:tableColumn id="4" name="Verified type"/>
+    <x:tableColumn id="5" name="Result"/>
+    <x:tableColumn id="6" name="Evidence finding"/>
+    <x:tableColumn id="7" name="Evidence pointers"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SupportiveParaphraseFlagsTable" displayName="SupportiveParaphraseFlagsTable" ref="A10:D37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="Supportive paraphrase flag"/>
+    <x:tableColumn id="2" name="Combined position"/>
+    <x:tableColumn id="3" name="Supportive realization"/>
+    <x:tableColumn id="4" name="Evidence pointers"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AspectMechanismsTable" displayName="AspectMechanismsTable" ref="A3:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Reader effect"/>
@@ -348,8 +398,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ModalityUnitsTable" displayName="ModalityUnitsTable" ref="A3:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ModalityUnitsTable" displayName="ModalityUnitsTable" ref="A3:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Reader effect"/>
@@ -367,8 +417,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ElementUnitsTable" displayName="ElementUnitsTable" ref="A3:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ElementUnitsTable" displayName="ElementUnitsTable" ref="A3:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Reader effect"/>
@@ -1029,6 +1079,736 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="3" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="64" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Wording-layer QA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="9" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="str">
+        <x:v>Cap</x:v>
+      </x:c>
+      <x:c r="D4" s="9" t="str">
+        <x:v>Manifestation occurrence count</x:v>
+      </x:c>
+      <x:c r="E4" s="9" t="str">
+        <x:v>Distinct bullets</x:v>
+      </x:c>
+      <x:c r="G4" s="9" t="str">
+        <x:v>Skeleton occurrence count</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="str">
+        <x:v>Distinct skeletons</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="14" t="str">
+        <x:v>Evidence-layer SHA-256</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>0ceb85f5897fb42238dfdd69e7b02271f87befe202f009da8659add9b9337c23</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>locked</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="10" t="n">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="G5" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H5" s="10" t="n">
+        <x:v>496</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="15" t="str">
+        <x:v>Mechanical join rows</x:v>
+      </x:c>
+      <x:c r="B6" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="15" t="str">
+        <x:v>Details copied from combined position</x:v>
+      </x:c>
+      <x:c r="B7" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="15" t="str">
+        <x:v>Maximum opening construction use</x:v>
+      </x:c>
+      <x:c r="B8" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C8" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="15" t="str">
+        <x:v>Maximum exact manifestation use</x:v>
+      </x:c>
+      <x:c r="B9" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="15" t="str">
+        <x:v>Maximum manifestation skeleton use</x:v>
+      </x:c>
+      <x:c r="B10" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="15" t="str">
+        <x:v>Maximum details-language use</x:v>
+      </x:c>
+      <x:c r="B11" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="15" t="str">
+        <x:v>Maximum connective n-gram use</x:v>
+      </x:c>
+      <x:c r="B12" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C12" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="15" t="str">
+        <x:v>Abstract-subject violations</x:v>
+      </x:c>
+      <x:c r="B13" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="15" t="str">
+        <x:v>Manifestation plainness violations</x:v>
+      </x:c>
+      <x:c r="B14" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="15" t="str">
+        <x:v>Owner-source verbatim matches (8+ words)</x:v>
+      </x:c>
+      <x:c r="B15" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C15" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="15" t="str">
+        <x:v>Units rechecked</x:v>
+      </x:c>
+      <x:c r="B16" s="15" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="C16" s="15" t="n">
+        <x:v>174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="15" t="str">
+        <x:v>Units changed</x:v>
+      </x:c>
+      <x:c r="B17" s="15" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="C17" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="15" t="str">
+        <x:v>One-sided before source-shadow pass</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C18" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="15" t="str">
+        <x:v>One-sided after source-shadow pass</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="15" t="str">
+        <x:v>Legacy ordered manifestation fields</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C20" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="15" t="str">
+        <x:v>Typed-array count shapes</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C21" s="15" t="str">
+        <x:v>&gt;= 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="15" t="str">
+        <x:v>Analytical-abstraction units changed</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C22" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="15" t="str">
+        <x:v>Assembled-construction units changed</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="15" t="str">
+        <x:v>Invented-motive units changed</x:v>
+      </x:c>
+      <x:c r="B24" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C24" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="15" t="str">
+        <x:v>Unsupported-vocabulary units changed</x:v>
+      </x:c>
+      <x:c r="B25" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C25" s="15" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="16" t="str">
+        <x:v>Generic-actor units simplified</x:v>
+      </x:c>
+      <x:c r="B26" s="16" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C26" s="16" t="str">
+        <x:v>report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="9" t="str">
+        <x:v>Opening construction</x:v>
+      </x:c>
+      <x:c r="B29" s="9" t="str">
+        <x:v>Uses</x:v>
+      </x:c>
+      <x:c r="D29" s="9" t="str">
+        <x:v>Repeated connective n-gram</x:v>
+      </x:c>
+      <x:c r="E29" s="9" t="str">
+        <x:v>Uses</x:v>
+      </x:c>
+      <x:c r="G29" s="9" t="str">
+        <x:v>Manifestation skeleton</x:v>
+      </x:c>
+      <x:c r="H29" s="9" t="str">
+        <x:v>Uses</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="19" t="str">
+        <x:v>people can</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D30" s="19" t="str">
+        <x:v>as the</x:v>
+      </x:c>
+      <x:c r="E30" s="19" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G30" s="19" t="str">
+        <x:v>{planet} becoming real when it is shown where others can see it</x:v>
+      </x:c>
+      <x:c r="H30" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="20" t="str">
+        <x:v>a group</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="str">
+        <x:v>before anyone</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G31" s="20" t="str">
+        <x:v>{planet} becoming unclear when many people shaped the same vision</x:v>
+      </x:c>
+      <x:c r="H31" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="20" t="str">
+        <x:v>a larger</x:v>
+      </x:c>
+      <x:c r="B32" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D32" s="20" t="str">
+        <x:v>until the</x:v>
+      </x:c>
+      <x:c r="E32" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G32" s="20" t="str">
+        <x:v>{planet} divided according to terms both sides must answer to</x:v>
+      </x:c>
+      <x:c r="H32" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="20" t="str">
+        <x:v>a new</x:v>
+      </x:c>
+      <x:c r="B33" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D33" s="20" t="str">
+        <x:v>when the</x:v>
+      </x:c>
+      <x:c r="E33" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G33" s="20" t="str">
+        <x:v>{planet} going to the work that protected what needed to last</x:v>
+      </x:c>
+      <x:c r="H33" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="20" t="str">
+        <x:v>people protect</x:v>
+      </x:c>
+      <x:c r="B34" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D34" s="20" t="str">
+        <x:v>while the</x:v>
+      </x:c>
+      <x:c r="E34" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G34" s="20" t="str">
+        <x:v>{planet} narrowed until every part can be checked</x:v>
+      </x:c>
+      <x:c r="H34" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="20" t="str">
+        <x:v>a sudden</x:v>
+      </x:c>
+      <x:c r="B35" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D35" s="20" t="str">
+        <x:v>with the</x:v>
+      </x:c>
+      <x:c r="E35" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G35" s="20" t="str">
+        <x:v>{planet} reduced to a transaction so uncertain terms stay under control</x:v>
+      </x:c>
+      <x:c r="H35" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="20" t="str">
+        <x:v>each side</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D36" s="20" t="str">
+        <x:v>around a</x:v>
+      </x:c>
+      <x:c r="E36" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G36" s="20" t="str">
+        <x:v>{planet} revised to distribute responsibility more fairly</x:v>
+      </x:c>
+      <x:c r="H36" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="20" t="str">
+        <x:v>people give</x:v>
+      </x:c>
+      <x:c r="B37" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D37" s="20" t="str">
+        <x:v>around the</x:v>
+      </x:c>
+      <x:c r="E37" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G37" s="20" t="str">
+        <x:v>{planet} spreading because the exception reveals a wider problem</x:v>
+      </x:c>
+      <x:c r="H37" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="20" t="str">
+        <x:v>people have</x:v>
+      </x:c>
+      <x:c r="B38" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D38" s="20" t="str">
+        <x:v>before anyone can</x:v>
+      </x:c>
+      <x:c r="E38" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G38" s="20" t="str">
+        <x:v>a {planet} announced before every objection has been heard</x:v>
+      </x:c>
+      <x:c r="H38" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="20" t="str">
+        <x:v>people make</x:v>
+      </x:c>
+      <x:c r="B39" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D39" s="20" t="str">
+        <x:v>boundary around</x:v>
+      </x:c>
+      <x:c r="E39" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G39" s="20" t="str">
+        <x:v>a {planet} becoming real when an authority records it</x:v>
+      </x:c>
+      <x:c r="H39" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="20" t="str">
+        <x:v>people refuse</x:v>
+      </x:c>
+      <x:c r="B40" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D40" s="20" t="str">
+        <x:v>by fixing</x:v>
+      </x:c>
+      <x:c r="E40" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G40" s="20" t="str">
+        <x:v>a {planet} blurred by sympathy for several incompatible {planet}</x:v>
+      </x:c>
+      <x:c r="H40" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="20" t="str">
+        <x:v>people stay</x:v>
+      </x:c>
+      <x:c r="B41" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D41" s="20" t="str">
+        <x:v>when it</x:v>
+      </x:c>
+      <x:c r="E41" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G41" s="20" t="str">
+        <x:v>a {planet} changing when one more fact enters the conversation</x:v>
+      </x:c>
+      <x:c r="H41" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="20" t="str">
+        <x:v>someone acts</x:v>
+      </x:c>
+      <x:c r="B42" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D42" s="21" t="str">
+        <x:v>with it</x:v>
+      </x:c>
+      <x:c r="E42" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G42" s="20" t="str">
+        <x:v>a {planet} forming around the body or resource others expect to use</x:v>
+      </x:c>
+      <x:c r="H42" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="20" t="str">
+        <x:v>the group</x:v>
+      </x:c>
+      <x:c r="B43" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G43" s="20" t="str">
+        <x:v>a {planet} given time to become clear before the plan changes again</x:v>
+      </x:c>
+      <x:c r="H43" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="20" t="str">
+        <x:v>the wording</x:v>
+      </x:c>
+      <x:c r="B44" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G44" s="20" t="str">
+        <x:v>a {planet} meant to apply equally</x:v>
+      </x:c>
+      <x:c r="H44" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="20" t="str">
+        <x:v>whoever defines</x:v>
+      </x:c>
+      <x:c r="B45" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G45" s="20" t="str">
+        <x:v>a {planet} moving only after both replies enter the record</x:v>
+      </x:c>
+      <x:c r="H45" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="20" t="str">
+        <x:v>whoever moves</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G46" s="20" t="str">
+        <x:v>a {planet} protecting access to information that cannot be taken back</x:v>
+      </x:c>
+      <x:c r="H46" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="20" t="str">
+        <x:v>a beautiful</x:v>
+      </x:c>
+      <x:c r="B47" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G47" s="20" t="str">
+        <x:v>a {planet} pursued carefully because it cannot be undone</x:v>
+      </x:c>
+      <x:c r="H47" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="20" t="str">
+        <x:v>a bigger</x:v>
+      </x:c>
+      <x:c r="B48" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G48" s="20" t="str">
+        <x:v>a {planet} stated before anyone grants the right to object</x:v>
+      </x:c>
+      <x:c r="H48" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="21" t="str">
+        <x:v>a choice</x:v>
+      </x:c>
+      <x:c r="B49" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G49" s="21" t="str">
+        <x:v>a {planet} stated clearly enough to force a quick answer</x:v>
+      </x:c>
+      <x:c r="H49" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1944,12 +2724,11 @@
       <x:c r="D12" s="45" t="str">
         <x:v>whoever names the larger purpose can become the face of it</x:v>
       </x:c>
-      <x:c r="E12" s="45" t="str">
-        <x:v>• a strong belief making one contribution stand for a larger cause</x:v>
-      </x:c>
+      <x:c r="E12" s="45" t="str"/>
       <x:c r="F12" s="45" t="str"/>
       <x:c r="G12" s="45" t="str">
-        <x:v>• the person who names the wider purpose becoming identified with it</x:v>
+        <x:v>• the person who names the wider purpose becoming identified with it
+• a strong belief making one contribution stand for a larger cause</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
         <x:v>• people carrying someone's work to an audience it was not made for</x:v>
@@ -5892,13 +6671,12 @@
       <x:c r="D86" s="45" t="str">
         <x:v>the same rule is expected to apply across the group, even when one case resists it</x:v>
       </x:c>
-      <x:c r="E86" s="45" t="str">
-        <x:v>• a standard meant to apply equally</x:v>
-      </x:c>
+      <x:c r="E86" s="45" t="str"/>
       <x:c r="F86" s="45" t="str"/>
       <x:c r="G86" s="45" t="str">
         <x:v>• policy applied across the group
-• precedent</x:v>
+• precedent
+• a standard meant to apply equally</x:v>
       </x:c>
       <x:c r="H86" s="45" t="str"/>
       <x:c r="I86" s="45" t="str">
@@ -7082,14 +7860,13 @@
       <x:c r="D108" s="45" t="str">
         <x:v>the promise grows beyond the facts that were meant to support it</x:v>
       </x:c>
-      <x:c r="E108" s="45" t="str">
-        <x:v>• a belief growing beyond what its supporting facts can carry</x:v>
-      </x:c>
+      <x:c r="E108" s="45" t="str"/>
       <x:c r="F108" s="45" t="str"/>
       <x:c r="G108" s="45" t="str"/>
       <x:c r="H108" s="45" t="str">
         <x:v>• people looking farther ahead while overlooking the practical distance
-• a collective ideal becoming difficult to separate from certainty</x:v>
+• a collective ideal becoming difficult to separate from certainty
+• a belief growing beyond what its supporting facts can carry</x:v>
       </x:c>
       <x:c r="I108" s="45" t="str">
         <x:v>belief outrunning supporting facts</x:v>
@@ -9150,7 +9927,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78792d434679476f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red5841d4f9d34c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11777,12 +12554,610 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b89693590e4523"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1065d684feab4963"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="72" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="72" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="72" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Targeted classification verification</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Targeted classification verification</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Targeted classification verification</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Targeted classification verification</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Targeted classification verification</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Targeted classification verification</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Targeted classification verification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>44 moved realizations checked: 42 hold, 2 corrected. Wording and evidence are unchanged.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>44 moved realizations checked: 42 hold, 2 corrected. Wording and evidence are unchanged.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>44 moved realizations checked: 42 hold, 2 corrected. Wording and evidence are unchanged.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>44 moved realizations checked: 42 hold, 2 corrected. Wording and evidence are unchanged.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>44 moved realizations checked: 42 hold, 2 corrected. Wording and evidence are unchanged.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>44 moved realizations checked: 42 hold, 2 corrected. Wording and evidence are unchanged.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>44 moved realizations checked: 42 hold, 2 corrected. Wording and evidence are unchanged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B3" s="35" t="str">
+        <x:v>Realization</x:v>
+      </x:c>
+      <x:c r="C3" s="35" t="str">
+        <x:v>Prior type</x:v>
+      </x:c>
+      <x:c r="D3" s="35" t="str">
+        <x:v>Verified type</x:v>
+      </x:c>
+      <x:c r="E3" s="35" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>Evidence finding</x:v>
+      </x:c>
+      <x:c r="G3" s="36" t="str">
+        <x:v>Evidence pointers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="44" t="str">
+        <x:v>sky-sign/sun/sagittarius</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
+        <x:v>a strong belief making one contribution stand for a larger cause</x:v>
+      </x:c>
+      <x:c r="C4" s="44" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="D4" s="44" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="E4" s="44" t="str">
+        <x:v>CORRECTED</x:v>
+      </x:c>
+      <x:c r="F4" s="44" t="str">
+        <x:v>The realization describes amplification, but neither governed source says that it helps or eases the situation. The matrix source instead warns that certainty can outrun the facts.</x:v>
+      </x:c>
+      <x:c r="G4" s="44" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/sagittarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!845</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>sky-sign/saturn/aquarius</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>a standard meant to apply equally</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>CORRECTED</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>The realization states the standard's intended scope. It does not show the placement helping or easing anything, and the governed source explicitly allows the rule to prove arbitrary.</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/aquarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!719</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="46" t="str">
+        <x:v>sky-sign/neptune/sagittarius</x:v>
+      </x:c>
+      <x:c r="B6" s="46" t="str">
+        <x:v>a belief growing beyond what its supporting facts can carry</x:v>
+      </x:c>
+      <x:c r="C6" s="46" t="str">
+        <x:v>supportive</x:v>
+      </x:c>
+      <x:c r="D6" s="46" t="str">
+        <x:v>shadow</x:v>
+      </x:c>
+      <x:c r="E6" s="46" t="str">
+        <x:v>CORRECTED (OWNER-REPORTED)</x:v>
+      </x:c>
+      <x:c r="F6" s="46" t="str">
+        <x:v>Growing beyond supporting facts is overreach. The governed sources describe a blank map, a leap without a parachute, and a promise that claims it can explain everything.</x:v>
+      </x:c>
+      <x:c r="G6" s="46" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/sagittarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!547</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="34" t="str">
+        <x:v>Supportive paraphrase flag</x:v>
+      </x:c>
+      <x:c r="B10" s="35" t="str">
+        <x:v>Combined position</x:v>
+      </x:c>
+      <x:c r="C10" s="35" t="str">
+        <x:v>Supportive realization</x:v>
+      </x:c>
+      <x:c r="D10" s="36" t="str">
+        <x:v>Evidence pointers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="44" t="str">
+        <x:v>sky-sign/sun/taurus</x:v>
+      </x:c>
+      <x:c r="B11" s="44" t="str">
+        <x:v>people give credit to the work that proves useful and lasts</x:v>
+      </x:c>
+      <x:c r="C11" s="44" t="str">
+        <x:v>a contribution valued because it keeps producing something useful</x:v>
+      </x:c>
+      <x:c r="D11" s="44" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!782</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="45" t="str">
+        <x:v>sky-sign/sun/taurus</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="str">
+        <x:v>people give credit to the work that proves useful and lasts</x:v>
+      </x:c>
+      <x:c r="C12" s="45" t="str">
+        <x:v>people waiting to give credit until the result proves it can last</x:v>
+      </x:c>
+      <x:c r="D12" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!782</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="45" t="str">
+        <x:v>sky-sign/sun/taurus</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>people give credit to the work that proves useful and lasts</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>credit going to the work that protected what needed to last</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!782</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="45" t="str">
+        <x:v>sky-sign/sun/gemini</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>the clearest explanation can decide who gets credit for the idea</x:v>
+      </x:c>
+      <x:c r="C14" s="45" t="str">
+        <x:v>the clearest explanation deciding who is seen as responsible</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!792</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="45" t="str">
+        <x:v>sky-sign/sun/leo</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="str">
+        <x:v>whoever did the work wants their name kept with it</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="str">
+        <x:v>wanting credit attached to the person who did the work</x:v>
+      </x:c>
+      <x:c r="D15" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/leo
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!813</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="45" t="str">
+        <x:v>sky-sign/sun/capricorn</x:v>
+      </x:c>
+      <x:c r="B16" s="45" t="str">
+        <x:v>a title goes to the person expected to carry the result</x:v>
+      </x:c>
+      <x:c r="C16" s="45" t="str">
+        <x:v>people giving credit to the person expected to answer for the result</x:v>
+      </x:c>
+      <x:c r="D16" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/capricorn
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!852</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="45" t="str">
+        <x:v>sky-sign/moon/aquarius</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="str">
+        <x:v>the group makes room for feeling by stepping back and looking at the pattern</x:v>
+      </x:c>
+      <x:c r="C17" s="45" t="str">
+        <x:v>someone stepping back from a reaction long enough to see the pattern clearly</x:v>
+      </x:c>
+      <x:c r="D17" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/moon/aquarius
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!118</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="45" t="str">
+        <x:v>sky-sign/mercury/aries</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="str">
+        <x:v>the first clear answer can move a decision before everyone has finished thinking</x:v>
+      </x:c>
+      <x:c r="C18" s="45" t="str">
+        <x:v>someone giving the clear answer that gets a stalled decision moving again</x:v>
+      </x:c>
+      <x:c r="D18" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mercury/aries
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!251
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!84</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="45" t="str">
+        <x:v>sky-sign/mercury/taurus</x:v>
+      </x:c>
+      <x:c r="B19" s="45" t="str">
+        <x:v>The wording gets slower and more specific until everyone knows what the terms actually mean.</x:v>
+      </x:c>
+      <x:c r="C19" s="45" t="str">
+        <x:v>an agreement slowing until the practical terms are clear</x:v>
+      </x:c>
+      <x:c r="D19" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mercury/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!275</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="45" t="str">
+        <x:v>sky-sign/mercury/pisces</x:v>
+      </x:c>
+      <x:c r="B20" s="45" t="str">
+        <x:v>people understand the tone or image sooner than they agree on the facts</x:v>
+      </x:c>
+      <x:c r="C20" s="45" t="str">
+        <x:v>people reading the tone when the stated facts remain incomplete</x:v>
+      </x:c>
+      <x:c r="D20" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mercury/pisces
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!466
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="45" t="str">
+        <x:v>sky-sign/venus/taurus</x:v>
+      </x:c>
+      <x:c r="B21" s="45" t="str">
+        <x:v>a choice feels worthwhile when it is pleasant, affordable, and built to last</x:v>
+      </x:c>
+      <x:c r="C21" s="45" t="str">
+        <x:v>someone choosing the arrangement that feels good and can still hold up over time</x:v>
+      </x:c>
+      <x:c r="D21" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/venus/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!978
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!61</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="45" t="str">
+        <x:v>sky-sign/venus/sagittarius</x:v>
+      </x:c>
+      <x:c r="B22" s="45" t="str">
+        <x:v>people choose the agreement that leaves more room to grow and explore</x:v>
+      </x:c>
+      <x:c r="C22" s="45" t="str">
+        <x:v>someone choosing a connection that leaves both people room to keep growing</x:v>
+      </x:c>
+      <x:c r="D22" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/venus/sagittarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!1061
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="45" t="str">
+        <x:v>sky-sign/venus/aquarius</x:v>
+      </x:c>
+      <x:c r="B23" s="45" t="str">
+        <x:v>people stay connected by giving each other room inside the group</x:v>
+      </x:c>
+      <x:c r="C23" s="45" t="str">
+        <x:v>people staying connected because the agreement leaves room for independence</x:v>
+      </x:c>
+      <x:c r="D23" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/venus/aquarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!1083</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="45" t="str">
+        <x:v>sky-sign/mars/cancer</x:v>
+      </x:c>
+      <x:c r="B24" s="45" t="str">
+        <x:v>someone protects the home or the people involved before explaining the anger</x:v>
+      </x:c>
+      <x:c r="C24" s="45" t="str">
+        <x:v>someone acting to protect another person before explaining why</x:v>
+      </x:c>
+      <x:c r="D24" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/cancer
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!159
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="45" t="str">
+        <x:v>sky-sign/mars/taurus</x:v>
+      </x:c>
+      <x:c r="B25" s="45" t="str">
+        <x:v>people keep pushing the same point until a material limit finally moves</x:v>
+      </x:c>
+      <x:c r="C25" s="45" t="str">
+        <x:v>someone working the same point until a material limit gives way</x:v>
+      </x:c>
+      <x:c r="D25" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!140
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="45" t="str">
+        <x:v>sky-sign/mars/scorpio</x:v>
+      </x:c>
+      <x:c r="B26" s="45" t="str">
+        <x:v>someone acts carefully because trust, control, and lasting consequences are involved</x:v>
+      </x:c>
+      <x:c r="C26" s="45" t="str">
+        <x:v>a result pursued carefully because it cannot be undone</x:v>
+      </x:c>
+      <x:c r="D26" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mars/scorpio
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!194</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="45" t="str">
+        <x:v>sky-sign/jupiter/libra</x:v>
+      </x:c>
+      <x:c r="B27" s="45" t="str">
+        <x:v>people find more room to move when the terms spread the benefit fairly</x:v>
+      </x:c>
+      <x:c r="C27" s="45" t="str">
+        <x:v>more people benefiting after the terms distribute the opportunity more fairly</x:v>
+      </x:c>
+      <x:c r="D27" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/jupiter/libra
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!80
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="45" t="str">
+        <x:v>sky-sign/saturn/gemini</x:v>
+      </x:c>
+      <x:c r="B28" s="45" t="str">
+        <x:v>The wording gets tighter once the decision has consequences and the record has to stay consistent.</x:v>
+      </x:c>
+      <x:c r="C28" s="45" t="str">
+        <x:v>revised language that still has to match the record</x:v>
+      </x:c>
+      <x:c r="D28" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!667
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!194</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="45" t="str">
+        <x:v>sky-sign/saturn/sagittarius</x:v>
+      </x:c>
+      <x:c r="B29" s="45" t="str">
+        <x:v>a large promise meets the test of what can be proved and delivered</x:v>
+      </x:c>
+      <x:c r="C29" s="45" t="str">
+        <x:v>a large promise reduced to what can be proved and delivered</x:v>
+      </x:c>
+      <x:c r="D29" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/saturn/sagittarius
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!690
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="45" t="str">
+        <x:v>sky-sign/uranus/gemini</x:v>
+      </x:c>
+      <x:c r="B30" s="45" t="str">
+        <x:v>new information rewrites the route before the standard method can catch up</x:v>
+      </x:c>
+      <x:c r="C30" s="45" t="str">
+        <x:v>new information altering the available routes almost immediately</x:v>
+      </x:c>
+      <x:c r="D30" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!930
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!218</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="45" t="str">
+        <x:v>sky-sign/neptune/leo</x:v>
+      </x:c>
+      <x:c r="B31" s="45" t="str">
+        <x:v>an image becomes larger than the private work or person behind it</x:v>
+      </x:c>
+      <x:c r="C31" s="45" t="str">
+        <x:v>a public image carrying more hope than the contribution can support</x:v>
+      </x:c>
+      <x:c r="D31" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/leo
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!539
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!244</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="45" t="str">
+        <x:v>sky-sign/chiron/virgo</x:v>
+      </x:c>
+      <x:c r="B32" s="45" t="str">
+        <x:v>a small mistake can reopen the fear that usefulness is the price of belonging</x:v>
+      </x:c>
+      <x:c r="C32" s="45" t="str">
+        <x:v>a small correction reopening the fear of never being useful enough</x:v>
+      </x:c>
+      <x:c r="D32" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/chiron/virgo
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="45" t="str">
+        <x:v>sky-sign/lilith/leo</x:v>
+      </x:c>
+      <x:c r="B33" s="45" t="str">
+        <x:v>someone claims visibility without making the difficult part more acceptable first</x:v>
+      </x:c>
+      <x:c r="C33" s="45" t="str">
+        <x:v>someone claiming visibility without making the contribution more acceptable first</x:v>
+      </x:c>
+      <x:c r="D33" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/leo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="45" t="str">
+        <x:v>sky-sign/lilith/virgo</x:v>
+      </x:c>
+      <x:c r="B34" s="45" t="str">
+        <x:v>people reject a standard that treats usefulness or purity as the price of worth</x:v>
+      </x:c>
+      <x:c r="C34" s="45" t="str">
+        <x:v>a standard refused because usefulness has become a condition of worth</x:v>
+      </x:c>
+      <x:c r="D34" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/virgo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="45" t="str">
+        <x:v>sky-sign/lilith/libra</x:v>
+      </x:c>
+      <x:c r="B35" s="45" t="str">
+        <x:v>someone challenges an agreement that calls repeated self-erasure fair</x:v>
+      </x:c>
+      <x:c r="C35" s="45" t="str">
+        <x:v>an agreement challenged after fairness becomes repeated self-erasure</x:v>
+      </x:c>
+      <x:c r="D35" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/libra</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="45" t="str">
+        <x:v>sky-sign/lilith/scorpio</x:v>
+      </x:c>
+      <x:c r="B36" s="45" t="str">
+        <x:v>people protect desire and private access from someone trying to take control</x:v>
+      </x:c>
+      <x:c r="C36" s="45" t="str">
+        <x:v>someone protecting desire from another person's claim to private access</x:v>
+      </x:c>
+      <x:c r="D36" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/scorpio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="46" t="str">
+        <x:v>sky-sign/lilith/capricorn</x:v>
+      </x:c>
+      <x:c r="B37" s="46" t="str">
+        <x:v>people confront an authority that uses duty or respectability to demand compliance</x:v>
+      </x:c>
+      <x:c r="C37" s="46" t="str">
+        <x:v>someone confronting an authority that has used respectability as control</x:v>
+      </x:c>
+      <x:c r="D37" s="46" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/capricorn</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="A4:G6">
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="PENDING OWNER"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="A11:D37">
+    <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING OWNER"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71fbcf869da84810"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4dc3a4fc83748ca"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -12075,7 +13450,7 @@
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:K8">
-    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="PENDING OWNER"/>
+    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="PENDING OWNER"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="J4:J8">
@@ -12084,464 +13459,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R116813ff029f4ccc"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="J1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="D2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="E2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="F2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="G2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="H2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="I2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="J2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="K2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="34" t="str">
-        <x:v>Key</x:v>
-      </x:c>
-      <x:c r="B3" s="35" t="str">
-        <x:v>Reader effect</x:v>
-      </x:c>
-      <x:c r="C3" s="35" t="str">
-        <x:v>Conflict behavior</x:v>
-      </x:c>
-      <x:c r="D3" s="35" t="str">
-        <x:v>Movement bias</x:v>
-      </x:c>
-      <x:c r="E3" s="35" t="str">
-        <x:v>Supportive realizations</x:v>
-      </x:c>
-      <x:c r="F3" s="35" t="str">
-        <x:v>Neutral realizations</x:v>
-      </x:c>
-      <x:c r="G3" s="35" t="str">
-        <x:v>Shadow realizations</x:v>
-      </x:c>
-      <x:c r="H3" s="35" t="str">
-        <x:v>Source IDs</x:v>
-      </x:c>
-      <x:c r="I3" s="35" t="str">
-        <x:v>Source hashes</x:v>
-      </x:c>
-      <x:c r="J3" s="35" t="str">
-        <x:v>Owner review status</x:v>
-      </x:c>
-      <x:c r="K3" s="36" t="str">
-        <x:v>Owner notes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="44" t="str">
-        <x:v>sky-how/modality/cardinal/cardinal</x:v>
-      </x:c>
-      <x:c r="B4" s="44" t="str">
-        <x:v>two attempts to set direction become visible at once</x:v>
-      </x:c>
-      <x:c r="C4" s="44" t="str">
-        <x:v>both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
-      </x:c>
-      <x:c r="D4" s="44" t="str">
-        <x:v>both sides need a shared first step or a clear decision about who leads</x:v>
-      </x:c>
-      <x:c r="E4" s="44" t="str">
-        <x:v>• both sides need a shared first step or a clear decision about who leads</x:v>
-      </x:c>
-      <x:c r="F4" s="44" t="str">
-        <x:v>• two attempts to set direction become visible at once</x:v>
-      </x:c>
-      <x:c r="G4" s="44" t="str">
-        <x:v>• both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
-      </x:c>
-      <x:c r="H4" s="44" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I4" s="44" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J4" s="44" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K4" s="44" t="str"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="45" t="str">
-        <x:v>sky-how/modality/cardinal/fixed</x:v>
-      </x:c>
-      <x:c r="B5" s="45" t="str">
-        <x:v>an immediate push runs into a limit meant to hold</x:v>
-      </x:c>
-      <x:c r="C5" s="45" t="str">
-        <x:v>one position keeps initiating while the other protects what cannot be surrendered</x:v>
-      </x:c>
-      <x:c r="D5" s="45" t="str">
-        <x:v>people need an action that preserves the fixed position's central limit</x:v>
-      </x:c>
-      <x:c r="E5" s="45" t="str">
-        <x:v>• people need an action that preserves the fixed position's central limit</x:v>
-      </x:c>
-      <x:c r="F5" s="45" t="str">
-        <x:v>• an immediate push runs into a limit meant to hold</x:v>
-      </x:c>
-      <x:c r="G5" s="45" t="str">
-        <x:v>• one position keeps initiating while the other protects what cannot be surrendered</x:v>
-      </x:c>
-      <x:c r="H5" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I5" s="45" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J5" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K5" s="45" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="45" t="str">
-        <x:v>sky-how/modality/cardinal/mutable</x:v>
-      </x:c>
-      <x:c r="B6" s="45" t="str">
-        <x:v>a first move keeps meeting revised terms</x:v>
-      </x:c>
-      <x:c r="C6" s="45" t="str">
-        <x:v>one position wants a decision while the other adapts as new conditions appear</x:v>
-      </x:c>
-      <x:c r="D6" s="45" t="str">
-        <x:v>the first step has to leave room for a defined adjustment</x:v>
-      </x:c>
-      <x:c r="E6" s="45" t="str">
-        <x:v>• the first step has to leave room for a defined adjustment</x:v>
-      </x:c>
-      <x:c r="F6" s="45" t="str">
-        <x:v>• a first move keeps meeting revised terms</x:v>
-      </x:c>
-      <x:c r="G6" s="45" t="str">
-        <x:v>• one position wants a decision while the other adapts as new conditions appear</x:v>
-      </x:c>
-      <x:c r="H6" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I6" s="45" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J6" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K6" s="45" t="str"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="45" t="str">
-        <x:v>sky-how/modality/fixed/cardinal</x:v>
-      </x:c>
-      <x:c r="B7" s="45" t="str">
-        <x:v>a protected position is pressed for immediate action</x:v>
-      </x:c>
-      <x:c r="C7" s="45" t="str">
-        <x:v>one side holds its ground while the other treats movement as urgent</x:v>
-      </x:c>
-      <x:c r="D7" s="45" t="str">
-        <x:v>the proposed action must work inside the limit that is not moving</x:v>
-      </x:c>
-      <x:c r="E7" s="45" t="str">
-        <x:v>• the proposed action must work inside the limit that is not moving</x:v>
-      </x:c>
-      <x:c r="F7" s="45" t="str">
-        <x:v>• a protected position is pressed for immediate action</x:v>
-      </x:c>
-      <x:c r="G7" s="45" t="str">
-        <x:v>• one side holds its ground while the other treats movement as urgent</x:v>
-      </x:c>
-      <x:c r="H7" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I7" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J7" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K7" s="45" t="str"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="45" t="str">
-        <x:v>sky-how/modality/fixed/fixed</x:v>
-      </x:c>
-      <x:c r="B8" s="45" t="str">
-        <x:v>the disagreement settles around two positions neither side considers expendable</x:v>
-      </x:c>
-      <x:c r="C8" s="45" t="str">
-        <x:v>neither side gives ground easily under pressure</x:v>
-      </x:c>
-      <x:c r="D8" s="45" t="str">
-        <x:v>people are more likely to change the terms or structure than to make either side back down</x:v>
-      </x:c>
-      <x:c r="E8" s="45" t="str">
-        <x:v>• people are more likely to change the terms or structure than to make either side back down</x:v>
-      </x:c>
-      <x:c r="F8" s="45" t="str">
-        <x:v>• the disagreement settles around two positions neither side considers expendable</x:v>
-      </x:c>
-      <x:c r="G8" s="45" t="str">
-        <x:v>• neither side gives ground easily under pressure</x:v>
-      </x:c>
-      <x:c r="H8" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I8" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J8" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K8" s="45" t="str"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="45" t="str">
-        <x:v>sky-how/modality/fixed/mutable</x:v>
-      </x:c>
-      <x:c r="B9" s="45" t="str">
-        <x:v>a firm limit keeps meeting a changing response</x:v>
-      </x:c>
-      <x:c r="C9" s="45" t="str">
-        <x:v>one position holds the line while the other revises around it</x:v>
-      </x:c>
-      <x:c r="D9" s="45" t="str">
-        <x:v>people have to name the nonnegotiable point instead of revising around it</x:v>
-      </x:c>
-      <x:c r="E9" s="45" t="str">
-        <x:v>• people have to name the nonnegotiable point instead of revising around it</x:v>
-      </x:c>
-      <x:c r="F9" s="45" t="str">
-        <x:v>• a firm limit keeps meeting a changing response</x:v>
-      </x:c>
-      <x:c r="G9" s="45" t="str">
-        <x:v>• one position holds the line while the other revises around it</x:v>
-      </x:c>
-      <x:c r="H9" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I9" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J9" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K9" s="45" t="str"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="45" t="str">
-        <x:v>sky-how/modality/mutable/cardinal</x:v>
-      </x:c>
-      <x:c r="B10" s="45" t="str">
-        <x:v>changing conditions are pushed toward a decision</x:v>
-      </x:c>
-      <x:c r="C10" s="45" t="str">
-        <x:v>one position keeps revising while the other insists that action cannot wait</x:v>
-      </x:c>
-      <x:c r="D10" s="45" t="str">
-        <x:v>a decision can move if it includes a defined point for review</x:v>
-      </x:c>
-      <x:c r="E10" s="45" t="str">
-        <x:v>• a decision can move if it includes a defined point for review</x:v>
-      </x:c>
-      <x:c r="F10" s="45" t="str">
-        <x:v>• changing conditions are pushed toward a decision</x:v>
-      </x:c>
-      <x:c r="G10" s="45" t="str">
-        <x:v>• one position keeps revising while the other insists that action cannot wait</x:v>
-      </x:c>
-      <x:c r="H10" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I10" s="45" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J10" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K10" s="45" t="str"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="45" t="str">
-        <x:v>sky-how/modality/mutable/fixed</x:v>
-      </x:c>
-      <x:c r="B11" s="45" t="str">
-        <x:v>continued adjustment reaches a demand that will not move</x:v>
-      </x:c>
-      <x:c r="C11" s="45" t="str">
-        <x:v>one position adapts repeatedly while the other protects a fixed requirement</x:v>
-      </x:c>
-      <x:c r="D11" s="45" t="str">
-        <x:v>people can move once the flexible side stops revising around an unnamed demand</x:v>
-      </x:c>
-      <x:c r="E11" s="45" t="str">
-        <x:v>• people can move once the flexible side stops revising around an unnamed demand</x:v>
-      </x:c>
-      <x:c r="F11" s="45" t="str">
-        <x:v>• continued adjustment reaches a demand that will not move</x:v>
-      </x:c>
-      <x:c r="G11" s="45" t="str">
-        <x:v>• one position adapts repeatedly while the other protects a fixed requirement</x:v>
-      </x:c>
-      <x:c r="H11" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I11" s="45" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J11" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K11" s="45" t="str"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="46" t="str">
-        <x:v>sky-how/modality/mutable/mutable</x:v>
-      </x:c>
-      <x:c r="B12" s="46" t="str">
-        <x:v>the terms remain open because both positions keep changing with the conditions</x:v>
-      </x:c>
-      <x:c r="C12" s="46" t="str">
-        <x:v>each answer creates another possible version before the last one can be tested</x:v>
-      </x:c>
-      <x:c r="D12" s="46" t="str">
-        <x:v>one workable version has to remain in place long enough to show what it does</x:v>
-      </x:c>
-      <x:c r="E12" s="46" t="str">
-        <x:v>• one workable version has to remain in place long enough to show what it does</x:v>
-      </x:c>
-      <x:c r="F12" s="46" t="str">
-        <x:v>• the terms remain open because both positions keep changing with the conditions</x:v>
-      </x:c>
-      <x:c r="G12" s="46" t="str">
-        <x:v>• each answer creates another possible version before the last one can be tested</x:v>
-      </x:c>
-      <x:c r="H12" s="46" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I12" s="46" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J12" s="46" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K12" s="46" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="A4:K12">
-    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="PENDING OWNER"/>
-  </x:conditionalFormatting>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="J4:J12">
-      <x:formula1>"PENDING OWNER,APPROVED,REVISE,REJECTED"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a55d96e22d74fbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f7fcb2804404992"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12565,6 +13483,463 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="I1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="J1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="K1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="I2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="J2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="K2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B3" s="35" t="str">
+        <x:v>Reader effect</x:v>
+      </x:c>
+      <x:c r="C3" s="35" t="str">
+        <x:v>Conflict behavior</x:v>
+      </x:c>
+      <x:c r="D3" s="35" t="str">
+        <x:v>Movement bias</x:v>
+      </x:c>
+      <x:c r="E3" s="35" t="str">
+        <x:v>Supportive realizations</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>Neutral realizations</x:v>
+      </x:c>
+      <x:c r="G3" s="35" t="str">
+        <x:v>Shadow realizations</x:v>
+      </x:c>
+      <x:c r="H3" s="35" t="str">
+        <x:v>Source IDs</x:v>
+      </x:c>
+      <x:c r="I3" s="35" t="str">
+        <x:v>Source hashes</x:v>
+      </x:c>
+      <x:c r="J3" s="35" t="str">
+        <x:v>Owner review status</x:v>
+      </x:c>
+      <x:c r="K3" s="36" t="str">
+        <x:v>Owner notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="44" t="str">
+        <x:v>sky-how/modality/cardinal/cardinal</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
+        <x:v>two attempts to set direction become visible at once</x:v>
+      </x:c>
+      <x:c r="C4" s="44" t="str">
+        <x:v>both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
+      </x:c>
+      <x:c r="D4" s="44" t="str">
+        <x:v>both sides need a shared first step or a clear decision about who leads</x:v>
+      </x:c>
+      <x:c r="E4" s="44" t="str">
+        <x:v>• both sides need a shared first step or a clear decision about who leads</x:v>
+      </x:c>
+      <x:c r="F4" s="44" t="str">
+        <x:v>• two attempts to set direction become visible at once</x:v>
+      </x:c>
+      <x:c r="G4" s="44" t="str">
+        <x:v>• both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
+      </x:c>
+      <x:c r="H4" s="44" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I4" s="44" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J4" s="44" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K4" s="44" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>sky-how/modality/cardinal/fixed</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>an immediate push runs into a limit meant to hold</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>one position keeps initiating while the other protects what cannot be surrendered</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>people need an action that preserves the fixed position's central limit</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>• people need an action that preserves the fixed position's central limit</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>• an immediate push runs into a limit meant to hold</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>• one position keeps initiating while the other protects what cannot be surrendered</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K5" s="45" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="45" t="str">
+        <x:v>sky-how/modality/cardinal/mutable</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>a first move keeps meeting revised terms</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>one position wants a decision while the other adapts as new conditions appear</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="str">
+        <x:v>the first step has to leave room for a defined adjustment</x:v>
+      </x:c>
+      <x:c r="E6" s="45" t="str">
+        <x:v>• the first step has to leave room for a defined adjustment</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="str">
+        <x:v>• a first move keeps meeting revised terms</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="str">
+        <x:v>• one position wants a decision while the other adapts as new conditions appear</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J6" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K6" s="45" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="45" t="str">
+        <x:v>sky-how/modality/fixed/cardinal</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>a protected position is pressed for immediate action</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>one side holds its ground while the other treats movement as urgent</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="str">
+        <x:v>the proposed action must work inside the limit that is not moving</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="str">
+        <x:v>• the proposed action must work inside the limit that is not moving</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str">
+        <x:v>• a protected position is pressed for immediate action</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>• one side holds its ground while the other treats movement as urgent</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K7" s="45" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="45" t="str">
+        <x:v>sky-how/modality/fixed/fixed</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>the disagreement settles around two positions neither side considers expendable</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="str">
+        <x:v>neither side gives ground easily under pressure</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="str">
+        <x:v>people are more likely to change the terms or structure than to make either side back down</x:v>
+      </x:c>
+      <x:c r="E8" s="45" t="str">
+        <x:v>• people are more likely to change the terms or structure than to make either side back down</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="str">
+        <x:v>• the disagreement settles around two positions neither side considers expendable</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="str">
+        <x:v>• neither side gives ground easily under pressure</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J8" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K8" s="45" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="45" t="str">
+        <x:v>sky-how/modality/fixed/mutable</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>a firm limit keeps meeting a changing response</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>one position holds the line while the other revises around it</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="str">
+        <x:v>people have to name the nonnegotiable point instead of revising around it</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="str">
+        <x:v>• people have to name the nonnegotiable point instead of revising around it</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="str">
+        <x:v>• a firm limit keeps meeting a changing response</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="str">
+        <x:v>• one position holds the line while the other revises around it</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J9" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K9" s="45" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="45" t="str">
+        <x:v>sky-how/modality/mutable/cardinal</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="str">
+        <x:v>changing conditions are pushed toward a decision</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="str">
+        <x:v>one position keeps revising while the other insists that action cannot wait</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="str">
+        <x:v>a decision can move if it includes a defined point for review</x:v>
+      </x:c>
+      <x:c r="E10" s="45" t="str">
+        <x:v>• a decision can move if it includes a defined point for review</x:v>
+      </x:c>
+      <x:c r="F10" s="45" t="str">
+        <x:v>• changing conditions are pushed toward a decision</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="str">
+        <x:v>• one position keeps revising while the other insists that action cannot wait</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J10" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K10" s="45" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="45" t="str">
+        <x:v>sky-how/modality/mutable/fixed</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>continued adjustment reaches a demand that will not move</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>one position adapts repeatedly while the other protects a fixed requirement</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="str">
+        <x:v>people can move once the flexible side stops revising around an unnamed demand</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="str">
+        <x:v>• people can move once the flexible side stops revising around an unnamed demand</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="str">
+        <x:v>• continued adjustment reaches a demand that will not move</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="str">
+        <x:v>• one position adapts repeatedly while the other protects a fixed requirement</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I11" s="45" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J11" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K11" s="45" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="46" t="str">
+        <x:v>sky-how/modality/mutable/mutable</x:v>
+      </x:c>
+      <x:c r="B12" s="46" t="str">
+        <x:v>the terms remain open because both positions keep changing with the conditions</x:v>
+      </x:c>
+      <x:c r="C12" s="46" t="str">
+        <x:v>each answer creates another possible version before the last one can be tested</x:v>
+      </x:c>
+      <x:c r="D12" s="46" t="str">
+        <x:v>one workable version has to remain in place long enough to show what it does</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="str">
+        <x:v>• one workable version has to remain in place long enough to show what it does</x:v>
+      </x:c>
+      <x:c r="F12" s="46" t="str">
+        <x:v>• the terms remain open because both positions keep changing with the conditions</x:v>
+      </x:c>
+      <x:c r="G12" s="46" t="str">
+        <x:v>• each answer creates another possible version before the last one can be tested</x:v>
+      </x:c>
+      <x:c r="H12" s="46" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I12" s="46" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J12" s="46" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K12" s="46" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="A4:K12">
+    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="PENDING OWNER"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="J4:J12">
+      <x:formula1>"PENDING OWNER,APPROVED,REVISE,REJECTED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3449e3b58884a0a"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
         <x:v>Element units (16)</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
@@ -13202,7 +14577,7 @@
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:K19">
-    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="PENDING OWNER"/>
+    <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="PENDING OWNER"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="J4:J19">
@@ -13211,12 +14586,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f714b0fcc7d45d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc450aae407cb4620"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -13555,734 +14930,4 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="3" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="64" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>Wording-layer QA</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-      <x:c r="D2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-      <x:c r="E2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-      <x:c r="F2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-      <x:c r="G2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-      <x:c r="H2" s="7" t="str">
-        <x:v>The evidence layer is hash-locked. These checks show whether fixed joins, repeated bullets, structural slot templates, or opener monoculture have returned.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="9" t="str">
-        <x:v>Measure</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>Result</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>Cap</x:v>
-      </x:c>
-      <x:c r="D4" s="9" t="str">
-        <x:v>Manifestation occurrence count</x:v>
-      </x:c>
-      <x:c r="E4" s="9" t="str">
-        <x:v>Distinct bullets</x:v>
-      </x:c>
-      <x:c r="G4" s="9" t="str">
-        <x:v>Skeleton occurrence count</x:v>
-      </x:c>
-      <x:c r="H4" s="9" t="str">
-        <x:v>Distinct skeletons</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Evidence-layer SHA-256</x:v>
-      </x:c>
-      <x:c r="B5" s="14" t="str">
-        <x:v>0ceb85f5897fb42238dfdd69e7b02271f87befe202f009da8659add9b9337c23</x:v>
-      </x:c>
-      <x:c r="C5" s="14" t="str">
-        <x:v>locked</x:v>
-      </x:c>
-      <x:c r="D5" s="10" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E5" s="10" t="n">
-        <x:v>496</x:v>
-      </x:c>
-      <x:c r="G5" s="10" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H5" s="10" t="n">
-        <x:v>496</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="15" t="str">
-        <x:v>Mechanical join rows</x:v>
-      </x:c>
-      <x:c r="B6" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C6" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="15" t="str">
-        <x:v>Details copied from combined position</x:v>
-      </x:c>
-      <x:c r="B7" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="15" t="str">
-        <x:v>Maximum opening construction use</x:v>
-      </x:c>
-      <x:c r="B8" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="15" t="str">
-        <x:v>Maximum exact manifestation use</x:v>
-      </x:c>
-      <x:c r="B9" s="15" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C9" s="15" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="15" t="str">
-        <x:v>Maximum manifestation skeleton use</x:v>
-      </x:c>
-      <x:c r="B10" s="15" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C10" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="15" t="str">
-        <x:v>Maximum details-language use</x:v>
-      </x:c>
-      <x:c r="B11" s="15" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C11" s="15" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="15" t="str">
-        <x:v>Maximum connective n-gram use</x:v>
-      </x:c>
-      <x:c r="B12" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C12" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="15" t="str">
-        <x:v>Abstract-subject violations</x:v>
-      </x:c>
-      <x:c r="B13" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C13" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="15" t="str">
-        <x:v>Manifestation plainness violations</x:v>
-      </x:c>
-      <x:c r="B14" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C14" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="15" t="str">
-        <x:v>Owner-source verbatim matches (8+ words)</x:v>
-      </x:c>
-      <x:c r="B15" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C15" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="15" t="str">
-        <x:v>Units rechecked</x:v>
-      </x:c>
-      <x:c r="B16" s="15" t="n">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="C16" s="15" t="n">
-        <x:v>174</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="15" t="str">
-        <x:v>Units changed</x:v>
-      </x:c>
-      <x:c r="B17" s="15" t="n">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="C17" s="15" t="str">
-        <x:v>report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="15" t="str">
-        <x:v>One-sided before source-shadow pass</x:v>
-      </x:c>
-      <x:c r="B18" s="15" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="C18" s="15" t="str">
-        <x:v>report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="15" t="str">
-        <x:v>One-sided after source-shadow pass</x:v>
-      </x:c>
-      <x:c r="B19" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C19" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="15" t="str">
-        <x:v>Legacy ordered manifestation fields</x:v>
-      </x:c>
-      <x:c r="B20" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C20" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="15" t="str">
-        <x:v>Typed-array count shapes</x:v>
-      </x:c>
-      <x:c r="B21" s="15" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C21" s="15" t="str">
-        <x:v>&gt;= 2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="15" t="str">
-        <x:v>Analytical-abstraction units changed</x:v>
-      </x:c>
-      <x:c r="B22" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C22" s="15" t="str">
-        <x:v>report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="15" t="str">
-        <x:v>Assembled-construction units changed</x:v>
-      </x:c>
-      <x:c r="B23" s="15" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C23" s="15" t="str">
-        <x:v>report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="15" t="str">
-        <x:v>Invented-motive units changed</x:v>
-      </x:c>
-      <x:c r="B24" s="15" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C24" s="15" t="str">
-        <x:v>report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="15" t="str">
-        <x:v>Unsupported-vocabulary units changed</x:v>
-      </x:c>
-      <x:c r="B25" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C25" s="15" t="str">
-        <x:v>report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="16" t="str">
-        <x:v>Generic-actor units simplified</x:v>
-      </x:c>
-      <x:c r="B26" s="16" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C26" s="16" t="str">
-        <x:v>report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="9" t="str">
-        <x:v>Opening construction</x:v>
-      </x:c>
-      <x:c r="B29" s="9" t="str">
-        <x:v>Uses</x:v>
-      </x:c>
-      <x:c r="D29" s="9" t="str">
-        <x:v>Repeated connective n-gram</x:v>
-      </x:c>
-      <x:c r="E29" s="9" t="str">
-        <x:v>Uses</x:v>
-      </x:c>
-      <x:c r="G29" s="9" t="str">
-        <x:v>Manifestation skeleton</x:v>
-      </x:c>
-      <x:c r="H29" s="9" t="str">
-        <x:v>Uses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="19" t="str">
-        <x:v>people can</x:v>
-      </x:c>
-      <x:c r="B30" s="19" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D30" s="19" t="str">
-        <x:v>as the</x:v>
-      </x:c>
-      <x:c r="E30" s="19" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G30" s="19" t="str">
-        <x:v>{planet} becoming real when it is shown where others can see it</x:v>
-      </x:c>
-      <x:c r="H30" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="20" t="str">
-        <x:v>a group</x:v>
-      </x:c>
-      <x:c r="B31" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D31" s="20" t="str">
-        <x:v>before anyone</x:v>
-      </x:c>
-      <x:c r="E31" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G31" s="20" t="str">
-        <x:v>{planet} becoming unclear when many people shaped the same vision</x:v>
-      </x:c>
-      <x:c r="H31" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="20" t="str">
-        <x:v>a larger</x:v>
-      </x:c>
-      <x:c r="B32" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D32" s="20" t="str">
-        <x:v>until the</x:v>
-      </x:c>
-      <x:c r="E32" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G32" s="20" t="str">
-        <x:v>{planet} divided according to terms both sides must answer to</x:v>
-      </x:c>
-      <x:c r="H32" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="20" t="str">
-        <x:v>a new</x:v>
-      </x:c>
-      <x:c r="B33" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D33" s="20" t="str">
-        <x:v>when the</x:v>
-      </x:c>
-      <x:c r="E33" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G33" s="20" t="str">
-        <x:v>{planet} going to the work that protected what needed to last</x:v>
-      </x:c>
-      <x:c r="H33" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="20" t="str">
-        <x:v>people protect</x:v>
-      </x:c>
-      <x:c r="B34" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D34" s="20" t="str">
-        <x:v>while the</x:v>
-      </x:c>
-      <x:c r="E34" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G34" s="20" t="str">
-        <x:v>{planet} narrowed until every part can be checked</x:v>
-      </x:c>
-      <x:c r="H34" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="20" t="str">
-        <x:v>a sudden</x:v>
-      </x:c>
-      <x:c r="B35" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D35" s="20" t="str">
-        <x:v>with the</x:v>
-      </x:c>
-      <x:c r="E35" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G35" s="20" t="str">
-        <x:v>{planet} reduced to a transaction so uncertain terms stay under control</x:v>
-      </x:c>
-      <x:c r="H35" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="20" t="str">
-        <x:v>each side</x:v>
-      </x:c>
-      <x:c r="B36" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D36" s="20" t="str">
-        <x:v>around a</x:v>
-      </x:c>
-      <x:c r="E36" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G36" s="20" t="str">
-        <x:v>{planet} revised to distribute responsibility more fairly</x:v>
-      </x:c>
-      <x:c r="H36" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="20" t="str">
-        <x:v>people give</x:v>
-      </x:c>
-      <x:c r="B37" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D37" s="20" t="str">
-        <x:v>around the</x:v>
-      </x:c>
-      <x:c r="E37" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G37" s="20" t="str">
-        <x:v>{planet} spreading because the exception reveals a wider problem</x:v>
-      </x:c>
-      <x:c r="H37" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="20" t="str">
-        <x:v>people have</x:v>
-      </x:c>
-      <x:c r="B38" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D38" s="20" t="str">
-        <x:v>before anyone can</x:v>
-      </x:c>
-      <x:c r="E38" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G38" s="20" t="str">
-        <x:v>a {planet} announced before every objection has been heard</x:v>
-      </x:c>
-      <x:c r="H38" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="20" t="str">
-        <x:v>people make</x:v>
-      </x:c>
-      <x:c r="B39" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D39" s="20" t="str">
-        <x:v>boundary around</x:v>
-      </x:c>
-      <x:c r="E39" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G39" s="20" t="str">
-        <x:v>a {planet} becoming real when an authority records it</x:v>
-      </x:c>
-      <x:c r="H39" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="20" t="str">
-        <x:v>people refuse</x:v>
-      </x:c>
-      <x:c r="B40" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D40" s="20" t="str">
-        <x:v>by fixing</x:v>
-      </x:c>
-      <x:c r="E40" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G40" s="20" t="str">
-        <x:v>a {planet} blurred by sympathy for several incompatible {planet}</x:v>
-      </x:c>
-      <x:c r="H40" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="20" t="str">
-        <x:v>people stay</x:v>
-      </x:c>
-      <x:c r="B41" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D41" s="20" t="str">
-        <x:v>when it</x:v>
-      </x:c>
-      <x:c r="E41" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G41" s="20" t="str">
-        <x:v>a {planet} changing when one more fact enters the conversation</x:v>
-      </x:c>
-      <x:c r="H41" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="20" t="str">
-        <x:v>someone acts</x:v>
-      </x:c>
-      <x:c r="B42" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D42" s="21" t="str">
-        <x:v>with it</x:v>
-      </x:c>
-      <x:c r="E42" s="21" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G42" s="20" t="str">
-        <x:v>a {planet} forming around the body or resource others expect to use</x:v>
-      </x:c>
-      <x:c r="H42" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="20" t="str">
-        <x:v>the group</x:v>
-      </x:c>
-      <x:c r="B43" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G43" s="20" t="str">
-        <x:v>a {planet} given time to become clear before the plan changes again</x:v>
-      </x:c>
-      <x:c r="H43" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="20" t="str">
-        <x:v>the wording</x:v>
-      </x:c>
-      <x:c r="B44" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G44" s="20" t="str">
-        <x:v>a {planet} meant to apply equally</x:v>
-      </x:c>
-      <x:c r="H44" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="20" t="str">
-        <x:v>whoever defines</x:v>
-      </x:c>
-      <x:c r="B45" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G45" s="20" t="str">
-        <x:v>a {planet} moving only after both replies enter the record</x:v>
-      </x:c>
-      <x:c r="H45" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="20" t="str">
-        <x:v>whoever moves</x:v>
-      </x:c>
-      <x:c r="B46" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G46" s="20" t="str">
-        <x:v>a {planet} protecting access to information that cannot be taken back</x:v>
-      </x:c>
-      <x:c r="H46" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="20" t="str">
-        <x:v>a beautiful</x:v>
-      </x:c>
-      <x:c r="B47" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G47" s="20" t="str">
-        <x:v>a {planet} pursued carefully because it cannot be undone</x:v>
-      </x:c>
-      <x:c r="H47" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="20" t="str">
-        <x:v>a bigger</x:v>
-      </x:c>
-      <x:c r="B48" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G48" s="20" t="str">
-        <x:v>a {planet} stated before anyone grants the right to object</x:v>
-      </x:c>
-      <x:c r="H48" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="21" t="str">
-        <x:v>a choice</x:v>
-      </x:c>
-      <x:c r="B49" s="21" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G49" s="21" t="str">
-        <x:v>a {planet} stated clearly enough to force a quick answer</x:v>
-      </x:c>
-      <x:c r="H49" s="21" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(content): close sky supportive coverage gaps
</commit_message>
<xml_diff>
--- a/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
+++ b/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re59bc0001e1b4ddb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R7699e6c81c824914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="R1b8a6c53e2454533"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Audit" sheetId="4" r:id="Rd25e47f202c5411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeted Verification" sheetId="5" r:id="R6c4dcb0abb9d4a43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="6" r:id="Rdc456446029c4507"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="7" r:id="Rbc676e3729324001"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="8" r:id="R9fc7a54080334053"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="9" r:id="R7dd328c624554cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="10" r:id="R97efc298562e40bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59e0b64fb54c47d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="2" r:id="R1e2d55da4ecd4926"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="3" r:id="R3895962a34644295"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Audit" sheetId="4" r:id="Radf5245da3894458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeted Verification" sheetId="5" r:id="R03cb4e45971f40fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Closing" sheetId="6" r:id="R1fcb13f355204601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="7" r:id="R80fbd9b683d74efb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="8" r:id="R1a4b8c2c974d4ad7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="9" r:id="R2e9b785781f44721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="10" r:id="Racc3f59117d946bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="11" r:id="Re617f4f6e5124dec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -227,7 +228,18 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="8">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF6B4F00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF7E8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -380,26 +392,22 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AspectMechanismsTable" displayName="AspectMechanismsTable" ref="A3:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="11">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SupportiveCoverageClosingTable" displayName="SupportiveCoverageClosingTable" ref="A3:G30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="Key"/>
-    <x:tableColumn id="2" name="Reader effect"/>
-    <x:tableColumn id="3" name="Conflict behavior"/>
-    <x:tableColumn id="4" name="Movement bias"/>
-    <x:tableColumn id="5" name="Supportive realizations"/>
-    <x:tableColumn id="6" name="Neutral realizations"/>
-    <x:tableColumn id="7" name="Shadow realizations"/>
-    <x:tableColumn id="8" name="Source IDs"/>
-    <x:tableColumn id="9" name="Source hashes"/>
-    <x:tableColumn id="10" name="Owner review status"/>
-    <x:tableColumn id="11" name="Owner notes"/>
+    <x:tableColumn id="2" name="Flagged realization"/>
+    <x:tableColumn id="3" name="Only supportive?"/>
+    <x:tableColumn id="4" name="Supportive count before"/>
+    <x:tableColumn id="5" name="Disposition"/>
+    <x:tableColumn id="6" name="Distinct supportive extraction"/>
+    <x:tableColumn id="7" name="Evidence pointers"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ModalityUnitsTable" displayName="ModalityUnitsTable" ref="A3:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AspectMechanismsTable" displayName="AspectMechanismsTable" ref="A3:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Reader effect"/>
@@ -418,7 +426,26 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ElementUnitsTable" displayName="ElementUnitsTable" ref="A3:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ModalityUnitsTable" displayName="ModalityUnitsTable" ref="A3:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Key"/>
+    <x:tableColumn id="2" name="Reader effect"/>
+    <x:tableColumn id="3" name="Conflict behavior"/>
+    <x:tableColumn id="4" name="Movement bias"/>
+    <x:tableColumn id="5" name="Supportive realizations"/>
+    <x:tableColumn id="6" name="Neutral realizations"/>
+    <x:tableColumn id="7" name="Shadow realizations"/>
+    <x:tableColumn id="8" name="Source IDs"/>
+    <x:tableColumn id="9" name="Source hashes"/>
+    <x:tableColumn id="10" name="Owner review status"/>
+    <x:tableColumn id="11" name="Owner notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ElementUnitsTable" displayName="ElementUnitsTable" ref="A3:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Reader effect"/>
@@ -823,10 +850,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="13" t="str">
-        <x:v>Empty supportive pools</x:v>
+        <x:v>Current empty supportive pools</x:v>
       </x:c>
       <x:c r="B15" s="13" t="n">
-        <x:v>64</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1080,6 +1107,347 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Frame uniqueness gate</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Frame uniqueness gate</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Frame uniqueness gate</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Frame uniqueness gate</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Frame uniqueness gate</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Frame uniqueness gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="18" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="B4" s="18" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="C4" s="18" t="str">
+        <x:v>Cap</x:v>
+      </x:c>
+      <x:c r="D4" s="18" t="str">
+        <x:v>Pass example</x:v>
+      </x:c>
+      <x:c r="E4" s="18" t="str">
+        <x:v>Fail example</x:v>
+      </x:c>
+      <x:c r="F4" s="18" t="str">
+        <x:v>Reason</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="25" t="str">
+        <x:v>Exact sentence uniqueness</x:v>
+      </x:c>
+      <x:c r="B5" s="25" t="str">
+        <x:v>Forecast + Details</x:v>
+      </x:c>
+      <x:c r="C5" s="25" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="25" t="str">
+        <x:v>Every sentence appears once</x:v>
+      </x:c>
+      <x:c r="E5" s="25" t="str">
+        <x:v>Same full sentence in two cards</x:v>
+      </x:c>
+      <x:c r="F5" s="25" t="str">
+        <x:v>Prevents copied frames</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="26" t="str">
+        <x:v>Forecast opener construction</x:v>
+      </x:c>
+      <x:c r="B6" s="26" t="str">
+        <x:v>Forecast first sentence</x:v>
+      </x:c>
+      <x:c r="C6" s="26" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D6" s="26" t="str">
+        <x:v>Four or fewer uses</x:v>
+      </x:c>
+      <x:c r="E6" s="26" t="str">
+        <x:v>Five cards begin with the same normalized opening</x:v>
+      </x:c>
+      <x:c r="F6" s="26" t="str">
+        <x:v>Prevents opener monoculture</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="26" t="str">
+        <x:v>Details opener construction</x:v>
+      </x:c>
+      <x:c r="B7" s="26" t="str">
+        <x:v>Details first composed sentence</x:v>
+      </x:c>
+      <x:c r="C7" s="26" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D7" s="26" t="str">
+        <x:v>Four or fewer uses</x:v>
+      </x:c>
+      <x:c r="E7" s="26" t="str">
+        <x:v>Five cards begin with the same normalized opening</x:v>
+      </x:c>
+      <x:c r="F7" s="26" t="str">
+        <x:v>Details must also compose both positions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="26" t="str">
+        <x:v>Connective construction</x:v>
+      </x:c>
+      <x:c r="B8" s="26" t="str">
+        <x:v>Later sentences</x:v>
+      </x:c>
+      <x:c r="C8" s="26" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="str">
+        <x:v>Four or fewer uses of one opening phrase</x:v>
+      </x:c>
+      <x:c r="E8" s="26" t="str">
+        <x:v>Repeated 'That can turn...' across five cards</x:v>
+      </x:c>
+      <x:c r="F8" s="26" t="str">
+        <x:v>Beats do not require fixed connective wording</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="26" t="str">
+        <x:v>Required forecast beats</x:v>
+      </x:c>
+      <x:c r="B9" s="26" t="str">
+        <x:v>Each forecast</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="str">
+        <x:v>All four meanings present</x:v>
+      </x:c>
+      <x:c r="E9" s="26" t="str">
+        <x:v>A moral replaces what can move</x:v>
+      </x:c>
+      <x:c r="F9" s="26" t="str">
+        <x:v>Meaning is required even when wording varies</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="26" t="str">
+        <x:v>Required Details beats</x:v>
+      </x:c>
+      <x:c r="B10" s="26" t="str">
+        <x:v>Each Details block</x:v>
+      </x:c>
+      <x:c r="C10" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="str">
+        <x:v>Explanation ends after behavior</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="str">
+        <x:v>Forecast conclusion repeated in Details</x:v>
+      </x:c>
+      <x:c r="F10" s="26" t="str">
+        <x:v>Forecast concludes; Details explains</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="26" t="str">
+        <x:v>Verbatim component emission</x:v>
+      </x:c>
+      <x:c r="B11" s="26" t="str">
+        <x:v>All components</x:v>
+      </x:c>
+      <x:c r="C11" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="str">
+        <x:v>Composer paraphrases and integrates</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="str">
+        <x:v>A stored component appears as a full sentence</x:v>
+      </x:c>
+      <x:c r="F11" s="26" t="str">
+        <x:v>Components govern meaning, not prose</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="26" t="str">
+        <x:v>Manifestation shape reuse</x:v>
+      </x:c>
+      <x:c r="B12" s="26" t="str">
+        <x:v>Sign-unit manifestations</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="str">
+        <x:v>Planet-sign events use distinct grammar</x:v>
+      </x:c>
+      <x:c r="E12" s="26" t="str">
+        <x:v>A sign frame survives after planet nouns are stripped</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
+        <x:v>String uniqueness alone does not catch slot templates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="26" t="str">
+        <x:v>Plain-register subject</x:v>
+      </x:c>
+      <x:c r="B13" s="26" t="str">
+        <x:v>Meaning components</x:v>
+      </x:c>
+      <x:c r="C13" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="26" t="str">
+        <x:v>People, deadlines, messages, rules, and other everyday actors lead</x:v>
+      </x:c>
+      <x:c r="E13" s="26" t="str">
+        <x:v>Recognition, autonomy, or pressure narrates itself</x:v>
+      </x:c>
+      <x:c r="F13" s="26" t="str">
+        <x:v>The owner's register uses active verbs and concrete nouns</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="26" t="str">
+        <x:v>Manifestation actor or act</x:v>
+      </x:c>
+      <x:c r="B14" s="26" t="str">
+        <x:v>All sign manifestations</x:v>
+      </x:c>
+      <x:c r="C14" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="26" t="str">
+        <x:v>A person acts or a concrete act is visible</x:v>
+      </x:c>
+      <x:c r="E14" s="26" t="str">
+        <x:v>Care turns into leverage</x:v>
+      </x:c>
+      <x:c r="F14" s="26" t="str">
+        <x:v>An abstraction may not perform the behavior</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="26" t="str">
+        <x:v>Source shadow coverage</x:v>
+      </x:c>
+      <x:c r="B15" s="26" t="str">
+        <x:v>All sign units</x:v>
+      </x:c>
+      <x:c r="C15" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="26" t="str">
+        <x:v>A supported cost or overreach remains available</x:v>
+      </x:c>
+      <x:c r="E15" s="26" t="str">
+        <x:v>Jupiter becomes uniformly beneficial</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="str">
+        <x:v>The component may not erase source challenge, shadow, or cost</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="26" t="str">
+        <x:v>Typed realization pools</x:v>
+      </x:c>
+      <x:c r="B16" s="26" t="str">
+        <x:v>All 174 units</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="str">
+        <x:v>Supportive, neutral, and shadow meanings live in named arrays</x:v>
+      </x:c>
+      <x:c r="E16" s="26" t="str">
+        <x:v>Useful/neutral/shadow is encoded as bullet position</x:v>
+      </x:c>
+      <x:c r="F16" s="26" t="str">
+        <x:v>The composer chooses meaning type; it never learns a three-item rhythm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="27" t="str">
+        <x:v>Owner-source conversion</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>All owner-voice evidence</x:v>
+      </x:c>
+      <x:c r="C17" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="str">
+        <x:v>Personal source meaning is converted for collective Sky</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="str">
+        <x:v>Eight or more source words are copied verbatim</x:v>
+      </x:c>
+      <x:c r="F17" s="27" t="str">
+        <x:v>Owner voice governs without leaking second-person source prose</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1182,13 +1550,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="10" t="n">
-        <x:v>496</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>496</x:v>
+        <x:v>514</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1361,7 +1729,7 @@
         <x:v>Typed-array count shapes</x:v>
       </x:c>
       <x:c r="B21" s="15" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C21" s="15" t="str">
         <x:v>&gt;= 2</x:v>
@@ -2531,9 +2899,13 @@
         <x:v>whoever did the work wants their name kept with it</x:v>
       </x:c>
       <x:c r="E8" s="45" t="str">
-        <x:v>• wanting credit attached to the person who did the work</x:v>
-      </x:c>
-      <x:c r="F8" s="45" t="str"/>
+        <x:v>• wanting credit attached to the person who did the work
+• someone showing work they are proud of instead of leaving it hidden</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="str">
+        <x:v>someone showing work they are proud of instead of leaving it hidden
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!813</x:v>
+      </x:c>
       <x:c r="G8" s="45" t="str">
         <x:v>• wanting effort acknowledged
 • wanting individual contribution distinguished from the group</x:v>
@@ -2724,8 +3096,13 @@
       <x:c r="D12" s="45" t="str">
         <x:v>whoever names the larger purpose can become the face of it</x:v>
       </x:c>
-      <x:c r="E12" s="45" t="str"/>
-      <x:c r="F12" s="45" t="str"/>
+      <x:c r="E12" s="45" t="str">
+        <x:v>• someone asking why until the larger purpose behind a decision becomes clear</x:v>
+      </x:c>
+      <x:c r="F12" s="45" t="str">
+        <x:v>someone asking why until the larger purpose behind a decision becomes clear
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/sagittarius</x:v>
+      </x:c>
       <x:c r="G12" s="45" t="str">
         <x:v>• the person who names the wider purpose becoming identified with it
 • a strong belief making one contribution stand for a larger cause</x:v>
@@ -3449,10 +3826,13 @@
         <x:v>the group makes room for feeling by stepping back and looking at the pattern</x:v>
       </x:c>
       <x:c r="E26" s="45" t="str">
-        <x:v>• someone stepping back from a reaction long enough to see the pattern clearly</x:v>
+        <x:v>• someone stepping back from a reaction long enough to see the pattern clearly
+• someone keeping track of what the whole group needs during a crisis</x:v>
       </x:c>
       <x:c r="F26" s="45" t="str">
         <x:v>someone stepping back from a reaction long enough to see the pattern clearly
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!118
+someone keeping track of what the whole group needs during a crisis
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!118</x:v>
       </x:c>
       <x:c r="G26" s="45" t="str">
@@ -3558,11 +3938,14 @@
         <x:v>the first clear answer can move a decision before everyone has finished thinking</x:v>
       </x:c>
       <x:c r="E28" s="45" t="str">
-        <x:v>• someone giving the clear answer that gets a stalled decision moving again</x:v>
+        <x:v>• someone giving the clear answer that gets a stalled decision moving again
+• someone stating the main point before the discussion gets lost in explanation</x:v>
       </x:c>
       <x:c r="F28" s="45" t="str">
         <x:v>someone giving the clear answer that gets a stalled decision moving again
-tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!251</x:v>
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!251
+someone stating the main point before the discussion gets lost in explanation
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!84</x:v>
       </x:c>
       <x:c r="G28" s="45" t="str">
         <x:v>• a decision announced before every objection has been heard
@@ -4132,9 +4515,13 @@
         <x:v>people understand the tone or image sooner than they agree on the facts</x:v>
       </x:c>
       <x:c r="E39" s="45" t="str">
-        <x:v>• people reading the tone when the stated facts remain incomplete</x:v>
-      </x:c>
-      <x:c r="F39" s="45" t="str"/>
+        <x:v>• people reading the tone when the stated facts remain incomplete
+• someone finding words for an image or hunch so other people can follow the reasoning</x:v>
+      </x:c>
+      <x:c r="F39" s="45" t="str">
+        <x:v>someone finding words for an image or hunch so other people can follow the reasoning
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!95</x:v>
+      </x:c>
       <x:c r="G39" s="45" t="str"/>
       <x:c r="H39" s="45" t="str">
         <x:v>• an implication spreading faster than anyone can verify it
@@ -4234,10 +4621,13 @@
         <x:v>a choice feels worthwhile when it is pleasant, affordable, and built to last</x:v>
       </x:c>
       <x:c r="E41" s="45" t="str">
-        <x:v>• someone choosing the arrangement that feels good and can still hold up over time</x:v>
+        <x:v>• someone choosing the arrangement that feels good and can still hold up over time
+• someone remembering the favorite snack and bringing it without being asked</x:v>
       </x:c>
       <x:c r="F41" s="45" t="str">
         <x:v>someone choosing the arrangement that feels good and can still hold up over time
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!61
+someone remembering the favorite snack and bringing it without being asked
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!61</x:v>
       </x:c>
       <x:c r="G41" s="45" t="str">
@@ -4610,10 +5000,13 @@
         <x:v>people choose the agreement that leaves more room to grow and explore</x:v>
       </x:c>
       <x:c r="E48" s="45" t="str">
-        <x:v>• someone choosing a connection that leaves both people room to keep growing</x:v>
+        <x:v>• someone choosing a connection that leaves both people room to keep growing
+• someone taking interest in an independent plan instead of treating it as a threat</x:v>
       </x:c>
       <x:c r="F48" s="45" t="str">
         <x:v>someone choosing a connection that leaves both people room to keep growing
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!68
+someone taking interest in an independent plan instead of treating it as a threat
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!68</x:v>
       </x:c>
       <x:c r="G48" s="45" t="str">
@@ -4726,9 +5119,13 @@
         <x:v>people stay connected by giving each other room inside the group</x:v>
       </x:c>
       <x:c r="E50" s="45" t="str">
-        <x:v>• people staying connected because the agreement leaves room for independence</x:v>
-      </x:c>
-      <x:c r="F50" s="45" t="str"/>
+        <x:v>• people staying connected because the agreement leaves room for independence
+• someone making room for an offbeat idea without asking the person behind it to explain themselves</x:v>
+      </x:c>
+      <x:c r="F50" s="45" t="str">
+        <x:v>someone making room for an offbeat idea without asking the person behind it to explain themselves
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/venus/aquarius</x:v>
+      </x:c>
       <x:c r="G50" s="45" t="str">
         <x:v>• people finding common value in a group commitment instead of private closeness</x:v>
       </x:c>
@@ -4884,9 +5281,13 @@
         <x:v>people keep pushing the same point until a material limit finally moves</x:v>
       </x:c>
       <x:c r="E53" s="45" t="str">
-        <x:v>• someone working the same point until a material limit gives way</x:v>
-      </x:c>
-      <x:c r="F53" s="45" t="str"/>
+        <x:v>• someone working the same point until a material limit gives way
+• someone finishing a careful repair instead of changing tactics halfway through</x:v>
+      </x:c>
+      <x:c r="F53" s="45" t="str">
+        <x:v>someone finishing a careful repair instead of changing tactics halfway through
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!37</x:v>
+      </x:c>
       <x:c r="G53" s="45" t="str">
         <x:v>• someone delaying action until they can keep the result</x:v>
       </x:c>
@@ -4991,9 +5392,13 @@
         <x:v>someone protects the home or the people involved before explaining the anger</x:v>
       </x:c>
       <x:c r="E55" s="45" t="str">
-        <x:v>• someone acting to protect another person before explaining why</x:v>
-      </x:c>
-      <x:c r="F55" s="45" t="str"/>
+        <x:v>• someone acting to protect another person before explaining why
+• someone separating the practical need from the feeling before choosing the next step</x:v>
+      </x:c>
+      <x:c r="F55" s="45" t="str">
+        <x:v>someone separating the practical need from the feeling before choosing the next step
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!159</x:v>
+      </x:c>
       <x:c r="G55" s="45" t="str">
         <x:v>• defense beginning when home or belonging feels exposed
 • someone defending a private vulnerability inside a public decision</x:v>
@@ -5214,9 +5619,13 @@
         <x:v>someone acts carefully because trust, control, and lasting consequences are involved</x:v>
       </x:c>
       <x:c r="E59" s="45" t="str">
-        <x:v>• a result pursued carefully because it cannot be undone</x:v>
-      </x:c>
-      <x:c r="F59" s="45" t="str"/>
+        <x:v>• a result pursued carefully because it cannot be undone
+• someone using what the delay revealed instead of starting the work over</x:v>
+      </x:c>
+      <x:c r="F59" s="45" t="str">
+        <x:v>someone using what the delay revealed instead of starting the work over
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!194</x:v>
+      </x:c>
       <x:c r="G59" s="45" t="str">
         <x:v>• someone withholding action until the source of control becomes clear</x:v>
       </x:c>
@@ -6237,9 +6646,13 @@
         <x:v>The wording gets tighter once the decision has consequences and the record has to stay consistent.</x:v>
       </x:c>
       <x:c r="E78" s="45" t="str">
-        <x:v>• revised language that still has to match the record</x:v>
-      </x:c>
-      <x:c r="F78" s="45" t="str"/>
+        <x:v>• revised language that still has to match the record
+• someone finishing the course or project they kept setting down</x:v>
+      </x:c>
+      <x:c r="F78" s="45" t="str">
+        <x:v>someone finishing the course or project they kept setting down
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!667</x:v>
+      </x:c>
       <x:c r="G78" s="45" t="str">
         <x:v>• a decision delayed while conflicting facts are documented</x:v>
       </x:c>
@@ -6563,9 +6976,13 @@
         <x:v>a large promise meets the test of what can be proved and delivered</x:v>
       </x:c>
       <x:c r="E84" s="45" t="str">
-        <x:v>• a large promise reduced to what can be proved and delivered</x:v>
-      </x:c>
-      <x:c r="F84" s="45" t="str"/>
+        <x:v>• a large promise reduced to what can be proved and delivered
+• someone turning a vague obligation into a deadline that can be met</x:v>
+      </x:c>
+      <x:c r="F84" s="45" t="str">
+        <x:v>someone turning a vague obligation into a deadline that can be met
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!690</x:v>
+      </x:c>
       <x:c r="G84" s="45" t="str"/>
       <x:c r="H84" s="45" t="str">
         <x:v>• someone testing a belief against the boundary of an institution or law
@@ -6671,8 +7088,13 @@
       <x:c r="D86" s="45" t="str">
         <x:v>the same rule is expected to apply across the group, even when one case resists it</x:v>
       </x:c>
-      <x:c r="E86" s="45" t="str"/>
-      <x:c r="F86" s="45" t="str"/>
+      <x:c r="E86" s="45" t="str">
+        <x:v>• someone proving a different method works before the old rule is treated as permanent</x:v>
+      </x:c>
+      <x:c r="F86" s="45" t="str">
+        <x:v>someone proving a different method works before the old rule is treated as permanent
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!719</x:v>
+      </x:c>
       <x:c r="G86" s="45" t="str">
         <x:v>• policy applied across the group
 • precedent
@@ -7860,8 +8282,13 @@
       <x:c r="D108" s="45" t="str">
         <x:v>the promise grows beyond the facts that were meant to support it</x:v>
       </x:c>
-      <x:c r="E108" s="45" t="str"/>
-      <x:c r="F108" s="45" t="str"/>
+      <x:c r="E108" s="45" t="str">
+        <x:v>• someone checking whether a belief is their own before making a decision around it</x:v>
+      </x:c>
+      <x:c r="F108" s="45" t="str">
+        <x:v>someone checking whether a belief is their own before making a decision around it
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!547</x:v>
+      </x:c>
       <x:c r="G108" s="45" t="str"/>
       <x:c r="H108" s="45" t="str">
         <x:v>• people looking farther ahead while overlooking the practical distance
@@ -8996,13 +9423,17 @@
         <x:v>a small mistake can reopen the fear that usefulness is the price of belonging</x:v>
       </x:c>
       <x:c r="E129" s="45" t="str">
-        <x:v>• a small correction reopening the fear of never being useful enough</x:v>
-      </x:c>
-      <x:c r="F129" s="45" t="str"/>
+        <x:v>• someone letting a finished task stand before every small flaw has been fixed</x:v>
+      </x:c>
+      <x:c r="F129" s="45" t="str">
+        <x:v>someone letting a finished task stand before every small flaw has been fixed
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!21</x:v>
+      </x:c>
       <x:c r="G129" s="45" t="str"/>
       <x:c r="H129" s="45" t="str">
         <x:v>• competence becoming a defense against being judged as a burden
-• someone focusing on the detail others dismiss because it once carried a real cost</x:v>
+• someone focusing on the detail others dismiss because it once carried a real cost
+• a small correction reopening the fear of never being useful enough</x:v>
       </x:c>
       <x:c r="I129" s="45" t="str">
         <x:v>sensitivity around usefulness and correction</x:v>
@@ -9640,9 +10071,13 @@
         <x:v>someone challenges an agreement that calls repeated self-erasure fair</x:v>
       </x:c>
       <x:c r="E142" s="45" t="str">
-        <x:v>• an agreement challenged after fairness becomes repeated self-erasure</x:v>
-      </x:c>
-      <x:c r="F142" s="45" t="str"/>
+        <x:v>• an agreement challenged after fairness becomes repeated self-erasure
+• someone saying plainly that an arrangement does not work for them</x:v>
+      </x:c>
+      <x:c r="F142" s="45" t="str">
+        <x:v>someone saying plainly that an arrangement does not work for them
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/libra</x:v>
+      </x:c>
       <x:c r="G142" s="45" t="str">
         <x:v>• someone demanding terms that do not depend on one side yielding</x:v>
       </x:c>
@@ -9686,9 +10121,13 @@
         <x:v>people protect desire and private access from someone trying to take control</x:v>
       </x:c>
       <x:c r="E143" s="45" t="str">
-        <x:v>• someone protecting desire from another person's claim to private access</x:v>
-      </x:c>
-      <x:c r="F143" s="45" t="str"/>
+        <x:v>• someone protecting desire from another person's claim to private access
+• someone naming the private agreement everybody has been organizing around</x:v>
+      </x:c>
+      <x:c r="F143" s="45" t="str">
+        <x:v>someone naming the private agreement everybody has been organizing around
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/scorpio</x:v>
+      </x:c>
       <x:c r="G143" s="45" t="str">
         <x:v>• someone ending the agreement after trust is used as leverage
 • someone keeping private what they could not safely recover once given</x:v>
@@ -9927,7 +10366,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red5841d4f9d34c86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2816db6eddd84fbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12554,7 +12993,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1065d684feab4963"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dcb0ec43db14f16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13151,13 +13590,719 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71fbcf869da84810"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4dc3a4fc83748ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b6664373b0140e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03387f4d0a554857"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="64" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="72" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Supportive coverage closing review</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Supportive coverage closing review</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Supportive coverage closing review</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Supportive coverage closing review</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Supportive coverage closing review</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Supportive coverage closing review</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Supportive coverage closing review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>27 flags checked; 15 were sole-support items. 18 evidence-backed supportive realizations added; blocked soft routes 98 -&gt; 0.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>27 flags checked; 15 were sole-support items. 18 evidence-backed supportive realizations added; blocked soft routes 98 -&gt; 0.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>27 flags checked; 15 were sole-support items. 18 evidence-backed supportive realizations added; blocked soft routes 98 -&gt; 0.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>27 flags checked; 15 were sole-support items. 18 evidence-backed supportive realizations added; blocked soft routes 98 -&gt; 0.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>27 flags checked; 15 were sole-support items. 18 evidence-backed supportive realizations added; blocked soft routes 98 -&gt; 0.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>27 flags checked; 15 were sole-support items. 18 evidence-backed supportive realizations added; blocked soft routes 98 -&gt; 0.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>27 flags checked; 15 were sole-support items. 18 evidence-backed supportive realizations added; blocked soft routes 98 -&gt; 0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B3" s="35" t="str">
+        <x:v>Flagged realization</x:v>
+      </x:c>
+      <x:c r="C3" s="35" t="str">
+        <x:v>Only supportive?</x:v>
+      </x:c>
+      <x:c r="D3" s="35" t="str">
+        <x:v>Supportive count before</x:v>
+      </x:c>
+      <x:c r="E3" s="35" t="str">
+        <x:v>Disposition</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>Distinct supportive extraction</x:v>
+      </x:c>
+      <x:c r="G3" s="36" t="str">
+        <x:v>Evidence pointers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="44" t="str">
+        <x:v>sky-sign/sun/taurus</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
+        <x:v>a contribution valued because it keeps producing something useful</x:v>
+      </x:c>
+      <x:c r="C4" s="44" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D4" s="44" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E4" s="44" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F4" s="44" t="str"/>
+      <x:c r="G4" s="44" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!782</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>sky-sign/sun/taurus</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>people waiting to give credit until the result proves it can last</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str"/>
+      <x:c r="G5" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!782</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="45" t="str">
+        <x:v>sky-sign/sun/taurus</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>credit going to the work that protected what needed to last</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E6" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="str"/>
+      <x:c r="G6" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!782</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="45" t="str">
+        <x:v>sky-sign/sun/gemini</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>the clearest explanation deciding who is seen as responsible</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str"/>
+      <x:c r="G7" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!792</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="45" t="str">
+        <x:v>sky-sign/sun/leo</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>wanting credit attached to the person who did the work</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="str">
+        <x:v>someone showing work they are proud of instead of leaving it hidden</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!813</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="45" t="str">
+        <x:v>sky-sign/sun/capricorn</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>people giving credit to the person expected to answer for the result</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="str"/>
+      <x:c r="G9" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/sun/capricorn
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!852</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="45" t="str">
+        <x:v>sky-sign/moon/aquarius</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="str">
+        <x:v>someone stepping back from a reaction long enough to see the pattern clearly</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F10" s="45" t="str">
+        <x:v>someone keeping track of what the whole group needs during a crisis</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!118</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="45" t="str">
+        <x:v>sky-sign/mercury/aries</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>someone giving the clear answer that gets a stalled decision moving again</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="str">
+        <x:v>someone stating the main point before the discussion gets lost in explanation</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!84</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="45" t="str">
+        <x:v>sky-sign/mercury/taurus</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="str">
+        <x:v>an agreement slowing until the practical terms are clear</x:v>
+      </x:c>
+      <x:c r="C12" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D12" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E12" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F12" s="45" t="str"/>
+      <x:c r="G12" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/mercury/taurus
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!275</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="45" t="str">
+        <x:v>sky-sign/mercury/pisces</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>people reading the tone when the stated facts remain incomplete</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E13" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F13" s="45" t="str">
+        <x:v>someone finding words for an image or hunch so other people can follow the reasoning</x:v>
+      </x:c>
+      <x:c r="G13" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="45" t="str">
+        <x:v>sky-sign/venus/taurus</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>someone choosing the arrangement that feels good and can still hold up over time</x:v>
+      </x:c>
+      <x:c r="C14" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F14" s="45" t="str">
+        <x:v>someone remembering the favorite snack and bringing it without being asked</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!61</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="45" t="str">
+        <x:v>sky-sign/venus/sagittarius</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="str">
+        <x:v>someone choosing a connection that leaves both people room to keep growing</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D15" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E15" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F15" s="45" t="str">
+        <x:v>someone taking interest in an independent plan instead of treating it as a threat</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="45" t="str">
+        <x:v>sky-sign/venus/aquarius</x:v>
+      </x:c>
+      <x:c r="B16" s="45" t="str">
+        <x:v>people staying connected because the agreement leaves room for independence</x:v>
+      </x:c>
+      <x:c r="C16" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D16" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F16" s="45" t="str">
+        <x:v>someone making room for an offbeat idea without asking the person behind it to explain themselves</x:v>
+      </x:c>
+      <x:c r="G16" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/venus/aquarius</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="45" t="str">
+        <x:v>sky-sign/mars/cancer</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="str">
+        <x:v>someone acting to protect another person before explaining why</x:v>
+      </x:c>
+      <x:c r="C17" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D17" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E17" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F17" s="45" t="str">
+        <x:v>someone separating the practical need from the feeling before choosing the next step</x:v>
+      </x:c>
+      <x:c r="G17" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!159</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="45" t="str">
+        <x:v>sky-sign/mars/taurus</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="str">
+        <x:v>someone working the same point until a material limit gives way</x:v>
+      </x:c>
+      <x:c r="C18" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D18" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F18" s="45" t="str">
+        <x:v>someone finishing a careful repair instead of changing tactics halfway through</x:v>
+      </x:c>
+      <x:c r="G18" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="45" t="str">
+        <x:v>sky-sign/mars/scorpio</x:v>
+      </x:c>
+      <x:c r="B19" s="45" t="str">
+        <x:v>a result pursued carefully because it cannot be undone</x:v>
+      </x:c>
+      <x:c r="C19" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D19" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F19" s="45" t="str">
+        <x:v>someone using what the delay revealed instead of starting the work over</x:v>
+      </x:c>
+      <x:c r="G19" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!194</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="45" t="str">
+        <x:v>sky-sign/jupiter/libra</x:v>
+      </x:c>
+      <x:c r="B20" s="45" t="str">
+        <x:v>more people benefiting after the terms distribute the opportunity more fairly</x:v>
+      </x:c>
+      <x:c r="C20" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D20" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E20" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F20" s="45" t="str"/>
+      <x:c r="G20" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/jupiter/libra
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!80
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="45" t="str">
+        <x:v>sky-sign/saturn/gemini</x:v>
+      </x:c>
+      <x:c r="B21" s="45" t="str">
+        <x:v>revised language that still has to match the record</x:v>
+      </x:c>
+      <x:c r="C21" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D21" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E21" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F21" s="45" t="str">
+        <x:v>someone finishing the course or project they kept setting down</x:v>
+      </x:c>
+      <x:c r="G21" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="45" t="str">
+        <x:v>sky-sign/saturn/sagittarius</x:v>
+      </x:c>
+      <x:c r="B22" s="45" t="str">
+        <x:v>a large promise reduced to what can be proved and delivered</x:v>
+      </x:c>
+      <x:c r="C22" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D22" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E22" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F22" s="45" t="str">
+        <x:v>someone turning a vague obligation into a deadline that can be met</x:v>
+      </x:c>
+      <x:c r="G22" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!690</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="45" t="str">
+        <x:v>sky-sign/uranus/gemini</x:v>
+      </x:c>
+      <x:c r="B23" s="45" t="str">
+        <x:v>new information altering the available routes almost immediately</x:v>
+      </x:c>
+      <x:c r="C23" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D23" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E23" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F23" s="45" t="str"/>
+      <x:c r="G23" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/uranus/gemini
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!930
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!218</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="45" t="str">
+        <x:v>sky-sign/neptune/leo</x:v>
+      </x:c>
+      <x:c r="B24" s="45" t="str">
+        <x:v>a public image carrying more hope than the contribution can support</x:v>
+      </x:c>
+      <x:c r="C24" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D24" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E24" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F24" s="45" t="str"/>
+      <x:c r="G24" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/neptune/leo
+tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!539
+tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!244</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="45" t="str">
+        <x:v>sky-sign/chiron/virgo</x:v>
+      </x:c>
+      <x:c r="B25" s="45" t="str">
+        <x:v>a small correction reopening the fear of never being useful enough</x:v>
+      </x:c>
+      <x:c r="C25" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D25" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E25" s="45" t="str">
+        <x:v>reclassified to shadow and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F25" s="45" t="str">
+        <x:v>someone letting a finished task stand before every small flaw has been fixed</x:v>
+      </x:c>
+      <x:c r="G25" s="45" t="str">
+        <x:v>tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="45" t="str">
+        <x:v>sky-sign/lilith/leo</x:v>
+      </x:c>
+      <x:c r="B26" s="45" t="str">
+        <x:v>someone claiming visibility without making the contribution more acceptable first</x:v>
+      </x:c>
+      <x:c r="C26" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D26" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E26" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F26" s="45" t="str"/>
+      <x:c r="G26" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/leo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="45" t="str">
+        <x:v>sky-sign/lilith/virgo</x:v>
+      </x:c>
+      <x:c r="B27" s="45" t="str">
+        <x:v>a standard refused because usefulness has become a condition of worth</x:v>
+      </x:c>
+      <x:c r="C27" s="45" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D27" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E27" s="45" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F27" s="45" t="str"/>
+      <x:c r="G27" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/virgo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="45" t="str">
+        <x:v>sky-sign/lilith/libra</x:v>
+      </x:c>
+      <x:c r="B28" s="45" t="str">
+        <x:v>an agreement challenged after fairness becomes repeated self-erasure</x:v>
+      </x:c>
+      <x:c r="C28" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D28" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E28" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F28" s="45" t="str">
+        <x:v>someone saying plainly that an arrangement does not work for them</x:v>
+      </x:c>
+      <x:c r="G28" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/libra</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="45" t="str">
+        <x:v>sky-sign/lilith/scorpio</x:v>
+      </x:c>
+      <x:c r="B29" s="45" t="str">
+        <x:v>someone protecting desire from another person's claim to private access</x:v>
+      </x:c>
+      <x:c r="C29" s="45" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D29" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E29" s="45" t="str">
+        <x:v>kept and distinct supportive extracted</x:v>
+      </x:c>
+      <x:c r="F29" s="45" t="str">
+        <x:v>someone naming the private agreement everybody has been organizing around</x:v>
+      </x:c>
+      <x:c r="G29" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/scorpio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="46" t="str">
+        <x:v>sky-sign/lilith/capricorn</x:v>
+      </x:c>
+      <x:c r="B30" s="46" t="str">
+        <x:v>someone confronting an authority that has used respectability as control</x:v>
+      </x:c>
+      <x:c r="C30" s="46" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D30" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E30" s="46" t="str">
+        <x:v>left unchanged other supportive available</x:v>
+      </x:c>
+      <x:c r="F30" s="46" t="str"/>
+      <x:c r="G30" s="46" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-hook/sky-placement-hook/lilith/capricorn</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="A4:G30">
+    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="PENDING OWNER"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3a962e17bdd4843"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -13450,7 +14595,7 @@
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:K8">
-    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="PENDING OWNER"/>
+    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="PENDING OWNER"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="J4:J8">
@@ -13459,464 +14604,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f7fcb2804404992"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="J1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="str">
-        <x:v>Modality units (9)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="D2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="E2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="F2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="G2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="H2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="I2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="J2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-      <x:c r="K2" s="7" t="str">
-        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="34" t="str">
-        <x:v>Key</x:v>
-      </x:c>
-      <x:c r="B3" s="35" t="str">
-        <x:v>Reader effect</x:v>
-      </x:c>
-      <x:c r="C3" s="35" t="str">
-        <x:v>Conflict behavior</x:v>
-      </x:c>
-      <x:c r="D3" s="35" t="str">
-        <x:v>Movement bias</x:v>
-      </x:c>
-      <x:c r="E3" s="35" t="str">
-        <x:v>Supportive realizations</x:v>
-      </x:c>
-      <x:c r="F3" s="35" t="str">
-        <x:v>Neutral realizations</x:v>
-      </x:c>
-      <x:c r="G3" s="35" t="str">
-        <x:v>Shadow realizations</x:v>
-      </x:c>
-      <x:c r="H3" s="35" t="str">
-        <x:v>Source IDs</x:v>
-      </x:c>
-      <x:c r="I3" s="35" t="str">
-        <x:v>Source hashes</x:v>
-      </x:c>
-      <x:c r="J3" s="35" t="str">
-        <x:v>Owner review status</x:v>
-      </x:c>
-      <x:c r="K3" s="36" t="str">
-        <x:v>Owner notes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="44" t="str">
-        <x:v>sky-how/modality/cardinal/cardinal</x:v>
-      </x:c>
-      <x:c r="B4" s="44" t="str">
-        <x:v>two attempts to set direction become visible at once</x:v>
-      </x:c>
-      <x:c r="C4" s="44" t="str">
-        <x:v>both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
-      </x:c>
-      <x:c r="D4" s="44" t="str">
-        <x:v>both sides need a shared first step or a clear decision about who leads</x:v>
-      </x:c>
-      <x:c r="E4" s="44" t="str">
-        <x:v>• both sides need a shared first step or a clear decision about who leads</x:v>
-      </x:c>
-      <x:c r="F4" s="44" t="str">
-        <x:v>• two attempts to set direction become visible at once</x:v>
-      </x:c>
-      <x:c r="G4" s="44" t="str">
-        <x:v>• both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
-      </x:c>
-      <x:c r="H4" s="44" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I4" s="44" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J4" s="44" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K4" s="44" t="str"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="45" t="str">
-        <x:v>sky-how/modality/cardinal/fixed</x:v>
-      </x:c>
-      <x:c r="B5" s="45" t="str">
-        <x:v>an immediate push runs into a limit meant to hold</x:v>
-      </x:c>
-      <x:c r="C5" s="45" t="str">
-        <x:v>one position keeps initiating while the other protects what cannot be surrendered</x:v>
-      </x:c>
-      <x:c r="D5" s="45" t="str">
-        <x:v>people need an action that preserves the fixed position's central limit</x:v>
-      </x:c>
-      <x:c r="E5" s="45" t="str">
-        <x:v>• people need an action that preserves the fixed position's central limit</x:v>
-      </x:c>
-      <x:c r="F5" s="45" t="str">
-        <x:v>• an immediate push runs into a limit meant to hold</x:v>
-      </x:c>
-      <x:c r="G5" s="45" t="str">
-        <x:v>• one position keeps initiating while the other protects what cannot be surrendered</x:v>
-      </x:c>
-      <x:c r="H5" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I5" s="45" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J5" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K5" s="45" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="45" t="str">
-        <x:v>sky-how/modality/cardinal/mutable</x:v>
-      </x:c>
-      <x:c r="B6" s="45" t="str">
-        <x:v>a first move keeps meeting revised terms</x:v>
-      </x:c>
-      <x:c r="C6" s="45" t="str">
-        <x:v>one position wants a decision while the other adapts as new conditions appear</x:v>
-      </x:c>
-      <x:c r="D6" s="45" t="str">
-        <x:v>the first step has to leave room for a defined adjustment</x:v>
-      </x:c>
-      <x:c r="E6" s="45" t="str">
-        <x:v>• the first step has to leave room for a defined adjustment</x:v>
-      </x:c>
-      <x:c r="F6" s="45" t="str">
-        <x:v>• a first move keeps meeting revised terms</x:v>
-      </x:c>
-      <x:c r="G6" s="45" t="str">
-        <x:v>• one position wants a decision while the other adapts as new conditions appear</x:v>
-      </x:c>
-      <x:c r="H6" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I6" s="45" t="str">
-        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J6" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K6" s="45" t="str"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="45" t="str">
-        <x:v>sky-how/modality/fixed/cardinal</x:v>
-      </x:c>
-      <x:c r="B7" s="45" t="str">
-        <x:v>a protected position is pressed for immediate action</x:v>
-      </x:c>
-      <x:c r="C7" s="45" t="str">
-        <x:v>one side holds its ground while the other treats movement as urgent</x:v>
-      </x:c>
-      <x:c r="D7" s="45" t="str">
-        <x:v>the proposed action must work inside the limit that is not moving</x:v>
-      </x:c>
-      <x:c r="E7" s="45" t="str">
-        <x:v>• the proposed action must work inside the limit that is not moving</x:v>
-      </x:c>
-      <x:c r="F7" s="45" t="str">
-        <x:v>• a protected position is pressed for immediate action</x:v>
-      </x:c>
-      <x:c r="G7" s="45" t="str">
-        <x:v>• one side holds its ground while the other treats movement as urgent</x:v>
-      </x:c>
-      <x:c r="H7" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I7" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J7" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K7" s="45" t="str"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="45" t="str">
-        <x:v>sky-how/modality/fixed/fixed</x:v>
-      </x:c>
-      <x:c r="B8" s="45" t="str">
-        <x:v>the disagreement settles around two positions neither side considers expendable</x:v>
-      </x:c>
-      <x:c r="C8" s="45" t="str">
-        <x:v>neither side gives ground easily under pressure</x:v>
-      </x:c>
-      <x:c r="D8" s="45" t="str">
-        <x:v>people are more likely to change the terms or structure than to make either side back down</x:v>
-      </x:c>
-      <x:c r="E8" s="45" t="str">
-        <x:v>• people are more likely to change the terms or structure than to make either side back down</x:v>
-      </x:c>
-      <x:c r="F8" s="45" t="str">
-        <x:v>• the disagreement settles around two positions neither side considers expendable</x:v>
-      </x:c>
-      <x:c r="G8" s="45" t="str">
-        <x:v>• neither side gives ground easily under pressure</x:v>
-      </x:c>
-      <x:c r="H8" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I8" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J8" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K8" s="45" t="str"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="45" t="str">
-        <x:v>sky-how/modality/fixed/mutable</x:v>
-      </x:c>
-      <x:c r="B9" s="45" t="str">
-        <x:v>a firm limit keeps meeting a changing response</x:v>
-      </x:c>
-      <x:c r="C9" s="45" t="str">
-        <x:v>one position holds the line while the other revises around it</x:v>
-      </x:c>
-      <x:c r="D9" s="45" t="str">
-        <x:v>people have to name the nonnegotiable point instead of revising around it</x:v>
-      </x:c>
-      <x:c r="E9" s="45" t="str">
-        <x:v>• people have to name the nonnegotiable point instead of revising around it</x:v>
-      </x:c>
-      <x:c r="F9" s="45" t="str">
-        <x:v>• a firm limit keeps meeting a changing response</x:v>
-      </x:c>
-      <x:c r="G9" s="45" t="str">
-        <x:v>• one position holds the line while the other revises around it</x:v>
-      </x:c>
-      <x:c r="H9" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I9" s="45" t="str">
-        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J9" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K9" s="45" t="str"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="45" t="str">
-        <x:v>sky-how/modality/mutable/cardinal</x:v>
-      </x:c>
-      <x:c r="B10" s="45" t="str">
-        <x:v>changing conditions are pushed toward a decision</x:v>
-      </x:c>
-      <x:c r="C10" s="45" t="str">
-        <x:v>one position keeps revising while the other insists that action cannot wait</x:v>
-      </x:c>
-      <x:c r="D10" s="45" t="str">
-        <x:v>a decision can move if it includes a defined point for review</x:v>
-      </x:c>
-      <x:c r="E10" s="45" t="str">
-        <x:v>• a decision can move if it includes a defined point for review</x:v>
-      </x:c>
-      <x:c r="F10" s="45" t="str">
-        <x:v>• changing conditions are pushed toward a decision</x:v>
-      </x:c>
-      <x:c r="G10" s="45" t="str">
-        <x:v>• one position keeps revising while the other insists that action cannot wait</x:v>
-      </x:c>
-      <x:c r="H10" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
-      </x:c>
-      <x:c r="I10" s="45" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
-      </x:c>
-      <x:c r="J10" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K10" s="45" t="str"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="45" t="str">
-        <x:v>sky-how/modality/mutable/fixed</x:v>
-      </x:c>
-      <x:c r="B11" s="45" t="str">
-        <x:v>continued adjustment reaches a demand that will not move</x:v>
-      </x:c>
-      <x:c r="C11" s="45" t="str">
-        <x:v>one position adapts repeatedly while the other protects a fixed requirement</x:v>
-      </x:c>
-      <x:c r="D11" s="45" t="str">
-        <x:v>people can move once the flexible side stops revising around an unnamed demand</x:v>
-      </x:c>
-      <x:c r="E11" s="45" t="str">
-        <x:v>• people can move once the flexible side stops revising around an unnamed demand</x:v>
-      </x:c>
-      <x:c r="F11" s="45" t="str">
-        <x:v>• continued adjustment reaches a demand that will not move</x:v>
-      </x:c>
-      <x:c r="G11" s="45" t="str">
-        <x:v>• one position adapts repeatedly while the other protects a fixed requirement</x:v>
-      </x:c>
-      <x:c r="H11" s="45" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
-      </x:c>
-      <x:c r="I11" s="45" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
-      </x:c>
-      <x:c r="J11" s="45" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K11" s="45" t="str"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="46" t="str">
-        <x:v>sky-how/modality/mutable/mutable</x:v>
-      </x:c>
-      <x:c r="B12" s="46" t="str">
-        <x:v>the terms remain open because both positions keep changing with the conditions</x:v>
-      </x:c>
-      <x:c r="C12" s="46" t="str">
-        <x:v>each answer creates another possible version before the last one can be tested</x:v>
-      </x:c>
-      <x:c r="D12" s="46" t="str">
-        <x:v>one workable version has to remain in place long enough to show what it does</x:v>
-      </x:c>
-      <x:c r="E12" s="46" t="str">
-        <x:v>• one workable version has to remain in place long enough to show what it does</x:v>
-      </x:c>
-      <x:c r="F12" s="46" t="str">
-        <x:v>• the terms remain open because both positions keep changing with the conditions</x:v>
-      </x:c>
-      <x:c r="G12" s="46" t="str">
-        <x:v>• each answer creates another possible version before the last one can be tested</x:v>
-      </x:c>
-      <x:c r="H12" s="46" t="str">
-        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
-apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
-      </x:c>
-      <x:c r="I12" s="46" t="str">
-        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
-1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
-      </x:c>
-      <x:c r="J12" s="46" t="str">
-        <x:v>PENDING OWNER</x:v>
-      </x:c>
-      <x:c r="K12" s="46" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="A4:K12">
-    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="PENDING OWNER"/>
-  </x:conditionalFormatting>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="J4:J12">
-      <x:formula1>"PENDING OWNER,APPROVED,REVISE,REJECTED"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3449e3b58884a0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae998a30f52841b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13940,6 +14628,463 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="I1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="J1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+      <x:c r="K1" s="3" t="str">
+        <x:v>Modality units (9)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="I2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="J2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+      <x:c r="K2" s="7" t="str">
+        <x:v>Ordered modality pairs. Each row composes reader effect, conflict behavior, and movement bias.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B3" s="35" t="str">
+        <x:v>Reader effect</x:v>
+      </x:c>
+      <x:c r="C3" s="35" t="str">
+        <x:v>Conflict behavior</x:v>
+      </x:c>
+      <x:c r="D3" s="35" t="str">
+        <x:v>Movement bias</x:v>
+      </x:c>
+      <x:c r="E3" s="35" t="str">
+        <x:v>Supportive realizations</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>Neutral realizations</x:v>
+      </x:c>
+      <x:c r="G3" s="35" t="str">
+        <x:v>Shadow realizations</x:v>
+      </x:c>
+      <x:c r="H3" s="35" t="str">
+        <x:v>Source IDs</x:v>
+      </x:c>
+      <x:c r="I3" s="35" t="str">
+        <x:v>Source hashes</x:v>
+      </x:c>
+      <x:c r="J3" s="35" t="str">
+        <x:v>Owner review status</x:v>
+      </x:c>
+      <x:c r="K3" s="36" t="str">
+        <x:v>Owner notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="44" t="str">
+        <x:v>sky-how/modality/cardinal/cardinal</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
+        <x:v>two attempts to set direction become visible at once</x:v>
+      </x:c>
+      <x:c r="C4" s="44" t="str">
+        <x:v>both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
+      </x:c>
+      <x:c r="D4" s="44" t="str">
+        <x:v>both sides need a shared first step or a clear decision about who leads</x:v>
+      </x:c>
+      <x:c r="E4" s="44" t="str">
+        <x:v>• both sides need a shared first step or a clear decision about who leads</x:v>
+      </x:c>
+      <x:c r="F4" s="44" t="str">
+        <x:v>• two attempts to set direction become visible at once</x:v>
+      </x:c>
+      <x:c r="G4" s="44" t="str">
+        <x:v>• both positions push to lead, so delay quickly becomes a contest over the first move</x:v>
+      </x:c>
+      <x:c r="H4" s="44" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I4" s="44" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J4" s="44" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K4" s="44" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>sky-how/modality/cardinal/fixed</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>an immediate push runs into a limit meant to hold</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>one position keeps initiating while the other protects what cannot be surrendered</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>people need an action that preserves the fixed position's central limit</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>• people need an action that preserves the fixed position's central limit</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>• an immediate push runs into a limit meant to hold</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>• one position keeps initiating while the other protects what cannot be surrendered</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K5" s="45" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="45" t="str">
+        <x:v>sky-how/modality/cardinal/mutable</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>a first move keeps meeting revised terms</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>one position wants a decision while the other adapts as new conditions appear</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="str">
+        <x:v>the first step has to leave room for a defined adjustment</x:v>
+      </x:c>
+      <x:c r="E6" s="45" t="str">
+        <x:v>• the first step has to leave room for a defined adjustment</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="str">
+        <x:v>• a first move keeps meeting revised terms</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="str">
+        <x:v>• one position wants a decision while the other adapts as new conditions appear</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="str">
+        <x:v>c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J6" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K6" s="45" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="45" t="str">
+        <x:v>sky-how/modality/fixed/cardinal</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>a protected position is pressed for immediate action</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>one side holds its ground while the other treats movement as urgent</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="str">
+        <x:v>the proposed action must work inside the limit that is not moving</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="str">
+        <x:v>• the proposed action must work inside the limit that is not moving</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str">
+        <x:v>• a protected position is pressed for immediate action</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>• one side holds its ground while the other treats movement as urgent</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K7" s="45" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="45" t="str">
+        <x:v>sky-how/modality/fixed/fixed</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>the disagreement settles around two positions neither side considers expendable</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="str">
+        <x:v>neither side gives ground easily under pressure</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="str">
+        <x:v>people are more likely to change the terms or structure than to make either side back down</x:v>
+      </x:c>
+      <x:c r="E8" s="45" t="str">
+        <x:v>• people are more likely to change the terms or structure than to make either side back down</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="str">
+        <x:v>• the disagreement settles around two positions neither side considers expendable</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="str">
+        <x:v>• neither side gives ground easily under pressure</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J8" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K8" s="45" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="45" t="str">
+        <x:v>sky-how/modality/fixed/mutable</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>a firm limit keeps meeting a changing response</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>one position holds the line while the other revises around it</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="str">
+        <x:v>people have to name the nonnegotiable point instead of revising around it</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="str">
+        <x:v>• people have to name the nonnegotiable point instead of revising around it</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="str">
+        <x:v>• a firm limit keeps meeting a changing response</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="str">
+        <x:v>• one position holds the line while the other revises around it</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="str">
+        <x:v>c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J9" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K9" s="45" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="45" t="str">
+        <x:v>sky-how/modality/mutable/cardinal</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="str">
+        <x:v>changing conditions are pushed toward a decision</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="str">
+        <x:v>one position keeps revising while the other insists that action cannot wait</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="str">
+        <x:v>a decision can move if it includes a defined point for review</x:v>
+      </x:c>
+      <x:c r="E10" s="45" t="str">
+        <x:v>• a decision can move if it includes a defined point for review</x:v>
+      </x:c>
+      <x:c r="F10" s="45" t="str">
+        <x:v>• changing conditions are pushed toward a decision</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="str">
+        <x:v>• one position keeps revising while the other insists that action cannot wait</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/cardinal</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+c8bb886bf5a7daf1cff047bb46e3b4c95c4ad46e3b7b5a0cb041d7fdeaf77349</x:v>
+      </x:c>
+      <x:c r="J10" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K10" s="45" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="45" t="str">
+        <x:v>sky-how/modality/mutable/fixed</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>continued adjustment reaches a demand that will not move</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>one position adapts repeatedly while the other protects a fixed requirement</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="str">
+        <x:v>people can move once the flexible side stops revising around an unnamed demand</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="str">
+        <x:v>• people can move once the flexible side stops revising around an unnamed demand</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="str">
+        <x:v>• continued adjustment reaches a demand that will not move</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="str">
+        <x:v>• one position adapts repeatedly while the other protects a fixed requirement</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/fixed</x:v>
+      </x:c>
+      <x:c r="I11" s="45" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+c1af5c2de3d3f5860119897ad43903f3b0214beeab6d10548a14663ec22de3ae</x:v>
+      </x:c>
+      <x:c r="J11" s="45" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K11" s="45" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="46" t="str">
+        <x:v>sky-how/modality/mutable/mutable</x:v>
+      </x:c>
+      <x:c r="B12" s="46" t="str">
+        <x:v>the terms remain open because both positions keep changing with the conditions</x:v>
+      </x:c>
+      <x:c r="C12" s="46" t="str">
+        <x:v>each answer creates another possible version before the last one can be tested</x:v>
+      </x:c>
+      <x:c r="D12" s="46" t="str">
+        <x:v>one workable version has to remain in place long enough to show what it does</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="str">
+        <x:v>• one workable version has to remain in place long enough to show what it does</x:v>
+      </x:c>
+      <x:c r="F12" s="46" t="str">
+        <x:v>• the terms remain open because both positions keep changing with the conditions</x:v>
+      </x:c>
+      <x:c r="G12" s="46" t="str">
+        <x:v>• each answer creates another possible version before the last one can be tested</x:v>
+      </x:c>
+      <x:c r="H12" s="46" t="str">
+        <x:v>apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable
+apps/web/src/content/fallbackArchitectureV3/source-rows/fallback-source-rows-v3.json#fallback-vocab/pattern-mode/mutable</x:v>
+      </x:c>
+      <x:c r="I12" s="46" t="str">
+        <x:v>1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41
+1d50f30d05d27a1dddaa3d0303836016780e89fa39b0749b6b4ee29dd3f37b41</x:v>
+      </x:c>
+      <x:c r="J12" s="46" t="str">
+        <x:v>PENDING OWNER</x:v>
+      </x:c>
+      <x:c r="K12" s="46" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="A4:K12">
+    <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="PENDING OWNER"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="J4:J12">
+      <x:formula1>"PENDING OWNER,APPROVED,REVISE,REJECTED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e245fc9dc3845d3"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="3" t="str">
         <x:v>Element units (16)</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
@@ -14577,7 +15722,7 @@
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:K19">
-    <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="PENDING OWNER"/>
+    <x:cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="PENDING OWNER"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="J4:J19">
@@ -14586,348 +15731,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc450aae407cb4620"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29ae295f65994f12"/>
   </x:tableParts>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Frame uniqueness gate</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Frame uniqueness gate</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
-        <x:v>Frame uniqueness gate</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>Frame uniqueness gate</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>Frame uniqueness gate</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>Frame uniqueness gate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="str">
-        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
-      </x:c>
-      <x:c r="D2" s="7" t="str">
-        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
-      </x:c>
-      <x:c r="E2" s="7" t="str">
-        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
-      </x:c>
-      <x:c r="F2" s="7" t="str">
-        <x:v>Beats are hidden logic, not sentence positions. Forecast concludes; Details explains and stops. The composer must vary openers, closers, entry modes, and connective constructions.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="18" t="str">
-        <x:v>Rule</x:v>
-      </x:c>
-      <x:c r="B4" s="18" t="str">
-        <x:v>Scope</x:v>
-      </x:c>
-      <x:c r="C4" s="18" t="str">
-        <x:v>Cap</x:v>
-      </x:c>
-      <x:c r="D4" s="18" t="str">
-        <x:v>Pass example</x:v>
-      </x:c>
-      <x:c r="E4" s="18" t="str">
-        <x:v>Fail example</x:v>
-      </x:c>
-      <x:c r="F4" s="18" t="str">
-        <x:v>Reason</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="25" t="str">
-        <x:v>Exact sentence uniqueness</x:v>
-      </x:c>
-      <x:c r="B5" s="25" t="str">
-        <x:v>Forecast + Details</x:v>
-      </x:c>
-      <x:c r="C5" s="25" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D5" s="25" t="str">
-        <x:v>Every sentence appears once</x:v>
-      </x:c>
-      <x:c r="E5" s="25" t="str">
-        <x:v>Same full sentence in two cards</x:v>
-      </x:c>
-      <x:c r="F5" s="25" t="str">
-        <x:v>Prevents copied frames</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="26" t="str">
-        <x:v>Forecast opener construction</x:v>
-      </x:c>
-      <x:c r="B6" s="26" t="str">
-        <x:v>Forecast first sentence</x:v>
-      </x:c>
-      <x:c r="C6" s="26" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D6" s="26" t="str">
-        <x:v>Four or fewer uses</x:v>
-      </x:c>
-      <x:c r="E6" s="26" t="str">
-        <x:v>Five cards begin with the same normalized opening</x:v>
-      </x:c>
-      <x:c r="F6" s="26" t="str">
-        <x:v>Prevents opener monoculture</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="26" t="str">
-        <x:v>Details opener construction</x:v>
-      </x:c>
-      <x:c r="B7" s="26" t="str">
-        <x:v>Details first composed sentence</x:v>
-      </x:c>
-      <x:c r="C7" s="26" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D7" s="26" t="str">
-        <x:v>Four or fewer uses</x:v>
-      </x:c>
-      <x:c r="E7" s="26" t="str">
-        <x:v>Five cards begin with the same normalized opening</x:v>
-      </x:c>
-      <x:c r="F7" s="26" t="str">
-        <x:v>Details must also compose both positions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="26" t="str">
-        <x:v>Connective construction</x:v>
-      </x:c>
-      <x:c r="B8" s="26" t="str">
-        <x:v>Later sentences</x:v>
-      </x:c>
-      <x:c r="C8" s="26" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D8" s="26" t="str">
-        <x:v>Four or fewer uses of one opening phrase</x:v>
-      </x:c>
-      <x:c r="E8" s="26" t="str">
-        <x:v>Repeated 'That can turn...' across five cards</x:v>
-      </x:c>
-      <x:c r="F8" s="26" t="str">
-        <x:v>Beats do not require fixed connective wording</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="26" t="str">
-        <x:v>Required forecast beats</x:v>
-      </x:c>
-      <x:c r="B9" s="26" t="str">
-        <x:v>Each forecast</x:v>
-      </x:c>
-      <x:c r="C9" s="26" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="str">
-        <x:v>All four meanings present</x:v>
-      </x:c>
-      <x:c r="E9" s="26" t="str">
-        <x:v>A moral replaces what can move</x:v>
-      </x:c>
-      <x:c r="F9" s="26" t="str">
-        <x:v>Meaning is required even when wording varies</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="26" t="str">
-        <x:v>Required Details beats</x:v>
-      </x:c>
-      <x:c r="B10" s="26" t="str">
-        <x:v>Each Details block</x:v>
-      </x:c>
-      <x:c r="C10" s="26" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D10" s="26" t="str">
-        <x:v>Explanation ends after behavior</x:v>
-      </x:c>
-      <x:c r="E10" s="26" t="str">
-        <x:v>Forecast conclusion repeated in Details</x:v>
-      </x:c>
-      <x:c r="F10" s="26" t="str">
-        <x:v>Forecast concludes; Details explains</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="26" t="str">
-        <x:v>Verbatim component emission</x:v>
-      </x:c>
-      <x:c r="B11" s="26" t="str">
-        <x:v>All components</x:v>
-      </x:c>
-      <x:c r="C11" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D11" s="26" t="str">
-        <x:v>Composer paraphrases and integrates</x:v>
-      </x:c>
-      <x:c r="E11" s="26" t="str">
-        <x:v>A stored component appears as a full sentence</x:v>
-      </x:c>
-      <x:c r="F11" s="26" t="str">
-        <x:v>Components govern meaning, not prose</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="26" t="str">
-        <x:v>Manifestation shape reuse</x:v>
-      </x:c>
-      <x:c r="B12" s="26" t="str">
-        <x:v>Sign-unit manifestations</x:v>
-      </x:c>
-      <x:c r="C12" s="26" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D12" s="26" t="str">
-        <x:v>Planet-sign events use distinct grammar</x:v>
-      </x:c>
-      <x:c r="E12" s="26" t="str">
-        <x:v>A sign frame survives after planet nouns are stripped</x:v>
-      </x:c>
-      <x:c r="F12" s="26" t="str">
-        <x:v>String uniqueness alone does not catch slot templates</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="26" t="str">
-        <x:v>Plain-register subject</x:v>
-      </x:c>
-      <x:c r="B13" s="26" t="str">
-        <x:v>Meaning components</x:v>
-      </x:c>
-      <x:c r="C13" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D13" s="26" t="str">
-        <x:v>People, deadlines, messages, rules, and other everyday actors lead</x:v>
-      </x:c>
-      <x:c r="E13" s="26" t="str">
-        <x:v>Recognition, autonomy, or pressure narrates itself</x:v>
-      </x:c>
-      <x:c r="F13" s="26" t="str">
-        <x:v>The owner's register uses active verbs and concrete nouns</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="26" t="str">
-        <x:v>Manifestation actor or act</x:v>
-      </x:c>
-      <x:c r="B14" s="26" t="str">
-        <x:v>All sign manifestations</x:v>
-      </x:c>
-      <x:c r="C14" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D14" s="26" t="str">
-        <x:v>A person acts or a concrete act is visible</x:v>
-      </x:c>
-      <x:c r="E14" s="26" t="str">
-        <x:v>Care turns into leverage</x:v>
-      </x:c>
-      <x:c r="F14" s="26" t="str">
-        <x:v>An abstraction may not perform the behavior</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="26" t="str">
-        <x:v>Source shadow coverage</x:v>
-      </x:c>
-      <x:c r="B15" s="26" t="str">
-        <x:v>All sign units</x:v>
-      </x:c>
-      <x:c r="C15" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D15" s="26" t="str">
-        <x:v>A supported cost or overreach remains available</x:v>
-      </x:c>
-      <x:c r="E15" s="26" t="str">
-        <x:v>Jupiter becomes uniformly beneficial</x:v>
-      </x:c>
-      <x:c r="F15" s="26" t="str">
-        <x:v>The component may not erase source challenge, shadow, or cost</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="26" t="str">
-        <x:v>Typed realization pools</x:v>
-      </x:c>
-      <x:c r="B16" s="26" t="str">
-        <x:v>All 174 units</x:v>
-      </x:c>
-      <x:c r="C16" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D16" s="26" t="str">
-        <x:v>Supportive, neutral, and shadow meanings live in named arrays</x:v>
-      </x:c>
-      <x:c r="E16" s="26" t="str">
-        <x:v>Useful/neutral/shadow is encoded as bullet position</x:v>
-      </x:c>
-      <x:c r="F16" s="26" t="str">
-        <x:v>The composer chooses meaning type; it never learns a three-item rhythm</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="27" t="str">
-        <x:v>Owner-source conversion</x:v>
-      </x:c>
-      <x:c r="B17" s="27" t="str">
-        <x:v>All owner-voice evidence</x:v>
-      </x:c>
-      <x:c r="C17" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D17" s="27" t="str">
-        <x:v>Personal source meaning is converted for collective Sky</x:v>
-      </x:c>
-      <x:c r="E17" s="27" t="str">
-        <x:v>Eight or more source words are copied verbatim</x:v>
-      </x:c>
-      <x:c r="F17" s="27" t="str">
-        <x:v>Owner voice governs without leaking second-person source prose</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A2:F2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(content): regenerate Calendar component evidence artifacts
</commit_message>
<xml_diff>
--- a/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
+++ b/outputs/sky-calendar-meaning-components-2026-08-14/sky-calendar-meaning-components-owner-review.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc6d7d3102cf745cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Record" sheetId="2" r:id="R8a60fb471d15439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="3" r:id="Rc5ee7b733f4a446c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="4" r:id="R3a1b374946e14a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Audit" sheetId="5" r:id="Re99bb7ce7c734f27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeted Verification" sheetId="6" r:id="R9176cd38e2d9451f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Closing" sheetId="7" r:id="R9614a99880894a4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="8" r:id="Rb6fb758c54314003"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="9" r:id="Re3440f18098444f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="10" r:id="Rede169688acf412a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="11" r:id="R26455853c2584994"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="12" r:id="R6c04b9a6c5ef4842"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0f8a09d066904666"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Record" sheetId="2" r:id="Rcb4f1f1d86714bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Voice Coverage" sheetId="3" r:id="R7eb15f64d479441a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign Units" sheetId="4" r:id="Rfa807c5ea27d4138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Audit" sheetId="5" r:id="R01f1d1a58a2c4c45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeted Verification" sheetId="6" r:id="Rae644e65dce44052"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Closing" sheetId="7" r:id="R3d73d49e758e4cd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aspect Mechanisms" sheetId="8" r:id="Rbf0be778f96144fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality Units" sheetId="9" r:id="Rcad560194a534b98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Element Units" sheetId="10" r:id="Rfc67c2764c04461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Gate" sheetId="11" r:id="Rb8bfb7bed9444574"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wording QA" sheetId="12" r:id="Rf106ca70d8b44039"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1823,7 +1823,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R107a458320cb4e1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85d578f2327145ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2263,7 +2263,7 @@
         <x:v>Evidence-layer SHA-256</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>0ceb85f5897fb42238dfdd69e7b02271f87befe202f009da8659add9b9337c23</x:v>
+        <x:v>4072572c3ba27afda4bdd27bddc70d892f53bd861bec9f4e52971ff279de8cd2</x:v>
       </x:c>
       <x:c r="C5" s="14" t="str">
         <x:v>locked</x:v>
@@ -6027,7 +6027,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e8c53504c4f467d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf676209a96f24417"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6582,7 +6582,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!770</x:v>
       </x:c>
       <x:c r="K4" s="47" t="str">
-        <x:v>b6232d9ff6b4bbf7745f7b2dcb6cb699eb804f90bbd24ae1a73f9a1d87ae0ebb
+        <x:v>72d5c14d8211a2ca2070f49f8b92516a9c1000fb66fa75c95a6125144955a028
 c60d047e15b9838a147ce7c505a86de4c94490b3365ae42e2f0bc5c12e6e2724</x:v>
       </x:c>
       <x:c r="L4" s="47" t="str">
@@ -6628,7 +6628,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!782</x:v>
       </x:c>
       <x:c r="K5" s="48" t="str">
-        <x:v>553a41030a43bdfdc8224a6f9e5bf830cf5b469939ba56fb10373861eb525748
+        <x:v>994355ada37f9004dc6d76eeaf7977bf97d84606f3031d2ffe3ecb48a4f51e7b
 b3e7ea4414f2a38f9a858223ebc978f2111167fd9f52b3cab9aa14397104fb0c</x:v>
       </x:c>
       <x:c r="L5" s="48" t="str">
@@ -6675,7 +6675,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!792</x:v>
       </x:c>
       <x:c r="K6" s="48" t="str">
-        <x:v>068670bda0c06889be61a6bb00ebeab5b0d5324f7b6c306bc410f990cc1e99af
+        <x:v>e5198d60bf28e1fba2dc33ac6bd11e860ee8836107d442dca360607b9a91bd26
 4f6ff1b1398f8366db74be688c6fa5370a54505eff49824ab86f451ecbd0ede2</x:v>
       </x:c>
       <x:c r="L6" s="48" t="str">
@@ -6822,7 +6822,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!822</x:v>
       </x:c>
       <x:c r="K9" s="48" t="str">
-        <x:v>a0792cdd2170c55212c6b071c49f8c19e9d02cd07675da471a6962567c4c5896
+        <x:v>d3c01ba605171012f790040a6cc663cc495ab1b5d16d95a76dfdd562e97d18cb
 6c441c45502b3eeebed5a6cda170d74281ce1c13ab7a8f4b5eb22d219a9aa5eb</x:v>
       </x:c>
       <x:c r="L9" s="48" t="str">
@@ -6869,7 +6869,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!830</x:v>
       </x:c>
       <x:c r="K10" s="48" t="str">
-        <x:v>9ddd5ab097f70084442c50cdb5f5099e990fccd53b45ce8acde980b95f249f90
+        <x:v>316e12c40ae2ab2081998a56be8f5ab502d84d3e302b01e5422cd2d5130210c0
 0e4c8c7929b3d06445e7042c5315a83e3a96d787f9d38546a1f4e1226e351ecd</x:v>
       </x:c>
       <x:c r="L10" s="48" t="str">
@@ -6921,7 +6921,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!838</x:v>
       </x:c>
       <x:c r="K11" s="48" t="str">
-        <x:v>b7f49ad5fec325bbe9b9a99a3883baaea32470f203979d8f69f56c8ceebb3e31
+        <x:v>81ae06f78c3562d9b6c029824c0301136aee280d389b034b88947997893dcdd9
 e58c141239bac2092c59cafde00a9758984ca8b477f2fb194c49e8e77ff3ffb3</x:v>
       </x:c>
       <x:c r="L11" s="48" t="str">
@@ -6973,7 +6973,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!845</x:v>
       </x:c>
       <x:c r="K12" s="48" t="str">
-        <x:v>ed83780b31908b7f8f73c92696bcf917542995f87449837b8a9b8ac82927b94b
+        <x:v>d75139cbc5eb4eaebc18c01626b2cb4a0c9a3b3cb6df9dfa2cbde6487b4d75d7
 9ab87f2efd1446de205628bb1124cc57309ec35d3937972afc1cc95655c1f3bc</x:v>
       </x:c>
       <x:c r="L12" s="48" t="str">
@@ -7020,7 +7020,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!852</x:v>
       </x:c>
       <x:c r="K13" s="48" t="str">
-        <x:v>2b7dcf125f2aed466ec0c2688edfc7a27b149e8ca31e3a3a71bd7299b08b74c9
+        <x:v>7f037fef1d72d96bebb1fc7ca60e348b308dbb91ea3586e710102bfd80d463f8
 19070167ec0dbb73cbdf52d47a0903992d464bfb93f4c8cc12f1c243aeb1bd8a</x:v>
       </x:c>
       <x:c r="L13" s="48" t="str">
@@ -7068,7 +7068,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!863</x:v>
       </x:c>
       <x:c r="K14" s="48" t="str">
-        <x:v>5edc0968f3ec70c427bb81a71a0783cae06e06f94e89eb88fd1b0af6153e29fe
+        <x:v>323093a171da7ba042f3ed46fa05813fd0af894a7bdd4eccd047fa22d7aad4b0
 52191403a1fa0ec5a4201498cddfffc7e59eae479ed265e25563c268a81fcc51</x:v>
       </x:c>
       <x:c r="L14" s="48" t="str">
@@ -7115,7 +7115,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!872</x:v>
       </x:c>
       <x:c r="K15" s="48" t="str">
-        <x:v>d0456b2d1906bfb3aca99ceb69f599a9382e2496d4c2802ca4be0c1a2201c16e
+        <x:v>a5af76ed9bc23a46e927282ae13ba60b05a9ce6a670add8a663acf9dbee6ab09
 5b692620db4bebd4b3973d1e3b111603af3f994deccc48d8e3287c932d546ab5</x:v>
       </x:c>
       <x:c r="L15" s="48" t="str">
@@ -7818,7 +7818,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!84</x:v>
       </x:c>
       <x:c r="K28" s="48" t="str">
-        <x:v>289a7cc6aa3899bf42c5df7bd43ea005e04111d5a6d455b9f0131c9af8fcd063
+        <x:v>e80eb19f823a69cb81735a7a9559024cdaa7746a523d20a0a178c65a60d3db34
 0ab8c1ff29ab1bc9658e67fd43c08ca864ff6dd2ef0bcf1dc070557091127af2
 50c5676f41167ea227c5ba13c29caebde9f3cfcf23ca7a482d9c1a4ad78858b3</x:v>
       </x:c>
@@ -7920,7 +7920,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!86</x:v>
       </x:c>
       <x:c r="K30" s="48" t="str">
-        <x:v>489bc7bd576cec0d98ac8f7e8d2b41a5d8ddb8489e2786be6eb5bf99ec4a9fbd
+        <x:v>eb16de0a1a53fb59a8bbfd75e6b00c6ac59084a39c3bc21bd5adf5b17d518e78
 2b78f98753e33c107bf6cac264cd8ecc994e12c661ddb8bafdbbbf907957edcc
 d188f1325ee54c49afbf5b184d3e1963252d64d22e1b021ff57754371f0c537c</x:v>
       </x:c>
@@ -8024,7 +8024,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!88</x:v>
       </x:c>
       <x:c r="K32" s="48" t="str">
-        <x:v>937e23a8c9ba648e1a9290e8ebaa235edd40917c6bc9b82aa6a792eeaf571cb6
+        <x:v>e187255ab7f1e2f5cb95a840c1cda714cdd7bcdbeef19c80e66ebbb644cddb50
 67004c39cec49a0595b6663d0b4578c9d3091665e98936da5e3c4350e198ebdb
 e1eabcbd2a676fc92b22f0727b2be8da6522f5bcb1988664bb2e21ce3685d668</x:v>
       </x:c>
@@ -8076,7 +8076,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!356</x:v>
       </x:c>
       <x:c r="K33" s="48" t="str">
-        <x:v>0cd51c8d151814d45abe7468de574441b8a26b71a78e893a4ee268cc7c838c14
+        <x:v>b73cef931ded7416f3bc1c48c68b271beda59c0263c0ef9625a68a73bec11db7
 3a2e89fb2229ce8c2d5a335b77842ed183cab3e9aa8700788cf2946496746532</x:v>
       </x:c>
       <x:c r="L33" s="48" t="str">
@@ -8126,7 +8126,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!378</x:v>
       </x:c>
       <x:c r="K34" s="48" t="str">
-        <x:v>d4b219c684feb9d19dc5b96eade0cc1c24a965af991d687cddc1650c8ab32bf7
+        <x:v>c29b2d83961d743f81447ea0bf41989ef179bec607baba7f48318ce693f2f723
 04269dbd62799d5409048836a61a9f73064941204e048aa5f7e890267b7e74e2</x:v>
       </x:c>
       <x:c r="L34" s="48" t="str">
@@ -8180,7 +8180,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!392</x:v>
       </x:c>
       <x:c r="K35" s="48" t="str">
-        <x:v>e94711013efedf38abfdf67cf233133fb1e14be23fdb5dd87e5776e27ae43119
+        <x:v>df9c0c2814a7e924ec344937e5e32a8f14ed4b2166f8f41e5d929a84fe75c87d
 379a1b9b2940ae97fb0fc26750e590d9c11e000a5717690ba726b32757af5416</x:v>
       </x:c>
       <x:c r="L35" s="48" t="str">
@@ -8391,7 +8391,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!95</x:v>
       </x:c>
       <x:c r="K39" s="48" t="str">
-        <x:v>916bb88d5657c0e00252a6bebbfa64a7f3bb14847a9e68dbb409ac19b463b13f
+        <x:v>ec66175968dd9709ee5cc8fdd47936a6c28634f3037fbb61b4449ebdec12d372
 28addf7e51a760c9506814d3da705c669326f3aae025a529f5156c152c52a3ee
 9350e839fe167dc84002c28847495d2c0f29ed14f588f8bc666560cecaed54ed</x:v>
       </x:c>
@@ -8443,7 +8443,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!963</x:v>
       </x:c>
       <x:c r="K40" s="48" t="str">
-        <x:v>2ce4fbb0f2e46fd671ab4b5fb41213943f420ef83c5669995a7e6fb30bddbec1
+        <x:v>db38a311aa838353fc52a6aeb5bdf54063eb0e2f1432c13bba331291de184862
 fbcdef2e2fc920ac0125b9daec59c68963ec32c764a9ea77c3a3ffd1a8bdc423</x:v>
       </x:c>
       <x:c r="L40" s="48" t="str">
@@ -8612,7 +8612,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!1006</x:v>
       </x:c>
       <x:c r="K43" s="48" t="str">
-        <x:v>598d6a053da1ee284db883d882b68103cd67a4b32d278b192bec1e16d430b3ea
+        <x:v>198544e12f0b5b4f5415e9733d583f343e211121de8c0fc3ee3c1fd7aa13a015
 79e029e05fef406e802fda91cf0ebbb6b0477538034a095cc64d0f5639d33026</x:v>
       </x:c>
       <x:c r="L43" s="48" t="str">
@@ -8663,7 +8663,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!64</x:v>
       </x:c>
       <x:c r="K44" s="48" t="str">
-        <x:v>a489df6bc53303970522c4b87ed5a5f8ee7040f67460c4a9d10020e07b166cc5
+        <x:v>13fbf54f774e71f88c3d6154be010c08f4844ca3a4e5bc2fbddddb3f67e1e0ab
 24bbe05a3593f9aebb7c7466bf9cec88d34094be8687b24c4119f63958ffb72f
 174fc05f9e43115ec7942c5a3388998483fcec1e0682e9e5a55f9f66a3389ba4</x:v>
       </x:c>
@@ -8880,7 +8880,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!68</x:v>
       </x:c>
       <x:c r="K48" s="48" t="str">
-        <x:v>cef7130a73e47e34fafaa3ad09e2b45cf6002bf2e1894da977693bab197255c6
+        <x:v>67ca60040e138c12c71a1f10166908b989c1c3206c818e4711127dad31f4cb33
 4a6d1bb3a44c756ddd5a8ea6526f23b9c433e8516dcd9710f7e1a78daa5e76d1
 8536df484d62507cd74941fb64d98a411d15c0878e56e1d3db660a9656426bae</x:v>
       </x:c>
@@ -8938,7 +8938,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!69</x:v>
       </x:c>
       <x:c r="K49" s="48" t="str">
-        <x:v>01dc72b3919b47bf93452f88dfa77ac86532745a5a85aac3bc1e44b888122e65
+        <x:v>9c82ffc87a83714229f1190d8f7d03e325ae3f129c306e92c4dda0ed0d75fc29
 4f89ed4ae84bb1152ca8958fa119e9d6d44cf597aea024909589240bd5480ffd
 8b125bf88f1aee6436760a54e01cd7005a62722d39fa6bb71a50c7715c57f107</x:v>
       </x:c>
@@ -8995,7 +8995,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!1083</x:v>
       </x:c>
       <x:c r="K50" s="48" t="str">
-        <x:v>cb1c7e3fd7b93583d6051822f082ba1babfe845d6aac761de0ab20eed276560a
+        <x:v>dd11f1b7f6f88f2affc279e870df078411bf2a5636f2544e74a7fa7f72aa14fd
 466bd6a866c2bc637a5b7239c315a8e57b480fd210552c20ea26dc78899941c3</x:v>
       </x:c>
       <x:c r="L50" s="48" t="str">
@@ -9049,7 +9049,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!1093</x:v>
       </x:c>
       <x:c r="K51" s="48" t="str">
-        <x:v>968c0e379bb064511c55a75b600c611031e6102809e504b263ba67e7cd10280d
+        <x:v>3f07dd5b18f4c59c02fe116fbbafb089f5c01aef206e0e34a805aeb3b0de38a4
 015929baf8822626da459cf3d1f3ae4ce64c685829f5d0149220131eb0c834ec</x:v>
       </x:c>
       <x:c r="L51" s="48" t="str">
@@ -9100,7 +9100,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!36</x:v>
       </x:c>
       <x:c r="K52" s="48" t="str">
-        <x:v>0ea369b65869f5b4f1ecb4750bac3e3ead379873da9720ae9c9fbd0b54418b5c
+        <x:v>49c049221e0d3b7a8e1fd36ba83888f424c24438b6cf66908d7041b228c24d83
 4997e05239b7bd200d99db9cc421ace94178b091988877da512f1e4f79b92e3d
 3ca4a4e07b787aa13e54168fda88000c6e63e18d04732c1226ba27f5f88af089</x:v>
       </x:c>
@@ -9158,7 +9158,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!37</x:v>
       </x:c>
       <x:c r="K53" s="48" t="str">
-        <x:v>ca33eb1746e7401defcc681220c5d0ef60755a1aed7365133ed1e7b40d7af68f
+        <x:v>bf97a72f7ed674efb35e0b0beafd2124a2b5c99f60ad0ba53d103988bbd92c8a
 ebbcbf7973f49ab721216ad240dad6d6d7f7d91952eacbdefd7209dea61a1a53
 eeae0d838c1ad19bfbc96d004795b6662cd50802af29f83072e4e90d10f7243b</x:v>
       </x:c>
@@ -9211,7 +9211,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!38</x:v>
       </x:c>
       <x:c r="K54" s="48" t="str">
-        <x:v>7cd7318205ce886660fdb11df01ffc66d92e3c2700c9a8548e485709afbbb077
+        <x:v>976b1d7c665a0eadd4694962720fb18374892c0bcb7efa2dadf50912dc212e01
 9eb24ef8b9e20ce56ae146bb8f056b2ac60def6c21d417fe3907c15aab20f322
 f0e89aa57c294d30065c6839b325ef4e37c1085868641c662503ce286f02a04b</x:v>
       </x:c>
@@ -9268,7 +9268,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!39</x:v>
       </x:c>
       <x:c r="K55" s="48" t="str">
-        <x:v>1aecaf23c0e38b83a9c55a6dd853900e92a669adfb1bac71ec5ba832ed0039c0
+        <x:v>7a5f11d98f8a05bd9aad89e1684ce28e39e2c8243c50e0cb3b2bd8794b66d99b
 af3858af454d9e5b5dcc6c54bf51f2791304f3c6f8a929023d7662fb9c16190e
 f9b8c94f27cf0bfdc575ea9a697b69285b3a2f6f7d842b88498d310bc854b25b</x:v>
       </x:c>
@@ -9380,7 +9380,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!41</x:v>
       </x:c>
       <x:c r="K57" s="48" t="str">
-        <x:v>f2fa7ac04c56ee24926cec000efbd4ebb374a8a42ebfa7b1a374ae289771293c
+        <x:v>455514125624dd41bda4237ebeb94b4699e7993ea96cad89482062d6c951f109
 b40ceca33a7a95ab4d4ac8065754fb60c790f61d0e9dde2bdcc4a4692aff138e
 450012d516db7ab086fe6777e27a2745c446b4eb86ca6fe8e090fbfa6bd1ed67</x:v>
       </x:c>
@@ -9438,7 +9438,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!42</x:v>
       </x:c>
       <x:c r="K58" s="48" t="str">
-        <x:v>9ff19d3cb104e5c919c7b64b523226c47d448ca7d97604feb371315f5ad0f06a
+        <x:v>414c655399a8aacccb8b9a0554093c2d941db203722b0c1d0bfcdba7e9b3812a
 c2b34fb98325e393268f9486ab423fccf5eb13678495cd9b3730eaa87e219233
 492b1f314d8a6df9b534e659ea4f3313edc71b437c6d1d7dd7d054ddb5576768</x:v>
       </x:c>
@@ -9495,7 +9495,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!194</x:v>
       </x:c>
       <x:c r="K59" s="48" t="str">
-        <x:v>e8bd257b9897adc676da748e3179db1bfced535618eece35baa96171abab7a2c
+        <x:v>9c400e385be8c586752b358f0164a98be7374f2839decacef9ff28212ffb5338
 cee20b568b72a43b2df40e3a0dfe84b6e42c81c96912d5010a5a5947c0029fab</x:v>
       </x:c>
       <x:c r="L59" s="48" t="str">
@@ -9551,7 +9551,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!203</x:v>
       </x:c>
       <x:c r="K60" s="48" t="str">
-        <x:v>c8312d3d1902a2d5ef1c47ca009062e20609672393a35b20b2d5ab72cfe7c3ba
+        <x:v>780cf7541ee4f622cd0c7095a5f1dbb4ff235dac7b830d489585fba009fe2230
 c51a9dab166de602ddf124b7a1f08aadc4f0639534c467e83e2d185ff101f9a0</x:v>
       </x:c>
       <x:c r="L60" s="48" t="str">
@@ -9604,7 +9604,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!45</x:v>
       </x:c>
       <x:c r="K61" s="48" t="str">
-        <x:v>11ba43a16e43e3c7922b93f753e14d9b0ad95d9e7f6b78e1ecddb3f0f16ae25e
+        <x:v>2696d17cb7fa13c59e7d163e01b63f66d67f415cf82c2058c605c23b48349b38
 8918ed2d4cbebd12f931e80ef6caada70a3e904436de36add9bd1a1d7db27536
 0f67b52d7020e236bac6cd2387e66d3c476dc0d4eeb3c3b963f68dadabe13e17</x:v>
       </x:c>
@@ -9661,7 +9661,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!223</x:v>
       </x:c>
       <x:c r="K62" s="48" t="str">
-        <x:v>5d559edeb0e33e0c586d8f504071982d1210824e456dc4b19075951b5bfaa177
+        <x:v>5a9c3c1284994788a81097b62d7d7209c6bf99da2a96a3ee3ee253f6cc7a88e4
 5f8ce9b7212e3b7cc14497b412a8162cbea650eba30c66985269448c79b0e229</x:v>
       </x:c>
       <x:c r="L62" s="48" t="str">
@@ -9718,7 +9718,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!47</x:v>
       </x:c>
       <x:c r="K63" s="48" t="str">
-        <x:v>e19f246c7f7b55e783872832ce679ee8b10407c35c73286bb3d284c139ae3fa3
+        <x:v>0589af9cee928ad361657b2bf33be24803c821fe1338b39f179fc4a95a88eb80
 bf69e5dd76e542280955500ef6a7dc370745ec7d867e90b811213ae02d08fb1c
 ce39b9484f05ee4b4de00ed7f559d9ec63c9799e6d15afed33154562b15b086e</x:v>
       </x:c>
@@ -9776,7 +9776,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!168</x:v>
       </x:c>
       <x:c r="K64" s="48" t="str">
-        <x:v>e1633e4fdc4773ddac329b619dd0e30f9a377d622a910796806136d678691032
+        <x:v>78c0943e9e028d2dbf4ef1d1bd09197bcccc8c3a83fb1fc901a5f8a0c213bfee
 31d7a4e11a2d261067bfc2441a9c6cc18d34661a91b1b54a3fe42cefe8314106
 e4f01e9514f9a57aed31a2fa97438e6aa6577e788da968121d2255064f671d06</x:v>
       </x:c>
@@ -9828,7 +9828,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!40</x:v>
       </x:c>
       <x:c r="K65" s="48" t="str">
-        <x:v>84eafbdcc3030e3f9f65f32a004510030346010f35dee5929a6a65323a310546
+        <x:v>07fcd85de9cdd483e9ad88aefe291f2b3657bb61b9ab261dd8cbb3d31be6ad3f
 2086de4eafed38fe396fdba2c4528e11061c495a7f711d96702ddad0d688dd65</x:v>
       </x:c>
       <x:c r="L65" s="48" t="str">
@@ -9881,7 +9881,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!170</x:v>
       </x:c>
       <x:c r="K66" s="48" t="str">
-        <x:v>17ad430f69d29d0ea3076f92d4e6b292f46c171353aea077dd58061bde73ee08
+        <x:v>6bf29641dd5ae58188a3729026780657f992245b061f526c5e4fc0f7e1ea694f
 ae1b8f04a0c6ab5eec68950935fa7da7a57c03000b03684c3c70dced1e33e330
 556f6465359353f692e1956a21329f2ea02a676cd1730f5ac0b11f9c46545c13</x:v>
       </x:c>
@@ -9933,7 +9933,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!58</x:v>
       </x:c>
       <x:c r="K67" s="48" t="str">
-        <x:v>4c0d47dc264d9269eaafcbf499d65d260f3040fcdf40be8981fa49ba1403a350
+        <x:v>f88609671b88e1d307fa2bec38502613b87adea2e895cb0112d5440b863437f6
 2e51b1ae2e9b898dac43d1971924f829c26bf17756805ca1b9b4c912d1cee2ee</x:v>
       </x:c>
       <x:c r="L67" s="48" t="str">
@@ -9985,7 +9985,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!68</x:v>
       </x:c>
       <x:c r="K68" s="48" t="str">
-        <x:v>2cc652baf7a93f906bf412496eeac4322fb1186bb7170378829cd7672794619f
+        <x:v>c7a721bd8714bae49ff994e7274bbc9394db763b09e7333eb3d2dd26ba2b5d53
 131842b5f88b8185e1a39ed479cf8e2dcec813aa384b28a98d2e52ad168c575f</x:v>
       </x:c>
       <x:c r="L68" s="48" t="str">
@@ -10036,7 +10036,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!74</x:v>
       </x:c>
       <x:c r="K69" s="48" t="str">
-        <x:v>c8c19ee447751865afa8421698f4a83d834acb363594c5da7e658efdfaf10865
+        <x:v>5fc448d807ea1a063e3738d5e5f4ba7baa9f155d919088f5edbf3b34897726be
 95686ec3c9fbb4e36392c04053039a68653116b41bbf5cd537cf431e76eb05cb</x:v>
       </x:c>
       <x:c r="L69" s="48" t="str">
@@ -10088,7 +10088,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!174</x:v>
       </x:c>
       <x:c r="K70" s="48" t="str">
-        <x:v>02af03797b130c48a565d0a4c048b0aedadda86b6b8838d21822cc08c9f3ff2e
+        <x:v>7fece516324cab686ccc5e85f7c36b40d399367023ec56575b4fe6c1a8e58534
 8d01bdbc30560a74f47b8ef60785711f011041cd9c393eb3b31e1892405d09fc
 7fef144a23fe2414ead57274a100c2ee44c18d2cdd76ed6d6a7e1c41d21ffa46</x:v>
       </x:c>
@@ -10145,7 +10145,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!89</x:v>
       </x:c>
       <x:c r="K71" s="48" t="str">
-        <x:v>5b6b1b28279631383476d50da072bd1b7e9aa6a136d2eb34f2599ba5c1dceb07
+        <x:v>a84f0a4fd85391bdc6bc5c85d914c674236d54c72a8baf129173b37d5d6169b7
 4f25fcfbf9248a585d7b669cb800935266a6eaabc0120128ad34bf78efb3c72a</x:v>
       </x:c>
       <x:c r="L71" s="48" t="str">
@@ -10196,7 +10196,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!95</x:v>
       </x:c>
       <x:c r="K72" s="48" t="str">
-        <x:v>823ca6d549e9b0c707184218a4884ee6f7872a0b72ab2584d3d1193ac889661b
+        <x:v>33e9ed73a3f6c747e692762d8b9f573bc1ece8e92b5e2d4fc3b163e099143833
 b96debd2f6c90354e63da57beb5831bc893ef2fe8a9ef1338bf197040ce2ebed</x:v>
       </x:c>
       <x:c r="L72" s="48" t="str">
@@ -10248,7 +10248,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!177</x:v>
       </x:c>
       <x:c r="K73" s="48" t="str">
-        <x:v>84878732c2158325a98f8914e7199c01d8b6f3cfa719554ec640f510f4bcf399
+        <x:v>31f8b30244274ea1b92029a3db4e71f56bc751e78040bee6719e29d9b6c87269
 5a6ed3ff832ffe11fcb6f6a676adbc4028dadce087bd59df02d469817c59c502
 a88f6ea5b6eb38dac954d8aa304c57970825b8f8bc184837b4a3f51d5c92a704</x:v>
       </x:c>
@@ -10300,7 +10300,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!109</x:v>
       </x:c>
       <x:c r="K74" s="48" t="str">
-        <x:v>d05e9ad71cb62ac7005fc1454284765e7188a0b31ac4adb9f3bd9f7de625b801
+        <x:v>d325825221cc592920f42f8f729e553471df73905681e7a7adf09f73ca9ed878
 103f3d87783939b0baa1a240d707b73a4f502d6c7e5b7a4a1d05d35e6032557a</x:v>
       </x:c>
       <x:c r="L74" s="48" t="str">
@@ -10352,7 +10352,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!116</x:v>
       </x:c>
       <x:c r="K75" s="48" t="str">
-        <x:v>c7c5bf507d8e41f98493a32f9fa409d766c85a62545fc4bd87395016e7c6b70e
+        <x:v>5dc7bee61e18f9800f58504fb66dd5232845f59008f6c842c422670ac6809333
 a3fdbac6ad21d9ed7034635f794a215a0d9499937924860f50ce7ae266c66008</x:v>
       </x:c>
       <x:c r="L75" s="48" t="str">
@@ -10408,7 +10408,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!654</x:v>
       </x:c>
       <x:c r="K76" s="48" t="str">
-        <x:v>0cbbca9571d4479ea00d4def0930f33607fe774ce6f5154b5d1246d6ce6ce2f0
+        <x:v>fcc05307f9ee30696783ffacf362eafeeb5e5b3d4a5315305675b7df2dd5c56d
 7e5fb724918b17ca3725051fbd9c0295cf672fe75c1d97e8c30c8b46df8dfc55</x:v>
       </x:c>
       <x:c r="L76" s="48" t="str">
@@ -10465,7 +10465,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!193</x:v>
       </x:c>
       <x:c r="K77" s="48" t="str">
-        <x:v>84b74e1c38d2eaf56a5aab53e0980e9d84fed0ab203745ee646fff7aaf0c23e3
+        <x:v>f5026e41cb1a3fe36df7e455ba21544eb61bcc667a293dd2bad952d43610d668
 cf9d28d34bc61fbf23cd7d388a18d982df243cbf888ff48ebbaef7dc1c087364
 3b0435cddd077f55c6ff8fd51efecf026f841287d6594bb384362db6d84aad16</x:v>
       </x:c>
@@ -10523,7 +10523,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!194</x:v>
       </x:c>
       <x:c r="K78" s="48" t="str">
-        <x:v>679137a6dd1dbfe617b5395d3fc3c0e5100db26b9261dcbc2964d6adf16aaeeb
+        <x:v>c526f5733c623e659f57e10e3f6377700e45f6d85da5655355b1302fe32f805f
 d867e451c4e3aad4e2c9cec4b15f972f1f2c0a2d64b91d8717944500f914f374
 450f7177700af840cac6531f6874331d6a879bf2e1cd70861c2c823704ea1534</x:v>
       </x:c>
@@ -10576,7 +10576,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!669</x:v>
       </x:c>
       <x:c r="K79" s="48" t="str">
-        <x:v>66f52a0e9eea5df4a5cc4e5aefdb8c3f78f04ddfa0fe6d56fe71e829c9a77f69
+        <x:v>3f5b7f4981d24e2fdfc7ea13402853af0e780ebc297ce11fada32293d74957a9
 c62b507ca44ae23b178b6dee971ff6e0a8c34cd3ff480b0b62187d7d9393212b</x:v>
       </x:c>
       <x:c r="L79" s="48" t="str">
@@ -10632,7 +10632,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!671</x:v>
       </x:c>
       <x:c r="K80" s="48" t="str">
-        <x:v>b978b4111efb041f0a6272971d443557d79b0817a436d195779c345dd015d651
+        <x:v>56548b8d22e8a5bc7e1aa91271618231934157613c8293a0c4e5be6b74ca541f
 73c4292b0b670c63064e19f4b8e0c8b029cf29910c4438116ef878683f905dae</x:v>
       </x:c>
       <x:c r="L80" s="48" t="str">
@@ -10688,7 +10688,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!673</x:v>
       </x:c>
       <x:c r="K81" s="48" t="str">
-        <x:v>99dcb7740497f0a18d769d9ba5fc793459fdd526a6ba8f04126939f0d1b4f380
+        <x:v>429add497d5f95f394b79117f333ec1f259ed4b72c7f72691e795ba1f3a8c691
 24fd7d31306750ccba043b18fe9c8f60523e5246ee4fb31b744b1413ef81d26c</x:v>
       </x:c>
       <x:c r="L81" s="48" t="str">
@@ -10744,7 +10744,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!676</x:v>
       </x:c>
       <x:c r="K82" s="48" t="str">
-        <x:v>84541e284a54a3f68ebaef81d279971b2f262df4a53c110a5aee39952b3075d3
+        <x:v>2fb6fd9f37cffb4ef4613935d753e6714e22124d11a329fc20ce88149a8ec8fc
 368bb13fb490aa824d76054f2495eefc059a67927e26ce94eef551955ae46f33</x:v>
       </x:c>
       <x:c r="L82" s="48" t="str">
@@ -10796,7 +10796,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!684</x:v>
       </x:c>
       <x:c r="K83" s="48" t="str">
-        <x:v>8a72f403cde754a9d771d7fa845d886305eb5e87d319caba0778ec1390000f6b
+        <x:v>031413ca105dbf56e96f96d45600afc4cfdd324c93085386b55578012ac05ae3
 a38fccfa21bc91e88f8c85eecc690812cb98c1f36dd274ddc3e3f0995265b2a3</x:v>
       </x:c>
       <x:c r="L83" s="48" t="str">
@@ -10852,7 +10852,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!200</x:v>
       </x:c>
       <x:c r="K84" s="48" t="str">
-        <x:v>f680e56d59eb99a38f7876a79652b7c786dd6ce7a7d8d8ebc17cc3cdb094b1e5
+        <x:v>8ed3c837cb244c624322d298650dc288bbbf14f6b2873049b0371556d5768107
 bf9303bb03e278d3e0fb235c8cd4a9dedfb1e7a4880c5d9f6f95355e48818e25
 45e592772b02bb544d31edd4197e85b74afef70793cf64d4f8a0482181b162a3</x:v>
       </x:c>
@@ -10909,7 +10909,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!705</x:v>
       </x:c>
       <x:c r="K85" s="48" t="str">
-        <x:v>2234e4f00d332cc3ea366f23b0e8c1305155161d3e471ffcdfc090c6523659ae
+        <x:v>a76e69808daac28276a1b1f7e7da78de93f5cba76de11ccb23ea883aefceb9e4
 51e474631540a435c287607a99ec26dbfab40e3c6d6ef5365a577a9a5cab4a92</x:v>
       </x:c>
       <x:c r="L85" s="48" t="str">
@@ -10964,7 +10964,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!719</x:v>
       </x:c>
       <x:c r="K86" s="48" t="str">
-        <x:v>fb7f855d3acc0efeeef9812657f11a9cd037276ee115ad8e28a8eb61baf43f6d
+        <x:v>8ed232d60b74485b0eec48b1f5d0b40c9eb956b296833e260cf88740db59959d
 ee211e5057deb529b7154fcf93a1bffadcae23ebd35ddb729eb76695eee4f753</x:v>
       </x:c>
       <x:c r="L86" s="48" t="str">
@@ -11016,7 +11016,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!733</x:v>
       </x:c>
       <x:c r="K87" s="48" t="str">
-        <x:v>13dba6d688a586c891b4fec795602ac3708328f7f12a28f4cc2c380c842afd03
+        <x:v>fbf5c17a4c1118a3f0576fe0ca76b4a84355c7ed3c34e5588416222de187c5fb
 6293712b2312e3ff52aa703d0e222ab22b75319fb79fbe592082adfb65b80ec9</x:v>
       </x:c>
       <x:c r="L87" s="48" t="str">
@@ -11068,7 +11068,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!216</x:v>
       </x:c>
       <x:c r="K88" s="48" t="str">
-        <x:v>9c16fafa7441d9fb654d1753d4d224c02ca88182b4f904e496696b34ada5bee0
+        <x:v>08270588c1c7db6f4fb66a0b2b30e989560fe665b16404d0a8a82d450fdfad1c
 6680d4966ab688befdb6aad74e208624a28bf1c8a6b6d5dd0d9b2b47a9287572
 4af33623a95a0ef2e145d311bb273368101fb28c403726088677af9274a0d2dc</x:v>
       </x:c>
@@ -11125,7 +11125,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!911</x:v>
       </x:c>
       <x:c r="K89" s="48" t="str">
-        <x:v>322266933455907d24063cd287620b9f45f006c2311c09aa012db0818b3ed1cc
+        <x:v>7045c70bca7deef91348d9a5217c6460379ba04f9a31164991d925ef03fd9e00
 447e068caf4b7ff17812902ea09095706df1053ccd80bd3161a07947288149eb</x:v>
       </x:c>
       <x:c r="L89" s="48" t="str">
@@ -11177,7 +11177,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!218</x:v>
       </x:c>
       <x:c r="K90" s="48" t="str">
-        <x:v>30fe088adad6e601a42100c23c007a337f5a4b6fdd62aba7ae0b1cb57bfbc591
+        <x:v>4ae1db63e0e76d0b74c60329921b72d49be0f0e0f4a9ccbc0b3c323eb906bc62
 9aef8201daf3e48d54a2b32bb5e3c279c92274f8e043db16a4c6ba7538484a45
 d7bc674bbc05b97ef2e6f8c0dec2eac0f69b35b585de1e8918c11eda772ef36b</x:v>
       </x:c>
@@ -11230,7 +11230,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!939</x:v>
       </x:c>
       <x:c r="K91" s="48" t="str">
-        <x:v>48d1a473c02c7e9deab09aa371b520554dc7dd8bcff5c85f43627ac303f82615
+        <x:v>559cbc380624bbba16848fe0ef163a91aad00c2b5d3e2185ed43c19fc268dded
 7ec94173da203fcdf642afae7e52c14607377a5f663e24fcde4905b5d67d6630</x:v>
       </x:c>
       <x:c r="L91" s="48" t="str">
@@ -11281,7 +11281,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!941</x:v>
       </x:c>
       <x:c r="K92" s="48" t="str">
-        <x:v>19232b34a4986f3653c7c07c58615a12a9532abc809ddfc93d0e34f3ab91ba43
+        <x:v>0d05197b09e358226504bc2daed90b7024f6fca37ccdf3087e747c7a1301ff2a
 547e4e741404de72f02abf1ed487b8f14767894f7737ef5dc26c2a5469a9b41b</x:v>
       </x:c>
       <x:c r="L92" s="48" t="str">
@@ -11332,7 +11332,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!943</x:v>
       </x:c>
       <x:c r="K93" s="48" t="str">
-        <x:v>04cde10745561cfd9ba26e384e75a47068c47544fd77506cb9d3653c36a23359
+        <x:v>d63dbd64a642e9a238c01907ada8d1a563edf63e8d4c5f88c160df9a4eba9046
 5b27aac9d232c1ed3c36be39c159f65241fc3f2892c1a828c1eb96f4dc2f68f1</x:v>
       </x:c>
       <x:c r="L93" s="48" t="str">
@@ -11383,7 +11383,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!945</x:v>
       </x:c>
       <x:c r="K94" s="48" t="str">
-        <x:v>e7013a98473a7a1ad1a548189a14e74d2bd6a65384842f69d7a09d95df7b4def
+        <x:v>c7a826b1d8270dee52a0721490b54e3ab60d58b89e39efa531f835f56028e42c
 3099753af1a94c4ac7e31c0d83e9b8c466707439a39d6e75875b6b9563fec488</x:v>
       </x:c>
       <x:c r="L94" s="48" t="str">
@@ -11439,7 +11439,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!947</x:v>
       </x:c>
       <x:c r="K95" s="48" t="str">
-        <x:v>aa152106f1e5b14fa091b7a0e33bc22b17ab6cb59f039b22010a0fbc1b636406
+        <x:v>81aed1eb666f48f2bb97789150cf3690245a8459a40901a458b68731a196f8eb
 a2d3ac8ff4c43961ef8985b236f50e5251c858f480b2d91596f0dd23933a6074</x:v>
       </x:c>
       <x:c r="L95" s="48" t="str">
@@ -11491,7 +11491,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!224</x:v>
       </x:c>
       <x:c r="K96" s="48" t="str">
-        <x:v>46ca873689700027117c082b950a61dfe5b123c77ff9559cbed7bc3551d5a867
+        <x:v>fe52599a065bf01c4a95cddac335a5621abd25c57b39950b0989fc27a87c1ad9
 798329d1aff3565ba920574245dcc0b3606582570d56b11345fa5b61cda78e8e
 99fbe75073bb695e32490ef58811a584de4c79a1c450a64700682f803615b074</x:v>
       </x:c>
@@ -11548,7 +11548,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!951</x:v>
       </x:c>
       <x:c r="K97" s="48" t="str">
-        <x:v>106d6b6f9c2421cb4ec3abf85792aae78ffc81fe058c73e3a160651639e52715
+        <x:v>ff23dce0d0048121bfd4799fce4a5bf3278e6685486b254d14402d5392081a1a
 7cc3fa6004b46427a26906c749a0ca0bd2125f28957eb5992c9cd116e286354c</x:v>
       </x:c>
       <x:c r="L97" s="48" t="str">
@@ -11604,7 +11604,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!953</x:v>
       </x:c>
       <x:c r="K98" s="48" t="str">
-        <x:v>d080be5f08b03a50156c015caca2d4a6e44c008dde341fe56edfa2714f0069d2
+        <x:v>882a51f49dbbcff11f530c3247b835bfcceb590fd7ea5de7b692a88d7a65ef65
 0b25fb329bb37dcb8844ef406f5c268075a7608a5de3a8a5a8ec47f5a53677b6</x:v>
       </x:c>
       <x:c r="L98" s="48" t="str">
@@ -11656,7 +11656,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!955</x:v>
       </x:c>
       <x:c r="K99" s="48" t="str">
-        <x:v>0b8b39acd10c828da4b79acf593a3adf919bc5b216c984ff348732059d2b2f9b
+        <x:v>154bd4fa3a89340dc8fcc0136ea77b278941231819746164a9b6093b749438d6
 d054b96cdd579838dae8808b49239a9351cd60833842a62e7af2b2bbb5508488</x:v>
       </x:c>
       <x:c r="L99" s="48" t="str">
@@ -11708,7 +11708,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!240</x:v>
       </x:c>
       <x:c r="K100" s="48" t="str">
-        <x:v>52d1a82bd9416e4324421def493c5a99cf88024b7552dece808502825cdc8c5b
+        <x:v>9f8b0b9c062632bfd559733c6daaab9b8e7e33c1319fe0dca2f9dc3a6e19a798
 736ef7deaaa6397e51ba3da95802e890431f793eea2df4566edf1333837fee55
 0aef56387e1e46a5d1156fd5dee71cb6962a3af58c458f91bb55f744a0e4f9b3</x:v>
       </x:c>
@@ -11766,7 +11766,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!241</x:v>
       </x:c>
       <x:c r="K101" s="48" t="str">
-        <x:v>8a3d22ff23a817382aa3fe46940d945910b50b010d63cc046509d142836f2f6a
+        <x:v>f1edb79238ac681ab9bcac5978ed39224011271b5f758e43ca59acf5263b5d2f
 8e1d1862f7db429b2e86969ed690df77f44b2920e338d42cb7f200bc570174d2
 a2347094d9321f6a196c01f6200e7986f65a2e463e2966c3a8ec4e785f785ac0</x:v>
       </x:c>
@@ -11824,7 +11824,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!242</x:v>
       </x:c>
       <x:c r="K102" s="48" t="str">
-        <x:v>094ebaa3361df2417cc88a80fafe21ebde98fb1b9033780d70b4c68a19b5f4a4
+        <x:v>ddb5434ca55e692841e0c63340215b6fc926ae4bfb7e67190a52ebf5764c4344
 e2e37cf7930ac87e8c00053a2657030d6333382f457d64e34feb684481aa50e1
 c0f8836c5c1a1172338e5acdf3cd097f45693271d06149b0a26c139d31098dfe</x:v>
       </x:c>
@@ -11881,7 +11881,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!537</x:v>
       </x:c>
       <x:c r="K103" s="48" t="str">
-        <x:v>338681432c422198625999859e6f7b56efac4d6c217ada4d5236f32ea9ddb79c
+        <x:v>3f5ceb27e54c58374f675398df59a8b2842747367668fba57287805dea28cfc9
 070f3cfc10da7ac3099e6eca89f82f3855914fd86896986d6d030dbe0ffc73f9</x:v>
       </x:c>
       <x:c r="L103" s="48" t="str">
@@ -11933,7 +11933,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!244</x:v>
       </x:c>
       <x:c r="K104" s="48" t="str">
-        <x:v>cc2d65484c7c13fdcdad59a3e74a785565619810f7b67f6dad351bb0d580683f
+        <x:v>21f7913cc18ddba9ee681ae7008bbd63f87007eaf69e655627d2b070c000279c
 59ba9db8b4a193860544c7a69a33999fd1f1c52c4919e1c60d3b286049f66023
 7f262b198bc95210d99058dd00039dca0a5d017fb59010569429bae2a6b802e1</x:v>
       </x:c>
@@ -11990,7 +11990,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!541</x:v>
       </x:c>
       <x:c r="K105" s="48" t="str">
-        <x:v>9c3b08ebc5c347e74e9a1281077c1355d153a395256763f6dc3e4f02508f62b3
+        <x:v>5af7c2f54821ad28ea15505a08e189fd688ce9bb9ba65631ad3b56ea3e082006
 d7bd95bf8533bc3079c5d81ae46eac40d254d5b2d6b578b42ea990f7a9294e39</x:v>
       </x:c>
       <x:c r="L105" s="48" t="str">
@@ -12045,7 +12045,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!543</x:v>
       </x:c>
       <x:c r="K106" s="48" t="str">
-        <x:v>fe4c8f516b973f81cfb65ab71f4279110a553a4f058cd349a3864b159ead719d
+        <x:v>328ee59ee5962f32312b6138284aa7c1612c8fd1a5b846e78f884ad509da1f3f
 ac71ce5dc69cda4540b6e94a12649ad377ea80775509fb3977b920ae326dd228</x:v>
       </x:c>
       <x:c r="L106" s="48" t="str">
@@ -12102,7 +12102,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!247</x:v>
       </x:c>
       <x:c r="K107" s="48" t="str">
-        <x:v>defbc7e710a5910b29a807f7e2014fbdfbe1f541e95dfa17f2834e3963293cfd
+        <x:v>e6225aeab2b352522ed4cf16182838636d019b3657d2b1d804b5e1612df3565b
 de3787a6c1595d6d5a6bf20872d2afc13ee9c0b383ed232b5206e0caa6be0ad1
 784d57f41ce8fb7f246e05203c322f24ab8f3dd71aa0211b950b1b35919d8c05</x:v>
       </x:c>
@@ -12158,7 +12158,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!547</x:v>
       </x:c>
       <x:c r="K108" s="48" t="str">
-        <x:v>6e46c62a0dccb569962c321e37821e54d1120cd922a89c1b49e3734486b4903d
+        <x:v>11429cc6fb958b4824ccd2d6d9a030c88128ad208922972ef2666f30b1b8d01a
 f32d1712124abc70f2b60d2ed0e2af485b346fe87854056a5a8fda31790ea7d9</x:v>
       </x:c>
       <x:c r="L108" s="48" t="str">
@@ -12214,7 +12214,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!549</x:v>
       </x:c>
       <x:c r="K109" s="48" t="str">
-        <x:v>a994b86ab7b43db2d36a15ece5dbf31569b3d485b1d2bbe11e37ee9db7bd5c89
+        <x:v>48310983a8ff62115128ced56353bacafb1e9dccc014788f17a8b878ef804160
 f0b963c36f04d533c99c313b29b5f145acda559523d2441dce5c7c90f77ecc26</x:v>
       </x:c>
       <x:c r="L109" s="48" t="str">
@@ -12266,7 +12266,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!551</x:v>
       </x:c>
       <x:c r="K110" s="48" t="str">
-        <x:v>13e248904965490eff67d7ada868f89854540374351cebdb3e9e2d3ddc512ef4
+        <x:v>20adac8936c3e0b52b4bdbfa13d30fc1f9c72de71a476f52f8277f3bf3935fb8
 c3a13cfc33422f94d250ceaca0e369283789df6172873964320491d28614bc2a</x:v>
       </x:c>
       <x:c r="L110" s="48" t="str">
@@ -12318,7 +12318,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!555</x:v>
       </x:c>
       <x:c r="K111" s="48" t="str">
-        <x:v>f600e536b24d68844e28d3688050fa0ed7c8e6106056440246da1af10ba28c3f
+        <x:v>78d7291041e0cd85e0cb3cbf6cbbeecb84e19f2d8ba2460b4225d923894707d2
 75b9e5741dfa3c949f4369f2ad8ca26fcf3604ac43625993390dff737112f609</x:v>
       </x:c>
       <x:c r="L111" s="48" t="str">
@@ -12374,7 +12374,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!599</x:v>
       </x:c>
       <x:c r="K112" s="48" t="str">
-        <x:v>4942cf6d921dc4e5d87b00708201e9ad20cc311c097a73ea29f0f43a0ef59934
+        <x:v>8099fe3729d15eec6cf37d5d67cabd502576a25660075c8fa4ef6461d3e4d635
 38151f49bf83f9963c6fd871a5a68b9804aed3ae6d498a67b2e215b076ec98c2</x:v>
       </x:c>
       <x:c r="L112" s="48" t="str">
@@ -12431,7 +12431,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!145</x:v>
       </x:c>
       <x:c r="K113" s="48" t="str">
-        <x:v>9740afd6b3304ff35c1106af36ff10639b89699afce23b7a01a23ea411153373
+        <x:v>a977b10b568f0d68b9f6f8cd36ac055c67c2ecc2908d2f620567632a6ce7e4e8
 210776fa92bc87f5045ba0d2f237581eb42335ea7a8ea06b3f0b9b065eb07e0a
 64165ec2596f36b2fa3cd46763ada25d4681c982b53f9581d11fc5de839aaeae</x:v>
       </x:c>
@@ -12488,7 +12488,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!603</x:v>
       </x:c>
       <x:c r="K114" s="48" t="str">
-        <x:v>dff07c5f573df4531b38378decb6cbeba250b97f8b95ea616e21e766ea237e8e
+        <x:v>1eadc6b5592a5e9f0ad37fb2bf7e52f415c29c998071a28621bfd94a68c4354c
 a9518abaec842c1f0de30f34c0888d93c846bc5de4c7bf2e266eb0d737cfbe6e</x:v>
       </x:c>
       <x:c r="L114" s="48" t="str">
@@ -12544,7 +12544,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!605</x:v>
       </x:c>
       <x:c r="K115" s="48" t="str">
-        <x:v>fdf95450b69e9bc8a0201e6f29fffe11c4d259bfb3e5798096fca010ca84c3f1
+        <x:v>83c5b097d0c10a16e565b01a61c703dcf2168fdab1f6f1c8dbd344676cb40f06
 20f1ef6fbf6b19bc2fd56e2b91c2f2347a4cb63c433fc84493349182ee15d0df</x:v>
       </x:c>
       <x:c r="L115" s="48" t="str">
@@ -12600,7 +12600,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!607</x:v>
       </x:c>
       <x:c r="K116" s="48" t="str">
-        <x:v>8ad2e3746b981472724799d6bdfa425e0f8d405b78b27ff07a1a0581ada24976
+        <x:v>4f3136156448c72b65ee36f5d1ccd9f94f07b0d66ef55427f7cbb54486f65f3b
 9adcd6ba13260b466db67a799b750d360f8a09ad42313c7df9a052c893263b27</x:v>
       </x:c>
       <x:c r="L116" s="48" t="str">
@@ -12653,7 +12653,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!149</x:v>
       </x:c>
       <x:c r="K117" s="48" t="str">
-        <x:v>c3bb4187f0af3a761a3c50a4d055f02e750db60b4bf5546d3d5fe658f378ee32
+        <x:v>1e16dcbc80e5697681fb3e015e9f36d93ac07f4019a0bbeb30f8df15b87475c8
 1af907bb8637e571e5c7d23856ad894851cf1090a3bc594c2ea2905d6eced2ed
 11f49398eb8446f1e6eae222e74818ae7f4dd226457e28a06676dcc05947354c</x:v>
       </x:c>
@@ -12710,7 +12710,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!611</x:v>
       </x:c>
       <x:c r="K118" s="48" t="str">
-        <x:v>059758551d4c21bc42094b33fea532380314c65ab0a6b1f2f912357ea49c9853
+        <x:v>b1b121bf131e0ec51f869e96ecca536edcffb061a3c854b0f9477d294b23fa41
 5a504ba7155cd45d03b0d4627458bb9d8198536da8024a5e248ccc99f96770fd</x:v>
       </x:c>
       <x:c r="L118" s="48" t="str">
@@ -12767,7 +12767,7 @@
 tldr-astro-phrasebank/TLDR-LL-KNOWLEDGE-MATRIX-V13-DIRECT-LANGUAGE-OWNER-APPROVED.xlsx#PlacementMeanings!151</x:v>
       </x:c>
       <x:c r="K119" s="48" t="str">
-        <x:v>e2b37463fd16dd8ca5da635b685980e764d4ccaaa38a59591537cb1804b78652
+        <x:v>acc51a9b9217881690d7106664693aeb17e5af366d6d5b97e078ec66db369620
 72b6e0bd25f8dc3a7806170a2ebf0beeb7d6a7446e654b938ad6514a6e7e2db4
 b3f845992e2a982a389e5d0292dc27dbc0635a259e98d115d8ae7540a4badaf0</x:v>
       </x:c>
@@ -12824,7 +12824,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!615</x:v>
       </x:c>
       <x:c r="K120" s="48" t="str">
-        <x:v>70e6b984495ffcfa380529cc12c41759ad86cf1fd12b9492b2782aa9a06d9675
+        <x:v>9994937af9d3db7b9a59cc927f27e76733f0465870dddabd8f90d9593428d2e8
 1ca242e50bf0e6785b30a34640ffca4cca814829c2ee54ed18b28db52ebf0e9a</x:v>
       </x:c>
       <x:c r="L120" s="48" t="str">
@@ -12880,7 +12880,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!617</x:v>
       </x:c>
       <x:c r="K121" s="48" t="str">
-        <x:v>67c9f93bc880c7e2e83c58a20d2d018c6c9b23fcd2047096ac1fd16aebb893f4
+        <x:v>1d8727c0ef52bd62cef50deaba7859538e590a04109bdffdfd569ef2ec035c84
 561ab8da2a85c422ac3be616352c3b5b5b514c39865886c11c6cf6fc94b141a3</x:v>
       </x:c>
       <x:c r="L121" s="48" t="str">
@@ -12932,7 +12932,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!635</x:v>
       </x:c>
       <x:c r="K122" s="48" t="str">
-        <x:v>4119ee519613e573061d2c66eb0349d8cd67390a01c0f9937ca193956a21b413
+        <x:v>13cb43dabab4c4ce944c302d0d6bec4e00853f42f6c22c99952f9d046233247c
 f65d42ab4532aa04b93bc1f5daf9d8f45f678de1d2f3096212e3c8eb3a3e7f30</x:v>
       </x:c>
       <x:c r="L122" s="48" t="str">
@@ -12988,7 +12988,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!647</x:v>
       </x:c>
       <x:c r="K123" s="48" t="str">
-        <x:v>53af71952c53f93907409379e17b80db93f3a6f82c6f23e88fb8a9f260d5006a
+        <x:v>fbfbee839d50061b5bf105e5676f3d5bd0821554aad111e0e99c88a57af57efd
 c37156cad7ff9a237bf0785b39b83107bd40d8f64297ac16e61bcefa3fab773d</x:v>
       </x:c>
       <x:c r="L123" s="48" t="str">
@@ -13044,7 +13044,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!4</x:v>
       </x:c>
       <x:c r="K124" s="48" t="str">
-        <x:v>9452114e243543efef2d1054d379d575d4478b4adaf7fee23b61c0703ab2b1e5
+        <x:v>665d19fb89ed1dfc711a6af7074a45747882286ca77b00351904eac8af3973a6
 b2cabb3951c0a2b65c79395a2f0e42f03e2f17d6fc7126ada780b5ccb20569cc</x:v>
       </x:c>
       <x:c r="L124" s="48" t="str">
@@ -13096,7 +13096,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!10</x:v>
       </x:c>
       <x:c r="K125" s="48" t="str">
-        <x:v>886ade5ac1be70e949b9b143fee510144367948b379fc2d666514f5c47eebc20
+        <x:v>bdac47354dc9d32683d9b8d7e9374dabedc65c87a2b2c8d01ed86c0dd14b905a
 dba3adff229b8043a48f7604a778f8fc29393b5dc7910bb21fe50f4cebc684d8</x:v>
       </x:c>
       <x:c r="L125" s="48" t="str">
@@ -13148,7 +13148,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!15</x:v>
       </x:c>
       <x:c r="K126" s="48" t="str">
-        <x:v>3ba7919f6a2d6f38ef96dfcbf8a6f0a118ab8d88d7571008d3002078456f716d
+        <x:v>b8d8a42e196812146d75d888099f473ec4c329d4779dde0ff5f8696a3ca4cd92
 78edaff067639521b44181d003467ca5cccaa5b8d381f08a95e8bbca9011e4c1</x:v>
       </x:c>
       <x:c r="L126" s="48" t="str">
@@ -13195,7 +13195,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!17</x:v>
       </x:c>
       <x:c r="K127" s="48" t="str">
-        <x:v>10f31581a59e13ccaeabf3c4246ff3991128a8e76e9bfa950dfde8c80a1bf108
+        <x:v>ebe46b2a6497d90a6ea3a4898674b099a201f7a7039c235f6475c8d0532d8cb7
 a3edc1497398fa1623f21973a0ebf6e9e9021fdf2f170f3ffa6789aaf6ed0e49</x:v>
       </x:c>
       <x:c r="L127" s="48" t="str">
@@ -13247,7 +13247,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!19</x:v>
       </x:c>
       <x:c r="K128" s="48" t="str">
-        <x:v>f400f333a592c4b9fa3babaf903f198028df36ed8521f100214f8dfdee1056d7
+        <x:v>c0c29f3f3de460f69dfb291ef91de9eb7f3e6330beb7c43cd199946d13883b2d
 009b737f732c579020195c6b992dac19f826715af6227895d676973202a80207</x:v>
       </x:c>
       <x:c r="L128" s="48" t="str">
@@ -13298,7 +13298,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!21</x:v>
       </x:c>
       <x:c r="K129" s="48" t="str">
-        <x:v>acd1b6bc3000385facef278464b3c82e242f54e0a6fbf57f2971817a94c8468f
+        <x:v>c86812319493dd6972e5595725997e2e4517e54ce329ddcebef76eca640ec44a
 e24b7e1d96a7ba688793694b4d58a2383c697e652d2e0edc984be800e00b32be</x:v>
       </x:c>
       <x:c r="L129" s="48" t="str">
@@ -13350,7 +13350,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!23</x:v>
       </x:c>
       <x:c r="K130" s="48" t="str">
-        <x:v>895e4bcaf9fcb47fcb0b56c90fc2eccfb8537a1d0728812ef5b693604e4880b2
+        <x:v>35874f6916cb8cda37a9ac1d93620ee12cd5fe69e9a50e1810933512801fc04d
 95c29facac24c9ec132ba8092cb83bf1a2b20941e1c37193c39a208f1eaedce7</x:v>
       </x:c>
       <x:c r="L130" s="48" t="str">
@@ -13402,7 +13402,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!25</x:v>
       </x:c>
       <x:c r="K131" s="48" t="str">
-        <x:v>25e28e9fd4bed6227f283498363a9addb5f0b9511773b581e8006116359550e6
+        <x:v>05131fbd09dbd56cd8f92d5b5bac7f19b68bd88ae066710ed6e8850c7d140ce9
 f82bbd6e0681e6c94ba555224695abe258d9faa2ffb78329d2f0750fbbf6cbb5</x:v>
       </x:c>
       <x:c r="L131" s="48" t="str">
@@ -13454,7 +13454,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!27</x:v>
       </x:c>
       <x:c r="K132" s="48" t="str">
-        <x:v>91c7fb716f1539c253df4ab0f5a4ee656e7b5a4b6baa138f0010f7173aa64f2c
+        <x:v>ec3fd6d004301d67a6c027ffc380bb087ced6ea9aa2c30c6e3e65866df88fe94
 96edddc9530f9f16866239920c92e516223b6d6ba683b90afef8667d6709addb</x:v>
       </x:c>
       <x:c r="L132" s="48" t="str">
@@ -13506,7 +13506,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!29</x:v>
       </x:c>
       <x:c r="K133" s="48" t="str">
-        <x:v>f15c68d6266ed25e740b7b2e70e1181cec598927d651c833a7f3ba36d06e1a6d
+        <x:v>0e710ad8ba4713a417c4f5d8f1e56e4f4ed42bf32522b7dd28d9d135794edc59
 e9a1fde6aaf473bf5e407f5ef9ade3769bcea4d9ebdb56134d53195f50a91b68</x:v>
       </x:c>
       <x:c r="L133" s="48" t="str">
@@ -13558,7 +13558,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!31</x:v>
       </x:c>
       <x:c r="K134" s="48" t="str">
-        <x:v>46b6aa5df58cdf932a787d7ab5192354bfe0128d9287e755b4cad0ab72c33d1c
+        <x:v>c4562228f9486b4bc73671d53ee20968c6d25de8cf8423a28a27d2c79425296b
 e90ad5413bd8cfc6a1adf1ad804faa1d46479f77ed63fc1959307297736d0325</x:v>
       </x:c>
       <x:c r="L134" s="48" t="str">
@@ -13610,7 +13610,7 @@
 tldr-astro-phrasebank/TLDR-CC-KNOWLEDGE-MATRIX-VOICED-AC-V9-OWNER-APPROVED-GOVERNANCE-LABELED.xlsx#TransitMeanings!33</x:v>
       </x:c>
       <x:c r="K135" s="48" t="str">
-        <x:v>3a48920d2af12e327e680b314e976b4dc914715b87d7ac3d073dd97933023802
+        <x:v>b2a1e864424d7350f4bf6a03f3b26e8fe4ac6f2cef8c0bf44e7be21fa0bbcb5e
 8978b0b7d8ad7dd7076fc2927c2ad508edc7887e3668de982bd0207149dfa945</x:v>
       </x:c>
       <x:c r="L135" s="48" t="str">
@@ -14221,7 +14221,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1494514efce413b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00aad3a53dd41f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16848,7 +16848,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R250b04bfb8694e80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb656d745c64797"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17445,8 +17445,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53a1a2a1caec404d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb44d54fab54d80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41413845db0844b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a06fd88a6f4168"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18152,7 +18152,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6fb217d02844f58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec1f85bde9ec40b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18459,7 +18459,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra48a402e180049d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8903480aeae45da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18916,7 +18916,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7468888cc9574332"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaebbd52a9354a34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>